<commit_message>
Atualização automática: 2026-07-06 13:17
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -1795,7 +1795,11 @@
       <c r="L13" s="1" t="n">
         <v>46213</v>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -1828,7 +1832,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr"/>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 12:40</t>
+        </is>
+      </c>
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr"/>
       <c r="Y13" t="inlineStr"/>
@@ -83553,8 +83561,16 @@
       <c r="AA789" t="inlineStr"/>
       <c r="AB789" t="inlineStr"/>
       <c r="AC789" t="inlineStr"/>
-      <c r="AD789" t="inlineStr"/>
-      <c r="AE789" t="inlineStr"/>
+      <c r="AD789" t="inlineStr">
+        <is>
+          <t>Atraso da operação, as coordenadoras Erika Santana e Isabella Nascimento informaram que os fechamentos serão concluídos até o final desta semana. - Data Comentário: 06/07/2026 12:41</t>
+        </is>
+      </c>
+      <c r="AE789" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
       <c r="AF789" t="inlineStr">
         <is>
           <t>Tarefa</t>
@@ -83662,12 +83678,12 @@
       <c r="AC790" t="inlineStr"/>
       <c r="AD790" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 25/06/2026. - Data Comentário: 24/06/2026 12:06</t>
+          <t>Atraso da operação, as coordenadoras Erika Santana e Isabella Nascimento informaram que os fechamentos serão concluídos até o final desta semana. - Data Comentário: 06/07/2026 12:41</t>
         </is>
       </c>
       <c r="AE790" t="inlineStr">
         <is>
-          <t>25/06/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="AF790" t="inlineStr">
@@ -83777,12 +83793,12 @@
       <c r="AC791" t="inlineStr"/>
       <c r="AD791" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 03/07/2026. - Data Comentário: 02/07/2026 07:32</t>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 06/07/2026. - Data Comentário: 06/07/2026 12:41</t>
         </is>
       </c>
       <c r="AE791" t="inlineStr">
         <is>
-          <t>03/07/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="AF791" t="inlineStr">
@@ -83892,12 +83908,12 @@
       <c r="AC792" t="inlineStr"/>
       <c r="AD792" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 30/06/2026. - Data Comentário: 29/06/2026 09:26</t>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 06/07/2026. - Data Comentário: 06/07/2026 12:41</t>
         </is>
       </c>
       <c r="AE792" t="inlineStr">
         <is>
-          <t>30/06/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="AF792" t="inlineStr">
@@ -84007,12 +84023,12 @@
       <c r="AC793" t="inlineStr"/>
       <c r="AD793" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 30/06/2026. - Data Comentário: 29/06/2026 09:23</t>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 06/07/2026. - Data Comentário: 06/07/2026 12:41</t>
         </is>
       </c>
       <c r="AE793" t="inlineStr">
         <is>
-          <t>30/06/2026</t>
+          <t>06/07/2026</t>
         </is>
       </c>
       <c r="AF793" t="inlineStr">
@@ -84119,12 +84135,12 @@
       <c r="AC794" t="inlineStr"/>
       <c r="AD794" t="inlineStr">
         <is>
-          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09 - Data Comentário: 25/06/2026 18:15</t>
+          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09 - Data Comentário: 06/07/2026 12:41</t>
         </is>
       </c>
       <c r="AE794" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="AF794" t="inlineStr">
@@ -84227,12 +84243,12 @@
       <c r="AC795" t="inlineStr"/>
       <c r="AD795" t="inlineStr">
         <is>
-          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09 - Data Comentário: 25/06/2026 18:15</t>
+          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09 - Data Comentário: 06/07/2026 12:41</t>
         </is>
       </c>
       <c r="AE795" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="AF795" t="inlineStr">
@@ -84333,8 +84349,16 @@
       <c r="AA796" t="inlineStr"/>
       <c r="AB796" t="inlineStr"/>
       <c r="AC796" t="inlineStr"/>
-      <c r="AD796" t="inlineStr"/>
-      <c r="AE796" t="inlineStr"/>
+      <c r="AD796" t="inlineStr">
+        <is>
+          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09 - Data Comentário: 06/07/2026 12:41</t>
+        </is>
+      </c>
+      <c r="AE796" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
       <c r="AF796" t="inlineStr">
         <is>
           <t>Tarefa</t>
@@ -84443,12 +84467,12 @@
       <c r="AC797" t="inlineStr"/>
       <c r="AD797" t="inlineStr">
         <is>
-          <t>Operação e GC validando as informações errôneas no sistema de análise - Data Comentário: 24/06/2026 14:39</t>
+          <t>A operação e o GC estão ajustando os créditos de meses anteriores para que o valor desse mês seja ajustado. A Gerente Priscila Volpe está em contato direto com o GC e informou que a tarefa deve ser concluída até o fim desta semana. - Data Comentário: 06/07/2026 12:41</t>
         </is>
       </c>
       <c r="AE797" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="AF797" t="inlineStr">
@@ -84554,12 +84578,12 @@
       <c r="AC798" t="inlineStr"/>
       <c r="AD798" t="inlineStr">
         <is>
-          <t>Atraso por parte do cliente, GC e GM acionado - CA03 - Data Comentário: 25/06/2026 18:14</t>
+          <t>Atraso do cliente, o atraso do cliente já é recorrente e de ciência do Master e do Gerente de Contas. - Data Comentário: 06/07/2026 12:41</t>
         </is>
       </c>
       <c r="AE798" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="AF798" t="inlineStr">
@@ -84669,12 +84693,12 @@
       <c r="AC799" t="inlineStr"/>
       <c r="AD799" t="inlineStr">
         <is>
-          <t>Atraso por parte do cliente, GC e GM acionados - Data Comentário: 25/06/2026 18:14</t>
+          <t>Atraso do cliente, o atraso do cliente já é recorrente e de ciência do Master e do Gerente de Contas. - Data Comentário: 06/07/2026 12:41</t>
         </is>
       </c>
       <c r="AE799" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>10/07/2026</t>
         </is>
       </c>
       <c r="AF799" t="inlineStr">
@@ -84778,8 +84802,16 @@
       <c r="AA800" t="inlineStr"/>
       <c r="AB800" t="inlineStr"/>
       <c r="AC800" t="inlineStr"/>
-      <c r="AD800" t="inlineStr"/>
-      <c r="AE800" t="inlineStr"/>
+      <c r="AD800" t="inlineStr">
+        <is>
+          <t>Claudineia cobrada a respeito das aplicações, ela informou que o atraso se deu ao fato de estar concluindo a distribuição da carteira de clientes do seu departamento, mas a tarefa será executada ainda hoje. - Data Comentário: 06/07/2026 12:41</t>
+        </is>
+      </c>
+      <c r="AE800" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
       <c r="AF800" t="inlineStr">
         <is>
           <t>Tarefa</t>
@@ -84888,12 +84920,12 @@
       <c r="AC801" t="inlineStr"/>
       <c r="AD801" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 01/07/2026. - Data Comentário: 30/06/2026 08:45</t>
+          <t>Os GC's estão respondendo as importações do Contábil conforme vão sendo realizadas, o GD Sérgio informou que a previsão é concluir na próxima semana - Data Comentário: 06/07/2026 12:42</t>
         </is>
       </c>
       <c r="AE801" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>13/07/2026</t>
         </is>
       </c>
       <c r="AF801" t="inlineStr">
@@ -85004,12 +85036,12 @@
       <c r="AC802" t="inlineStr"/>
       <c r="AD802" t="inlineStr">
         <is>
-          <t>Tarefa reaberta e já passadas para o GO Sérgio que disse que as mesmas serão conclupidas até o fim da semana - Data Comentário: 22/06/2026 17:05</t>
+          <t>Os GC's estão respondendo as importações do Contábil conforme vão sendo realizadas, o GD Sérgio informou que a previsão é concluir na próxima semana - Data Comentário: 06/07/2026 12:42</t>
         </is>
       </c>
       <c r="AE802" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>13/07/2026</t>
         </is>
       </c>
       <c r="AF802" t="inlineStr">
@@ -85111,12 +85143,12 @@
       <c r="AC803" t="inlineStr"/>
       <c r="AD803" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 04/07/2026. - Data Comentário: 03/07/2026 17:02</t>
+          <t>Os GC's estão respondendo as importações do Contábil conforme vão sendo realizadas, o GD Sérgio informou que a previsão é concluir na próxima semana - Data Comentário: 06/07/2026 12:42</t>
         </is>
       </c>
       <c r="AE803" t="inlineStr">
         <is>
-          <t>04/07/2026</t>
+          <t>13/07/2026</t>
         </is>
       </c>
       <c r="AF803" t="inlineStr">
@@ -85227,12 +85259,12 @@
       <c r="AC804" t="inlineStr"/>
       <c r="AD804" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 01/07/2026. - Data Comentário: 30/06/2026 08:50</t>
+          <t>Os GC's estão respondendo as importações do Contábil conforme vão sendo realizadas, o GD Sérgio informou que a previsão é concluir na próxima semana - Data Comentário: 06/07/2026 12:42</t>
         </is>
       </c>
       <c r="AE804" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>13/07/2026</t>
         </is>
       </c>
       <c r="AF804" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-07 10:15
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG804"/>
+  <dimension ref="A1:AG803"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85036,11 +85036,11 @@
     </row>
     <row r="801">
       <c r="A801" t="n">
-        <v>6981</v>
+        <v>6404</v>
       </c>
       <c r="B801" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUIZ GOMES DA SILVA - O GOIANO </t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="C801" t="inlineStr">
@@ -85050,7 +85050,7 @@
       </c>
       <c r="D801" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E801" t="inlineStr">
@@ -85060,41 +85060,45 @@
       </c>
       <c r="F801" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G801" t="n">
-        <v>9793</v>
+        <v>11001</v>
       </c>
       <c r="H801" t="n">
         <v>0</v>
       </c>
       <c r="I801" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J801" t="inlineStr">
         <is>
-          <t>Aplicação de Modelo - Pendente - SP</t>
+          <t>Movimento - Analise de Balanço Lucro Presumido</t>
         </is>
       </c>
       <c r="K801" t="inlineStr"/>
       <c r="L801" s="1" t="n">
-        <v>46205</v>
-      </c>
-      <c r="M801" t="inlineStr"/>
+        <v>46202</v>
+      </c>
+      <c r="M801" t="inlineStr">
+        <is>
+          <t>02/07/2026</t>
+        </is>
+      </c>
       <c r="N801" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="O801" t="n">
-        <v>18195069</v>
+        <v>16962451</v>
       </c>
       <c r="P801" t="inlineStr">
         <is>
-          <t>Claudineia Rodrigues</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="Q801" t="inlineStr">
@@ -85104,17 +85108,22 @@
       </c>
       <c r="R801" t="inlineStr"/>
       <c r="S801" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="T801" t="inlineStr">
         <is>
-          <t>SUPERMERCADO AVENIDA</t>
-        </is>
-      </c>
-      <c r="U801" t="inlineStr"/>
+          <t>SOLAR INVESTIMENTOS</t>
+        </is>
+      </c>
+      <c r="U801" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="V801" t="inlineStr">
         <is>
-          <t>Rotina de Cliente Sem Modelo - CodCliente: 6981; Tarefa Incluida: 9793; Vencimento: 02/07/2026 00:00:00; UsuarioResponsavel: Claudineia - Data Comentário: 01/07/2026 09:04</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/07/2026 
+Analisar até 02/07/2026 - Data Comentário: 01/07/2026 07:26</t>
         </is>
       </c>
       <c r="W801" t="inlineStr"/>
@@ -85126,12 +85135,12 @@
       <c r="AC801" t="inlineStr"/>
       <c r="AD801" t="inlineStr">
         <is>
-          <t>Claudineia cobrada a respeito das aplicações, ela informou que o atraso se deu ao fato de estar concluindo a distribuição da carteira de clientes do seu departamento, mas a tarefa será executada ainda hoje. - Data Comentário: 06/07/2026 12:41</t>
+          <t>Os GC's estão respondendo as importações do Contábil conforme vão sendo realizadas, o GD Sérgio informou que a previsão é concluir na próxima semana - Data Comentário: 06/07/2026 12:42</t>
         </is>
       </c>
       <c r="AE801" t="inlineStr">
         <is>
-          <t>06/07/2026</t>
+          <t>13/07/2026</t>
         </is>
       </c>
       <c r="AF801" t="inlineStr">
@@ -85143,11 +85152,11 @@
     </row>
     <row r="802">
       <c r="A802" t="n">
-        <v>6404</v>
+        <v>6224</v>
       </c>
       <c r="B802" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C802" t="inlineStr">
@@ -85157,7 +85166,7 @@
       </c>
       <c r="D802" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E802" t="inlineStr">
@@ -85167,11 +85176,11 @@
       </c>
       <c r="F802" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G802" t="n">
-        <v>11001</v>
+        <v>7877</v>
       </c>
       <c r="H802" t="n">
         <v>0</v>
@@ -85183,25 +85192,25 @@
       </c>
       <c r="J802" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Lucro Presumido</t>
+          <t>Movimento - Analise de Balanço Lucro Real</t>
         </is>
       </c>
       <c r="K802" t="inlineStr"/>
       <c r="L802" s="1" t="n">
-        <v>46202</v>
+        <v>46171</v>
       </c>
       <c r="M802" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>03/07/2026</t>
         </is>
       </c>
       <c r="N802" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="O802" t="n">
-        <v>16962451</v>
+        <v>18076566</v>
       </c>
       <c r="P802" t="inlineStr">
         <is>
@@ -85215,11 +85224,11 @@
       </c>
       <c r="R802" t="inlineStr"/>
       <c r="S802" t="n">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="T802" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U802" t="inlineStr">
@@ -85229,8 +85238,8 @@
       </c>
       <c r="V802" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/07/2026 
-Analisar até 02/07/2026 - Data Comentário: 01/07/2026 07:26</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 03/07/2026 
+Devido as ocorrências com Cbenef e atendimetnos a cliente precisamos reprogramar conclusão para 03/07/2026 - Data Comentário: 03/07/2026 08:15</t>
         </is>
       </c>
       <c r="W802" t="inlineStr"/>
@@ -85259,11 +85268,11 @@
     </row>
     <row r="803">
       <c r="A803" t="n">
-        <v>6224</v>
+        <v>6486</v>
       </c>
       <c r="B803" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C803" t="inlineStr">
@@ -85283,11 +85292,11 @@
       </c>
       <c r="F803" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G803" t="n">
-        <v>7877</v>
+        <v>9774</v>
       </c>
       <c r="H803" t="n">
         <v>0</v>
@@ -85299,25 +85308,25 @@
       </c>
       <c r="J803" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Lucro Real</t>
+          <t>Movimento - Analise de Balanço Simples Nacional</t>
         </is>
       </c>
       <c r="K803" t="inlineStr"/>
       <c r="L803" s="1" t="n">
-        <v>46171</v>
+        <v>46189</v>
       </c>
       <c r="M803" t="inlineStr">
         <is>
-          <t>03/07/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="N803" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="O803" t="n">
-        <v>18076566</v>
+        <v>16976318</v>
       </c>
       <c r="P803" t="inlineStr">
         <is>
@@ -85331,11 +85340,11 @@
       </c>
       <c r="R803" t="inlineStr"/>
       <c r="S803" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="T803" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U803" t="inlineStr">
@@ -85345,8 +85354,8 @@
       </c>
       <c r="V803" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 03/07/2026 
-Devido as ocorrências com Cbenef e atendimetnos a cliente precisamos reprogramar conclusão para 03/07/2026 - Data Comentário: 03/07/2026 08:15</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/07/2026 
+Priorização na análise - Data Comentário: 01/07/2026 08:13</t>
         </is>
       </c>
       <c r="W803" t="inlineStr"/>
@@ -85373,122 +85382,6 @@
       </c>
       <c r="AG803" t="inlineStr"/>
     </row>
-    <row r="804">
-      <c r="A804" t="n">
-        <v>6486</v>
-      </c>
-      <c r="B804" t="inlineStr">
-        <is>
-          <t>PC GAMER GOIANIA LTDA</t>
-        </is>
-      </c>
-      <c r="C804" t="inlineStr">
-        <is>
-          <t>GOIAS</t>
-        </is>
-      </c>
-      <c r="D804" t="inlineStr">
-        <is>
-          <t>Federal - L Real -Trimestral</t>
-        </is>
-      </c>
-      <c r="E804" t="inlineStr">
-        <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="F804" t="inlineStr">
-        <is>
-          <t>Edimir Santos</t>
-        </is>
-      </c>
-      <c r="G804" t="n">
-        <v>9774</v>
-      </c>
-      <c r="H804" t="n">
-        <v>0</v>
-      </c>
-      <c r="I804" t="inlineStr">
-        <is>
-          <t>GERENCIA DE CONTAS</t>
-        </is>
-      </c>
-      <c r="J804" t="inlineStr">
-        <is>
-          <t>Movimento - Analise de Balanço Simples Nacional</t>
-        </is>
-      </c>
-      <c r="K804" t="inlineStr"/>
-      <c r="L804" s="1" t="n">
-        <v>46189</v>
-      </c>
-      <c r="M804" t="inlineStr">
-        <is>
-          <t>02/07/2026</t>
-        </is>
-      </c>
-      <c r="N804" t="inlineStr">
-        <is>
-          <t>05/2026</t>
-        </is>
-      </c>
-      <c r="O804" t="n">
-        <v>16976318</v>
-      </c>
-      <c r="P804" t="inlineStr">
-        <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="Q804" t="inlineStr">
-        <is>
-          <t>Em Atraso</t>
-        </is>
-      </c>
-      <c r="R804" t="inlineStr"/>
-      <c r="S804" t="n">
-        <v>21</v>
-      </c>
-      <c r="T804" t="inlineStr">
-        <is>
-          <t>PC GAMER</t>
-        </is>
-      </c>
-      <c r="U804" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="V804" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/07/2026 
-Priorização na análise - Data Comentário: 01/07/2026 08:13</t>
-        </is>
-      </c>
-      <c r="W804" t="inlineStr"/>
-      <c r="X804" t="inlineStr"/>
-      <c r="Y804" t="inlineStr"/>
-      <c r="Z804" t="inlineStr"/>
-      <c r="AA804" t="inlineStr"/>
-      <c r="AB804" t="inlineStr"/>
-      <c r="AC804" t="inlineStr"/>
-      <c r="AD804" t="inlineStr">
-        <is>
-          <t>Os GC's estão respondendo as importações do Contábil conforme vão sendo realizadas, o GD Sérgio informou que a previsão é concluir na próxima semana - Data Comentário: 06/07/2026 12:42</t>
-        </is>
-      </c>
-      <c r="AE804" t="inlineStr">
-        <is>
-          <t>13/07/2026</t>
-        </is>
-      </c>
-      <c r="AF804" t="inlineStr">
-        <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AG804" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-10 10:09
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -3954,7 +3954,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>14/07/2026</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -3987,8 +3987,8 @@
       <c r="U33" t="inlineStr"/>
       <c r="V33" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 10/07/2026 
-ESocial fechado, antecipação de envio. - Data Comentário: 08/07/2026 14:21</t>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 14/07/2026 
+ESocial fechado, antecipação de envio. - Data Comentário: 10/07/2026 09:19</t>
         </is>
       </c>
       <c r="W33" t="inlineStr"/>
@@ -7281,10 +7281,10 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>1793</v>
+        <v>6294</v>
       </c>
       <c r="H65" t="n">
-        <v>0</v>
+        <v>1788</v>
       </c>
       <c r="I65" t="inlineStr">
         <is>
@@ -7293,25 +7293,21 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Mun - ISS Serv. Tomados</t>
+          <t>Recebimento NFCE</t>
         </is>
       </c>
       <c r="K65" t="inlineStr"/>
       <c r="L65" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="M65" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
+        <v>46216</v>
+      </c>
+      <c r="M65" t="inlineStr"/>
       <c r="N65" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O65" t="n">
-        <v>17948926</v>
+        <v>17948997</v>
       </c>
       <c r="P65" t="inlineStr">
         <is>
@@ -7325,7 +7321,7 @@
       </c>
       <c r="R65" t="inlineStr"/>
       <c r="S65" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="T65" t="inlineStr">
         <is>
@@ -7337,11 +7333,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V65" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 15:51</t>
-        </is>
-      </c>
+      <c r="V65" t="inlineStr"/>
       <c r="W65" t="inlineStr"/>
       <c r="X65" t="inlineStr"/>
       <c r="Y65" t="inlineStr"/>
@@ -7355,7 +7347,7 @@
       <c r="AE65" t="inlineStr"/>
       <c r="AF65" t="inlineStr">
         <is>
-          <t>Imposto</t>
+          <t>Tarefa</t>
         </is>
       </c>
       <c r="AG65" t="inlineStr">
@@ -7366,11 +7358,11 @@
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>6779</v>
+        <v>5617</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>CORDEIRO E CIA LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -7380,7 +7372,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -7394,7 +7386,7 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>1793</v>
+        <v>11303</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
@@ -7406,25 +7398,21 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Mun - ISS Serv. Tomados</t>
+          <t>Retorno do Check-List Fiscal</t>
         </is>
       </c>
       <c r="K66" t="inlineStr"/>
       <c r="L66" s="1" t="n">
-        <v>46213</v>
-      </c>
-      <c r="M66" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
+        <v>46218</v>
+      </c>
+      <c r="M66" t="inlineStr"/>
       <c r="N66" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O66" t="n">
-        <v>18084953</v>
+        <v>17407963</v>
       </c>
       <c r="P66" t="inlineStr">
         <is>
@@ -7438,19 +7426,19 @@
       </c>
       <c r="R66" t="inlineStr"/>
       <c r="S66" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
-        </is>
-      </c>
-      <c r="U66" t="inlineStr"/>
-      <c r="V66" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 15:51</t>
-        </is>
-      </c>
+          <t>SUPER MAIS DO GOIÁS</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr"/>
       <c r="W66" t="inlineStr"/>
       <c r="X66" t="inlineStr"/>
       <c r="Y66" t="inlineStr"/>
@@ -7464,7 +7452,7 @@
       <c r="AE66" t="inlineStr"/>
       <c r="AF66" t="inlineStr">
         <is>
-          <t>Imposto</t>
+          <t>Tarefa</t>
         </is>
       </c>
       <c r="AG66" t="inlineStr">
@@ -7475,11 +7463,11 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>6885</v>
+        <v>6962</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
+          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -7489,7 +7477,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -7499,45 +7487,41 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G67" t="n">
-        <v>1793</v>
+        <v>950</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Mun - ISS Serv. Tomados</t>
+          <t>Confirm Rec - ISS Prestados</t>
         </is>
       </c>
       <c r="K67" t="inlineStr"/>
       <c r="L67" s="1" t="n">
         <v>46213</v>
       </c>
-      <c r="M67" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
+      <c r="M67" t="inlineStr"/>
       <c r="N67" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O67" t="n">
-        <v>18134033</v>
+        <v>18188715</v>
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>Cristina Leite</t>
+          <t>Victoria Virgens</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
@@ -7551,13 +7535,13 @@
       </c>
       <c r="T67" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>PROMOTORAS GYN</t>
         </is>
       </c>
       <c r="U67" t="inlineStr"/>
       <c r="V67" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 15:51</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1866] sendo a ultima baixa feita [1866]-08/07/2026 18:25:05.. - Data Comentário: 08/07/2026 18:24</t>
         </is>
       </c>
       <c r="W67" t="inlineStr"/>
@@ -7576,19 +7560,15 @@
           <t>Imposto</t>
         </is>
       </c>
-      <c r="AG67" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
+      <c r="AG67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>6705</v>
+        <v>6963</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>NARCIZO ALVES CORDEIRO</t>
+          <t>PROMOTORAS GYN LTDA</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -7598,7 +7578,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -7608,28 +7588,28 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G68" t="n">
-        <v>6294</v>
+        <v>950</v>
       </c>
       <c r="H68" t="n">
-        <v>1788</v>
+        <v>0</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Recebimento NFCE</t>
+          <t>Confirm Rec - ISS Prestados</t>
         </is>
       </c>
       <c r="K68" t="inlineStr"/>
       <c r="L68" s="1" t="n">
-        <v>46216</v>
+        <v>46213</v>
       </c>
       <c r="M68" t="inlineStr"/>
       <c r="N68" t="inlineStr">
@@ -7638,11 +7618,11 @@
         </is>
       </c>
       <c r="O68" t="n">
-        <v>17948997</v>
+        <v>18188621</v>
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>Cristina Leite</t>
+          <t>Victoria Virgens</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
@@ -7652,19 +7632,19 @@
       </c>
       <c r="R68" t="inlineStr"/>
       <c r="S68" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="T68" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
-        </is>
-      </c>
-      <c r="U68" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="V68" t="inlineStr"/>
+          <t>PROMOTORAS GYN</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr"/>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1866] sendo a ultima baixa feita [1866]-08/07/2026 18:24:46.. - Data Comentário: 08/07/2026 18:24</t>
+        </is>
+      </c>
       <c r="W68" t="inlineStr"/>
       <c r="X68" t="inlineStr"/>
       <c r="Y68" t="inlineStr"/>
@@ -7678,22 +7658,18 @@
       <c r="AE68" t="inlineStr"/>
       <c r="AF68" t="inlineStr">
         <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AG68" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
+          <t>Imposto</t>
+        </is>
+      </c>
+      <c r="AG68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>5617</v>
+        <v>6705</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>NARCIZO ALVES CORDEIRO</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -7703,7 +7679,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -7717,24 +7693,24 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>11303</v>
+        <v>951</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Retorno do Check-List Fiscal</t>
+          <t>Confirm Rec - ISS Tomados</t>
         </is>
       </c>
       <c r="K69" t="inlineStr"/>
       <c r="L69" s="1" t="n">
-        <v>46218</v>
+        <v>46213</v>
       </c>
       <c r="M69" t="inlineStr"/>
       <c r="N69" t="inlineStr">
@@ -7743,11 +7719,11 @@
         </is>
       </c>
       <c r="O69" t="n">
-        <v>17407963</v>
+        <v>17952533</v>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Cristina Leite</t>
+          <t>Victoria Virgens</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -7757,11 +7733,11 @@
       </c>
       <c r="R69" t="inlineStr"/>
       <c r="S69" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="T69" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U69" t="inlineStr">
@@ -7769,7 +7745,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V69" t="inlineStr"/>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1793] sendo a ultima baixa feita [1793]-10/07/2026 09:57:11.. - Data Comentário: 10/07/2026 09:56</t>
+        </is>
+      </c>
       <c r="W69" t="inlineStr"/>
       <c r="X69" t="inlineStr"/>
       <c r="Y69" t="inlineStr"/>
@@ -7783,22 +7763,18 @@
       <c r="AE69" t="inlineStr"/>
       <c r="AF69" t="inlineStr">
         <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AG69" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
+          <t>Imposto</t>
+        </is>
+      </c>
+      <c r="AG69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>6962</v>
+        <v>6779</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
+          <t>CORDEIRO E CIA LTDA</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -7808,7 +7784,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -7818,11 +7794,11 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G70" t="n">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="H70" t="n">
         <v>0</v>
@@ -7834,7 +7810,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Confirm Rec - ISS Prestados</t>
+          <t>Confirm Rec - ISS Tomados</t>
         </is>
       </c>
       <c r="K70" t="inlineStr"/>
@@ -7848,7 +7824,7 @@
         </is>
       </c>
       <c r="O70" t="n">
-        <v>18188715</v>
+        <v>18056703</v>
       </c>
       <c r="P70" t="inlineStr">
         <is>
@@ -7866,13 +7842,13 @@
       </c>
       <c r="T70" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U70" t="inlineStr"/>
       <c r="V70" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1866] sendo a ultima baixa feita [1866]-08/07/2026 18:25:05.. - Data Comentário: 08/07/2026 18:24</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1793] sendo a ultima baixa feita [1793]-10/07/2026 09:57:11.. - Data Comentário: 10/07/2026 09:56</t>
         </is>
       </c>
       <c r="W70" t="inlineStr"/>
@@ -7895,11 +7871,11 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>6963</v>
+        <v>6885</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN LTDA</t>
+          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -7909,7 +7885,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -7919,11 +7895,11 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G71" t="n">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="H71" t="n">
         <v>0</v>
@@ -7935,7 +7911,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Confirm Rec - ISS Prestados</t>
+          <t>Confirm Rec - ISS Tomados</t>
         </is>
       </c>
       <c r="K71" t="inlineStr"/>
@@ -7949,7 +7925,7 @@
         </is>
       </c>
       <c r="O71" t="n">
-        <v>18188621</v>
+        <v>18128657</v>
       </c>
       <c r="P71" t="inlineStr">
         <is>
@@ -7967,13 +7943,13 @@
       </c>
       <c r="T71" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U71" t="inlineStr"/>
       <c r="V71" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1866] sendo a ultima baixa feita [1866]-08/07/2026 18:24:46.. - Data Comentário: 08/07/2026 18:24</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1793] sendo a ultima baixa feita [1793]-10/07/2026 09:57:12.. - Data Comentário: 10/07/2026 09:56</t>
         </is>
       </c>
       <c r="W71" t="inlineStr"/>
@@ -31687,11 +31663,11 @@
     </row>
     <row r="287">
       <c r="A287" t="n">
-        <v>6703</v>
+        <v>6705</v>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>NARCIZO ALVES CORDEIRO</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -31701,7 +31677,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E287" t="inlineStr">
@@ -31715,7 +31691,7 @@
         </is>
       </c>
       <c r="G287" t="n">
-        <v>1796</v>
+        <v>1793</v>
       </c>
       <c r="H287" t="n">
         <v>0</v>
@@ -31727,12 +31703,12 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>Produtor Rural</t>
+          <t>Mun - ISS Serv. Tomados</t>
         </is>
       </c>
       <c r="K287" t="inlineStr"/>
       <c r="L287" s="1" t="n">
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="M287" t="inlineStr">
         <is>
@@ -31745,7 +31721,7 @@
         </is>
       </c>
       <c r="O287" t="n">
-        <v>18073096</v>
+        <v>17948926</v>
       </c>
       <c r="P287" t="inlineStr">
         <is>
@@ -31758,14 +31734,14 @@
         </is>
       </c>
       <c r="R287" s="1" t="n">
-        <v>46211.67827373843</v>
+        <v>46213.41471872685</v>
       </c>
       <c r="S287" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T287" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U287" t="inlineStr">
@@ -31775,7 +31751,7 @@
       </c>
       <c r="V287" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 14:49</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 15:51</t>
         </is>
       </c>
       <c r="W287" t="inlineStr"/>
@@ -31795,7 +31771,7 @@
       <c r="AE287" t="inlineStr"/>
       <c r="AF287" t="inlineStr">
         <is>
-          <t>Tarefa</t>
+          <t>Imposto</t>
         </is>
       </c>
       <c r="AG287" t="inlineStr">
@@ -31806,11 +31782,11 @@
     </row>
     <row r="288">
       <c r="A288" t="n">
-        <v>6486</v>
+        <v>6779</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>PC GAMER GOIANIA LTDA</t>
+          <t>CORDEIRO E CIA LTDA</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -31820,7 +31796,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -31834,7 +31810,7 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>11359</v>
+        <v>1793</v>
       </c>
       <c r="H288" t="n">
         <v>0</v>
@@ -31846,21 +31822,25 @@
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recebimento - Sped ICMS </t>
+          <t>Mun - ISS Serv. Tomados</t>
         </is>
       </c>
       <c r="K288" t="inlineStr"/>
       <c r="L288" s="1" t="n">
-        <v>46205</v>
-      </c>
-      <c r="M288" t="inlineStr"/>
+        <v>46213</v>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
       <c r="N288" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O288" t="n">
-        <v>18155343</v>
+        <v>18084953</v>
       </c>
       <c r="P288" t="inlineStr">
         <is>
@@ -31873,22 +31853,22 @@
         </is>
       </c>
       <c r="R288" s="1" t="n">
-        <v>46205.45901570602</v>
+        <v>46213.41472034722</v>
       </c>
       <c r="S288" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="T288" t="inlineStr">
         <is>
-          <t>PC GAMER</t>
-        </is>
-      </c>
-      <c r="U288" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="V288" t="inlineStr"/>
+          <t>TECNO COM</t>
+        </is>
+      </c>
+      <c r="U288" t="inlineStr"/>
+      <c r="V288" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 15:51</t>
+        </is>
+      </c>
       <c r="W288" t="inlineStr"/>
       <c r="X288" t="inlineStr"/>
       <c r="Y288" t="inlineStr"/>
@@ -31906,7 +31886,7 @@
       <c r="AE288" t="inlineStr"/>
       <c r="AF288" t="inlineStr">
         <is>
-          <t>Tarefa</t>
+          <t>Imposto</t>
         </is>
       </c>
       <c r="AG288" t="inlineStr">
@@ -31917,11 +31897,11 @@
     </row>
     <row r="289">
       <c r="A289" t="n">
-        <v>6279</v>
+        <v>6885</v>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>DIENNYFER DA S PEREIRA</t>
+          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -31931,7 +31911,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
@@ -31941,14 +31921,14 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G289" t="n">
-        <v>6884</v>
+        <v>1793</v>
       </c>
       <c r="H289" t="n">
-        <v>1788</v>
+        <v>0</v>
       </c>
       <c r="I289" t="inlineStr">
         <is>
@@ -31957,21 +31937,25 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>Recebimento de NF Serviços Tomados</t>
+          <t>Mun - ISS Serv. Tomados</t>
         </is>
       </c>
       <c r="K289" t="inlineStr"/>
       <c r="L289" s="1" t="n">
-        <v>46211</v>
-      </c>
-      <c r="M289" t="inlineStr"/>
+        <v>46213</v>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
       <c r="N289" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O289" t="n">
-        <v>17071044</v>
+        <v>18134033</v>
       </c>
       <c r="P289" t="inlineStr">
         <is>
@@ -31984,22 +31968,22 @@
         </is>
       </c>
       <c r="R289" s="1" t="n">
-        <v>46206.79257369213</v>
+        <v>46213.41472866898</v>
       </c>
       <c r="S289" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T289" t="inlineStr">
         <is>
           <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
-      <c r="U289" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="V289" t="inlineStr"/>
+      <c r="U289" t="inlineStr"/>
+      <c r="V289" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 15:51</t>
+        </is>
+      </c>
       <c r="W289" t="inlineStr"/>
       <c r="X289" t="inlineStr"/>
       <c r="Y289" t="inlineStr"/>
@@ -32008,7 +31992,7 @@
       </c>
       <c r="AA289" t="inlineStr">
         <is>
-          <t>Ricardo Fischer</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="AB289" t="inlineStr"/>
@@ -32017,7 +32001,7 @@
       <c r="AE289" t="inlineStr"/>
       <c r="AF289" t="inlineStr">
         <is>
-          <t>Tarefa</t>
+          <t>Imposto</t>
         </is>
       </c>
       <c r="AG289" t="inlineStr">
@@ -32028,11 +32012,11 @@
     </row>
     <row r="290">
       <c r="A290" t="n">
-        <v>6486</v>
+        <v>6703</v>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>PC GAMER GOIANIA LTDA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -32042,7 +32026,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -32056,10 +32040,10 @@
         </is>
       </c>
       <c r="G290" t="n">
-        <v>6884</v>
+        <v>1796</v>
       </c>
       <c r="H290" t="n">
-        <v>1788</v>
+        <v>0</v>
       </c>
       <c r="I290" t="inlineStr">
         <is>
@@ -32068,21 +32052,25 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>Recebimento de NF Serviços Tomados</t>
+          <t>Produtor Rural</t>
         </is>
       </c>
       <c r="K290" t="inlineStr"/>
       <c r="L290" s="1" t="n">
         <v>46211</v>
       </c>
-      <c r="M290" t="inlineStr"/>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
       <c r="N290" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O290" t="n">
-        <v>16976205</v>
+        <v>18073096</v>
       </c>
       <c r="P290" t="inlineStr">
         <is>
@@ -32095,14 +32083,14 @@
         </is>
       </c>
       <c r="R290" s="1" t="n">
-        <v>46205.45918969908</v>
+        <v>46211.67827373843</v>
       </c>
       <c r="S290" t="n">
         <v>2</v>
       </c>
       <c r="T290" t="inlineStr">
         <is>
-          <t>PC GAMER</t>
+          <t>LIMA MOTA</t>
         </is>
       </c>
       <c r="U290" t="inlineStr">
@@ -32110,7 +32098,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V290" t="inlineStr"/>
+      <c r="V290" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 14:49</t>
+        </is>
+      </c>
       <c r="W290" t="inlineStr"/>
       <c r="X290" t="inlineStr"/>
       <c r="Y290" t="inlineStr"/>
@@ -32139,11 +32131,11 @@
     </row>
     <row r="291">
       <c r="A291" t="n">
-        <v>6705</v>
+        <v>6486</v>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>NARCIZO ALVES CORDEIRO</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -32153,7 +32145,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -32167,10 +32159,10 @@
         </is>
       </c>
       <c r="G291" t="n">
-        <v>6884</v>
+        <v>11359</v>
       </c>
       <c r="H291" t="n">
-        <v>1788</v>
+        <v>0</v>
       </c>
       <c r="I291" t="inlineStr">
         <is>
@@ -32179,25 +32171,21 @@
       </c>
       <c r="J291" t="inlineStr">
         <is>
-          <t>Recebimento de NF Serviços Tomados</t>
+          <t xml:space="preserve">Recebimento - Sped ICMS </t>
         </is>
       </c>
       <c r="K291" t="inlineStr"/>
       <c r="L291" s="1" t="n">
-        <v>46211</v>
-      </c>
-      <c r="M291" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
+        <v>46205</v>
+      </c>
+      <c r="M291" t="inlineStr"/>
       <c r="N291" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O291" t="n">
-        <v>17949037</v>
+        <v>18155343</v>
       </c>
       <c r="P291" t="inlineStr">
         <is>
@@ -32210,14 +32198,14 @@
         </is>
       </c>
       <c r="R291" s="1" t="n">
-        <v>46211.37590150463</v>
+        <v>46205.45901570602</v>
       </c>
       <c r="S291" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="T291" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U291" t="inlineStr">
@@ -32225,11 +32213,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V291" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 15:52</t>
-        </is>
-      </c>
+      <c r="V291" t="inlineStr"/>
       <c r="W291" t="inlineStr"/>
       <c r="X291" t="inlineStr"/>
       <c r="Y291" t="inlineStr"/>
@@ -32258,11 +32242,11 @@
     </row>
     <row r="292">
       <c r="A292" t="n">
-        <v>6885</v>
+        <v>6279</v>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
+          <t>DIENNYFER DA S PEREIRA</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -32272,7 +32256,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E292" t="inlineStr">
@@ -32282,7 +32266,7 @@
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G292" t="n">
@@ -32312,7 +32296,7 @@
         </is>
       </c>
       <c r="O292" t="n">
-        <v>18134133</v>
+        <v>17071044</v>
       </c>
       <c r="P292" t="inlineStr">
         <is>
@@ -32325,7 +32309,7 @@
         </is>
       </c>
       <c r="R292" s="1" t="n">
-        <v>46206.79256712963</v>
+        <v>46206.79257369213</v>
       </c>
       <c r="S292" t="n">
         <v>2</v>
@@ -32335,7 +32319,11 @@
           <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
-      <c r="U292" t="inlineStr"/>
+      <c r="U292" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="V292" t="inlineStr"/>
       <c r="W292" t="inlineStr"/>
       <c r="X292" t="inlineStr"/>
@@ -32365,11 +32353,11 @@
     </row>
     <row r="293">
       <c r="A293" t="n">
-        <v>6279</v>
+        <v>6486</v>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>DIENNYFER DA S PEREIRA</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -32379,7 +32367,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E293" t="inlineStr">
@@ -32389,11 +32377,11 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G293" t="n">
-        <v>6294</v>
+        <v>6884</v>
       </c>
       <c r="H293" t="n">
         <v>1788</v>
@@ -32405,12 +32393,12 @@
       </c>
       <c r="J293" t="inlineStr">
         <is>
-          <t>Recebimento NFCE</t>
+          <t>Recebimento de NF Serviços Tomados</t>
         </is>
       </c>
       <c r="K293" t="inlineStr"/>
       <c r="L293" s="1" t="n">
-        <v>46216</v>
+        <v>46211</v>
       </c>
       <c r="M293" t="inlineStr"/>
       <c r="N293" t="inlineStr">
@@ -32419,7 +32407,7 @@
         </is>
       </c>
       <c r="O293" t="n">
-        <v>17070959</v>
+        <v>16976205</v>
       </c>
       <c r="P293" t="inlineStr">
         <is>
@@ -32432,14 +32420,14 @@
         </is>
       </c>
       <c r="R293" s="1" t="n">
-        <v>46206.7921721875</v>
+        <v>46205.45918969908</v>
       </c>
       <c r="S293" t="n">
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="T293" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U293" t="inlineStr">
@@ -32456,7 +32444,7 @@
       </c>
       <c r="AA293" t="inlineStr">
         <is>
-          <t>Ricardo Fischer</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="AB293" t="inlineStr"/>
@@ -32476,11 +32464,11 @@
     </row>
     <row r="294">
       <c r="A294" t="n">
-        <v>6885</v>
+        <v>6705</v>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
+          <t>NARCIZO ALVES CORDEIRO</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -32504,7 +32492,7 @@
         </is>
       </c>
       <c r="G294" t="n">
-        <v>6294</v>
+        <v>6884</v>
       </c>
       <c r="H294" t="n">
         <v>1788</v>
@@ -32516,21 +32504,25 @@
       </c>
       <c r="J294" t="inlineStr">
         <is>
-          <t>Recebimento NFCE</t>
+          <t>Recebimento de NF Serviços Tomados</t>
         </is>
       </c>
       <c r="K294" t="inlineStr"/>
       <c r="L294" s="1" t="n">
-        <v>46216</v>
-      </c>
-      <c r="M294" t="inlineStr"/>
+        <v>46211</v>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
       <c r="N294" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O294" t="n">
-        <v>18134097</v>
+        <v>17949037</v>
       </c>
       <c r="P294" t="inlineStr">
         <is>
@@ -32543,18 +32535,26 @@
         </is>
       </c>
       <c r="R294" s="1" t="n">
-        <v>46206.7921681713</v>
+        <v>46211.37590150463</v>
       </c>
       <c r="S294" t="n">
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="T294" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
-        </is>
-      </c>
-      <c r="U294" t="inlineStr"/>
-      <c r="V294" t="inlineStr"/>
+          <t>TECNO COM</t>
+        </is>
+      </c>
+      <c r="U294" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V294" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 15:52</t>
+        </is>
+      </c>
       <c r="W294" t="inlineStr"/>
       <c r="X294" t="inlineStr"/>
       <c r="Y294" t="inlineStr"/>
@@ -32563,7 +32563,7 @@
       </c>
       <c r="AA294" t="inlineStr">
         <is>
-          <t>Ricardo Fischer</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="AB294" t="inlineStr"/>
@@ -32583,11 +32583,11 @@
     </row>
     <row r="295">
       <c r="A295" t="n">
-        <v>5417</v>
+        <v>6885</v>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -32597,7 +32597,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E295" t="inlineStr">
@@ -32607,14 +32607,14 @@
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G295" t="n">
-        <v>11303</v>
+        <v>6884</v>
       </c>
       <c r="H295" t="n">
-        <v>0</v>
+        <v>1788</v>
       </c>
       <c r="I295" t="inlineStr">
         <is>
@@ -32623,12 +32623,12 @@
       </c>
       <c r="J295" t="inlineStr">
         <is>
-          <t>Retorno do Check-List Fiscal</t>
+          <t>Recebimento de NF Serviços Tomados</t>
         </is>
       </c>
       <c r="K295" t="inlineStr"/>
       <c r="L295" s="1" t="n">
-        <v>46218</v>
+        <v>46211</v>
       </c>
       <c r="M295" t="inlineStr"/>
       <c r="N295" t="inlineStr">
@@ -32637,7 +32637,7 @@
         </is>
       </c>
       <c r="O295" t="n">
-        <v>17399452</v>
+        <v>18134133</v>
       </c>
       <c r="P295" t="inlineStr">
         <is>
@@ -32650,26 +32650,18 @@
         </is>
       </c>
       <c r="R295" s="1" t="n">
-        <v>46210.37424872685</v>
+        <v>46206.79256712963</v>
       </c>
       <c r="S295" t="n">
-        <v>-5</v>
+        <v>2</v>
       </c>
       <c r="T295" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
-        </is>
-      </c>
-      <c r="U295" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="V295" t="inlineStr">
-        <is>
-          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 07/07/2026 08:56:44. - Data Comentário: 07/07/2026 08:55</t>
-        </is>
-      </c>
+          <t>EMPORIO DOS FRIOS</t>
+        </is>
+      </c>
+      <c r="U295" t="inlineStr"/>
+      <c r="V295" t="inlineStr"/>
       <c r="W295" t="inlineStr"/>
       <c r="X295" t="inlineStr"/>
       <c r="Y295" t="inlineStr"/>
@@ -32678,7 +32670,7 @@
       </c>
       <c r="AA295" t="inlineStr">
         <is>
-          <t>ex-funcionario</t>
+          <t>Ricardo Fischer</t>
         </is>
       </c>
       <c r="AB295" t="inlineStr"/>
@@ -32726,10 +32718,10 @@
         </is>
       </c>
       <c r="G296" t="n">
-        <v>11303</v>
+        <v>6294</v>
       </c>
       <c r="H296" t="n">
-        <v>0</v>
+        <v>1788</v>
       </c>
       <c r="I296" t="inlineStr">
         <is>
@@ -32738,12 +32730,12 @@
       </c>
       <c r="J296" t="inlineStr">
         <is>
-          <t>Retorno do Check-List Fiscal</t>
+          <t>Recebimento NFCE</t>
         </is>
       </c>
       <c r="K296" t="inlineStr"/>
       <c r="L296" s="1" t="n">
-        <v>46218</v>
+        <v>46216</v>
       </c>
       <c r="M296" t="inlineStr"/>
       <c r="N296" t="inlineStr">
@@ -32752,7 +32744,7 @@
         </is>
       </c>
       <c r="O296" t="n">
-        <v>17071101</v>
+        <v>17070959</v>
       </c>
       <c r="P296" t="inlineStr">
         <is>
@@ -32765,10 +32757,10 @@
         </is>
       </c>
       <c r="R296" s="1" t="n">
-        <v>46205.76232731481</v>
+        <v>46206.7921721875</v>
       </c>
       <c r="S296" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="T296" t="inlineStr">
         <is>
@@ -32789,7 +32781,7 @@
       </c>
       <c r="AA296" t="inlineStr">
         <is>
-          <t>Juan Rodrigues</t>
+          <t>Ricardo Fischer</t>
         </is>
       </c>
       <c r="AB296" t="inlineStr"/>
@@ -32809,11 +32801,11 @@
     </row>
     <row r="297">
       <c r="A297" t="n">
-        <v>6486</v>
+        <v>6885</v>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>PC GAMER GOIANIA LTDA</t>
+          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -32823,7 +32815,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -32837,10 +32829,10 @@
         </is>
       </c>
       <c r="G297" t="n">
-        <v>11303</v>
+        <v>6294</v>
       </c>
       <c r="H297" t="n">
-        <v>0</v>
+        <v>1788</v>
       </c>
       <c r="I297" t="inlineStr">
         <is>
@@ -32849,12 +32841,12 @@
       </c>
       <c r="J297" t="inlineStr">
         <is>
-          <t>Retorno do Check-List Fiscal</t>
+          <t>Recebimento NFCE</t>
         </is>
       </c>
       <c r="K297" t="inlineStr"/>
       <c r="L297" s="1" t="n">
-        <v>46218</v>
+        <v>46216</v>
       </c>
       <c r="M297" t="inlineStr"/>
       <c r="N297" t="inlineStr">
@@ -32863,7 +32855,7 @@
         </is>
       </c>
       <c r="O297" t="n">
-        <v>16976349</v>
+        <v>18134097</v>
       </c>
       <c r="P297" t="inlineStr">
         <is>
@@ -32876,21 +32868,17 @@
         </is>
       </c>
       <c r="R297" s="1" t="n">
-        <v>46205.7623278588</v>
+        <v>46206.7921681713</v>
       </c>
       <c r="S297" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="T297" t="inlineStr">
         <is>
-          <t>PC GAMER</t>
-        </is>
-      </c>
-      <c r="U297" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+          <t>EMPORIO DOS FRIOS</t>
+        </is>
+      </c>
+      <c r="U297" t="inlineStr"/>
       <c r="V297" t="inlineStr"/>
       <c r="W297" t="inlineStr"/>
       <c r="X297" t="inlineStr"/>
@@ -32900,7 +32888,7 @@
       </c>
       <c r="AA297" t="inlineStr">
         <is>
-          <t>Juan Rodrigues</t>
+          <t>Ricardo Fischer</t>
         </is>
       </c>
       <c r="AB297" t="inlineStr"/>
@@ -32920,11 +32908,11 @@
     </row>
     <row r="298">
       <c r="A298" t="n">
-        <v>6705</v>
+        <v>5417</v>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>NARCIZO ALVES CORDEIRO</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -32934,7 +32922,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
@@ -32944,7 +32932,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G298" t="n">
@@ -32974,7 +32962,7 @@
         </is>
       </c>
       <c r="O298" t="n">
-        <v>17949077</v>
+        <v>17399452</v>
       </c>
       <c r="P298" t="inlineStr">
         <is>
@@ -32987,14 +32975,14 @@
         </is>
       </c>
       <c r="R298" s="1" t="n">
-        <v>46205.76232913195</v>
+        <v>46210.37424872685</v>
       </c>
       <c r="S298" t="n">
         <v>-5</v>
       </c>
       <c r="T298" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U298" t="inlineStr">
@@ -33002,7 +32990,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V298" t="inlineStr"/>
+      <c r="V298" t="inlineStr">
+        <is>
+          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 07/07/2026 08:56:44. - Data Comentário: 07/07/2026 08:55</t>
+        </is>
+      </c>
       <c r="W298" t="inlineStr"/>
       <c r="X298" t="inlineStr"/>
       <c r="Y298" t="inlineStr"/>
@@ -33011,7 +33003,7 @@
       </c>
       <c r="AA298" t="inlineStr">
         <is>
-          <t>Juan Rodrigues</t>
+          <t>ex-funcionario</t>
         </is>
       </c>
       <c r="AB298" t="inlineStr"/>
@@ -33031,11 +33023,11 @@
     </row>
     <row r="299">
       <c r="A299" t="n">
-        <v>6885</v>
+        <v>6279</v>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
+          <t>DIENNYFER DA S PEREIRA</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -33045,7 +33037,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -33055,7 +33047,7 @@
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G299" t="n">
@@ -33085,7 +33077,7 @@
         </is>
       </c>
       <c r="O299" t="n">
-        <v>18134169</v>
+        <v>17071101</v>
       </c>
       <c r="P299" t="inlineStr">
         <is>
@@ -33098,7 +33090,7 @@
         </is>
       </c>
       <c r="R299" s="1" t="n">
-        <v>46211.39581168981</v>
+        <v>46205.76232731481</v>
       </c>
       <c r="S299" t="n">
         <v>-5</v>
@@ -33108,12 +33100,12 @@
           <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
-      <c r="U299" t="inlineStr"/>
-      <c r="V299" t="inlineStr">
-        <is>
-          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 08/07/2026 09:27:45. - Data Comentário: 08/07/2026 09:26</t>
-        </is>
-      </c>
+      <c r="U299" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V299" t="inlineStr"/>
       <c r="W299" t="inlineStr"/>
       <c r="X299" t="inlineStr"/>
       <c r="Y299" t="inlineStr"/>
@@ -33122,7 +33114,7 @@
       </c>
       <c r="AA299" t="inlineStr">
         <is>
-          <t>ex-funcionario</t>
+          <t>Juan Rodrigues</t>
         </is>
       </c>
       <c r="AB299" t="inlineStr"/>
@@ -33142,11 +33134,11 @@
     </row>
     <row r="300">
       <c r="A300" t="n">
-        <v>6703</v>
+        <v>6486</v>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -33156,7 +33148,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -33170,24 +33162,24 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>950</v>
+        <v>11303</v>
       </c>
       <c r="H300" t="n">
         <v>0</v>
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J300" t="inlineStr">
         <is>
-          <t>Confirm Rec - ISS Prestados</t>
+          <t>Retorno do Check-List Fiscal</t>
         </is>
       </c>
       <c r="K300" t="inlineStr"/>
       <c r="L300" s="1" t="n">
-        <v>46213</v>
+        <v>46218</v>
       </c>
       <c r="M300" t="inlineStr"/>
       <c r="N300" t="inlineStr">
@@ -33196,11 +33188,11 @@
         </is>
       </c>
       <c r="O300" t="n">
-        <v>17941144</v>
+        <v>16976349</v>
       </c>
       <c r="P300" t="inlineStr">
         <is>
-          <t>Victoria Virgens</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="Q300" t="inlineStr">
@@ -33209,14 +33201,14 @@
         </is>
       </c>
       <c r="R300" s="1" t="n">
-        <v>46210.67626055556</v>
+        <v>46205.7623278588</v>
       </c>
       <c r="S300" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="T300" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U300" t="inlineStr">
@@ -33224,11 +33216,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V300" t="inlineStr">
-        <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1792] sendo a ultima baixa feita [1792]-06/07/2026 17:54:38.. - Data Comentário: 06/07/2026 17:53</t>
-        </is>
-      </c>
+      <c r="V300" t="inlineStr"/>
       <c r="W300" t="inlineStr"/>
       <c r="X300" t="inlineStr"/>
       <c r="Y300" t="inlineStr"/>
@@ -33237,7 +33225,7 @@
       </c>
       <c r="AA300" t="inlineStr">
         <is>
-          <t>Victoria Virgens</t>
+          <t>Juan Rodrigues</t>
         </is>
       </c>
       <c r="AB300" t="inlineStr"/>
@@ -33246,18 +33234,22 @@
       <c r="AE300" t="inlineStr"/>
       <c r="AF300" t="inlineStr">
         <is>
-          <t>Imposto</t>
-        </is>
-      </c>
-      <c r="AG300" t="inlineStr"/>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AG300" t="inlineStr">
+        <is>
+          <t>Ricardo Fischer</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="n">
-        <v>6704</v>
+        <v>6705</v>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>NARCIZO ALVES CORDEIRO</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -33267,7 +33259,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
@@ -33281,24 +33273,24 @@
         </is>
       </c>
       <c r="G301" t="n">
-        <v>950</v>
+        <v>11303</v>
       </c>
       <c r="H301" t="n">
         <v>0</v>
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J301" t="inlineStr">
         <is>
-          <t>Confirm Rec - ISS Prestados</t>
+          <t>Retorno do Check-List Fiscal</t>
         </is>
       </c>
       <c r="K301" t="inlineStr"/>
       <c r="L301" s="1" t="n">
-        <v>46213</v>
+        <v>46218</v>
       </c>
       <c r="M301" t="inlineStr"/>
       <c r="N301" t="inlineStr">
@@ -33307,11 +33299,11 @@
         </is>
       </c>
       <c r="O301" t="n">
-        <v>17952338</v>
+        <v>17949077</v>
       </c>
       <c r="P301" t="inlineStr">
         <is>
-          <t>Victoria Virgens</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="Q301" t="inlineStr">
@@ -33320,10 +33312,10 @@
         </is>
       </c>
       <c r="R301" s="1" t="n">
-        <v>46210.60626501157</v>
+        <v>46205.76232913195</v>
       </c>
       <c r="S301" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="T301" t="inlineStr">
         <is>
@@ -33335,11 +33327,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V301" t="inlineStr">
-        <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1792] sendo a ultima baixa feita [1792]-06/07/2026 14:56:57.. - Data Comentário: 06/07/2026 14:56</t>
-        </is>
-      </c>
+      <c r="V301" t="inlineStr"/>
       <c r="W301" t="inlineStr"/>
       <c r="X301" t="inlineStr"/>
       <c r="Y301" t="inlineStr"/>
@@ -33348,7 +33336,7 @@
       </c>
       <c r="AA301" t="inlineStr">
         <is>
-          <t>Victoria Virgens</t>
+          <t>Juan Rodrigues</t>
         </is>
       </c>
       <c r="AB301" t="inlineStr"/>
@@ -33357,18 +33345,22 @@
       <c r="AE301" t="inlineStr"/>
       <c r="AF301" t="inlineStr">
         <is>
-          <t>Imposto</t>
-        </is>
-      </c>
-      <c r="AG301" t="inlineStr"/>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AG301" t="inlineStr">
+        <is>
+          <t>Ricardo Fischer</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="n">
-        <v>6548</v>
+        <v>6885</v>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM LTDA</t>
+          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -33378,7 +33370,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
@@ -33392,24 +33384,24 @@
         </is>
       </c>
       <c r="G302" t="n">
-        <v>951</v>
+        <v>11303</v>
       </c>
       <c r="H302" t="n">
         <v>0</v>
       </c>
       <c r="I302" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J302" t="inlineStr">
         <is>
-          <t>Confirm Rec - ISS Tomados</t>
+          <t>Retorno do Check-List Fiscal</t>
         </is>
       </c>
       <c r="K302" t="inlineStr"/>
       <c r="L302" s="1" t="n">
-        <v>46213</v>
+        <v>46218</v>
       </c>
       <c r="M302" t="inlineStr"/>
       <c r="N302" t="inlineStr">
@@ -33418,11 +33410,11 @@
         </is>
       </c>
       <c r="O302" t="n">
-        <v>17222400</v>
+        <v>18134169</v>
       </c>
       <c r="P302" t="inlineStr">
         <is>
-          <t>Victoria Virgens</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="Q302" t="inlineStr">
@@ -33431,24 +33423,20 @@
         </is>
       </c>
       <c r="R302" s="1" t="n">
-        <v>46210.76622931713</v>
+        <v>46211.39581168981</v>
       </c>
       <c r="S302" t="n">
-        <v>0</v>
+        <v>-5</v>
       </c>
       <c r="T302" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM</t>
-        </is>
-      </c>
-      <c r="U302" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+          <t>EMPORIO DOS FRIOS</t>
+        </is>
+      </c>
+      <c r="U302" t="inlineStr"/>
       <c r="V302" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-07/07/2026 15:21:27.. - Data Comentário: 07/07/2026 15:20</t>
+          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 08/07/2026 09:27:45. - Data Comentário: 08/07/2026 09:26</t>
         </is>
       </c>
       <c r="W302" t="inlineStr"/>
@@ -33459,7 +33447,7 @@
       </c>
       <c r="AA302" t="inlineStr">
         <is>
-          <t>Victoria Virgens</t>
+          <t>ex-funcionario</t>
         </is>
       </c>
       <c r="AB302" t="inlineStr"/>
@@ -33468,18 +33456,22 @@
       <c r="AE302" t="inlineStr"/>
       <c r="AF302" t="inlineStr">
         <is>
-          <t>Imposto</t>
-        </is>
-      </c>
-      <c r="AG302" t="inlineStr"/>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AG302" t="inlineStr">
+        <is>
+          <t>Ricardo Fischer</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="n">
-        <v>6628</v>
+        <v>6703</v>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -33489,12 +33481,12 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
@@ -33503,7 +33495,7 @@
         </is>
       </c>
       <c r="G303" t="n">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H303" t="n">
         <v>0</v>
@@ -33515,7 +33507,7 @@
       </c>
       <c r="J303" t="inlineStr">
         <is>
-          <t>Confirm Rec - ISS Tomados</t>
+          <t>Confirm Rec - ISS Prestados</t>
         </is>
       </c>
       <c r="K303" t="inlineStr"/>
@@ -33529,7 +33521,7 @@
         </is>
       </c>
       <c r="O303" t="n">
-        <v>16959948</v>
+        <v>17941144</v>
       </c>
       <c r="P303" t="inlineStr">
         <is>
@@ -33542,14 +33534,14 @@
         </is>
       </c>
       <c r="R303" s="1" t="n">
-        <v>46210.6898024537</v>
+        <v>46210.67626055556</v>
       </c>
       <c r="S303" t="n">
         <v>0</v>
       </c>
       <c r="T303" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>LIMA MOTA</t>
         </is>
       </c>
       <c r="U303" t="inlineStr">
@@ -33557,7 +33549,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V303" t="inlineStr"/>
+      <c r="V303" t="inlineStr">
+        <is>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1792] sendo a ultima baixa feita [1792]-06/07/2026 17:54:38.. - Data Comentário: 06/07/2026 17:53</t>
+        </is>
+      </c>
       <c r="W303" t="inlineStr"/>
       <c r="X303" t="inlineStr"/>
       <c r="Y303" t="inlineStr"/>
@@ -33582,11 +33578,11 @@
     </row>
     <row r="304">
       <c r="A304" t="n">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -33596,7 +33592,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
@@ -33610,7 +33606,7 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="H304" t="n">
         <v>0</v>
@@ -33622,7 +33618,7 @@
       </c>
       <c r="J304" t="inlineStr">
         <is>
-          <t>Confirm Rec - ISS Tomados</t>
+          <t>Confirm Rec - ISS Prestados</t>
         </is>
       </c>
       <c r="K304" t="inlineStr"/>
@@ -33636,7 +33632,7 @@
         </is>
       </c>
       <c r="O304" t="n">
-        <v>17941154</v>
+        <v>17952338</v>
       </c>
       <c r="P304" t="inlineStr">
         <is>
@@ -33649,14 +33645,14 @@
         </is>
       </c>
       <c r="R304" s="1" t="n">
-        <v>46210.76516364583</v>
+        <v>46210.60626501157</v>
       </c>
       <c r="S304" t="n">
         <v>0</v>
       </c>
       <c r="T304" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U304" t="inlineStr">
@@ -33666,7 +33662,7 @@
       </c>
       <c r="V304" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1793] sendo a ultima baixa feita [1793]-03/07/2026 12:03:31.. - Data Comentário: 03/07/2026 12:02</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1792] sendo a ultima baixa feita [1792]-06/07/2026 14:56:57.. - Data Comentário: 06/07/2026 14:56</t>
         </is>
       </c>
       <c r="W304" t="inlineStr"/>
@@ -33693,11 +33689,11 @@
     </row>
     <row r="305">
       <c r="A305" t="n">
-        <v>6704</v>
+        <v>6548</v>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>GOIAS SILAGEM LTDA</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -33747,7 +33743,7 @@
         </is>
       </c>
       <c r="O305" t="n">
-        <v>17952349</v>
+        <v>17222400</v>
       </c>
       <c r="P305" t="inlineStr">
         <is>
@@ -33760,14 +33756,14 @@
         </is>
       </c>
       <c r="R305" s="1" t="n">
-        <v>46213.34372746528</v>
+        <v>46210.76622931713</v>
       </c>
       <c r="S305" t="n">
         <v>0</v>
       </c>
       <c r="T305" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>GOIAS SILAGEM</t>
         </is>
       </c>
       <c r="U305" t="inlineStr">
@@ -33777,7 +33773,7 @@
       </c>
       <c r="V305" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1793] sendo a ultima baixa feita [1793]-07/07/2026 19:15:35.. - Data Comentário: 07/07/2026 19:15</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-07/07/2026 15:21:27.. - Data Comentário: 07/07/2026 15:20</t>
         </is>
       </c>
       <c r="W305" t="inlineStr"/>
@@ -33804,11 +33800,11 @@
     </row>
     <row r="306">
       <c r="A306" t="n">
-        <v>6705</v>
+        <v>6628</v>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>NARCIZO ALVES CORDEIRO</t>
+          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -33823,7 +33819,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
@@ -33858,7 +33854,7 @@
         </is>
       </c>
       <c r="O306" t="n">
-        <v>17952533</v>
+        <v>16959948</v>
       </c>
       <c r="P306" t="inlineStr">
         <is>
@@ -33871,14 +33867,14 @@
         </is>
       </c>
       <c r="R306" s="1" t="n">
-        <v>46057.4012012963</v>
+        <v>46210.6898024537</v>
       </c>
       <c r="S306" t="n">
         <v>0</v>
       </c>
       <c r="T306" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U306" t="inlineStr">
@@ -33895,7 +33891,7 @@
       </c>
       <c r="AA306" t="inlineStr">
         <is>
-          <t>ex-funcionario</t>
+          <t>Victoria Virgens</t>
         </is>
       </c>
       <c r="AB306" t="inlineStr"/>
@@ -33911,11 +33907,11 @@
     </row>
     <row r="307">
       <c r="A307" t="n">
-        <v>6779</v>
+        <v>6703</v>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>CORDEIRO E CIA LTDA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -33925,7 +33921,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
@@ -33965,7 +33961,7 @@
         </is>
       </c>
       <c r="O307" t="n">
-        <v>18056703</v>
+        <v>17941154</v>
       </c>
       <c r="P307" t="inlineStr">
         <is>
@@ -33978,20 +33974,24 @@
         </is>
       </c>
       <c r="R307" s="1" t="n">
-        <v>46204.41790648148</v>
+        <v>46210.76516364583</v>
       </c>
       <c r="S307" t="n">
         <v>0</v>
       </c>
       <c r="T307" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
-        </is>
-      </c>
-      <c r="U307" t="inlineStr"/>
+          <t>LIMA MOTA</t>
+        </is>
+      </c>
+      <c r="U307" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="V307" t="inlineStr">
         <is>
-          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1793]. - Data Comentário: 01/07/2026 10:00</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1793] sendo a ultima baixa feita [1793]-03/07/2026 12:03:31.. - Data Comentário: 03/07/2026 12:02</t>
         </is>
       </c>
       <c r="W307" t="inlineStr"/>
@@ -34002,7 +34002,7 @@
       </c>
       <c r="AA307" t="inlineStr">
         <is>
-          <t>ex-funcionario</t>
+          <t>Victoria Virgens</t>
         </is>
       </c>
       <c r="AB307" t="inlineStr"/>
@@ -34018,11 +34018,11 @@
     </row>
     <row r="308">
       <c r="A308" t="n">
-        <v>6885</v>
+        <v>6704</v>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -34032,7 +34032,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
@@ -34072,7 +34072,7 @@
         </is>
       </c>
       <c r="O308" t="n">
-        <v>18128657</v>
+        <v>17952349</v>
       </c>
       <c r="P308" t="inlineStr">
         <is>
@@ -34085,20 +34085,24 @@
         </is>
       </c>
       <c r="R308" s="1" t="n">
-        <v>46204.4179340625</v>
+        <v>46213.34372746528</v>
       </c>
       <c r="S308" t="n">
         <v>0</v>
       </c>
       <c r="T308" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
-        </is>
-      </c>
-      <c r="U308" t="inlineStr"/>
+          <t>TECNO COM</t>
+        </is>
+      </c>
+      <c r="U308" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="V308" t="inlineStr">
         <is>
-          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1793]. - Data Comentário: 01/07/2026 10:00</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1793] sendo a ultima baixa feita [1793]-07/07/2026 19:15:35.. - Data Comentário: 07/07/2026 19:15</t>
         </is>
       </c>
       <c r="W308" t="inlineStr"/>
@@ -34109,7 +34113,7 @@
       </c>
       <c r="AA308" t="inlineStr">
         <is>
-          <t>ex-funcionario</t>
+          <t>Victoria Virgens</t>
         </is>
       </c>
       <c r="AB308" t="inlineStr"/>
@@ -85545,7 +85549,7 @@
       <c r="V800" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 10/07/2026 
-Previsão de Conclusão 10/07/2026 - Data Comentário: 08/07/2026 14:46</t>
+Em decorrência das alterações da cbenef iremos concluir em 10/07 - Data Comentário: 10/07/2026 09:38</t>
         </is>
       </c>
       <c r="W800" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-10 17:49
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -2572,7 +2572,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>13/07/2026</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2605,8 +2605,8 @@
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 10/07/2026 
-Empresa Implantação em processamento. - Data Comentário: 07/07/2026 15:25</t>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 13/07/2026 
+Empresa Implantação em processamento. - Data Comentário: 10/07/2026 17:01</t>
         </is>
       </c>
       <c r="W20" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-12 00:08
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -84502,7 +84502,7 @@
       </c>
       <c r="R789" t="inlineStr"/>
       <c r="S789" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T789" t="inlineStr">
         <is>
@@ -84606,7 +84606,7 @@
       </c>
       <c r="R790" t="inlineStr"/>
       <c r="S790" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T790" t="inlineStr">
         <is>
@@ -84710,7 +84710,7 @@
       </c>
       <c r="R791" t="inlineStr"/>
       <c r="S791" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T791" t="inlineStr">
         <is>
@@ -84810,7 +84810,7 @@
       </c>
       <c r="R792" t="inlineStr"/>
       <c r="S792" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T792" t="inlineStr">
         <is>
@@ -84918,7 +84918,7 @@
       </c>
       <c r="R793" t="inlineStr"/>
       <c r="S793" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T793" t="inlineStr">
         <is>
@@ -85026,7 +85026,7 @@
       </c>
       <c r="R794" t="inlineStr"/>
       <c r="S794" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T794" t="inlineStr">
         <is>
@@ -85138,7 +85138,7 @@
       </c>
       <c r="R795" t="inlineStr"/>
       <c r="S795" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T795" t="inlineStr">
         <is>
@@ -85242,7 +85242,7 @@
       </c>
       <c r="R796" t="inlineStr"/>
       <c r="S796" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T796" t="inlineStr">
         <is>
@@ -85346,7 +85346,7 @@
       </c>
       <c r="R797" t="inlineStr"/>
       <c r="S797" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T797" t="inlineStr">
         <is>
@@ -85450,7 +85450,7 @@
       </c>
       <c r="R798" t="inlineStr"/>
       <c r="S798" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="T798" t="inlineStr">
         <is>
@@ -85565,7 +85565,7 @@
       </c>
       <c r="R799" t="inlineStr"/>
       <c r="S799" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="T799" t="inlineStr">
         <is>
@@ -85680,7 +85680,7 @@
       </c>
       <c r="R800" t="inlineStr"/>
       <c r="S800" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="T800" t="inlineStr">
         <is>
@@ -85795,7 +85795,7 @@
       </c>
       <c r="R801" t="inlineStr"/>
       <c r="S801" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T801" t="inlineStr">
         <is>
@@ -85898,7 +85898,7 @@
       </c>
       <c r="R802" t="inlineStr"/>
       <c r="S802" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T802" t="inlineStr">
         <is>
@@ -86001,7 +86001,7 @@
       </c>
       <c r="R803" t="inlineStr"/>
       <c r="S803" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T803" t="inlineStr">
         <is>
@@ -86108,7 +86108,7 @@
       </c>
       <c r="R804" t="inlineStr"/>
       <c r="S804" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="T804" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-13 00:08
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -84556,7 +84556,7 @@
       </c>
       <c r="R789" t="inlineStr"/>
       <c r="S789" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T789" t="inlineStr">
         <is>
@@ -84660,7 +84660,7 @@
       </c>
       <c r="R790" t="inlineStr"/>
       <c r="S790" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T790" t="inlineStr">
         <is>
@@ -84764,7 +84764,7 @@
       </c>
       <c r="R791" t="inlineStr"/>
       <c r="S791" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T791" t="inlineStr">
         <is>
@@ -84864,7 +84864,7 @@
       </c>
       <c r="R792" t="inlineStr"/>
       <c r="S792" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T792" t="inlineStr">
         <is>
@@ -84972,7 +84972,7 @@
       </c>
       <c r="R793" t="inlineStr"/>
       <c r="S793" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="T793" t="inlineStr">
         <is>
@@ -85080,7 +85080,7 @@
       </c>
       <c r="R794" t="inlineStr"/>
       <c r="S794" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T794" t="inlineStr">
         <is>
@@ -85192,7 +85192,7 @@
       </c>
       <c r="R795" t="inlineStr"/>
       <c r="S795" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T795" t="inlineStr">
         <is>
@@ -85296,7 +85296,7 @@
       </c>
       <c r="R796" t="inlineStr"/>
       <c r="S796" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T796" t="inlineStr">
         <is>
@@ -85400,7 +85400,7 @@
       </c>
       <c r="R797" t="inlineStr"/>
       <c r="S797" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T797" t="inlineStr">
         <is>
@@ -85504,7 +85504,7 @@
       </c>
       <c r="R798" t="inlineStr"/>
       <c r="S798" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="T798" t="inlineStr">
         <is>
@@ -85619,7 +85619,7 @@
       </c>
       <c r="R799" t="inlineStr"/>
       <c r="S799" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="T799" t="inlineStr">
         <is>
@@ -85734,7 +85734,7 @@
       </c>
       <c r="R800" t="inlineStr"/>
       <c r="S800" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="T800" t="inlineStr">
         <is>
@@ -85849,7 +85849,7 @@
       </c>
       <c r="R801" t="inlineStr"/>
       <c r="S801" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T801" t="inlineStr">
         <is>
@@ -85952,7 +85952,7 @@
       </c>
       <c r="R802" t="inlineStr"/>
       <c r="S802" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T802" t="inlineStr">
         <is>
@@ -86055,7 +86055,7 @@
       </c>
       <c r="R803" t="inlineStr"/>
       <c r="S803" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T803" t="inlineStr">
         <is>
@@ -86162,7 +86162,7 @@
       </c>
       <c r="R804" t="inlineStr"/>
       <c r="S804" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="T804" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-13 10:09
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -2366,7 +2366,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>13/07/2026</t>
+          <t>14/07/2026</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2403,8 +2403,8 @@
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 13/07/2026 
-Foi enviada para a empresa planilha de reajuste e informações sobre termo aditivo do sindicato. Estamos aguardando retorno para aplicação e calculo das complementares. - Data Comentário: 07/07/2026 16:24</t>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 14/07/2026 
+Foi enviada para a empresa planilha de reajuste e informações sobre termo aditivo do sindicato. Estamos aguardando retorno para aplicação e calculo das complementares. - Data Comentário: 13/07/2026 09:43</t>
         </is>
       </c>
       <c r="W18" t="inlineStr"/>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>13/07/2026</t>
+          <t>14/07/2026</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2828,8 +2828,8 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 
-PREVISÃO DE CONCLUSÃO: 13/07/2026 - Data Comentário: 07/07/2026 16:32</t>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 14/07/2026 
+PREVISÃO DE CONCLUSÃO: 14/07/2026 - Data Comentário: 13/07/2026 09:52</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -2905,7 +2905,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>14/07/2026</t>
+          <t>15/07/2026</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2942,8 +2942,8 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 14/07/2026 
-Previsão pra finalizar em 14/07/2026 - Data Comentário: 13/07/2026 08:27</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 15/07/2026 
+Previsão pra finalizar em 15/07/2026 - Data Comentário: 13/07/2026 09:06</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -3468,7 +3468,11 @@
       <c r="L28" s="1" t="n">
         <v>46218</v>
       </c>
-      <c r="M28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
       <c r="N28" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -3497,7 +3501,12 @@
         </is>
       </c>
       <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr"/>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 14/07/2026 
+Previsão de conclusão: 14/07/2026 - Data Comentário: 13/07/2026 09:31</t>
+        </is>
+      </c>
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr"/>
       <c r="Y28" t="inlineStr"/>
@@ -3569,7 +3578,11 @@
       <c r="L29" s="1" t="n">
         <v>46218</v>
       </c>
-      <c r="M29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
       <c r="N29" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -3598,7 +3611,12 @@
         </is>
       </c>
       <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 14/07/2026 
+Empresa em implantação. - Data Comentário: 13/07/2026 09:25</t>
+        </is>
+      </c>
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
       <c r="Y29" t="inlineStr"/>
@@ -84601,12 +84619,12 @@
       <c r="AC789" t="inlineStr"/>
       <c r="AD789" t="inlineStr">
         <is>
-          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09 - Data Comentário: 06/07/2026 12:41</t>
+          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09. - Data Comentário: 13/07/2026 09:09</t>
         </is>
       </c>
       <c r="AE789" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>17/07/2026</t>
         </is>
       </c>
       <c r="AF789" t="inlineStr">
@@ -84709,12 +84727,12 @@
       <c r="AC790" t="inlineStr"/>
       <c r="AD790" t="inlineStr">
         <is>
-          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09 - Data Comentário: 06/07/2026 12:41</t>
+          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09. - Data Comentário: 13/07/2026 09:09</t>
         </is>
       </c>
       <c r="AE790" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>17/07/2026</t>
         </is>
       </c>
       <c r="AF790" t="inlineStr">
@@ -84817,12 +84835,12 @@
       <c r="AC791" t="inlineStr"/>
       <c r="AD791" t="inlineStr">
         <is>
-          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09 - Data Comentário: 06/07/2026 12:41</t>
+          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09. - Data Comentário: 13/07/2026 09:09</t>
         </is>
       </c>
       <c r="AE791" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>17/07/2026</t>
         </is>
       </c>
       <c r="AF791" t="inlineStr">
@@ -84932,12 +84950,12 @@
       <c r="AC792" t="inlineStr"/>
       <c r="AD792" t="inlineStr">
         <is>
-          <t>A operação e o GC estão ajustando os créditos de meses anteriores para que o valor desse mês seja ajustado. A Gerente Priscila Volpe está em contato direto com o GC e informou que a tarefa deve ser concluída até o fim desta semana. - Data Comentário: 06/07/2026 12:41</t>
+          <t>A operação e o GC estão ajustando os créditos de meses anteriores para que o valor desse mês seja ajustado. A Gerente Priscila Volpe está em contato direto com o GC e informou que a tarefa será concluída o quanto antes - Data Comentário: 13/07/2026 09:09</t>
         </is>
       </c>
       <c r="AE792" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>17/07/2026</t>
         </is>
       </c>
       <c r="AF792" t="inlineStr">
@@ -85162,12 +85180,12 @@
       <c r="AC794" t="inlineStr"/>
       <c r="AD794" t="inlineStr">
         <is>
-          <t>Atraso do cliente, o atraso do cliente já é recorrente e de ciência do Master e do Gerente de Contas. - Data Comentário: 10/07/2026 10:23</t>
+          <t>Atraso do cliente, o atraso do cliente já é recorrente e de ciência do Master e do Gerente de Contas. - Data Comentário: 10/07/2026 10:23 - Data Comentário: 13/07/2026 09:09</t>
         </is>
       </c>
       <c r="AE794" t="inlineStr">
         <is>
-          <t>10/07/2026</t>
+          <t>17/07/2026</t>
         </is>
       </c>
       <c r="AF794" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-13 13:09
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -2478,7 +2478,11 @@
       <c r="L19" s="1" t="n">
         <v>46218</v>
       </c>
-      <c r="M19" t="inlineStr"/>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -2511,7 +2515,12 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr"/>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 14/07/2026 
+Em processo de emissão - Data Comentário: 13/07/2026 11:58</t>
+        </is>
+      </c>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
       <c r="Y19" t="inlineStr"/>
@@ -4767,7 +4776,11 @@
       <c r="L40" s="1" t="n">
         <v>46218</v>
       </c>
-      <c r="M40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="N40" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -4800,7 +4813,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V40" t="inlineStr"/>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 15/07/2026 - Data Comentário: 13/07/2026 12:06</t>
+        </is>
+      </c>
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr"/>
       <c r="Y40" t="inlineStr"/>
@@ -4872,7 +4889,11 @@
       <c r="L41" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="M41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
       <c r="N41" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -4905,7 +4926,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V41" t="inlineStr"/>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
+        </is>
+      </c>
       <c r="W41" t="inlineStr"/>
       <c r="X41" t="inlineStr"/>
       <c r="Y41" t="inlineStr"/>
@@ -4977,7 +5002,11 @@
       <c r="L42" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="M42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
       <c r="N42" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -5010,7 +5039,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V42" t="inlineStr"/>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
+        </is>
+      </c>
       <c r="W42" t="inlineStr"/>
       <c r="X42" t="inlineStr"/>
       <c r="Y42" t="inlineStr"/>
@@ -5082,7 +5115,11 @@
       <c r="L43" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
       <c r="N43" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -5115,7 +5152,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr"/>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
+        </is>
+      </c>
       <c r="W43" t="inlineStr"/>
       <c r="X43" t="inlineStr"/>
       <c r="Y43" t="inlineStr"/>
@@ -5187,7 +5228,11 @@
       <c r="L44" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="M44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
       <c r="N44" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -5220,7 +5265,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V44" t="inlineStr"/>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
+        </is>
+      </c>
       <c r="W44" t="inlineStr"/>
       <c r="X44" t="inlineStr"/>
       <c r="Y44" t="inlineStr"/>
@@ -5292,7 +5341,11 @@
       <c r="L45" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="M45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
       <c r="N45" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -5325,7 +5378,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr"/>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
+        </is>
+      </c>
       <c r="W45" t="inlineStr"/>
       <c r="X45" t="inlineStr"/>
       <c r="Y45" t="inlineStr"/>
@@ -5397,7 +5454,11 @@
       <c r="L46" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="M46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
       <c r="N46" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -5430,7 +5491,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr"/>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
+        </is>
+      </c>
       <c r="W46" t="inlineStr"/>
       <c r="X46" t="inlineStr"/>
       <c r="Y46" t="inlineStr"/>
@@ -5502,7 +5567,11 @@
       <c r="L47" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="M47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
       <c r="N47" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -5535,7 +5604,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V47" t="inlineStr"/>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
+        </is>
+      </c>
       <c r="W47" t="inlineStr"/>
       <c r="X47" t="inlineStr"/>
       <c r="Y47" t="inlineStr"/>
@@ -5607,7 +5680,11 @@
       <c r="L48" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="M48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
       <c r="N48" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -5640,7 +5717,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V48" t="inlineStr"/>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
+        </is>
+      </c>
       <c r="W48" t="inlineStr"/>
       <c r="X48" t="inlineStr"/>
       <c r="Y48" t="inlineStr"/>
@@ -5712,7 +5793,11 @@
       <c r="L49" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="M49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
       <c r="N49" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -5745,7 +5830,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V49" t="inlineStr"/>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
+        </is>
+      </c>
       <c r="W49" t="inlineStr"/>
       <c r="X49" t="inlineStr"/>
       <c r="Y49" t="inlineStr"/>
@@ -5817,7 +5906,11 @@
       <c r="L50" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="M50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
       <c r="N50" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -5850,7 +5943,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V50" t="inlineStr"/>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
+        </is>
+      </c>
       <c r="W50" t="inlineStr"/>
       <c r="X50" t="inlineStr"/>
       <c r="Y50" t="inlineStr"/>
@@ -5922,7 +6019,11 @@
       <c r="L51" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="M51" t="inlineStr"/>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
       <c r="N51" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -5951,7 +6052,11 @@
         </is>
       </c>
       <c r="U51" t="inlineStr"/>
-      <c r="V51" t="inlineStr"/>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
+        </is>
+      </c>
       <c r="W51" t="inlineStr"/>
       <c r="X51" t="inlineStr"/>
       <c r="Y51" t="inlineStr"/>
@@ -6023,7 +6128,11 @@
       <c r="L52" s="1" t="n">
         <v>46216</v>
       </c>
-      <c r="M52" t="inlineStr"/>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
       <c r="N52" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -6052,7 +6161,11 @@
         </is>
       </c>
       <c r="U52" t="inlineStr"/>
-      <c r="V52" t="inlineStr"/>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
+        </is>
+      </c>
       <c r="W52" t="inlineStr"/>
       <c r="X52" t="inlineStr"/>
       <c r="Y52" t="inlineStr"/>
@@ -52707,7 +52820,11 @@
       <c r="L483" s="1" t="n">
         <v>46220</v>
       </c>
-      <c r="M483" t="inlineStr"/>
+      <c r="M483" t="inlineStr">
+        <is>
+          <t>16/07/2026</t>
+        </is>
+      </c>
       <c r="N483" t="inlineStr">
         <is>
           <t>07/2026</t>
@@ -52740,7 +52857,12 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V483" t="inlineStr"/>
+      <c r="V483" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 16/07/2026 
+Em processamento - Data Comentário: 13/07/2026 12:01</t>
+        </is>
+      </c>
       <c r="W483" t="inlineStr"/>
       <c r="X483" t="inlineStr"/>
       <c r="Y483" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-13 16:09
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -53182,7 +53182,11 @@
       <c r="L486" s="1" t="n">
         <v>46220</v>
       </c>
-      <c r="M486" t="inlineStr"/>
+      <c r="M486" t="inlineStr">
+        <is>
+          <t>15/07/2026</t>
+        </is>
+      </c>
       <c r="N486" t="inlineStr">
         <is>
           <t>07/2026</t>
@@ -53211,7 +53215,12 @@
         </is>
       </c>
       <c r="U486" t="inlineStr"/>
-      <c r="V486" t="inlineStr"/>
+      <c r="V486" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 15/07/2026 
+Previsão de conclusão 15/07/2026 - Data Comentário: 13/07/2026 15:28</t>
+        </is>
+      </c>
       <c r="W486" t="inlineStr"/>
       <c r="X486" t="inlineStr"/>
       <c r="Y486" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-13 17:09
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -17131,11 +17131,7 @@
       <c r="O151" t="n">
         <v>18199991</v>
       </c>
-      <c r="P151" t="inlineStr">
-        <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
+      <c r="P151" t="inlineStr"/>
       <c r="Q151" t="inlineStr">
         <is>
           <t>Baixado</t>
@@ -17179,11 +17175,7 @@
           <t>Imposto</t>
         </is>
       </c>
-      <c r="AG151" t="inlineStr">
-        <is>
-          <t>Leandro Matos</t>
-        </is>
-      </c>
+      <c r="AG151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -17243,11 +17235,7 @@
       <c r="O152" t="n">
         <v>18201961</v>
       </c>
-      <c r="P152" t="inlineStr">
-        <is>
-          <t>Gabriela Peres</t>
-        </is>
-      </c>
+      <c r="P152" t="inlineStr"/>
       <c r="Q152" t="inlineStr">
         <is>
           <t>Baixado</t>
@@ -17290,11 +17278,7 @@
           <t>Imposto</t>
         </is>
       </c>
-      <c r="AG152" t="inlineStr">
-        <is>
-          <t>Leandro Matos</t>
-        </is>
-      </c>
+      <c r="AG152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-13 20:17
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -3583,7 +3583,11 @@
       <c r="L29" s="1" t="n">
         <v>46218</v>
       </c>
-      <c r="M29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
       <c r="N29" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -3616,7 +3620,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 14/07/2026 - Data Comentário: 13/07/2026 19:28</t>
+        </is>
+      </c>
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr"/>
       <c r="Y29" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-14 00:09
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -42837,7 +42837,7 @@
       </c>
       <c r="R386" t="inlineStr"/>
       <c r="S386" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T386" t="inlineStr">
         <is>
@@ -42942,7 +42942,7 @@
       </c>
       <c r="R387" t="inlineStr"/>
       <c r="S387" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T387" t="inlineStr">
         <is>
@@ -43047,7 +43047,7 @@
       </c>
       <c r="R388" t="inlineStr"/>
       <c r="S388" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T388" t="inlineStr">
         <is>
@@ -43152,7 +43152,7 @@
       </c>
       <c r="R389" t="inlineStr"/>
       <c r="S389" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T389" t="inlineStr">
         <is>
@@ -43253,7 +43253,7 @@
       </c>
       <c r="R390" t="inlineStr"/>
       <c r="S390" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T390" t="inlineStr">
         <is>
@@ -43354,7 +43354,7 @@
       </c>
       <c r="R391" t="inlineStr"/>
       <c r="S391" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T391" t="inlineStr">
         <is>
@@ -43455,7 +43455,7 @@
       </c>
       <c r="R392" t="inlineStr"/>
       <c r="S392" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T392" t="inlineStr">
         <is>
@@ -43560,7 +43560,7 @@
       </c>
       <c r="R393" t="inlineStr"/>
       <c r="S393" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T393" t="inlineStr">
         <is>
@@ -43665,7 +43665,7 @@
       </c>
       <c r="R394" t="inlineStr"/>
       <c r="S394" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T394" t="inlineStr">
         <is>
@@ -43770,7 +43770,7 @@
       </c>
       <c r="R395" t="inlineStr"/>
       <c r="S395" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T395" t="inlineStr">
         <is>
@@ -43875,7 +43875,7 @@
       </c>
       <c r="R396" t="inlineStr"/>
       <c r="S396" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T396" t="inlineStr">
         <is>
@@ -43980,7 +43980,7 @@
       </c>
       <c r="R397" t="inlineStr"/>
       <c r="S397" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T397" t="inlineStr">
         <is>
@@ -44081,7 +44081,7 @@
       </c>
       <c r="R398" t="inlineStr"/>
       <c r="S398" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T398" t="inlineStr">
         <is>
@@ -44182,7 +44182,7 @@
       </c>
       <c r="R399" t="inlineStr"/>
       <c r="S399" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T399" t="inlineStr">
         <is>
@@ -44283,7 +44283,7 @@
       </c>
       <c r="R400" t="inlineStr"/>
       <c r="S400" t="n">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="T400" t="inlineStr">
         <is>
@@ -44388,7 +44388,7 @@
       </c>
       <c r="R401" t="inlineStr"/>
       <c r="S401" t="n">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="T401" t="inlineStr">
         <is>
@@ -44493,7 +44493,7 @@
       </c>
       <c r="R402" t="inlineStr"/>
       <c r="S402" t="n">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="T402" t="inlineStr">
         <is>
@@ -44594,7 +44594,7 @@
       </c>
       <c r="R403" t="inlineStr"/>
       <c r="S403" t="n">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="T403" t="inlineStr">
         <is>
@@ -44695,7 +44695,7 @@
       </c>
       <c r="R404" t="inlineStr"/>
       <c r="S404" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T404" t="inlineStr">
         <is>
@@ -44800,7 +44800,7 @@
       </c>
       <c r="R405" t="inlineStr"/>
       <c r="S405" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T405" t="inlineStr">
         <is>
@@ -44905,7 +44905,7 @@
       </c>
       <c r="R406" t="inlineStr"/>
       <c r="S406" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T406" t="inlineStr">
         <is>
@@ -45006,7 +45006,7 @@
       </c>
       <c r="R407" t="inlineStr"/>
       <c r="S407" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T407" t="inlineStr">
         <is>
@@ -45107,7 +45107,7 @@
       </c>
       <c r="R408" t="inlineStr"/>
       <c r="S408" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T408" t="inlineStr">
         <is>
@@ -45212,7 +45212,7 @@
       </c>
       <c r="R409" t="inlineStr"/>
       <c r="S409" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T409" t="inlineStr">
         <is>
@@ -45317,7 +45317,7 @@
       </c>
       <c r="R410" t="inlineStr"/>
       <c r="S410" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T410" t="inlineStr">
         <is>
@@ -45418,7 +45418,7 @@
       </c>
       <c r="R411" t="inlineStr"/>
       <c r="S411" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T411" t="inlineStr">
         <is>
@@ -45519,7 +45519,7 @@
       </c>
       <c r="R412" t="inlineStr"/>
       <c r="S412" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T412" t="inlineStr">
         <is>
@@ -45624,7 +45624,7 @@
       </c>
       <c r="R413" t="inlineStr"/>
       <c r="S413" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T413" t="inlineStr">
         <is>
@@ -45725,7 +45725,7 @@
       </c>
       <c r="R414" t="inlineStr"/>
       <c r="S414" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T414" t="inlineStr">
         <is>
@@ -45830,7 +45830,7 @@
       </c>
       <c r="R415" t="inlineStr"/>
       <c r="S415" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T415" t="inlineStr">
         <is>
@@ -45935,7 +45935,7 @@
       </c>
       <c r="R416" t="inlineStr"/>
       <c r="S416" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T416" t="inlineStr">
         <is>
@@ -46036,7 +46036,7 @@
       </c>
       <c r="R417" t="inlineStr"/>
       <c r="S417" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T417" t="inlineStr">
         <is>
@@ -46137,7 +46137,7 @@
       </c>
       <c r="R418" t="inlineStr"/>
       <c r="S418" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T418" t="inlineStr">
         <is>
@@ -46242,7 +46242,7 @@
       </c>
       <c r="R419" t="inlineStr"/>
       <c r="S419" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T419" t="inlineStr">
         <is>
@@ -46347,7 +46347,7 @@
       </c>
       <c r="R420" t="inlineStr"/>
       <c r="S420" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T420" t="inlineStr">
         <is>
@@ -46452,7 +46452,7 @@
       </c>
       <c r="R421" t="inlineStr"/>
       <c r="S421" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T421" t="inlineStr">
         <is>
@@ -46557,7 +46557,7 @@
       </c>
       <c r="R422" t="inlineStr"/>
       <c r="S422" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T422" t="inlineStr">
         <is>
@@ -46662,7 +46662,7 @@
       </c>
       <c r="R423" t="inlineStr"/>
       <c r="S423" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T423" t="inlineStr">
         <is>
@@ -46767,7 +46767,7 @@
       </c>
       <c r="R424" t="inlineStr"/>
       <c r="S424" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T424" t="inlineStr">
         <is>
@@ -46872,7 +46872,7 @@
       </c>
       <c r="R425" t="inlineStr"/>
       <c r="S425" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T425" t="inlineStr">
         <is>
@@ -46977,7 +46977,7 @@
       </c>
       <c r="R426" t="inlineStr"/>
       <c r="S426" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T426" t="inlineStr">
         <is>
@@ -47082,7 +47082,7 @@
       </c>
       <c r="R427" t="inlineStr"/>
       <c r="S427" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T427" t="inlineStr">
         <is>
@@ -47187,7 +47187,7 @@
       </c>
       <c r="R428" t="inlineStr"/>
       <c r="S428" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T428" t="inlineStr">
         <is>
@@ -47288,7 +47288,7 @@
       </c>
       <c r="R429" t="inlineStr"/>
       <c r="S429" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T429" t="inlineStr">
         <is>
@@ -47389,7 +47389,7 @@
       </c>
       <c r="R430" t="inlineStr"/>
       <c r="S430" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T430" t="inlineStr">
         <is>
@@ -47494,7 +47494,7 @@
       </c>
       <c r="R431" t="inlineStr"/>
       <c r="S431" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T431" t="inlineStr">
         <is>
@@ -47599,7 +47599,7 @@
       </c>
       <c r="R432" t="inlineStr"/>
       <c r="S432" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T432" t="inlineStr">
         <is>
@@ -47704,7 +47704,7 @@
       </c>
       <c r="R433" t="inlineStr"/>
       <c r="S433" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T433" t="inlineStr">
         <is>
@@ -47809,7 +47809,7 @@
       </c>
       <c r="R434" t="inlineStr"/>
       <c r="S434" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T434" t="inlineStr">
         <is>
@@ -47914,7 +47914,7 @@
       </c>
       <c r="R435" t="inlineStr"/>
       <c r="S435" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T435" t="inlineStr">
         <is>
@@ -48019,7 +48019,7 @@
       </c>
       <c r="R436" t="inlineStr"/>
       <c r="S436" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T436" t="inlineStr">
         <is>
@@ -48124,7 +48124,7 @@
       </c>
       <c r="R437" t="inlineStr"/>
       <c r="S437" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T437" t="inlineStr">
         <is>
@@ -48229,7 +48229,7 @@
       </c>
       <c r="R438" t="inlineStr"/>
       <c r="S438" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T438" t="inlineStr">
         <is>
@@ -48334,7 +48334,7 @@
       </c>
       <c r="R439" t="inlineStr"/>
       <c r="S439" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T439" t="inlineStr">
         <is>
@@ -48439,7 +48439,7 @@
       </c>
       <c r="R440" t="inlineStr"/>
       <c r="S440" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T440" t="inlineStr">
         <is>
@@ -48544,7 +48544,7 @@
       </c>
       <c r="R441" t="inlineStr"/>
       <c r="S441" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T441" t="inlineStr">
         <is>
@@ -48649,7 +48649,7 @@
       </c>
       <c r="R442" t="inlineStr"/>
       <c r="S442" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T442" t="inlineStr">
         <is>
@@ -48754,7 +48754,7 @@
       </c>
       <c r="R443" t="inlineStr"/>
       <c r="S443" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T443" t="inlineStr">
         <is>
@@ -48859,7 +48859,7 @@
       </c>
       <c r="R444" t="inlineStr"/>
       <c r="S444" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T444" t="inlineStr">
         <is>
@@ -48964,7 +48964,7 @@
       </c>
       <c r="R445" t="inlineStr"/>
       <c r="S445" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T445" t="inlineStr">
         <is>
@@ -49065,7 +49065,7 @@
       </c>
       <c r="R446" t="inlineStr"/>
       <c r="S446" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T446" t="inlineStr">
         <is>
@@ -49166,7 +49166,7 @@
       </c>
       <c r="R447" t="inlineStr"/>
       <c r="S447" t="n">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="T447" t="inlineStr">
         <is>
@@ -49271,7 +49271,7 @@
       </c>
       <c r="R448" t="inlineStr"/>
       <c r="S448" t="n">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="T448" t="inlineStr">
         <is>
@@ -49376,7 +49376,7 @@
       </c>
       <c r="R449" t="inlineStr"/>
       <c r="S449" t="n">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="T449" t="inlineStr">
         <is>
@@ -49481,7 +49481,7 @@
       </c>
       <c r="R450" t="inlineStr"/>
       <c r="S450" t="n">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="T450" t="inlineStr">
         <is>
@@ -49586,7 +49586,7 @@
       </c>
       <c r="R451" t="inlineStr"/>
       <c r="S451" t="n">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="T451" t="inlineStr">
         <is>
@@ -49691,7 +49691,7 @@
       </c>
       <c r="R452" t="inlineStr"/>
       <c r="S452" t="n">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="T452" t="inlineStr">
         <is>
@@ -49796,7 +49796,7 @@
       </c>
       <c r="R453" t="inlineStr"/>
       <c r="S453" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T453" t="inlineStr">
         <is>
@@ -49901,7 +49901,7 @@
       </c>
       <c r="R454" t="inlineStr"/>
       <c r="S454" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T454" t="inlineStr">
         <is>
@@ -50006,7 +50006,7 @@
       </c>
       <c r="R455" t="inlineStr"/>
       <c r="S455" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T455" t="inlineStr">
         <is>
@@ -50111,7 +50111,7 @@
       </c>
       <c r="R456" t="inlineStr"/>
       <c r="S456" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T456" t="inlineStr">
         <is>
@@ -50216,7 +50216,7 @@
       </c>
       <c r="R457" t="inlineStr"/>
       <c r="S457" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T457" t="inlineStr">
         <is>
@@ -50321,7 +50321,7 @@
       </c>
       <c r="R458" t="inlineStr"/>
       <c r="S458" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T458" t="inlineStr">
         <is>
@@ -50426,7 +50426,7 @@
       </c>
       <c r="R459" t="inlineStr"/>
       <c r="S459" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T459" t="inlineStr">
         <is>
@@ -50531,7 +50531,7 @@
       </c>
       <c r="R460" t="inlineStr"/>
       <c r="S460" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T460" t="inlineStr">
         <is>
@@ -50636,7 +50636,7 @@
       </c>
       <c r="R461" t="inlineStr"/>
       <c r="S461" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T461" t="inlineStr">
         <is>
@@ -50741,7 +50741,7 @@
       </c>
       <c r="R462" t="inlineStr"/>
       <c r="S462" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T462" t="inlineStr">
         <is>
@@ -50846,7 +50846,7 @@
       </c>
       <c r="R463" t="inlineStr"/>
       <c r="S463" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T463" t="inlineStr">
         <is>
@@ -50951,7 +50951,7 @@
       </c>
       <c r="R464" t="inlineStr"/>
       <c r="S464" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T464" t="inlineStr">
         <is>
@@ -51056,7 +51056,7 @@
       </c>
       <c r="R465" t="inlineStr"/>
       <c r="S465" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T465" t="inlineStr">
         <is>
@@ -51161,7 +51161,7 @@
       </c>
       <c r="R466" t="inlineStr"/>
       <c r="S466" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T466" t="inlineStr">
         <is>
@@ -51266,7 +51266,7 @@
       </c>
       <c r="R467" t="inlineStr"/>
       <c r="S467" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T467" t="inlineStr">
         <is>
@@ -51371,7 +51371,7 @@
       </c>
       <c r="R468" t="inlineStr"/>
       <c r="S468" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T468" t="inlineStr">
         <is>
@@ -51476,7 +51476,7 @@
       </c>
       <c r="R469" t="inlineStr"/>
       <c r="S469" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T469" t="inlineStr">
         <is>
@@ -51581,7 +51581,7 @@
       </c>
       <c r="R470" t="inlineStr"/>
       <c r="S470" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T470" t="inlineStr">
         <is>
@@ -51686,7 +51686,7 @@
       </c>
       <c r="R471" t="inlineStr"/>
       <c r="S471" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T471" t="inlineStr">
         <is>
@@ -51791,7 +51791,7 @@
       </c>
       <c r="R472" t="inlineStr"/>
       <c r="S472" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T472" t="inlineStr">
         <is>
@@ -51896,7 +51896,7 @@
       </c>
       <c r="R473" t="inlineStr"/>
       <c r="S473" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T473" t="inlineStr">
         <is>
@@ -52001,7 +52001,7 @@
       </c>
       <c r="R474" t="inlineStr"/>
       <c r="S474" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T474" t="inlineStr">
         <is>
@@ -52106,7 +52106,7 @@
       </c>
       <c r="R475" t="inlineStr"/>
       <c r="S475" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T475" t="inlineStr">
         <is>
@@ -52207,7 +52207,7 @@
       </c>
       <c r="R476" t="inlineStr"/>
       <c r="S476" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T476" t="inlineStr">
         <is>
@@ -52308,7 +52308,7 @@
       </c>
       <c r="R477" t="inlineStr"/>
       <c r="S477" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T477" t="inlineStr">
         <is>
@@ -52413,7 +52413,7 @@
       </c>
       <c r="R478" t="inlineStr"/>
       <c r="S478" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T478" t="inlineStr">
         <is>
@@ -52518,7 +52518,7 @@
       </c>
       <c r="R479" t="inlineStr"/>
       <c r="S479" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T479" t="inlineStr">
         <is>
@@ -52623,7 +52623,7 @@
       </c>
       <c r="R480" t="inlineStr"/>
       <c r="S480" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T480" t="inlineStr">
         <is>
@@ -52728,7 +52728,7 @@
       </c>
       <c r="R481" t="inlineStr"/>
       <c r="S481" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T481" t="inlineStr">
         <is>
@@ -52833,7 +52833,7 @@
       </c>
       <c r="R482" t="inlineStr"/>
       <c r="S482" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T482" t="inlineStr">
         <is>
@@ -52942,7 +52942,7 @@
       </c>
       <c r="R483" t="inlineStr"/>
       <c r="S483" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T483" t="inlineStr">
         <is>
@@ -53052,7 +53052,7 @@
       </c>
       <c r="R484" t="inlineStr"/>
       <c r="S484" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T484" t="inlineStr">
         <is>
@@ -53166,7 +53166,7 @@
       </c>
       <c r="R485" t="inlineStr"/>
       <c r="S485" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T485" t="inlineStr">
         <is>
@@ -53280,7 +53280,7 @@
       </c>
       <c r="R486" t="inlineStr"/>
       <c r="S486" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T486" t="inlineStr">
         <is>
@@ -53386,7 +53386,7 @@
       </c>
       <c r="R487" t="inlineStr"/>
       <c r="S487" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T487" t="inlineStr">
         <is>
@@ -53495,7 +53495,7 @@
       </c>
       <c r="R488" t="inlineStr"/>
       <c r="S488" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T488" t="inlineStr">
         <is>
@@ -53604,7 +53604,7 @@
       </c>
       <c r="R489" t="inlineStr"/>
       <c r="S489" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T489" t="inlineStr">
         <is>
@@ -53717,7 +53717,7 @@
       </c>
       <c r="R490" t="inlineStr"/>
       <c r="S490" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T490" t="inlineStr">
         <is>
@@ -53831,7 +53831,7 @@
       </c>
       <c r="R491" t="inlineStr"/>
       <c r="S491" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T491" t="inlineStr">
         <is>
@@ -53941,7 +53941,7 @@
       </c>
       <c r="R492" t="inlineStr"/>
       <c r="S492" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T492" t="inlineStr">
         <is>
@@ -54046,7 +54046,7 @@
       </c>
       <c r="R493" t="inlineStr"/>
       <c r="S493" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T493" t="inlineStr">
         <is>
@@ -54147,7 +54147,7 @@
       </c>
       <c r="R494" t="inlineStr"/>
       <c r="S494" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T494" t="inlineStr">
         <is>
@@ -54248,7 +54248,7 @@
       </c>
       <c r="R495" t="inlineStr"/>
       <c r="S495" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T495" t="inlineStr">
         <is>
@@ -54353,7 +54353,7 @@
       </c>
       <c r="R496" t="inlineStr"/>
       <c r="S496" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T496" t="inlineStr">
         <is>
@@ -54458,7 +54458,7 @@
       </c>
       <c r="R497" t="inlineStr"/>
       <c r="S497" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T497" t="inlineStr">
         <is>
@@ -54563,7 +54563,7 @@
       </c>
       <c r="R498" t="inlineStr"/>
       <c r="S498" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T498" t="inlineStr">
         <is>
@@ -54668,7 +54668,7 @@
       </c>
       <c r="R499" t="inlineStr"/>
       <c r="S499" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T499" t="inlineStr">
         <is>
@@ -54773,7 +54773,7 @@
       </c>
       <c r="R500" t="inlineStr"/>
       <c r="S500" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T500" t="inlineStr">
         <is>
@@ -54878,7 +54878,7 @@
       </c>
       <c r="R501" t="inlineStr"/>
       <c r="S501" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T501" t="inlineStr">
         <is>
@@ -54983,7 +54983,7 @@
       </c>
       <c r="R502" t="inlineStr"/>
       <c r="S502" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T502" t="inlineStr">
         <is>
@@ -55084,7 +55084,7 @@
       </c>
       <c r="R503" t="inlineStr"/>
       <c r="S503" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T503" t="inlineStr">
         <is>
@@ -55185,7 +55185,7 @@
       </c>
       <c r="R504" t="inlineStr"/>
       <c r="S504" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T504" t="inlineStr">
         <is>
@@ -55286,7 +55286,7 @@
       </c>
       <c r="R505" t="inlineStr"/>
       <c r="S505" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T505" t="inlineStr">
         <is>
@@ -55387,7 +55387,7 @@
       </c>
       <c r="R506" t="inlineStr"/>
       <c r="S506" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T506" t="inlineStr">
         <is>
@@ -55488,7 +55488,7 @@
       </c>
       <c r="R507" t="inlineStr"/>
       <c r="S507" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T507" t="inlineStr">
         <is>
@@ -55593,7 +55593,7 @@
       </c>
       <c r="R508" t="inlineStr"/>
       <c r="S508" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T508" t="inlineStr">
         <is>
@@ -55698,7 +55698,7 @@
       </c>
       <c r="R509" t="inlineStr"/>
       <c r="S509" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T509" t="inlineStr">
         <is>
@@ -55803,7 +55803,7 @@
       </c>
       <c r="R510" t="inlineStr"/>
       <c r="S510" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T510" t="inlineStr">
         <is>
@@ -55908,7 +55908,7 @@
       </c>
       <c r="R511" t="inlineStr"/>
       <c r="S511" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T511" t="inlineStr">
         <is>
@@ -56013,7 +56013,7 @@
       </c>
       <c r="R512" t="inlineStr"/>
       <c r="S512" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T512" t="inlineStr">
         <is>
@@ -56118,7 +56118,7 @@
       </c>
       <c r="R513" t="inlineStr"/>
       <c r="S513" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T513" t="inlineStr">
         <is>
@@ -56223,7 +56223,7 @@
       </c>
       <c r="R514" t="inlineStr"/>
       <c r="S514" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T514" t="inlineStr">
         <is>
@@ -56324,7 +56324,7 @@
       </c>
       <c r="R515" t="inlineStr"/>
       <c r="S515" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T515" t="inlineStr">
         <is>
@@ -56425,7 +56425,7 @@
       </c>
       <c r="R516" t="inlineStr"/>
       <c r="S516" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T516" t="inlineStr">
         <is>
@@ -56526,7 +56526,7 @@
       </c>
       <c r="R517" t="inlineStr"/>
       <c r="S517" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T517" t="inlineStr">
         <is>
@@ -56627,7 +56627,7 @@
       </c>
       <c r="R518" t="inlineStr"/>
       <c r="S518" t="n">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="T518" t="inlineStr">
         <is>
@@ -56732,7 +56732,7 @@
       </c>
       <c r="R519" t="inlineStr"/>
       <c r="S519" t="n">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="T519" t="inlineStr">
         <is>
@@ -56837,7 +56837,7 @@
       </c>
       <c r="R520" t="inlineStr"/>
       <c r="S520" t="n">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="T520" t="inlineStr">
         <is>
@@ -56942,7 +56942,7 @@
       </c>
       <c r="R521" t="inlineStr"/>
       <c r="S521" t="n">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="T521" t="inlineStr">
         <is>
@@ -57043,7 +57043,7 @@
       </c>
       <c r="R522" t="inlineStr"/>
       <c r="S522" t="n">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="T522" t="inlineStr">
         <is>
@@ -57148,7 +57148,7 @@
       </c>
       <c r="R523" t="inlineStr"/>
       <c r="S523" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T523" t="inlineStr">
         <is>
@@ -57253,7 +57253,7 @@
       </c>
       <c r="R524" t="inlineStr"/>
       <c r="S524" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T524" t="inlineStr">
         <is>
@@ -57354,7 +57354,7 @@
       </c>
       <c r="R525" t="inlineStr"/>
       <c r="S525" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T525" t="inlineStr">
         <is>
@@ -57455,7 +57455,7 @@
       </c>
       <c r="R526" t="inlineStr"/>
       <c r="S526" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T526" t="inlineStr">
         <is>
@@ -57560,7 +57560,7 @@
       </c>
       <c r="R527" t="inlineStr"/>
       <c r="S527" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T527" t="inlineStr">
         <is>
@@ -57665,7 +57665,7 @@
       </c>
       <c r="R528" t="inlineStr"/>
       <c r="S528" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T528" t="inlineStr">
         <is>
@@ -57770,7 +57770,7 @@
       </c>
       <c r="R529" t="inlineStr"/>
       <c r="S529" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T529" t="inlineStr">
         <is>
@@ -57875,7 +57875,7 @@
       </c>
       <c r="R530" t="inlineStr"/>
       <c r="S530" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T530" t="inlineStr">
         <is>
@@ -57984,7 +57984,7 @@
       </c>
       <c r="R531" t="inlineStr"/>
       <c r="S531" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T531" t="inlineStr">
         <is>
@@ -58093,7 +58093,7 @@
       </c>
       <c r="R532" t="inlineStr"/>
       <c r="S532" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T532" t="inlineStr">
         <is>
@@ -58194,7 +58194,7 @@
       </c>
       <c r="R533" t="inlineStr"/>
       <c r="S533" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T533" t="inlineStr">
         <is>
@@ -58295,7 +58295,7 @@
       </c>
       <c r="R534" t="inlineStr"/>
       <c r="S534" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T534" t="inlineStr">
         <is>
@@ -58396,7 +58396,7 @@
       </c>
       <c r="R535" t="inlineStr"/>
       <c r="S535" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T535" t="inlineStr">
         <is>
@@ -58497,7 +58497,7 @@
       </c>
       <c r="R536" t="inlineStr"/>
       <c r="S536" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T536" t="inlineStr">
         <is>
@@ -58602,7 +58602,7 @@
       </c>
       <c r="R537" t="inlineStr"/>
       <c r="S537" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T537" t="inlineStr">
         <is>
@@ -58707,7 +58707,7 @@
       </c>
       <c r="R538" t="inlineStr"/>
       <c r="S538" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T538" t="inlineStr">
         <is>
@@ -58812,7 +58812,7 @@
       </c>
       <c r="R539" t="inlineStr"/>
       <c r="S539" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T539" t="inlineStr">
         <is>
@@ -58917,7 +58917,7 @@
       </c>
       <c r="R540" t="inlineStr"/>
       <c r="S540" t="n">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="T540" t="inlineStr">
         <is>
@@ -59022,7 +59022,7 @@
       </c>
       <c r="R541" t="inlineStr"/>
       <c r="S541" t="n">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="T541" t="inlineStr">
         <is>
@@ -59127,7 +59127,7 @@
       </c>
       <c r="R542" t="inlineStr"/>
       <c r="S542" t="n">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="T542" t="inlineStr">
         <is>
@@ -59232,7 +59232,7 @@
       </c>
       <c r="R543" t="inlineStr"/>
       <c r="S543" t="n">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="T543" t="inlineStr">
         <is>
@@ -59333,7 +59333,7 @@
       </c>
       <c r="R544" t="inlineStr"/>
       <c r="S544" t="n">
-        <v>-18</v>
+        <v>-17</v>
       </c>
       <c r="T544" t="inlineStr">
         <is>
@@ -59434,7 +59434,7 @@
       </c>
       <c r="R545" t="inlineStr"/>
       <c r="S545" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T545" t="inlineStr">
         <is>
@@ -59535,7 +59535,7 @@
       </c>
       <c r="R546" t="inlineStr"/>
       <c r="S546" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T546" t="inlineStr">
         <is>
@@ -59640,7 +59640,7 @@
       </c>
       <c r="R547" t="inlineStr"/>
       <c r="S547" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T547" t="inlineStr">
         <is>
@@ -59745,7 +59745,7 @@
       </c>
       <c r="R548" t="inlineStr"/>
       <c r="S548" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T548" t="inlineStr">
         <is>
@@ -59850,7 +59850,7 @@
       </c>
       <c r="R549" t="inlineStr"/>
       <c r="S549" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T549" t="inlineStr">
         <is>
@@ -59955,7 +59955,7 @@
       </c>
       <c r="R550" t="inlineStr"/>
       <c r="S550" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T550" t="inlineStr">
         <is>
@@ -60060,7 +60060,7 @@
       </c>
       <c r="R551" t="inlineStr"/>
       <c r="S551" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T551" t="inlineStr">
         <is>
@@ -60161,7 +60161,7 @@
       </c>
       <c r="R552" t="inlineStr"/>
       <c r="S552" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T552" t="inlineStr">
         <is>
@@ -60262,7 +60262,7 @@
       </c>
       <c r="R553" t="inlineStr"/>
       <c r="S553" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T553" t="inlineStr">
         <is>
@@ -60367,7 +60367,7 @@
       </c>
       <c r="R554" t="inlineStr"/>
       <c r="S554" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T554" t="inlineStr">
         <is>
@@ -60468,7 +60468,7 @@
       </c>
       <c r="R555" t="inlineStr"/>
       <c r="S555" t="n">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="T555" t="inlineStr">
         <is>
@@ -60569,7 +60569,7 @@
       </c>
       <c r="R556" t="inlineStr"/>
       <c r="S556" t="n">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="T556" t="inlineStr">
         <is>
@@ -60670,7 +60670,7 @@
       </c>
       <c r="R557" t="inlineStr"/>
       <c r="S557" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T557" t="inlineStr">
         <is>
@@ -60775,7 +60775,7 @@
       </c>
       <c r="R558" t="inlineStr"/>
       <c r="S558" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T558" t="inlineStr">
         <is>
@@ -60880,7 +60880,7 @@
       </c>
       <c r="R559" t="inlineStr"/>
       <c r="S559" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T559" t="inlineStr">
         <is>
@@ -60981,7 +60981,7 @@
       </c>
       <c r="R560" t="inlineStr"/>
       <c r="S560" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T560" t="inlineStr">
         <is>
@@ -61086,7 +61086,7 @@
       </c>
       <c r="R561" t="inlineStr"/>
       <c r="S561" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T561" t="inlineStr">
         <is>
@@ -61191,7 +61191,7 @@
       </c>
       <c r="R562" t="inlineStr"/>
       <c r="S562" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T562" t="inlineStr">
         <is>
@@ -61296,7 +61296,7 @@
       </c>
       <c r="R563" t="inlineStr"/>
       <c r="S563" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T563" t="inlineStr">
         <is>
@@ -61401,7 +61401,7 @@
       </c>
       <c r="R564" t="inlineStr"/>
       <c r="S564" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="T564" t="inlineStr">
         <is>
@@ -61506,7 +61506,7 @@
       </c>
       <c r="R565" t="inlineStr"/>
       <c r="S565" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="T565" t="inlineStr">
         <is>
@@ -61611,7 +61611,7 @@
       </c>
       <c r="R566" t="inlineStr"/>
       <c r="S566" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="T566" t="inlineStr">
         <is>
@@ -61712,7 +61712,7 @@
       </c>
       <c r="R567" t="inlineStr"/>
       <c r="S567" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="T567" t="inlineStr">
         <is>
@@ -61817,7 +61817,7 @@
       </c>
       <c r="R568" t="inlineStr"/>
       <c r="S568" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T568" t="inlineStr">
         <is>
@@ -61927,7 +61927,7 @@
       </c>
       <c r="R569" t="inlineStr"/>
       <c r="S569" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T569" t="inlineStr">
         <is>
@@ -62037,7 +62037,7 @@
       </c>
       <c r="R570" t="inlineStr"/>
       <c r="S570" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T570" t="inlineStr">
         <is>
@@ -62147,7 +62147,7 @@
       </c>
       <c r="R571" t="inlineStr"/>
       <c r="S571" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T571" t="inlineStr">
         <is>
@@ -62261,7 +62261,7 @@
       </c>
       <c r="R572" t="inlineStr"/>
       <c r="S572" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T572" t="inlineStr">
         <is>
@@ -62375,7 +62375,7 @@
       </c>
       <c r="R573" t="inlineStr"/>
       <c r="S573" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T573" t="inlineStr">
         <is>
@@ -62485,7 +62485,7 @@
       </c>
       <c r="R574" t="inlineStr"/>
       <c r="S574" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T574" t="inlineStr">
         <is>
@@ -62590,7 +62590,7 @@
       </c>
       <c r="R575" t="inlineStr"/>
       <c r="S575" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T575" t="inlineStr">
         <is>
@@ -62695,7 +62695,7 @@
       </c>
       <c r="R576" t="inlineStr"/>
       <c r="S576" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T576" t="inlineStr">
         <is>
@@ -62796,7 +62796,7 @@
       </c>
       <c r="R577" t="inlineStr"/>
       <c r="S577" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T577" t="inlineStr">
         <is>
@@ -62897,7 +62897,7 @@
       </c>
       <c r="R578" t="inlineStr"/>
       <c r="S578" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="T578" t="inlineStr">
         <is>
@@ -63002,7 +63002,7 @@
       </c>
       <c r="R579" t="inlineStr"/>
       <c r="S579" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="T579" t="inlineStr">
         <is>
@@ -63111,7 +63111,7 @@
       </c>
       <c r="R580" t="inlineStr"/>
       <c r="S580" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="T580" t="inlineStr">
         <is>
@@ -63221,7 +63221,7 @@
       </c>
       <c r="R581" t="inlineStr"/>
       <c r="S581" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="T581" t="inlineStr">
         <is>
@@ -63326,7 +63326,7 @@
       </c>
       <c r="R582" t="inlineStr"/>
       <c r="S582" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="T582" t="inlineStr">
         <is>
@@ -63427,7 +63427,7 @@
       </c>
       <c r="R583" t="inlineStr"/>
       <c r="S583" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="T583" t="inlineStr">
         <is>
@@ -63528,7 +63528,7 @@
       </c>
       <c r="R584" t="inlineStr"/>
       <c r="S584" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T584" t="inlineStr">
         <is>
@@ -63633,7 +63633,7 @@
       </c>
       <c r="R585" t="inlineStr"/>
       <c r="S585" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T585" t="inlineStr">
         <is>
@@ -63738,7 +63738,7 @@
       </c>
       <c r="R586" t="inlineStr"/>
       <c r="S586" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T586" t="inlineStr">
         <is>
@@ -63843,7 +63843,7 @@
       </c>
       <c r="R587" t="inlineStr"/>
       <c r="S587" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T587" t="inlineStr">
         <is>
@@ -63952,7 +63952,7 @@
       </c>
       <c r="R588" t="inlineStr"/>
       <c r="S588" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T588" t="inlineStr">
         <is>
@@ -64065,7 +64065,7 @@
       </c>
       <c r="R589" t="inlineStr"/>
       <c r="S589" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T589" t="inlineStr">
         <is>
@@ -64178,7 +64178,7 @@
       </c>
       <c r="R590" t="inlineStr"/>
       <c r="S590" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T590" t="inlineStr">
         <is>
@@ -64291,7 +64291,7 @@
       </c>
       <c r="R591" t="inlineStr"/>
       <c r="S591" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T591" t="inlineStr">
         <is>
@@ -64404,7 +64404,7 @@
       </c>
       <c r="R592" t="inlineStr"/>
       <c r="S592" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T592" t="inlineStr">
         <is>
@@ -64517,7 +64517,7 @@
       </c>
       <c r="R593" t="inlineStr"/>
       <c r="S593" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T593" t="inlineStr">
         <is>
@@ -64626,7 +64626,7 @@
       </c>
       <c r="R594" t="inlineStr"/>
       <c r="S594" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T594" t="inlineStr">
         <is>
@@ -64731,7 +64731,7 @@
       </c>
       <c r="R595" t="inlineStr"/>
       <c r="S595" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T595" t="inlineStr">
         <is>
@@ -64836,7 +64836,7 @@
       </c>
       <c r="R596" t="inlineStr"/>
       <c r="S596" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T596" t="inlineStr">
         <is>
@@ -64941,7 +64941,7 @@
       </c>
       <c r="R597" t="inlineStr"/>
       <c r="S597" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T597" t="inlineStr">
         <is>
@@ -65046,7 +65046,7 @@
       </c>
       <c r="R598" t="inlineStr"/>
       <c r="S598" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T598" t="inlineStr">
         <is>
@@ -65151,7 +65151,7 @@
       </c>
       <c r="R599" t="inlineStr"/>
       <c r="S599" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T599" t="inlineStr">
         <is>
@@ -65256,7 +65256,7 @@
       </c>
       <c r="R600" t="inlineStr"/>
       <c r="S600" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T600" t="inlineStr">
         <is>
@@ -65361,7 +65361,7 @@
       </c>
       <c r="R601" t="inlineStr"/>
       <c r="S601" t="n">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="T601" t="inlineStr">
         <is>
@@ -65470,7 +65470,7 @@
       </c>
       <c r="R602" t="inlineStr"/>
       <c r="S602" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T602" t="inlineStr">
         <is>
@@ -65583,7 +65583,7 @@
       </c>
       <c r="R603" t="inlineStr"/>
       <c r="S603" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T603" t="inlineStr">
         <is>
@@ -65692,7 +65692,7 @@
       </c>
       <c r="R604" t="inlineStr"/>
       <c r="S604" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T604" t="inlineStr">
         <is>
@@ -65797,7 +65797,7 @@
       </c>
       <c r="R605" t="inlineStr"/>
       <c r="S605" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T605" t="inlineStr">
         <is>
@@ -65902,7 +65902,7 @@
       </c>
       <c r="R606" t="inlineStr"/>
       <c r="S606" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T606" t="inlineStr">
         <is>
@@ -66007,7 +66007,7 @@
       </c>
       <c r="R607" t="inlineStr"/>
       <c r="S607" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T607" t="inlineStr">
         <is>
@@ -66112,7 +66112,7 @@
       </c>
       <c r="R608" t="inlineStr"/>
       <c r="S608" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T608" t="inlineStr">
         <is>
@@ -66217,7 +66217,7 @@
       </c>
       <c r="R609" t="inlineStr"/>
       <c r="S609" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T609" t="inlineStr">
         <is>
@@ -66322,7 +66322,7 @@
       </c>
       <c r="R610" t="inlineStr"/>
       <c r="S610" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T610" t="inlineStr">
         <is>
@@ -66427,7 +66427,7 @@
       </c>
       <c r="R611" t="inlineStr"/>
       <c r="S611" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T611" t="inlineStr">
         <is>
@@ -66532,7 +66532,7 @@
       </c>
       <c r="R612" t="inlineStr"/>
       <c r="S612" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T612" t="inlineStr">
         <is>
@@ -66637,7 +66637,7 @@
       </c>
       <c r="R613" t="inlineStr"/>
       <c r="S613" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T613" t="inlineStr">
         <is>
@@ -66742,7 +66742,7 @@
       </c>
       <c r="R614" t="inlineStr"/>
       <c r="S614" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T614" t="inlineStr">
         <is>
@@ -66847,7 +66847,7 @@
       </c>
       <c r="R615" t="inlineStr"/>
       <c r="S615" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T615" t="inlineStr">
         <is>
@@ -66952,7 +66952,7 @@
       </c>
       <c r="R616" t="inlineStr"/>
       <c r="S616" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T616" t="inlineStr">
         <is>
@@ -67057,7 +67057,7 @@
       </c>
       <c r="R617" t="inlineStr"/>
       <c r="S617" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="T617" t="inlineStr">
         <is>
@@ -67162,7 +67162,7 @@
       </c>
       <c r="R618" t="inlineStr"/>
       <c r="S618" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="T618" t="inlineStr">
         <is>
@@ -67267,7 +67267,7 @@
       </c>
       <c r="R619" t="inlineStr"/>
       <c r="S619" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="T619" t="inlineStr">
         <is>
@@ -67372,7 +67372,7 @@
       </c>
       <c r="R620" t="inlineStr"/>
       <c r="S620" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="T620" t="inlineStr">
         <is>
@@ -67477,7 +67477,7 @@
       </c>
       <c r="R621" t="inlineStr"/>
       <c r="S621" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="T621" t="inlineStr">
         <is>
@@ -67582,7 +67582,7 @@
       </c>
       <c r="R622" t="inlineStr"/>
       <c r="S622" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="T622" t="inlineStr">
         <is>
@@ -67693,7 +67693,7 @@
       </c>
       <c r="R623" t="inlineStr"/>
       <c r="S623" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T623" t="inlineStr">
         <is>
@@ -67794,7 +67794,7 @@
       </c>
       <c r="R624" t="inlineStr"/>
       <c r="S624" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T624" t="inlineStr">
         <is>
@@ -67891,7 +67891,7 @@
       </c>
       <c r="R625" t="inlineStr"/>
       <c r="S625" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T625" t="inlineStr">
         <is>
@@ -67992,7 +67992,7 @@
       </c>
       <c r="R626" t="inlineStr"/>
       <c r="S626" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T626" t="inlineStr">
         <is>
@@ -68093,7 +68093,7 @@
       </c>
       <c r="R627" t="inlineStr"/>
       <c r="S627" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T627" t="inlineStr">
         <is>
@@ -68194,7 +68194,7 @@
       </c>
       <c r="R628" t="inlineStr"/>
       <c r="S628" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T628" t="inlineStr">
         <is>
@@ -68295,7 +68295,7 @@
       </c>
       <c r="R629" t="inlineStr"/>
       <c r="S629" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T629" t="inlineStr">
         <is>
@@ -68396,7 +68396,7 @@
       </c>
       <c r="R630" t="inlineStr"/>
       <c r="S630" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T630" t="inlineStr">
         <is>
@@ -68497,7 +68497,7 @@
       </c>
       <c r="R631" t="inlineStr"/>
       <c r="S631" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T631" t="inlineStr">
         <is>
@@ -68598,7 +68598,7 @@
       </c>
       <c r="R632" t="inlineStr"/>
       <c r="S632" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T632" t="inlineStr">
         <is>
@@ -68699,7 +68699,7 @@
       </c>
       <c r="R633" t="inlineStr"/>
       <c r="S633" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T633" t="inlineStr">
         <is>
@@ -68800,7 +68800,7 @@
       </c>
       <c r="R634" t="inlineStr"/>
       <c r="S634" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T634" t="inlineStr">
         <is>
@@ -68901,7 +68901,7 @@
       </c>
       <c r="R635" t="inlineStr"/>
       <c r="S635" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T635" t="inlineStr">
         <is>
@@ -69002,7 +69002,7 @@
       </c>
       <c r="R636" t="inlineStr"/>
       <c r="S636" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T636" t="inlineStr">
         <is>
@@ -69103,7 +69103,7 @@
       </c>
       <c r="R637" t="inlineStr"/>
       <c r="S637" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T637" t="inlineStr">
         <is>
@@ -69204,7 +69204,7 @@
       </c>
       <c r="R638" t="inlineStr"/>
       <c r="S638" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T638" t="inlineStr">
         <is>
@@ -69301,7 +69301,7 @@
       </c>
       <c r="R639" t="inlineStr"/>
       <c r="S639" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T639" t="inlineStr">
         <is>
@@ -69398,7 +69398,7 @@
       </c>
       <c r="R640" t="inlineStr"/>
       <c r="S640" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T640" t="inlineStr">
         <is>
@@ -69495,7 +69495,7 @@
       </c>
       <c r="R641" t="inlineStr"/>
       <c r="S641" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T641" t="inlineStr">
         <is>
@@ -69592,7 +69592,7 @@
       </c>
       <c r="R642" t="inlineStr"/>
       <c r="S642" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T642" t="inlineStr">
         <is>
@@ -69689,7 +69689,7 @@
       </c>
       <c r="R643" t="inlineStr"/>
       <c r="S643" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T643" t="inlineStr">
         <is>
@@ -69786,7 +69786,7 @@
       </c>
       <c r="R644" t="inlineStr"/>
       <c r="S644" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T644" t="inlineStr">
         <is>
@@ -69887,7 +69887,7 @@
       </c>
       <c r="R645" t="inlineStr"/>
       <c r="S645" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T645" t="inlineStr">
         <is>
@@ -69988,7 +69988,7 @@
       </c>
       <c r="R646" t="inlineStr"/>
       <c r="S646" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T646" t="inlineStr">
         <is>
@@ -70089,7 +70089,7 @@
       </c>
       <c r="R647" t="inlineStr"/>
       <c r="S647" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T647" t="inlineStr">
         <is>
@@ -70190,7 +70190,7 @@
       </c>
       <c r="R648" t="inlineStr"/>
       <c r="S648" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T648" t="inlineStr">
         <is>
@@ -70291,7 +70291,7 @@
       </c>
       <c r="R649" t="inlineStr"/>
       <c r="S649" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T649" t="inlineStr">
         <is>
@@ -70392,7 +70392,7 @@
       </c>
       <c r="R650" t="inlineStr"/>
       <c r="S650" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T650" t="inlineStr">
         <is>
@@ -70493,7 +70493,7 @@
       </c>
       <c r="R651" t="inlineStr"/>
       <c r="S651" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T651" t="inlineStr">
         <is>
@@ -70590,7 +70590,7 @@
       </c>
       <c r="R652" t="inlineStr"/>
       <c r="S652" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T652" t="inlineStr">
         <is>
@@ -70687,7 +70687,7 @@
       </c>
       <c r="R653" t="inlineStr"/>
       <c r="S653" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T653" t="inlineStr">
         <is>
@@ -70784,7 +70784,7 @@
       </c>
       <c r="R654" t="inlineStr"/>
       <c r="S654" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T654" t="inlineStr">
         <is>
@@ -70881,7 +70881,7 @@
       </c>
       <c r="R655" t="inlineStr"/>
       <c r="S655" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T655" t="inlineStr">
         <is>
@@ -70978,7 +70978,7 @@
       </c>
       <c r="R656" t="inlineStr"/>
       <c r="S656" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T656" t="inlineStr">
         <is>
@@ -71075,7 +71075,7 @@
       </c>
       <c r="R657" t="inlineStr"/>
       <c r="S657" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T657" t="inlineStr">
         <is>
@@ -71176,7 +71176,7 @@
       </c>
       <c r="R658" t="inlineStr"/>
       <c r="S658" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T658" t="inlineStr">
         <is>
@@ -71277,7 +71277,7 @@
       </c>
       <c r="R659" t="inlineStr"/>
       <c r="S659" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T659" t="inlineStr">
         <is>
@@ -71378,7 +71378,7 @@
       </c>
       <c r="R660" t="inlineStr"/>
       <c r="S660" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T660" t="inlineStr">
         <is>
@@ -71479,7 +71479,7 @@
       </c>
       <c r="R661" t="inlineStr"/>
       <c r="S661" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T661" t="inlineStr">
         <is>
@@ -71580,7 +71580,7 @@
       </c>
       <c r="R662" t="inlineStr"/>
       <c r="S662" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T662" t="inlineStr">
         <is>
@@ -71681,7 +71681,7 @@
       </c>
       <c r="R663" t="inlineStr"/>
       <c r="S663" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T663" t="inlineStr">
         <is>
@@ -71782,7 +71782,7 @@
       </c>
       <c r="R664" t="inlineStr"/>
       <c r="S664" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T664" t="inlineStr">
         <is>
@@ -71883,7 +71883,7 @@
       </c>
       <c r="R665" t="inlineStr"/>
       <c r="S665" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T665" t="inlineStr">
         <is>
@@ -71984,7 +71984,7 @@
       </c>
       <c r="R666" t="inlineStr"/>
       <c r="S666" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T666" t="inlineStr">
         <is>
@@ -72081,7 +72081,7 @@
       </c>
       <c r="R667" t="inlineStr"/>
       <c r="S667" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T667" t="inlineStr">
         <is>
@@ -72178,7 +72178,7 @@
       </c>
       <c r="R668" t="inlineStr"/>
       <c r="S668" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T668" t="inlineStr">
         <is>
@@ -72275,7 +72275,7 @@
       </c>
       <c r="R669" t="inlineStr"/>
       <c r="S669" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T669" t="inlineStr">
         <is>
@@ -72376,7 +72376,7 @@
       </c>
       <c r="R670" t="inlineStr"/>
       <c r="S670" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T670" t="inlineStr">
         <is>
@@ -72477,7 +72477,7 @@
       </c>
       <c r="R671" t="inlineStr"/>
       <c r="S671" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T671" t="inlineStr">
         <is>
@@ -72578,7 +72578,7 @@
       </c>
       <c r="R672" t="inlineStr"/>
       <c r="S672" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T672" t="inlineStr">
         <is>
@@ -72679,7 +72679,7 @@
       </c>
       <c r="R673" t="inlineStr"/>
       <c r="S673" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T673" t="inlineStr">
         <is>
@@ -72780,7 +72780,7 @@
       </c>
       <c r="R674" t="inlineStr"/>
       <c r="S674" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T674" t="inlineStr">
         <is>
@@ -72881,7 +72881,7 @@
       </c>
       <c r="R675" t="inlineStr"/>
       <c r="S675" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T675" t="inlineStr">
         <is>
@@ -72982,7 +72982,7 @@
       </c>
       <c r="R676" t="inlineStr"/>
       <c r="S676" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T676" t="inlineStr">
         <is>
@@ -73083,7 +73083,7 @@
       </c>
       <c r="R677" t="inlineStr"/>
       <c r="S677" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T677" t="inlineStr">
         <is>
@@ -73184,7 +73184,7 @@
       </c>
       <c r="R678" t="inlineStr"/>
       <c r="S678" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T678" t="inlineStr">
         <is>
@@ -73285,7 +73285,7 @@
       </c>
       <c r="R679" t="inlineStr"/>
       <c r="S679" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T679" t="inlineStr">
         <is>
@@ -73386,7 +73386,7 @@
       </c>
       <c r="R680" t="inlineStr"/>
       <c r="S680" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T680" t="inlineStr">
         <is>
@@ -73487,7 +73487,7 @@
       </c>
       <c r="R681" t="inlineStr"/>
       <c r="S681" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T681" t="inlineStr">
         <is>
@@ -73588,7 +73588,7 @@
       </c>
       <c r="R682" t="inlineStr"/>
       <c r="S682" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T682" t="inlineStr">
         <is>
@@ -73685,7 +73685,7 @@
       </c>
       <c r="R683" t="inlineStr"/>
       <c r="S683" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T683" t="inlineStr">
         <is>
@@ -73782,7 +73782,7 @@
       </c>
       <c r="R684" t="inlineStr"/>
       <c r="S684" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T684" t="inlineStr">
         <is>
@@ -73879,7 +73879,7 @@
       </c>
       <c r="R685" t="inlineStr"/>
       <c r="S685" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T685" t="inlineStr">
         <is>
@@ -73976,7 +73976,7 @@
       </c>
       <c r="R686" t="inlineStr"/>
       <c r="S686" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T686" t="inlineStr">
         <is>
@@ -74073,7 +74073,7 @@
       </c>
       <c r="R687" t="inlineStr"/>
       <c r="S687" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T687" t="inlineStr">
         <is>
@@ -74170,7 +74170,7 @@
       </c>
       <c r="R688" t="inlineStr"/>
       <c r="S688" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T688" t="inlineStr">
         <is>
@@ -74271,7 +74271,7 @@
       </c>
       <c r="R689" t="inlineStr"/>
       <c r="S689" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T689" t="inlineStr">
         <is>
@@ -74372,7 +74372,7 @@
       </c>
       <c r="R690" t="inlineStr"/>
       <c r="S690" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T690" t="inlineStr">
         <is>
@@ -74473,7 +74473,7 @@
       </c>
       <c r="R691" t="inlineStr"/>
       <c r="S691" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T691" t="inlineStr">
         <is>
@@ -74574,7 +74574,7 @@
       </c>
       <c r="R692" t="inlineStr"/>
       <c r="S692" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T692" t="inlineStr">
         <is>
@@ -74675,7 +74675,7 @@
       </c>
       <c r="R693" t="inlineStr"/>
       <c r="S693" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T693" t="inlineStr">
         <is>
@@ -74776,7 +74776,7 @@
       </c>
       <c r="R694" t="inlineStr"/>
       <c r="S694" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T694" t="inlineStr">
         <is>
@@ -74877,7 +74877,7 @@
       </c>
       <c r="R695" t="inlineStr"/>
       <c r="S695" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T695" t="inlineStr">
         <is>
@@ -74974,7 +74974,7 @@
       </c>
       <c r="R696" t="inlineStr"/>
       <c r="S696" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T696" t="inlineStr">
         <is>
@@ -75071,7 +75071,7 @@
       </c>
       <c r="R697" t="inlineStr"/>
       <c r="S697" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T697" t="inlineStr">
         <is>
@@ -75168,7 +75168,7 @@
       </c>
       <c r="R698" t="inlineStr"/>
       <c r="S698" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T698" t="inlineStr">
         <is>
@@ -75265,7 +75265,7 @@
       </c>
       <c r="R699" t="inlineStr"/>
       <c r="S699" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T699" t="inlineStr">
         <is>
@@ -75362,7 +75362,7 @@
       </c>
       <c r="R700" t="inlineStr"/>
       <c r="S700" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T700" t="inlineStr">
         <is>
@@ -75459,7 +75459,7 @@
       </c>
       <c r="R701" t="inlineStr"/>
       <c r="S701" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T701" t="inlineStr">
         <is>
@@ -75560,7 +75560,7 @@
       </c>
       <c r="R702" t="inlineStr"/>
       <c r="S702" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T702" t="inlineStr">
         <is>
@@ -75661,7 +75661,7 @@
       </c>
       <c r="R703" t="inlineStr"/>
       <c r="S703" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T703" t="inlineStr">
         <is>
@@ -75760,7 +75760,7 @@
         <v>46209.66158305555</v>
       </c>
       <c r="S704" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T704" t="inlineStr">
         <is>
@@ -75863,7 +75863,7 @@
         <v>46203.00285659722</v>
       </c>
       <c r="S705" t="n">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="T705" t="inlineStr">
         <is>
@@ -75974,7 +75974,7 @@
         <v>46203.00296711805</v>
       </c>
       <c r="S706" t="n">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="T706" t="inlineStr">
         <is>
@@ -76081,7 +76081,7 @@
         <v>46204.72937350695</v>
       </c>
       <c r="S707" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T707" t="inlineStr">
         <is>
@@ -76192,7 +76192,7 @@
         <v>46206.41464283565</v>
       </c>
       <c r="S708" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T708" t="inlineStr">
         <is>
@@ -76303,7 +76303,7 @@
         <v>46206.70573774305</v>
       </c>
       <c r="S709" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T709" t="inlineStr">
         <is>
@@ -76414,7 +76414,7 @@
         <v>46206.70573846065</v>
       </c>
       <c r="S710" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T710" t="inlineStr">
         <is>
@@ -76525,7 +76525,7 @@
         <v>46211.41697137732</v>
       </c>
       <c r="S711" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T711" t="inlineStr">
         <is>
@@ -76636,7 +76636,7 @@
         <v>46203.3758668287</v>
       </c>
       <c r="S712" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T712" t="inlineStr">
         <is>
@@ -76747,7 +76747,7 @@
         <v>46203.37586737268</v>
       </c>
       <c r="S713" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T713" t="inlineStr">
         <is>
@@ -76858,7 +76858,7 @@
         <v>46203.37586936342</v>
       </c>
       <c r="S714" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T714" t="inlineStr">
         <is>
@@ -76969,7 +76969,7 @@
         <v>46205.45020773148</v>
       </c>
       <c r="S715" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T715" t="inlineStr">
         <is>
@@ -77080,7 +77080,7 @@
         <v>46205.45020809027</v>
       </c>
       <c r="S716" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T716" t="inlineStr">
         <is>
@@ -77191,7 +77191,7 @@
         <v>46205.45020880787</v>
       </c>
       <c r="S717" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T717" t="inlineStr">
         <is>
@@ -77298,7 +77298,7 @@
         <v>46203.37587081019</v>
       </c>
       <c r="S718" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T718" t="inlineStr">
         <is>
@@ -77405,7 +77405,7 @@
         <v>46216.44618675926</v>
       </c>
       <c r="S719" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T719" t="inlineStr">
         <is>
@@ -77512,7 +77512,7 @@
         <v>46206.62907918981</v>
       </c>
       <c r="S720" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T720" t="inlineStr">
         <is>
@@ -77623,7 +77623,7 @@
         <v>46204.00354291667</v>
       </c>
       <c r="S721" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T721" t="inlineStr">
         <is>
@@ -77734,7 +77734,7 @@
         <v>46216.76160721065</v>
       </c>
       <c r="S722" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T722" t="inlineStr">
         <is>
@@ -77841,7 +77841,7 @@
         <v>46206.44786171296</v>
       </c>
       <c r="S723" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T723" t="inlineStr">
         <is>
@@ -77952,7 +77952,7 @@
         <v>46203.71390146991</v>
       </c>
       <c r="S724" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T724" t="inlineStr">
         <is>
@@ -78063,7 +78063,7 @@
         <v>46203.00370568287</v>
       </c>
       <c r="S725" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T725" t="inlineStr">
         <is>
@@ -78174,7 +78174,7 @@
         <v>46216.46069332176</v>
       </c>
       <c r="S726" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T726" t="inlineStr">
         <is>
@@ -78285,7 +78285,7 @@
         <v>46209.779275</v>
       </c>
       <c r="S727" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T727" t="inlineStr">
         <is>
@@ -78400,7 +78400,7 @@
         <v>46188.33599649306</v>
       </c>
       <c r="S728" t="n">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="T728" t="inlineStr">
         <is>
@@ -78511,7 +78511,7 @@
         <v>46204.3759534375</v>
       </c>
       <c r="S729" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T729" t="inlineStr">
         <is>
@@ -78622,7 +78622,7 @@
         <v>46206.79235917824</v>
       </c>
       <c r="S730" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T730" t="inlineStr">
         <is>
@@ -78733,7 +78733,7 @@
         <v>46206.79235393518</v>
       </c>
       <c r="S731" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T731" t="inlineStr">
         <is>
@@ -78844,7 +78844,7 @@
         <v>46210.75621153935</v>
       </c>
       <c r="S732" t="n">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="T732" t="inlineStr">
         <is>
@@ -78963,7 +78963,7 @@
         <v>46213.36370773148</v>
       </c>
       <c r="S733" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T733" t="inlineStr">
         <is>
@@ -79078,7 +79078,7 @@
         <v>46204.04179737269</v>
       </c>
       <c r="S734" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T734" t="inlineStr">
         <is>
@@ -79189,7 +79189,7 @@
         <v>46057.40119486111</v>
       </c>
       <c r="S735" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T735" t="inlineStr">
         <is>
@@ -79296,7 +79296,7 @@
         <v>46204.04187399305</v>
       </c>
       <c r="S736" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T736" t="inlineStr">
         <is>
@@ -79403,7 +79403,7 @@
         <v>46204.04188738426</v>
       </c>
       <c r="S737" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T737" t="inlineStr">
         <is>
@@ -79510,7 +79510,7 @@
         <v>46210.80007584491</v>
       </c>
       <c r="S738" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T738" t="inlineStr">
         <is>
@@ -79613,7 +79613,7 @@
         <v>46204.16684155093</v>
       </c>
       <c r="S739" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T739" t="inlineStr">
         <is>
@@ -79724,7 +79724,7 @@
         <v>46023.15052158565</v>
       </c>
       <c r="S740" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T740" t="inlineStr">
         <is>
@@ -79831,7 +79831,7 @@
         <v>46204.12510590278</v>
       </c>
       <c r="S741" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T741" t="inlineStr">
         <is>
@@ -79942,7 +79942,7 @@
         <v>46204.37521674769</v>
       </c>
       <c r="S742" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T742" t="inlineStr">
         <is>
@@ -80053,7 +80053,7 @@
         <v>46057.39078310185</v>
       </c>
       <c r="S743" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T743" t="inlineStr">
         <is>
@@ -80160,7 +80160,7 @@
         <v>46216.49331971065</v>
       </c>
       <c r="S744" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T744" t="inlineStr">
         <is>
@@ -80263,7 +80263,7 @@
         <v>46216.49332078703</v>
       </c>
       <c r="S745" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T745" t="inlineStr">
         <is>
@@ -80366,7 +80366,7 @@
         <v>46204.29183217593</v>
       </c>
       <c r="S746" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T746" t="inlineStr">
         <is>
@@ -80477,7 +80477,7 @@
         <v>46204.33341168981</v>
       </c>
       <c r="S747" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T747" t="inlineStr">
         <is>
@@ -80588,7 +80588,7 @@
         <v>46204.25011258102</v>
       </c>
       <c r="S748" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T748" t="inlineStr">
         <is>
@@ -80699,7 +80699,7 @@
         <v>46204.37522271991</v>
       </c>
       <c r="S749" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T749" t="inlineStr">
         <is>
@@ -80810,7 +80810,7 @@
         <v>46204.25009074074</v>
       </c>
       <c r="S750" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T750" t="inlineStr">
         <is>
@@ -80921,7 +80921,7 @@
         <v>46204.37521859954</v>
       </c>
       <c r="S751" t="n">
-        <v>-17</v>
+        <v>-16</v>
       </c>
       <c r="T751" t="inlineStr">
         <is>
@@ -81032,7 +81032,7 @@
         <v>46204.41730355324</v>
       </c>
       <c r="S752" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T752" t="inlineStr">
         <is>
@@ -81143,7 +81143,7 @@
         <v>46023.15053034722</v>
       </c>
       <c r="S753" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T753" t="inlineStr">
         <is>
@@ -81250,7 +81250,7 @@
         <v>46204.41680613426</v>
       </c>
       <c r="S754" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T754" t="inlineStr">
         <is>
@@ -81361,7 +81361,7 @@
         <v>46204.41687068287</v>
       </c>
       <c r="S755" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T755" t="inlineStr">
         <is>
@@ -81472,7 +81472,7 @@
         <v>46204.41788634259</v>
       </c>
       <c r="S756" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T756" t="inlineStr">
         <is>
@@ -81583,7 +81583,7 @@
         <v>46057.3907997338</v>
       </c>
       <c r="S757" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T757" t="inlineStr">
         <is>
@@ -81686,7 +81686,7 @@
         <v>46192.56685792824</v>
       </c>
       <c r="S758" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T758" t="inlineStr">
         <is>
@@ -81785,7 +81785,7 @@
         <v>46192.56339828703</v>
       </c>
       <c r="S759" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T759" t="inlineStr">
         <is>
@@ -81888,7 +81888,7 @@
         <v>46204.41730447917</v>
       </c>
       <c r="S760" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T760" t="inlineStr">
         <is>
@@ -81999,7 +81999,7 @@
         <v>46204.41751620371</v>
       </c>
       <c r="S761" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T761" t="inlineStr">
         <is>
@@ -82110,7 +82110,7 @@
         <v>46204.41687126157</v>
       </c>
       <c r="S762" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T762" t="inlineStr">
         <is>
@@ -82221,7 +82221,7 @@
         <v>46204.41788753472</v>
       </c>
       <c r="S763" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T763" t="inlineStr">
         <is>
@@ -82332,7 +82332,7 @@
         <v>46204.41788796296</v>
       </c>
       <c r="S764" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T764" t="inlineStr">
         <is>
@@ -82439,7 +82439,7 @@
         <v>46168.72822039352</v>
       </c>
       <c r="S765" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T765" t="inlineStr">
         <is>
@@ -82538,7 +82538,7 @@
         <v>46192.56687770833</v>
       </c>
       <c r="S766" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T766" t="inlineStr">
         <is>
@@ -82637,7 +82637,7 @@
         <v>46192.56342578704</v>
       </c>
       <c r="S767" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="T767" t="inlineStr">
         <is>
@@ -82740,7 +82740,7 @@
         <v>46213.75219915509</v>
       </c>
       <c r="S768" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T768" t="inlineStr">
         <is>
@@ -82847,7 +82847,7 @@
         <v>46213.75220699074</v>
       </c>
       <c r="S769" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T769" t="inlineStr">
         <is>
@@ -82954,7 +82954,7 @@
         <v>46213.75224594907</v>
       </c>
       <c r="S770" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T770" t="inlineStr">
         <is>
@@ -83061,7 +83061,7 @@
         <v>46213.75225217592</v>
       </c>
       <c r="S771" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T771" t="inlineStr">
         <is>
@@ -83168,7 +83168,7 @@
         <v>46213.75219873842</v>
       </c>
       <c r="S772" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T772" t="inlineStr">
         <is>
@@ -83275,7 +83275,7 @@
         <v>46213.75220643519</v>
       </c>
       <c r="S773" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T773" t="inlineStr">
         <is>
@@ -83382,7 +83382,7 @@
         <v>46213.75224560185</v>
       </c>
       <c r="S774" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T774" t="inlineStr">
         <is>
@@ -83489,7 +83489,7 @@
         <v>46213.75225246528</v>
       </c>
       <c r="S775" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="T775" t="inlineStr">
         <is>
@@ -83596,7 +83596,7 @@
         <v>46174.04914510417</v>
       </c>
       <c r="S776" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T776" t="inlineStr">
         <is>
@@ -83707,7 +83707,7 @@
         <v>46174.04916258102</v>
       </c>
       <c r="S777" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T777" t="inlineStr">
         <is>
@@ -83818,7 +83818,7 @@
         <v>46174.04899652778</v>
       </c>
       <c r="S778" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T778" t="inlineStr">
         <is>
@@ -83929,7 +83929,7 @@
         <v>46174.04886894676</v>
       </c>
       <c r="S779" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T779" t="inlineStr">
         <is>
@@ -84040,7 +84040,7 @@
         <v>46174.04901342592</v>
       </c>
       <c r="S780" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T780" t="inlineStr">
         <is>
@@ -84151,7 +84151,7 @@
         <v>46174.04899452546</v>
       </c>
       <c r="S781" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T781" t="inlineStr">
         <is>
@@ -84262,7 +84262,7 @@
         <v>46174.04894753472</v>
       </c>
       <c r="S782" t="n">
-        <v>-14</v>
+        <v>-13</v>
       </c>
       <c r="T782" t="inlineStr">
         <is>
@@ -84373,7 +84373,7 @@
         <v>46174.0003128125</v>
       </c>
       <c r="S783" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T783" t="inlineStr">
         <is>
@@ -84480,7 +84480,7 @@
         <v>46174.0003128125</v>
       </c>
       <c r="S784" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T784" t="inlineStr">
         <is>
@@ -84583,7 +84583,7 @@
         <v>46174.0003128125</v>
       </c>
       <c r="S785" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T785" t="inlineStr">
         <is>
@@ -84690,7 +84690,7 @@
         <v>46174.0003128125</v>
       </c>
       <c r="S786" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T786" t="inlineStr">
         <is>
@@ -84797,7 +84797,7 @@
         <v>46174.0003128125</v>
       </c>
       <c r="S787" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T787" t="inlineStr">
         <is>
@@ -84904,7 +84904,7 @@
         <v>46211.76825706018</v>
       </c>
       <c r="S788" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T788" t="inlineStr">
         <is>
@@ -85015,7 +85015,7 @@
         <v>46209.77926392361</v>
       </c>
       <c r="S789" t="n">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="T789" t="inlineStr">
         <is>
@@ -85126,7 +85126,7 @@
       </c>
       <c r="R790" t="inlineStr"/>
       <c r="S790" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T790" t="inlineStr">
         <is>
@@ -85234,7 +85234,7 @@
       </c>
       <c r="R791" t="inlineStr"/>
       <c r="S791" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="T791" t="inlineStr">
         <is>
@@ -85342,7 +85342,7 @@
       </c>
       <c r="R792" t="inlineStr"/>
       <c r="S792" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="T792" t="inlineStr">
         <is>
@@ -85454,7 +85454,7 @@
       </c>
       <c r="R793" t="inlineStr"/>
       <c r="S793" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="T793" t="inlineStr">
         <is>
@@ -85569,7 +85569,7 @@
       </c>
       <c r="R794" t="inlineStr"/>
       <c r="S794" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="T794" t="inlineStr">
         <is>
@@ -85684,7 +85684,7 @@
       </c>
       <c r="R795" t="inlineStr"/>
       <c r="S795" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="T795" t="inlineStr">
         <is>
@@ -85803,7 +85803,7 @@
       </c>
       <c r="R796" t="inlineStr"/>
       <c r="S796" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="T796" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-20 15:58
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -43367,7 +43367,11 @@
       <c r="L395" s="1" t="n">
         <v>46227</v>
       </c>
-      <c r="M395" t="inlineStr"/>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
       <c r="N395" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -43400,7 +43404,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V395" t="inlineStr"/>
+      <c r="V395" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 20/07/2026 15:29</t>
+        </is>
+      </c>
       <c r="W395" t="inlineStr"/>
       <c r="X395" t="inlineStr"/>
       <c r="Y395" t="inlineStr"/>
@@ -43472,7 +43480,11 @@
       <c r="L396" s="1" t="n">
         <v>46227</v>
       </c>
-      <c r="M396" t="inlineStr"/>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>24/07/2026</t>
+        </is>
+      </c>
       <c r="N396" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -43505,7 +43517,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V396" t="inlineStr"/>
+      <c r="V396" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 24/07/2026 - Data Comentário: 20/07/2026 15:10</t>
+        </is>
+      </c>
       <c r="W396" t="inlineStr"/>
       <c r="X396" t="inlineStr"/>
       <c r="Y396" t="inlineStr"/>
@@ -43577,7 +43593,11 @@
       <c r="L397" s="1" t="n">
         <v>46227</v>
       </c>
-      <c r="M397" t="inlineStr"/>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>24/07/2026</t>
+        </is>
+      </c>
       <c r="N397" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -43610,7 +43630,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V397" t="inlineStr"/>
+      <c r="V397" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 24/07/2026 - Data Comentário: 20/07/2026 15:10</t>
+        </is>
+      </c>
       <c r="W397" t="inlineStr"/>
       <c r="X397" t="inlineStr"/>
       <c r="Y397" t="inlineStr"/>
@@ -44397,7 +44421,11 @@
       <c r="L405" s="1" t="n">
         <v>46227</v>
       </c>
-      <c r="M405" t="inlineStr"/>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
       <c r="N405" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -44430,7 +44458,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V405" t="inlineStr"/>
+      <c r="V405" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 20/07/2026 15:31</t>
+        </is>
+      </c>
       <c r="W405" t="inlineStr"/>
       <c r="X405" t="inlineStr"/>
       <c r="Y405" t="inlineStr"/>
@@ -44502,7 +44534,11 @@
       <c r="L406" s="1" t="n">
         <v>46227</v>
       </c>
-      <c r="M406" t="inlineStr"/>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>24/07/2026</t>
+        </is>
+      </c>
       <c r="N406" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -44535,7 +44571,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V406" t="inlineStr"/>
+      <c r="V406" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 24/07/2026 - Data Comentário: 20/07/2026 15:12</t>
+        </is>
+      </c>
       <c r="W406" t="inlineStr"/>
       <c r="X406" t="inlineStr"/>
       <c r="Y406" t="inlineStr"/>
@@ -50152,7 +50192,11 @@
       <c r="L460" s="1" t="n">
         <v>46223</v>
       </c>
-      <c r="M460" t="inlineStr"/>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t>20/07/2026</t>
+        </is>
+      </c>
       <c r="N460" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -50185,7 +50229,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V460" t="inlineStr"/>
+      <c r="V460" t="inlineStr">
+        <is>
+          <t>Atraso da Operação, processo em elaboração conforme data prevista  Previsão para conclusão dia 20/07/2026 - Data Comentário: 20/07/2026 15:26</t>
+        </is>
+      </c>
       <c r="W460" t="inlineStr"/>
       <c r="X460" t="inlineStr"/>
       <c r="Y460" t="inlineStr"/>
@@ -50500,7 +50548,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V463" t="inlineStr"/>
+      <c r="V463" t="inlineStr">
+        <is>
+          <t>Aguardando a Liberação da Gerência de Contas - Data Comentário: 20/07/2026 15:32</t>
+        </is>
+      </c>
       <c r="W463" t="inlineStr"/>
       <c r="X463" t="inlineStr"/>
       <c r="Y463" t="inlineStr"/>
@@ -61558,11 +61610,7 @@
       <c r="O566" t="n">
         <v>17688651</v>
       </c>
-      <c r="P566" t="inlineStr">
-        <is>
-          <t>Jackson Silva</t>
-        </is>
-      </c>
+      <c r="P566" t="inlineStr"/>
       <c r="Q566" t="inlineStr">
         <is>
           <t>Baixado</t>
@@ -61605,11 +61653,7 @@
           <t>Tarefa</t>
         </is>
       </c>
-      <c r="AG566" t="inlineStr">
-        <is>
-          <t>Edileide Dias</t>
-        </is>
-      </c>
+      <c r="AG566" t="inlineStr"/>
     </row>
     <row r="567">
       <c r="A567" t="n">
@@ -70294,11 +70338,7 @@
       <c r="O645" t="n">
         <v>17407769</v>
       </c>
-      <c r="P645" t="inlineStr">
-        <is>
-          <t>Cristina Leite</t>
-        </is>
-      </c>
+      <c r="P645" t="inlineStr"/>
       <c r="Q645" t="inlineStr">
         <is>
           <t>Baixado</t>
@@ -70346,11 +70386,7 @@
           <t>Imposto</t>
         </is>
       </c>
-      <c r="AG645" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
+      <c r="AG645" t="inlineStr"/>
     </row>
     <row r="646">
       <c r="A646" t="n">
@@ -70414,11 +70450,7 @@
       <c r="O646" t="n">
         <v>17688897</v>
       </c>
-      <c r="P646" t="inlineStr">
-        <is>
-          <t>Cristina Leite</t>
-        </is>
-      </c>
+      <c r="P646" t="inlineStr"/>
       <c r="Q646" t="inlineStr">
         <is>
           <t>Baixado</t>
@@ -70466,11 +70498,7 @@
           <t>Imposto</t>
         </is>
       </c>
-      <c r="AG646" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
+      <c r="AG646" t="inlineStr"/>
     </row>
     <row r="647">
       <c r="A647" t="n">
@@ -70530,11 +70558,7 @@
       <c r="O647" t="n">
         <v>18087644</v>
       </c>
-      <c r="P647" t="inlineStr">
-        <is>
-          <t>Cristina Leite</t>
-        </is>
-      </c>
+      <c r="P647" t="inlineStr"/>
       <c r="Q647" t="inlineStr">
         <is>
           <t>Baixado</t>
@@ -70581,11 +70605,7 @@
           <t>Imposto</t>
         </is>
       </c>
-      <c r="AG647" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
+      <c r="AG647" t="inlineStr"/>
     </row>
     <row r="648">
       <c r="A648" t="n">
@@ -72092,11 +72112,7 @@
       <c r="O661" t="n">
         <v>17539708</v>
       </c>
-      <c r="P661" t="inlineStr">
-        <is>
-          <t>Victoria Virgens</t>
-        </is>
-      </c>
+      <c r="P661" t="inlineStr"/>
       <c r="Q661" t="inlineStr">
         <is>
           <t>Baixado</t>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-22 12:21
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -52048,11 +52048,7 @@
       <c r="L477" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="M477" t="inlineStr">
-        <is>
-          <t>21/07/2026</t>
-        </is>
-      </c>
+      <c r="M477" t="inlineStr"/>
       <c r="N477" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -52087,7 +52083,7 @@
       </c>
       <c r="V477" t="inlineStr">
         <is>
-          <t>Tarefa reaberta, imposto não publicado no SCI - Data Comentário: 20/07/2026 18:05</t>
+          <t>Imposto enviado via SCI Report - Data Comentário: 22/07/2026 11:55</t>
         </is>
       </c>
       <c r="W477" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-22 13:21
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -52001,11 +52001,11 @@
     </row>
     <row r="477">
       <c r="A477" t="n">
-        <v>6704</v>
+        <v>5617</v>
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="C477" t="inlineStr">
@@ -52029,7 +52029,7 @@
         </is>
       </c>
       <c r="G477" t="n">
-        <v>1808</v>
+        <v>7025</v>
       </c>
       <c r="H477" t="n">
         <v>0</v>
@@ -52041,12 +52041,12 @@
       </c>
       <c r="J477" t="inlineStr">
         <is>
-          <t>Fed - PIS/COFINS Não Cumul/Mon - 5856</t>
+          <t>Movimento - Sistema de Análise</t>
         </is>
       </c>
       <c r="K477" t="inlineStr"/>
       <c r="L477" s="1" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="M477" t="inlineStr"/>
       <c r="N477" t="inlineStr">
@@ -52055,7 +52055,7 @@
         </is>
       </c>
       <c r="O477" t="n">
-        <v>18085207</v>
+        <v>17407819</v>
       </c>
       <c r="P477" t="inlineStr">
         <is>
@@ -52069,11 +52069,11 @@
       </c>
       <c r="R477" t="inlineStr"/>
       <c r="S477" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T477" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U477" t="inlineStr">
@@ -52083,7 +52083,9 @@
       </c>
       <c r="V477" t="inlineStr">
         <is>
-          <t>Imposto enviado via SCI Report - Data Comentário: 22/07/2026 11:55</t>
+          <t>Integração com Sistema de Análise 
+ICMS liberado, aguardo a validação do SPED Contribuições. 
+Data Simulação: 16/07/2026 16:40:46 - Data Comentário: 16/07/2026 17:06</t>
         </is>
       </c>
       <c r="W477" t="inlineStr"/>
@@ -52099,7 +52101,7 @@
       <c r="AE477" t="inlineStr"/>
       <c r="AF477" t="inlineStr">
         <is>
-          <t>Imposto</t>
+          <t>Tarefa</t>
         </is>
       </c>
       <c r="AG477" t="inlineStr">
@@ -52110,11 +52112,11 @@
     </row>
     <row r="478">
       <c r="A478" t="n">
-        <v>5617</v>
+        <v>5417</v>
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
@@ -52134,28 +52136,28 @@
       </c>
       <c r="F478" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G478" t="n">
-        <v>7025</v>
+        <v>953</v>
       </c>
       <c r="H478" t="n">
         <v>0</v>
       </c>
       <c r="I478" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GC - ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="J478" t="inlineStr">
         <is>
-          <t>Movimento - Sistema de Análise</t>
+          <t>Confirm Rec - PIS/COFINS</t>
         </is>
       </c>
       <c r="K478" t="inlineStr"/>
       <c r="L478" s="1" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="M478" t="inlineStr"/>
       <c r="N478" t="inlineStr">
@@ -52164,11 +52166,11 @@
         </is>
       </c>
       <c r="O478" t="n">
-        <v>17407819</v>
+        <v>17398881</v>
       </c>
       <c r="P478" t="inlineStr">
         <is>
-          <t>Cristina Leite</t>
+          <t>Victoria Virgens</t>
         </is>
       </c>
       <c r="Q478" t="inlineStr">
@@ -52178,11 +52180,11 @@
       </c>
       <c r="R478" t="inlineStr"/>
       <c r="S478" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="T478" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U478" t="inlineStr">
@@ -52192,9 +52194,7 @@
       </c>
       <c r="V478" t="inlineStr">
         <is>
-          <t>Integração com Sistema de Análise 
-ICMS liberado, aguardo a validação do SPED Contribuições. 
-Data Simulação: 16/07/2026 16:40:46 - Data Comentário: 16/07/2026 17:06</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1808] sendo a ultima baixa feita [1808]-20/07/2026 08:20:32.. - Data Comentário: 20/07/2026 08:19</t>
         </is>
       </c>
       <c r="W478" t="inlineStr"/>
@@ -52210,22 +52210,18 @@
       <c r="AE478" t="inlineStr"/>
       <c r="AF478" t="inlineStr">
         <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AG478" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
+          <t>Imposto</t>
+        </is>
+      </c>
+      <c r="AG478" t="inlineStr"/>
     </row>
     <row r="479">
       <c r="A479" t="n">
-        <v>5417</v>
+        <v>6703</v>
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
@@ -52235,7 +52231,7 @@
       </c>
       <c r="D479" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E479" t="inlineStr">
@@ -52245,7 +52241,7 @@
       </c>
       <c r="F479" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G479" t="n">
@@ -52275,7 +52271,7 @@
         </is>
       </c>
       <c r="O479" t="n">
-        <v>17398881</v>
+        <v>17941164</v>
       </c>
       <c r="P479" t="inlineStr">
         <is>
@@ -52293,7 +52289,7 @@
       </c>
       <c r="T479" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>LIMA MOTA</t>
         </is>
       </c>
       <c r="U479" t="inlineStr">
@@ -52303,7 +52299,7 @@
       </c>
       <c r="V479" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1808] sendo a ultima baixa feita [1808]-20/07/2026 08:20:32.. - Data Comentário: 20/07/2026 08:19</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1807] sendo a ultima baixa feita [1807]-20/07/2026 08:20:29.. - Data Comentário: 20/07/2026 08:19</t>
         </is>
       </c>
       <c r="W479" t="inlineStr"/>
@@ -52326,11 +52322,11 @@
     </row>
     <row r="480">
       <c r="A480" t="n">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
@@ -52340,7 +52336,7 @@
       </c>
       <c r="D480" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E480" t="inlineStr">
@@ -52380,7 +52376,7 @@
         </is>
       </c>
       <c r="O480" t="n">
-        <v>17941164</v>
+        <v>17952360</v>
       </c>
       <c r="P480" t="inlineStr">
         <is>
@@ -52398,7 +52394,7 @@
       </c>
       <c r="T480" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U480" t="inlineStr">
@@ -52408,7 +52404,7 @@
       </c>
       <c r="V480" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1807] sendo a ultima baixa feita [1807]-20/07/2026 08:20:29.. - Data Comentário: 20/07/2026 08:19</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1808] sendo a ultima baixa feita [1808]-22/07/2026 12:44:41.. - Data Comentário: 22/07/2026 12:43</t>
         </is>
       </c>
       <c r="W480" t="inlineStr"/>
@@ -69610,11 +69606,11 @@
     </row>
     <row r="636">
       <c r="A636" t="n">
-        <v>5417</v>
+        <v>6704</v>
       </c>
       <c r="B636" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C636" t="inlineStr">
@@ -69634,11 +69630,11 @@
       </c>
       <c r="F636" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G636" t="n">
-        <v>7025</v>
+        <v>1808</v>
       </c>
       <c r="H636" t="n">
         <v>0</v>
@@ -69650,12 +69646,12 @@
       </c>
       <c r="J636" t="inlineStr">
         <is>
-          <t>Movimento - Sistema de Análise</t>
+          <t>Fed - PIS/COFINS Não Cumul/Mon - 5856</t>
         </is>
       </c>
       <c r="K636" t="inlineStr"/>
       <c r="L636" s="1" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="M636" t="inlineStr"/>
       <c r="N636" t="inlineStr">
@@ -69664,7 +69660,7 @@
         </is>
       </c>
       <c r="O636" t="n">
-        <v>17399278</v>
+        <v>18085207</v>
       </c>
       <c r="P636" t="inlineStr">
         <is>
@@ -69677,14 +69673,14 @@
         </is>
       </c>
       <c r="R636" s="1" t="n">
-        <v>46217.51638267361</v>
+        <v>46225.5310378125</v>
       </c>
       <c r="S636" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T636" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U636" t="inlineStr">
@@ -69694,7 +69690,7 @@
       </c>
       <c r="V636" t="inlineStr">
         <is>
-          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 14/07/2026 12:21:15. - Data Comentário: 14/07/2026 12:20</t>
+          <t>Imposto enviado via SCI Report - Data Comentário: 22/07/2026 11:55</t>
         </is>
       </c>
       <c r="W636" t="inlineStr"/>
@@ -69705,7 +69701,7 @@
       </c>
       <c r="AA636" t="inlineStr">
         <is>
-          <t>ex-funcionario</t>
+          <t>Juan Rodrigues</t>
         </is>
       </c>
       <c r="AB636" t="inlineStr"/>
@@ -69714,7 +69710,7 @@
       <c r="AE636" t="inlineStr"/>
       <c r="AF636" t="inlineStr">
         <is>
-          <t>Tarefa</t>
+          <t>Imposto</t>
         </is>
       </c>
       <c r="AG636" t="inlineStr">
@@ -69725,11 +69721,11 @@
     </row>
     <row r="637">
       <c r="A637" t="n">
-        <v>6278</v>
+        <v>5417</v>
       </c>
       <c r="B637" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C637" t="inlineStr">
@@ -69739,7 +69735,7 @@
       </c>
       <c r="D637" t="inlineStr">
         <is>
-          <t>Federal - Lucro Real - Anual</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E637" t="inlineStr">
@@ -69749,7 +69745,7 @@
       </c>
       <c r="F637" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G637" t="n">
@@ -69779,7 +69775,7 @@
         </is>
       </c>
       <c r="O637" t="n">
-        <v>17539786</v>
+        <v>17399278</v>
       </c>
       <c r="P637" t="inlineStr">
         <is>
@@ -69792,14 +69788,14 @@
         </is>
       </c>
       <c r="R637" s="1" t="n">
-        <v>46225.36690239584</v>
+        <v>46217.51638267361</v>
       </c>
       <c r="S637" t="n">
         <v>-1</v>
       </c>
       <c r="T637" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U637" t="inlineStr">
@@ -69809,7 +69805,7 @@
       </c>
       <c r="V637" t="inlineStr">
         <is>
-          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 22/07/2026 08:51:07. - Data Comentário: 22/07/2026 08:46</t>
+          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 14/07/2026 12:21:15. - Data Comentário: 14/07/2026 12:20</t>
         </is>
       </c>
       <c r="W637" t="inlineStr"/>
@@ -69840,11 +69836,11 @@
     </row>
     <row r="638">
       <c r="A638" t="n">
-        <v>6279</v>
+        <v>6278</v>
       </c>
       <c r="B638" t="inlineStr">
         <is>
-          <t>DIENNYFER DA S PEREIRA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="C638" t="inlineStr">
@@ -69854,7 +69850,7 @@
       </c>
       <c r="D638" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - Lucro Real - Anual</t>
         </is>
       </c>
       <c r="E638" t="inlineStr">
@@ -69864,7 +69860,7 @@
       </c>
       <c r="F638" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G638" t="n">
@@ -69894,16 +69890,20 @@
         </is>
       </c>
       <c r="O638" t="n">
-        <v>17646092</v>
-      </c>
-      <c r="P638" t="inlineStr"/>
+        <v>17539786</v>
+      </c>
+      <c r="P638" t="inlineStr">
+        <is>
+          <t>Cristina Leite</t>
+        </is>
+      </c>
       <c r="Q638" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R638" s="1" t="n">
-        <v>46219.46361605324</v>
+        <v>46225.36690239584</v>
       </c>
       <c r="S638" t="n">
         <v>-1</v>
@@ -69920,7 +69920,7 @@
       </c>
       <c r="V638" t="inlineStr">
         <is>
-          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 16/07/2026 11:08:58. - Data Comentário: 16/07/2026 11:04</t>
+          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 22/07/2026 08:51:07. - Data Comentário: 22/07/2026 08:46</t>
         </is>
       </c>
       <c r="W638" t="inlineStr"/>
@@ -69943,15 +69943,19 @@
           <t>Tarefa</t>
         </is>
       </c>
-      <c r="AG638" t="inlineStr"/>
+      <c r="AG638" t="inlineStr">
+        <is>
+          <t>Ricardo Fischer</t>
+        </is>
+      </c>
     </row>
     <row r="639">
       <c r="A639" t="n">
-        <v>6404</v>
+        <v>6279</v>
       </c>
       <c r="B639" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>DIENNYFER DA S PEREIRA</t>
         </is>
       </c>
       <c r="C639" t="inlineStr">
@@ -69971,7 +69975,7 @@
       </c>
       <c r="F639" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G639" t="n">
@@ -70001,27 +70005,23 @@
         </is>
       </c>
       <c r="O639" t="n">
-        <v>16962336</v>
-      </c>
-      <c r="P639" t="inlineStr">
-        <is>
-          <t>Cristina Leite</t>
-        </is>
-      </c>
+        <v>17646092</v>
+      </c>
+      <c r="P639" t="inlineStr"/>
       <c r="Q639" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R639" s="1" t="n">
-        <v>46210.75621153935</v>
+        <v>46219.46361605324</v>
       </c>
       <c r="S639" t="n">
         <v>-1</v>
       </c>
       <c r="T639" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U639" t="inlineStr">
@@ -70031,7 +70031,7 @@
       </c>
       <c r="V639" t="inlineStr">
         <is>
-          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 07/07/2026 18:06:44. - Data Comentário: 07/07/2026 18:05</t>
+          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 16/07/2026 11:08:58. - Data Comentário: 16/07/2026 11:04</t>
         </is>
       </c>
       <c r="W639" t="inlineStr"/>
@@ -70054,19 +70054,15 @@
           <t>Tarefa</t>
         </is>
       </c>
-      <c r="AG639" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
+      <c r="AG639" t="inlineStr"/>
     </row>
     <row r="640">
       <c r="A640" t="n">
-        <v>6486</v>
+        <v>6404</v>
       </c>
       <c r="B640" t="inlineStr">
         <is>
-          <t>PC GAMER GOIANIA LTDA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="C640" t="inlineStr">
@@ -70076,7 +70072,7 @@
       </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E640" t="inlineStr">
@@ -70116,7 +70112,7 @@
         </is>
       </c>
       <c r="O640" t="n">
-        <v>16976225</v>
+        <v>16962336</v>
       </c>
       <c r="P640" t="inlineStr">
         <is>
@@ -70129,14 +70125,14 @@
         </is>
       </c>
       <c r="R640" s="1" t="n">
-        <v>46224.47371898148</v>
+        <v>46210.75621153935</v>
       </c>
       <c r="S640" t="n">
         <v>-1</v>
       </c>
       <c r="T640" t="inlineStr">
         <is>
-          <t>PC GAMER</t>
+          <t>SOLAR INVESTIMENTOS</t>
         </is>
       </c>
       <c r="U640" t="inlineStr">
@@ -70146,7 +70142,7 @@
       </c>
       <c r="V640" t="inlineStr">
         <is>
-          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 21/07/2026 11:25:23. - Data Comentário: 21/07/2026 11:20</t>
+          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 07/07/2026 18:06:44. - Data Comentário: 07/07/2026 18:05</t>
         </is>
       </c>
       <c r="W640" t="inlineStr"/>
@@ -70177,11 +70173,11 @@
     </row>
     <row r="641">
       <c r="A641" t="n">
-        <v>5417</v>
+        <v>6486</v>
       </c>
       <c r="B641" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C641" t="inlineStr">
@@ -70201,11 +70197,11 @@
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G641" t="n">
-        <v>1793</v>
+        <v>7025</v>
       </c>
       <c r="H641" t="n">
         <v>0</v>
@@ -70217,25 +70213,21 @@
       </c>
       <c r="J641" t="inlineStr">
         <is>
-          <t>Mun - ISS Serv. Tomados</t>
+          <t>Movimento - Sistema de Análise</t>
         </is>
       </c>
       <c r="K641" t="inlineStr"/>
       <c r="L641" s="1" t="n">
-        <v>46220</v>
-      </c>
-      <c r="M641" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
+        <v>46226</v>
+      </c>
+      <c r="M641" t="inlineStr"/>
       <c r="N641" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O641" t="n">
-        <v>17398943</v>
+        <v>16976225</v>
       </c>
       <c r="P641" t="inlineStr">
         <is>
@@ -70248,14 +70240,14 @@
         </is>
       </c>
       <c r="R641" s="1" t="n">
-        <v>46213.36370773148</v>
+        <v>46224.47371898148</v>
       </c>
       <c r="S641" t="n">
-        <v>5</v>
+        <v>-1</v>
       </c>
       <c r="T641" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U641" t="inlineStr">
@@ -70265,7 +70257,7 @@
       </c>
       <c r="V641" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 15:51</t>
+          <t>Baixado via API integração MGC x Sistema de Analise Fiscal em 21/07/2026 11:25:23. - Data Comentário: 21/07/2026 11:20</t>
         </is>
       </c>
       <c r="W641" t="inlineStr"/>
@@ -70276,7 +70268,7 @@
       </c>
       <c r="AA641" t="inlineStr">
         <is>
-          <t>Cristina Leite</t>
+          <t>ex-funcionario</t>
         </is>
       </c>
       <c r="AB641" t="inlineStr"/>
@@ -70285,7 +70277,7 @@
       <c r="AE641" t="inlineStr"/>
       <c r="AF641" t="inlineStr">
         <is>
-          <t>Imposto</t>
+          <t>Tarefa</t>
         </is>
       </c>
       <c r="AG641" t="inlineStr">
@@ -70296,11 +70288,11 @@
     </row>
     <row r="642">
       <c r="A642" t="n">
-        <v>6628</v>
+        <v>5417</v>
       </c>
       <c r="B642" t="inlineStr">
         <is>
-          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C642" t="inlineStr">
@@ -70310,51 +70302,55 @@
       </c>
       <c r="D642" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E642" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F642" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G642" t="n">
-        <v>945</v>
+        <v>1793</v>
       </c>
       <c r="H642" t="n">
         <v>0</v>
       </c>
       <c r="I642" t="inlineStr">
         <is>
-          <t>GC - ADMINISTRATIVO</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J642" t="inlineStr">
         <is>
-          <t>Confirm Rec - DAS</t>
+          <t>Mun - ISS Serv. Tomados</t>
         </is>
       </c>
       <c r="K642" t="inlineStr"/>
       <c r="L642" s="1" t="n">
-        <v>46223</v>
-      </c>
-      <c r="M642" t="inlineStr"/>
+        <v>46220</v>
+      </c>
+      <c r="M642" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
       <c r="N642" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O642" t="n">
-        <v>16959936</v>
+        <v>17398943</v>
       </c>
       <c r="P642" t="inlineStr">
         <is>
-          <t>Victoria Virgens</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="Q642" t="inlineStr">
@@ -70363,14 +70359,14 @@
         </is>
       </c>
       <c r="R642" s="1" t="n">
-        <v>46219.69905140046</v>
+        <v>46213.36370773148</v>
       </c>
       <c r="S642" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T642" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U642" t="inlineStr">
@@ -70380,7 +70376,7 @@
       </c>
       <c r="V642" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1879] sendo a ultima baixa feita [1879]-16/07/2026 16:08:46.. - Data Comentário: 16/07/2026 16:07</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 15:51</t>
         </is>
       </c>
       <c r="W642" t="inlineStr"/>
@@ -70391,7 +70387,7 @@
       </c>
       <c r="AA642" t="inlineStr">
         <is>
-          <t>Victoria Virgens</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="AB642" t="inlineStr"/>
@@ -70403,15 +70399,19 @@
           <t>Imposto</t>
         </is>
       </c>
-      <c r="AG642" t="inlineStr"/>
+      <c r="AG642" t="inlineStr">
+        <is>
+          <t>Ricardo Fischer</t>
+        </is>
+      </c>
     </row>
     <row r="643">
       <c r="A643" t="n">
-        <v>6705</v>
+        <v>6628</v>
       </c>
       <c r="B643" t="inlineStr">
         <is>
-          <t>NARCIZO ALVES CORDEIRO</t>
+          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
         </is>
       </c>
       <c r="C643" t="inlineStr">
@@ -70426,7 +70426,7 @@
       </c>
       <c r="E643" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F643" t="inlineStr">
@@ -70461,23 +70461,27 @@
         </is>
       </c>
       <c r="O643" t="n">
-        <v>17952522</v>
-      </c>
-      <c r="P643" t="inlineStr"/>
+        <v>16959936</v>
+      </c>
+      <c r="P643" t="inlineStr">
+        <is>
+          <t>Victoria Virgens</t>
+        </is>
+      </c>
       <c r="Q643" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R643" s="1" t="n">
-        <v>46218.72615659722</v>
+        <v>46219.69905140046</v>
       </c>
       <c r="S643" t="n">
         <v>2</v>
       </c>
       <c r="T643" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U643" t="inlineStr">
@@ -70487,7 +70491,7 @@
       </c>
       <c r="V643" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1805] sendo a ultima baixa feita [1805]-14/07/2026 10:55:51.. - Data Comentário: 14/07/2026 10:54</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1879] sendo a ultima baixa feita [1879]-16/07/2026 16:08:46.. - Data Comentário: 16/07/2026 16:07</t>
         </is>
       </c>
       <c r="W643" t="inlineStr"/>
@@ -70514,11 +70518,11 @@
     </row>
     <row r="644">
       <c r="A644" t="n">
-        <v>6779</v>
+        <v>6705</v>
       </c>
       <c r="B644" t="inlineStr">
         <is>
-          <t>CORDEIRO E CIA LTDA</t>
+          <t>NARCIZO ALVES CORDEIRO</t>
         </is>
       </c>
       <c r="C644" t="inlineStr">
@@ -70568,20 +70572,16 @@
         </is>
       </c>
       <c r="O644" t="n">
-        <v>18056693</v>
-      </c>
-      <c r="P644" t="inlineStr">
-        <is>
-          <t>Victoria Virgens</t>
-        </is>
-      </c>
+        <v>17952522</v>
+      </c>
+      <c r="P644" t="inlineStr"/>
       <c r="Q644" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R644" s="1" t="n">
-        <v>46218.7261571412</v>
+        <v>46218.72615659722</v>
       </c>
       <c r="S644" t="n">
         <v>2</v>
@@ -70591,10 +70591,14 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U644" t="inlineStr"/>
+      <c r="U644" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="V644" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1805] sendo a ultima baixa feita [1805]-14/07/2026 10:55:52.. - Data Comentário: 14/07/2026 10:54</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1805] sendo a ultima baixa feita [1805]-14/07/2026 10:55:51.. - Data Comentário: 14/07/2026 10:54</t>
         </is>
       </c>
       <c r="W644" t="inlineStr"/>
@@ -70621,11 +70625,11 @@
     </row>
     <row r="645">
       <c r="A645" t="n">
-        <v>6885</v>
+        <v>6779</v>
       </c>
       <c r="B645" t="inlineStr">
         <is>
-          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
+          <t>CORDEIRO E CIA LTDA</t>
         </is>
       </c>
       <c r="C645" t="inlineStr">
@@ -70675,29 +70679,33 @@
         </is>
       </c>
       <c r="O645" t="n">
-        <v>18128639</v>
-      </c>
-      <c r="P645" t="inlineStr"/>
+        <v>18056693</v>
+      </c>
+      <c r="P645" t="inlineStr">
+        <is>
+          <t>Victoria Virgens</t>
+        </is>
+      </c>
       <c r="Q645" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R645" s="1" t="n">
-        <v>46218.72455349537</v>
+        <v>46218.7261571412</v>
       </c>
       <c r="S645" t="n">
         <v>2</v>
       </c>
       <c r="T645" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U645" t="inlineStr"/>
       <c r="V645" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1805] sendo a ultima baixa feita [1805]-14/07/2026 09:05:39.. - Data Comentário: 14/07/2026 09:04</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1805] sendo a ultima baixa feita [1805]-14/07/2026 10:55:52.. - Data Comentário: 14/07/2026 10:54</t>
         </is>
       </c>
       <c r="W645" t="inlineStr"/>
@@ -70724,11 +70732,11 @@
     </row>
     <row r="646">
       <c r="A646" t="n">
-        <v>6945</v>
+        <v>6885</v>
       </c>
       <c r="B646" t="inlineStr">
         <is>
-          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
+          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
         </is>
       </c>
       <c r="C646" t="inlineStr">
@@ -70743,7 +70751,7 @@
       </c>
       <c r="E646" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F646" t="inlineStr">
@@ -70778,31 +70786,31 @@
         </is>
       </c>
       <c r="O646" t="n">
-        <v>18164485</v>
-      </c>
-      <c r="P646" t="inlineStr">
-        <is>
-          <t>Victoria Virgens</t>
-        </is>
-      </c>
+        <v>18128639</v>
+      </c>
+      <c r="P646" t="inlineStr"/>
       <c r="Q646" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R646" s="1" t="n">
-        <v>46210.80007584491</v>
+        <v>46218.72455349537</v>
       </c>
       <c r="S646" t="n">
         <v>2</v>
       </c>
       <c r="T646" t="inlineStr">
         <is>
-          <t>BRASIL DISTRIBUIDORA</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U646" t="inlineStr"/>
-      <c r="V646" t="inlineStr"/>
+      <c r="V646" t="inlineStr">
+        <is>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1805] sendo a ultima baixa feita [1805]-14/07/2026 09:05:39.. - Data Comentário: 14/07/2026 09:04</t>
+        </is>
+      </c>
       <c r="W646" t="inlineStr"/>
       <c r="X646" t="inlineStr"/>
       <c r="Y646" t="inlineStr"/>
@@ -70827,11 +70835,11 @@
     </row>
     <row r="647">
       <c r="A647" t="n">
-        <v>5417</v>
+        <v>6945</v>
       </c>
       <c r="B647" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
         </is>
       </c>
       <c r="C647" t="inlineStr">
@@ -70841,21 +70849,21 @@
       </c>
       <c r="D647" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E647" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F647" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G647" t="n">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="H647" t="n">
         <v>0</v>
@@ -70867,7 +70875,7 @@
       </c>
       <c r="J647" t="inlineStr">
         <is>
-          <t>Confirm Rec - ICMS RPA</t>
+          <t>Confirm Rec - DAS</t>
         </is>
       </c>
       <c r="K647" t="inlineStr"/>
@@ -70881,7 +70889,7 @@
         </is>
       </c>
       <c r="O647" t="n">
-        <v>17398867</v>
+        <v>18164485</v>
       </c>
       <c r="P647" t="inlineStr">
         <is>
@@ -70894,26 +70902,18 @@
         </is>
       </c>
       <c r="R647" s="1" t="n">
-        <v>46223.52112873842</v>
+        <v>46210.80007584491</v>
       </c>
       <c r="S647" t="n">
         <v>2</v>
       </c>
       <c r="T647" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
-        </is>
-      </c>
-      <c r="U647" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="V647" t="inlineStr">
-        <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [11286] sendo a ultima baixa feita [11286]-17/07/2026 10:29:09.. - Data Comentário: 17/07/2026 10:28</t>
-        </is>
-      </c>
+          <t>BRASIL DISTRIBUIDORA</t>
+        </is>
+      </c>
+      <c r="U647" t="inlineStr"/>
+      <c r="V647" t="inlineStr"/>
       <c r="W647" t="inlineStr"/>
       <c r="X647" t="inlineStr"/>
       <c r="Y647" t="inlineStr"/>
@@ -70938,11 +70938,11 @@
     </row>
     <row r="648">
       <c r="A648" t="n">
-        <v>6278</v>
+        <v>5417</v>
       </c>
       <c r="B648" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C648" t="inlineStr">
@@ -70952,7 +70952,7 @@
       </c>
       <c r="D648" t="inlineStr">
         <is>
-          <t>Federal - Lucro Real - Anual</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E648" t="inlineStr">
@@ -70962,7 +70962,7 @@
       </c>
       <c r="F648" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G648" t="n">
@@ -70992,23 +70992,27 @@
         </is>
       </c>
       <c r="O648" t="n">
-        <v>17539708</v>
-      </c>
-      <c r="P648" t="inlineStr"/>
+        <v>17398867</v>
+      </c>
+      <c r="P648" t="inlineStr">
+        <is>
+          <t>Victoria Virgens</t>
+        </is>
+      </c>
       <c r="Q648" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R648" s="1" t="n">
-        <v>46223.52113091435</v>
+        <v>46223.52112873842</v>
       </c>
       <c r="S648" t="n">
         <v>2</v>
       </c>
       <c r="T648" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U648" t="inlineStr">
@@ -71018,7 +71022,7 @@
       </c>
       <c r="V648" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [11286] sendo a ultima baixa feita [11286]-17/07/2026 10:29:10.. - Data Comentário: 17/07/2026 10:28</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [11286] sendo a ultima baixa feita [11286]-17/07/2026 10:29:09.. - Data Comentário: 17/07/2026 10:28</t>
         </is>
       </c>
       <c r="W648" t="inlineStr"/>
@@ -71045,11 +71049,11 @@
     </row>
     <row r="649">
       <c r="A649" t="n">
-        <v>6404</v>
+        <v>6278</v>
       </c>
       <c r="B649" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="C649" t="inlineStr">
@@ -71059,7 +71063,7 @@
       </c>
       <c r="D649" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - Lucro Real - Anual</t>
         </is>
       </c>
       <c r="E649" t="inlineStr">
@@ -71099,27 +71103,23 @@
         </is>
       </c>
       <c r="O649" t="n">
-        <v>16962091</v>
-      </c>
-      <c r="P649" t="inlineStr">
-        <is>
-          <t>Victoria Virgens</t>
-        </is>
-      </c>
+        <v>17539708</v>
+      </c>
+      <c r="P649" t="inlineStr"/>
       <c r="Q649" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R649" s="1" t="n">
-        <v>46223.52113200232</v>
+        <v>46223.52113091435</v>
       </c>
       <c r="S649" t="n">
         <v>2</v>
       </c>
       <c r="T649" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U649" t="inlineStr">
@@ -71156,11 +71156,11 @@
     </row>
     <row r="650">
       <c r="A650" t="n">
-        <v>6627</v>
+        <v>6404</v>
       </c>
       <c r="B650" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="C650" t="inlineStr">
@@ -71170,12 +71170,12 @@
       </c>
       <c r="D650" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E650" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F650" t="inlineStr">
@@ -71210,7 +71210,7 @@
         </is>
       </c>
       <c r="O650" t="n">
-        <v>17042267</v>
+        <v>16962091</v>
       </c>
       <c r="P650" t="inlineStr">
         <is>
@@ -71223,14 +71223,14 @@
         </is>
       </c>
       <c r="R650" s="1" t="n">
-        <v>46219.51514050926</v>
+        <v>46223.52113200232</v>
       </c>
       <c r="S650" t="n">
         <v>2</v>
       </c>
       <c r="T650" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>SOLAR INVESTIMENTOS</t>
         </is>
       </c>
       <c r="U650" t="inlineStr">
@@ -71238,7 +71238,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V650" t="inlineStr"/>
+      <c r="V650" t="inlineStr">
+        <is>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [11286] sendo a ultima baixa feita [11286]-17/07/2026 10:29:10.. - Data Comentário: 17/07/2026 10:28</t>
+        </is>
+      </c>
       <c r="W650" t="inlineStr"/>
       <c r="X650" t="inlineStr"/>
       <c r="Y650" t="inlineStr"/>
@@ -71263,11 +71267,11 @@
     </row>
     <row r="651">
       <c r="A651" t="n">
-        <v>6703</v>
+        <v>6627</v>
       </c>
       <c r="B651" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C651" t="inlineStr">
@@ -71277,12 +71281,12 @@
       </c>
       <c r="D651" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E651" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F651" t="inlineStr">
@@ -71317,7 +71321,7 @@
         </is>
       </c>
       <c r="O651" t="n">
-        <v>17941130</v>
+        <v>17042267</v>
       </c>
       <c r="P651" t="inlineStr">
         <is>
@@ -71330,14 +71334,14 @@
         </is>
       </c>
       <c r="R651" s="1" t="n">
-        <v>46223.52113940972</v>
+        <v>46219.51514050926</v>
       </c>
       <c r="S651" t="n">
         <v>2</v>
       </c>
       <c r="T651" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U651" t="inlineStr">
@@ -71345,11 +71349,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V651" t="inlineStr">
-        <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1802] sendo a ultima baixa feita [1802]-17/07/2026 10:29:09.. - Data Comentário: 17/07/2026 10:28</t>
-        </is>
-      </c>
+      <c r="V651" t="inlineStr"/>
       <c r="W651" t="inlineStr"/>
       <c r="X651" t="inlineStr"/>
       <c r="Y651" t="inlineStr"/>
@@ -71374,11 +71374,11 @@
     </row>
     <row r="652">
       <c r="A652" t="n">
-        <v>6704</v>
+        <v>6703</v>
       </c>
       <c r="B652" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C652" t="inlineStr">
@@ -71388,7 +71388,7 @@
       </c>
       <c r="D652" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E652" t="inlineStr">
@@ -71428,23 +71428,27 @@
         </is>
       </c>
       <c r="O652" t="n">
-        <v>17952323</v>
-      </c>
-      <c r="P652" t="inlineStr"/>
+        <v>17941130</v>
+      </c>
+      <c r="P652" t="inlineStr">
+        <is>
+          <t>Victoria Virgens</t>
+        </is>
+      </c>
       <c r="Q652" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R652" s="1" t="n">
-        <v>46223.52114085648</v>
+        <v>46223.52113940972</v>
       </c>
       <c r="S652" t="n">
         <v>2</v>
       </c>
       <c r="T652" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>LIMA MOTA</t>
         </is>
       </c>
       <c r="U652" t="inlineStr">
@@ -71454,7 +71458,7 @@
       </c>
       <c r="V652" t="inlineStr">
         <is>
-          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1802] sendo a ultima baixa feita [1802]-20/07/2026 09:58:46.. - Data Comentário: 20/07/2026 09:57</t>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1802] sendo a ultima baixa feita [1802]-17/07/2026 10:29:09.. - Data Comentário: 17/07/2026 10:28</t>
         </is>
       </c>
       <c r="W652" t="inlineStr"/>
@@ -71481,11 +71485,11 @@
     </row>
     <row r="653">
       <c r="A653" t="n">
-        <v>6885</v>
+        <v>6704</v>
       </c>
       <c r="B653" t="inlineStr">
         <is>
-          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C653" t="inlineStr">
@@ -71495,7 +71499,7 @@
       </c>
       <c r="D653" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E653" t="inlineStr">
@@ -71535,7 +71539,7 @@
         </is>
       </c>
       <c r="O653" t="n">
-        <v>18128648</v>
+        <v>17952323</v>
       </c>
       <c r="P653" t="inlineStr"/>
       <c r="Q653" t="inlineStr">
@@ -71544,18 +71548,26 @@
         </is>
       </c>
       <c r="R653" s="1" t="n">
-        <v>46216.49331971065</v>
+        <v>46223.52114085648</v>
       </c>
       <c r="S653" t="n">
         <v>2</v>
       </c>
       <c r="T653" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
-        </is>
-      </c>
-      <c r="U653" t="inlineStr"/>
-      <c r="V653" t="inlineStr"/>
+          <t>TECNO COM</t>
+        </is>
+      </c>
+      <c r="U653" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V653" t="inlineStr">
+        <is>
+          <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1802] sendo a ultima baixa feita [1802]-20/07/2026 09:58:46.. - Data Comentário: 20/07/2026 09:57</t>
+        </is>
+      </c>
       <c r="W653" t="inlineStr"/>
       <c r="X653" t="inlineStr"/>
       <c r="Y653" t="inlineStr"/>
@@ -71580,11 +71592,11 @@
     </row>
     <row r="654">
       <c r="A654" t="n">
-        <v>6945</v>
+        <v>6885</v>
       </c>
       <c r="B654" t="inlineStr">
         <is>
-          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
+          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
         </is>
       </c>
       <c r="C654" t="inlineStr">
@@ -71599,7 +71611,7 @@
       </c>
       <c r="E654" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F654" t="inlineStr">
@@ -71634,27 +71646,23 @@
         </is>
       </c>
       <c r="O654" t="n">
-        <v>18164492</v>
-      </c>
-      <c r="P654" t="inlineStr">
-        <is>
-          <t>Victoria Virgens</t>
-        </is>
-      </c>
+        <v>18128648</v>
+      </c>
+      <c r="P654" t="inlineStr"/>
       <c r="Q654" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R654" s="1" t="n">
-        <v>46216.49332078703</v>
+        <v>46216.49331971065</v>
       </c>
       <c r="S654" t="n">
         <v>2</v>
       </c>
       <c r="T654" t="inlineStr">
         <is>
-          <t>BRASIL DISTRIBUIDORA</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U654" t="inlineStr"/>
@@ -71683,11 +71691,11 @@
     </row>
     <row r="655">
       <c r="A655" t="n">
-        <v>5417</v>
+        <v>6945</v>
       </c>
       <c r="B655" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
         </is>
       </c>
       <c r="C655" t="inlineStr">
@@ -71697,21 +71705,21 @@
       </c>
       <c r="D655" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E655" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F655" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G655" t="n">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="H655" t="n">
         <v>0</v>
@@ -71723,12 +71731,12 @@
       </c>
       <c r="J655" t="inlineStr">
         <is>
-          <t>Confirm Rec - IRPJ/CSLL (CTB)</t>
+          <t>Confirm Rec - ICMS RPA</t>
         </is>
       </c>
       <c r="K655" t="inlineStr"/>
       <c r="L655" s="1" t="n">
-        <v>46233</v>
+        <v>46223</v>
       </c>
       <c r="M655" t="inlineStr"/>
       <c r="N655" t="inlineStr">
@@ -71737,7 +71745,7 @@
         </is>
       </c>
       <c r="O655" t="n">
-        <v>17398875</v>
+        <v>18164492</v>
       </c>
       <c r="P655" t="inlineStr">
         <is>
@@ -71750,26 +71758,18 @@
         </is>
       </c>
       <c r="R655" s="1" t="n">
-        <v>46204.29183217593</v>
+        <v>46216.49332078703</v>
       </c>
       <c r="S655" t="n">
-        <v>-8</v>
+        <v>2</v>
       </c>
       <c r="T655" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
-        </is>
-      </c>
-      <c r="U655" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="V655" t="inlineStr">
-        <is>
-          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1582]. - Data Comentário: 01/07/2026 06:59</t>
-        </is>
-      </c>
+          <t>BRASIL DISTRIBUIDORA</t>
+        </is>
+      </c>
+      <c r="U655" t="inlineStr"/>
+      <c r="V655" t="inlineStr"/>
       <c r="W655" t="inlineStr"/>
       <c r="X655" t="inlineStr"/>
       <c r="Y655" t="inlineStr"/>
@@ -71778,7 +71778,7 @@
       </c>
       <c r="AA655" t="inlineStr">
         <is>
-          <t>ex-funcionario</t>
+          <t>Victoria Virgens</t>
         </is>
       </c>
       <c r="AB655" t="inlineStr"/>
@@ -71794,11 +71794,11 @@
     </row>
     <row r="656">
       <c r="A656" t="n">
-        <v>6278</v>
+        <v>5417</v>
       </c>
       <c r="B656" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C656" t="inlineStr">
@@ -71808,7 +71808,7 @@
       </c>
       <c r="D656" t="inlineStr">
         <is>
-          <t>Federal - Lucro Real - Anual</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E656" t="inlineStr">
@@ -71818,7 +71818,7 @@
       </c>
       <c r="F656" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G656" t="n">
@@ -71848,23 +71848,27 @@
         </is>
       </c>
       <c r="O656" t="n">
-        <v>17539716</v>
-      </c>
-      <c r="P656" t="inlineStr"/>
+        <v>17398875</v>
+      </c>
+      <c r="P656" t="inlineStr">
+        <is>
+          <t>Victoria Virgens</t>
+        </is>
+      </c>
       <c r="Q656" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R656" s="1" t="n">
-        <v>46204.33341168981</v>
+        <v>46204.29183217593</v>
       </c>
       <c r="S656" t="n">
         <v>-8</v>
       </c>
       <c r="T656" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U656" t="inlineStr">
@@ -71874,7 +71878,7 @@
       </c>
       <c r="V656" t="inlineStr">
         <is>
-          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1582]. - Data Comentário: 01/07/2026 07:59</t>
+          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1582]. - Data Comentário: 01/07/2026 06:59</t>
         </is>
       </c>
       <c r="W656" t="inlineStr"/>
@@ -71901,11 +71905,11 @@
     </row>
     <row r="657">
       <c r="A657" t="n">
-        <v>6627</v>
+        <v>6278</v>
       </c>
       <c r="B657" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="C657" t="inlineStr">
@@ -71915,12 +71919,12 @@
       </c>
       <c r="D657" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Real - Anual</t>
         </is>
       </c>
       <c r="E657" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F657" t="inlineStr">
@@ -71955,27 +71959,23 @@
         </is>
       </c>
       <c r="O657" t="n">
-        <v>17042295</v>
-      </c>
-      <c r="P657" t="inlineStr">
-        <is>
-          <t>Victoria Virgens</t>
-        </is>
-      </c>
+        <v>17539716</v>
+      </c>
+      <c r="P657" t="inlineStr"/>
       <c r="Q657" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R657" s="1" t="n">
-        <v>46204.25011258102</v>
+        <v>46204.33341168981</v>
       </c>
       <c r="S657" t="n">
         <v>-8</v>
       </c>
       <c r="T657" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U657" t="inlineStr">
@@ -71985,7 +71985,7 @@
       </c>
       <c r="V657" t="inlineStr">
         <is>
-          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1651]. - Data Comentário: 01/07/2026 05:59</t>
+          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1582]. - Data Comentário: 01/07/2026 07:59</t>
         </is>
       </c>
       <c r="W657" t="inlineStr"/>
@@ -72012,11 +72012,11 @@
     </row>
     <row r="658">
       <c r="A658" t="n">
-        <v>6704</v>
+        <v>6627</v>
       </c>
       <c r="B658" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C658" t="inlineStr">
@@ -72031,7 +72031,7 @@
       </c>
       <c r="E658" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F658" t="inlineStr">
@@ -72066,7 +72066,7 @@
         </is>
       </c>
       <c r="O658" t="n">
-        <v>17952331</v>
+        <v>17042295</v>
       </c>
       <c r="P658" t="inlineStr">
         <is>
@@ -72079,14 +72079,14 @@
         </is>
       </c>
       <c r="R658" s="1" t="n">
-        <v>46204.37522271991</v>
+        <v>46204.25011258102</v>
       </c>
       <c r="S658" t="n">
         <v>-8</v>
       </c>
       <c r="T658" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U658" t="inlineStr">
@@ -72096,7 +72096,7 @@
       </c>
       <c r="V658" t="inlineStr">
         <is>
-          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1582]. - Data Comentário: 01/07/2026 08:59</t>
+          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1651]. - Data Comentário: 01/07/2026 05:59</t>
         </is>
       </c>
       <c r="W658" t="inlineStr"/>
@@ -72123,11 +72123,11 @@
     </row>
     <row r="659">
       <c r="A659" t="n">
-        <v>6404</v>
+        <v>6704</v>
       </c>
       <c r="B659" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C659" t="inlineStr">
@@ -72137,7 +72137,7 @@
       </c>
       <c r="D659" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E659" t="inlineStr">
@@ -72151,7 +72151,7 @@
         </is>
       </c>
       <c r="G659" t="n">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="H659" t="n">
         <v>0</v>
@@ -72163,7 +72163,7 @@
       </c>
       <c r="J659" t="inlineStr">
         <is>
-          <t>Confirm Rec - IRPJ/CSLL (EF)</t>
+          <t>Confirm Rec - IRPJ/CSLL (CTB)</t>
         </is>
       </c>
       <c r="K659" t="inlineStr"/>
@@ -72177,7 +72177,7 @@
         </is>
       </c>
       <c r="O659" t="n">
-        <v>16962099</v>
+        <v>17952331</v>
       </c>
       <c r="P659" t="inlineStr">
         <is>
@@ -72190,14 +72190,14 @@
         </is>
       </c>
       <c r="R659" s="1" t="n">
-        <v>46204.25009074074</v>
+        <v>46204.37522271991</v>
       </c>
       <c r="S659" t="n">
         <v>-8</v>
       </c>
       <c r="T659" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U659" t="inlineStr">
@@ -72207,7 +72207,7 @@
       </c>
       <c r="V659" t="inlineStr">
         <is>
-          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1810]. - Data Comentário: 01/07/2026 05:59</t>
+          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1582]. - Data Comentário: 01/07/2026 08:59</t>
         </is>
       </c>
       <c r="W659" t="inlineStr"/>
@@ -72234,11 +72234,11 @@
     </row>
     <row r="660">
       <c r="A660" t="n">
-        <v>6703</v>
+        <v>6404</v>
       </c>
       <c r="B660" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="C660" t="inlineStr">
@@ -72288,7 +72288,7 @@
         </is>
       </c>
       <c r="O660" t="n">
-        <v>17941138</v>
+        <v>16962099</v>
       </c>
       <c r="P660" t="inlineStr">
         <is>
@@ -72301,14 +72301,14 @@
         </is>
       </c>
       <c r="R660" s="1" t="n">
-        <v>46204.37521859954</v>
+        <v>46204.25009074074</v>
       </c>
       <c r="S660" t="n">
         <v>-8</v>
       </c>
       <c r="T660" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t>SOLAR INVESTIMENTOS</t>
         </is>
       </c>
       <c r="U660" t="inlineStr">
@@ -72318,7 +72318,7 @@
       </c>
       <c r="V660" t="inlineStr">
         <is>
-          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1810]. - Data Comentário: 01/07/2026 08:59</t>
+          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1810]. - Data Comentário: 01/07/2026 05:59</t>
         </is>
       </c>
       <c r="W660" t="inlineStr"/>
@@ -72345,11 +72345,11 @@
     </row>
     <row r="661">
       <c r="A661" t="n">
-        <v>6278</v>
+        <v>6703</v>
       </c>
       <c r="B661" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C661" t="inlineStr">
@@ -72359,7 +72359,7 @@
       </c>
       <c r="D661" t="inlineStr">
         <is>
-          <t>Federal - Lucro Real - Anual</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E661" t="inlineStr">
@@ -72373,7 +72373,7 @@
         </is>
       </c>
       <c r="G661" t="n">
-        <v>953</v>
+        <v>948</v>
       </c>
       <c r="H661" t="n">
         <v>0</v>
@@ -72385,12 +72385,12 @@
       </c>
       <c r="J661" t="inlineStr">
         <is>
-          <t>Confirm Rec - PIS/COFINS</t>
+          <t>Confirm Rec - IRPJ/CSLL (EF)</t>
         </is>
       </c>
       <c r="K661" t="inlineStr"/>
       <c r="L661" s="1" t="n">
-        <v>46227</v>
+        <v>46233</v>
       </c>
       <c r="M661" t="inlineStr"/>
       <c r="N661" t="inlineStr">
@@ -72399,23 +72399,27 @@
         </is>
       </c>
       <c r="O661" t="n">
-        <v>17539722</v>
-      </c>
-      <c r="P661" t="inlineStr"/>
+        <v>17941138</v>
+      </c>
+      <c r="P661" t="inlineStr">
+        <is>
+          <t>Victoria Virgens</t>
+        </is>
+      </c>
       <c r="Q661" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R661" s="1" t="n">
-        <v>46023.15053034722</v>
+        <v>46204.37521859954</v>
       </c>
       <c r="S661" t="n">
-        <v>-2</v>
+        <v>-8</v>
       </c>
       <c r="T661" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>LIMA MOTA</t>
         </is>
       </c>
       <c r="U661" t="inlineStr">
@@ -72423,7 +72427,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V661" t="inlineStr"/>
+      <c r="V661" t="inlineStr">
+        <is>
+          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1810]. - Data Comentário: 01/07/2026 08:59</t>
+        </is>
+      </c>
       <c r="W661" t="inlineStr"/>
       <c r="X661" t="inlineStr"/>
       <c r="Y661" t="inlineStr"/>
@@ -72448,11 +72456,11 @@
     </row>
     <row r="662">
       <c r="A662" t="n">
-        <v>6404</v>
+        <v>6278</v>
       </c>
       <c r="B662" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="C662" t="inlineStr">
@@ -72462,7 +72470,7 @@
       </c>
       <c r="D662" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - Lucro Real - Anual</t>
         </is>
       </c>
       <c r="E662" t="inlineStr">
@@ -72502,27 +72510,23 @@
         </is>
       </c>
       <c r="O662" t="n">
-        <v>16962105</v>
-      </c>
-      <c r="P662" t="inlineStr">
-        <is>
-          <t>Victoria Virgens</t>
-        </is>
-      </c>
+        <v>17539722</v>
+      </c>
+      <c r="P662" t="inlineStr"/>
       <c r="Q662" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R662" s="1" t="n">
-        <v>46204.41680613426</v>
+        <v>46023.15053034722</v>
       </c>
       <c r="S662" t="n">
         <v>-2</v>
       </c>
       <c r="T662" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U662" t="inlineStr">
@@ -72530,11 +72534,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V662" t="inlineStr">
-        <is>
-          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1807]. - Data Comentário: 01/07/2026 09:59</t>
-        </is>
-      </c>
+      <c r="V662" t="inlineStr"/>
       <c r="W662" t="inlineStr"/>
       <c r="X662" t="inlineStr"/>
       <c r="Y662" t="inlineStr"/>
@@ -72559,11 +72559,11 @@
     </row>
     <row r="663">
       <c r="A663" t="n">
-        <v>6627</v>
+        <v>6404</v>
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="C663" t="inlineStr">
@@ -72573,12 +72573,12 @@
       </c>
       <c r="D663" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E663" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F663" t="inlineStr">
@@ -72613,7 +72613,7 @@
         </is>
       </c>
       <c r="O663" t="n">
-        <v>17042311</v>
+        <v>16962105</v>
       </c>
       <c r="P663" t="inlineStr">
         <is>
@@ -72626,14 +72626,14 @@
         </is>
       </c>
       <c r="R663" s="1" t="n">
-        <v>46204.41687068287</v>
+        <v>46204.41680613426</v>
       </c>
       <c r="S663" t="n">
         <v>-2</v>
       </c>
       <c r="T663" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>SOLAR INVESTIMENTOS</t>
         </is>
       </c>
       <c r="U663" t="inlineStr">
@@ -72643,7 +72643,7 @@
       </c>
       <c r="V663" t="inlineStr">
         <is>
-          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1882]. - Data Comentário: 01/07/2026 09:59</t>
+          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1807]. - Data Comentário: 01/07/2026 09:59</t>
         </is>
       </c>
       <c r="W663" t="inlineStr"/>
@@ -72670,11 +72670,11 @@
     </row>
     <row r="664">
       <c r="A664" t="n">
-        <v>6704</v>
+        <v>6627</v>
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C664" t="inlineStr">
@@ -72689,7 +72689,7 @@
       </c>
       <c r="E664" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F664" t="inlineStr">
@@ -72724,23 +72724,27 @@
         </is>
       </c>
       <c r="O664" t="n">
-        <v>17952360</v>
-      </c>
-      <c r="P664" t="inlineStr"/>
+        <v>17042311</v>
+      </c>
+      <c r="P664" t="inlineStr">
+        <is>
+          <t>Victoria Virgens</t>
+        </is>
+      </c>
       <c r="Q664" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R664" s="1" t="n">
-        <v>46223.79178935185</v>
+        <v>46204.41687068287</v>
       </c>
       <c r="S664" t="n">
         <v>-2</v>
       </c>
       <c r="T664" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U664" t="inlineStr">
@@ -72750,7 +72754,7 @@
       </c>
       <c r="V664" t="inlineStr">
         <is>
-          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1808]. - Data Comentário: 20/07/2026 18:59</t>
+          <t>Baixado via Rotina Configuração Após Baixa de tarefa, tarefas estão pedentes:[1882]. - Data Comentário: 01/07/2026 09:59</t>
         </is>
       </c>
       <c r="W664" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-22 17:21
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -47886,7 +47886,11 @@
       <c r="L437" s="1" t="n">
         <v>46230</v>
       </c>
-      <c r="M437" t="inlineStr"/>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
       <c r="N437" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -47919,7 +47923,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V437" t="inlineStr"/>
+      <c r="V437" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 22/07/2026 16:28</t>
+        </is>
+      </c>
       <c r="W437" t="inlineStr"/>
       <c r="X437" t="inlineStr"/>
       <c r="Y437" t="inlineStr"/>
@@ -47991,7 +47999,11 @@
       <c r="L438" s="1" t="n">
         <v>46230</v>
       </c>
-      <c r="M438" t="inlineStr"/>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
       <c r="N438" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -48024,7 +48036,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V438" t="inlineStr"/>
+      <c r="V438" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 22/07/2026 16:28</t>
+        </is>
+      </c>
       <c r="W438" t="inlineStr"/>
       <c r="X438" t="inlineStr"/>
       <c r="Y438" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-23 16:47
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -51542,7 +51542,11 @@
       <c r="O471" t="n">
         <v>17407829</v>
       </c>
-      <c r="P471" t="inlineStr"/>
+      <c r="P471" t="inlineStr">
+        <is>
+          <t>Sergio Fernandes</t>
+        </is>
+      </c>
       <c r="Q471" t="inlineStr">
         <is>
           <t>Em Aberto</t>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-27 13:20
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -42130,11 +42130,11 @@
     </row>
     <row r="386">
       <c r="A386" t="n">
-        <v>6486</v>
+        <v>6224</v>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>PC GAMER GOIANIA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -42154,45 +42154,41 @@
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G386" t="n">
-        <v>5800</v>
+        <v>1808</v>
       </c>
       <c r="H386" t="n">
-        <v>5776</v>
+        <v>0</v>
       </c>
       <c r="I386" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J386" t="inlineStr">
         <is>
-          <t>CCT Lançamento Sd.663</t>
+          <t>Fed - PIS/COFINS Não Cumul/Mon - 5856</t>
         </is>
       </c>
       <c r="K386" t="inlineStr"/>
       <c r="L386" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="M386" t="inlineStr">
-        <is>
-          <t>30/07/2026</t>
-        </is>
-      </c>
+      <c r="M386" t="inlineStr"/>
       <c r="N386" t="inlineStr">
         <is>
-          <t>00/2026</t>
+          <t>06/2026</t>
         </is>
       </c>
       <c r="O386" t="n">
-        <v>17901201</v>
+        <v>17688691</v>
       </c>
       <c r="P386" t="inlineStr">
         <is>
-          <t>Jakeline Silva</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="Q386" t="inlineStr">
@@ -42206,7 +42202,7 @@
       </c>
       <c r="T386" t="inlineStr">
         <is>
-          <t>PC GAMER</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U386" t="inlineStr">
@@ -42216,8 +42212,7 @@
       </c>
       <c r="V386" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 30/07/2026 
-O retorno do cliente foi recebido. Estamos realizando os trâmites para a aplicação do reajuste. - Data Comentário: 27/07/2026 09:51</t>
+          <t>Atraso de envio do cliente, consultar pendências no check list - Data Comentário: 22/07/2026 18:22</t>
         </is>
       </c>
       <c r="W386" t="inlineStr"/>
@@ -42233,22 +42228,22 @@
       <c r="AE386" t="inlineStr"/>
       <c r="AF386" t="inlineStr">
         <is>
-          <t>Tarefa</t>
+          <t>Imposto</t>
         </is>
       </c>
       <c r="AG386" t="inlineStr">
         <is>
-          <t>David Bragança</t>
+          <t>Ricardo Fischer</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="n">
-        <v>6224</v>
+        <v>6548</v>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>GOIAS SILAGEM LTDA</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
@@ -42268,55 +42263,59 @@
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G387" t="n">
-        <v>1808</v>
+        <v>6892</v>
       </c>
       <c r="H387" t="n">
         <v>0</v>
       </c>
       <c r="I387" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="J387" t="inlineStr">
         <is>
-          <t>Fed - PIS/COFINS Não Cumul/Mon - 5856</t>
+          <t>Fed - DCTFWEB</t>
         </is>
       </c>
       <c r="K387" t="inlineStr"/>
       <c r="L387" s="1" t="n">
-        <v>46225</v>
-      </c>
-      <c r="M387" t="inlineStr"/>
+        <v>46233</v>
+      </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
       <c r="N387" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O387" t="n">
-        <v>17688691</v>
+        <v>17968015</v>
       </c>
       <c r="P387" t="inlineStr">
         <is>
-          <t>Cristina Leite</t>
+          <t>Thais Souza</t>
         </is>
       </c>
       <c r="Q387" t="inlineStr">
         <is>
-          <t>Em Atraso</t>
+          <t>Em Aberto</t>
         </is>
       </c>
       <c r="R387" t="inlineStr"/>
       <c r="S387" t="n">
-        <v>5</v>
+        <v>-3</v>
       </c>
       <c r="T387" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>GOIAS SILAGEM</t>
         </is>
       </c>
       <c r="U387" t="inlineStr">
@@ -42326,7 +42325,7 @@
       </c>
       <c r="V387" t="inlineStr">
         <is>
-          <t>Atraso de envio do cliente, consultar pendências no check list - Data Comentário: 22/07/2026 18:22</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 20/07/2026 15:29</t>
         </is>
       </c>
       <c r="W387" t="inlineStr"/>
@@ -42342,22 +42341,22 @@
       <c r="AE387" t="inlineStr"/>
       <c r="AF387" t="inlineStr">
         <is>
-          <t>Imposto</t>
+          <t>Obrigação Acessória</t>
         </is>
       </c>
       <c r="AG387" t="inlineStr">
         <is>
-          <t>Ricardo Fischer</t>
+          <t>Erika Santana</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="n">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
@@ -42372,7 +42371,7 @@
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
@@ -42402,7 +42401,7 @@
       </c>
       <c r="M388" t="inlineStr">
         <is>
-          <t>23/07/2026</t>
+          <t>24/07/2026</t>
         </is>
       </c>
       <c r="N388" t="inlineStr">
@@ -42411,11 +42410,11 @@
         </is>
       </c>
       <c r="O388" t="n">
-        <v>17968015</v>
+        <v>17042482</v>
       </c>
       <c r="P388" t="inlineStr">
         <is>
-          <t>Thais Souza</t>
+          <t>Nathalia Lourenco</t>
         </is>
       </c>
       <c r="Q388" t="inlineStr">
@@ -42429,7 +42428,7 @@
       </c>
       <c r="T388" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U388" t="inlineStr">
@@ -42439,7 +42438,7 @@
       </c>
       <c r="V388" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 20/07/2026 15:29</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 24/07/2026 - Data Comentário: 20/07/2026 15:10</t>
         </is>
       </c>
       <c r="W388" t="inlineStr"/>
@@ -42460,17 +42459,17 @@
       </c>
       <c r="AG388" t="inlineStr">
         <is>
-          <t>Erika Santana</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="n">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
@@ -42480,7 +42479,7 @@
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E389" t="inlineStr">
@@ -42524,7 +42523,7 @@
         </is>
       </c>
       <c r="O389" t="n">
-        <v>17042482</v>
+        <v>16960022</v>
       </c>
       <c r="P389" t="inlineStr">
         <is>
@@ -42579,11 +42578,11 @@
     </row>
     <row r="390">
       <c r="A390" t="n">
-        <v>6628</v>
+        <v>6962</v>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
+          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
@@ -42593,17 +42592,17 @@
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G390" t="n">
@@ -42628,7 +42627,7 @@
       </c>
       <c r="M390" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="N390" t="inlineStr">
@@ -42637,11 +42636,11 @@
         </is>
       </c>
       <c r="O390" t="n">
-        <v>16960022</v>
+        <v>18187953</v>
       </c>
       <c r="P390" t="inlineStr">
         <is>
-          <t>Nathalia Lourenco</t>
+          <t>Mirian Lima</t>
         </is>
       </c>
       <c r="Q390" t="inlineStr">
@@ -42655,17 +42654,14 @@
       </c>
       <c r="T390" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
-        </is>
-      </c>
-      <c r="U390" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+          <t>PROMOTORAS GYN</t>
+        </is>
+      </c>
+      <c r="U390" t="inlineStr"/>
       <c r="V390" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 24/07/2026 - Data Comentário: 20/07/2026 15:10</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 
+Aguardando apurações PIS/COFINS/IRPJ/CSLL - Data Comentário: 21/07/2026 10:05</t>
         </is>
       </c>
       <c r="W390" t="inlineStr"/>
@@ -42692,11 +42688,11 @@
     </row>
     <row r="391">
       <c r="A391" t="n">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
+          <t>PROMOTORAS GYN LTDA</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
@@ -42750,7 +42746,7 @@
         </is>
       </c>
       <c r="O391" t="n">
-        <v>18187953</v>
+        <v>18187891</v>
       </c>
       <c r="P391" t="inlineStr">
         <is>
@@ -42802,11 +42798,11 @@
     </row>
     <row r="392">
       <c r="A392" t="n">
-        <v>6963</v>
+        <v>6548</v>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN LTDA</t>
+          <t>GOIAS SILAGEM LTDA</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
@@ -42826,11 +42822,11 @@
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G392" t="n">
-        <v>6892</v>
+        <v>1651</v>
       </c>
       <c r="H392" t="n">
         <v>0</v>
@@ -42842,29 +42838,25 @@
       </c>
       <c r="J392" t="inlineStr">
         <is>
-          <t>Fed - DCTFWEB</t>
+          <t>Fed - IRPJ/CSLL</t>
         </is>
       </c>
       <c r="K392" t="inlineStr"/>
       <c r="L392" s="1" t="n">
-        <v>46233</v>
-      </c>
-      <c r="M392" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
+        <v>46232</v>
+      </c>
+      <c r="M392" t="inlineStr"/>
       <c r="N392" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O392" t="n">
-        <v>18187891</v>
+        <v>17967985</v>
       </c>
       <c r="P392" t="inlineStr">
         <is>
-          <t>Mirian Lima</t>
+          <t>Thais Souza</t>
         </is>
       </c>
       <c r="Q392" t="inlineStr">
@@ -42874,20 +42866,19 @@
       </c>
       <c r="R392" t="inlineStr"/>
       <c r="S392" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T392" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN</t>
-        </is>
-      </c>
-      <c r="U392" t="inlineStr"/>
-      <c r="V392" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 
-Aguardando apurações PIS/COFINS/IRPJ/CSLL - Data Comentário: 21/07/2026 10:05</t>
-        </is>
-      </c>
+          <t>GOIAS SILAGEM</t>
+        </is>
+      </c>
+      <c r="U392" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V392" t="inlineStr"/>
       <c r="W392" t="inlineStr"/>
       <c r="X392" t="inlineStr"/>
       <c r="Y392" t="inlineStr"/>
@@ -42901,22 +42892,22 @@
       <c r="AE392" t="inlineStr"/>
       <c r="AF392" t="inlineStr">
         <is>
-          <t>Obrigação Acessória</t>
+          <t>Imposto</t>
         </is>
       </c>
       <c r="AG392" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Erika Santana</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="n">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
@@ -42931,7 +42922,7 @@
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
@@ -42966,11 +42957,11 @@
         </is>
       </c>
       <c r="O393" t="n">
-        <v>17967985</v>
+        <v>17042385</v>
       </c>
       <c r="P393" t="inlineStr">
         <is>
-          <t>Thais Souza</t>
+          <t>Nathalia Lourenco</t>
         </is>
       </c>
       <c r="Q393" t="inlineStr">
@@ -42984,7 +42975,7 @@
       </c>
       <c r="T393" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U393" t="inlineStr">
@@ -43011,17 +43002,17 @@
       </c>
       <c r="AG393" t="inlineStr">
         <is>
-          <t>Erika Santana</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="n">
-        <v>6627</v>
+        <v>6962</v>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -43036,12 +43027,12 @@
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G394" t="n">
@@ -43071,11 +43062,11 @@
         </is>
       </c>
       <c r="O394" t="n">
-        <v>17042385</v>
+        <v>18187935</v>
       </c>
       <c r="P394" t="inlineStr">
         <is>
-          <t>Nathalia Lourenco</t>
+          <t>Mirian Lima</t>
         </is>
       </c>
       <c r="Q394" t="inlineStr">
@@ -43089,14 +43080,10 @@
       </c>
       <c r="T394" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
-        </is>
-      </c>
-      <c r="U394" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+          <t>PROMOTORAS GYN</t>
+        </is>
+      </c>
+      <c r="U394" t="inlineStr"/>
       <c r="V394" t="inlineStr"/>
       <c r="W394" t="inlineStr"/>
       <c r="X394" t="inlineStr"/>
@@ -43122,11 +43109,11 @@
     </row>
     <row r="395">
       <c r="A395" t="n">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
+          <t>PROMOTORAS GYN LTDA</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
@@ -43176,7 +43163,7 @@
         </is>
       </c>
       <c r="O395" t="n">
-        <v>18187935</v>
+        <v>18187873</v>
       </c>
       <c r="P395" t="inlineStr">
         <is>
@@ -43223,11 +43210,11 @@
     </row>
     <row r="396">
       <c r="A396" t="n">
-        <v>6963</v>
+        <v>6548</v>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN LTDA</t>
+          <t>GOIAS SILAGEM LTDA</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
@@ -43247,11 +43234,11 @@
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G396" t="n">
-        <v>1651</v>
+        <v>11516</v>
       </c>
       <c r="H396" t="n">
         <v>0</v>
@@ -43263,25 +43250,29 @@
       </c>
       <c r="J396" t="inlineStr">
         <is>
-          <t>Fed - IRPJ/CSLL</t>
+          <t>Módulo de Inclusão Tributária (MIT)</t>
         </is>
       </c>
       <c r="K396" t="inlineStr"/>
       <c r="L396" s="1" t="n">
-        <v>46232</v>
-      </c>
-      <c r="M396" t="inlineStr"/>
+        <v>46233</v>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
       <c r="N396" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O396" t="n">
-        <v>18187873</v>
+        <v>17968051</v>
       </c>
       <c r="P396" t="inlineStr">
         <is>
-          <t>Mirian Lima</t>
+          <t>Thais Souza</t>
         </is>
       </c>
       <c r="Q396" t="inlineStr">
@@ -43291,15 +43282,23 @@
       </c>
       <c r="R396" t="inlineStr"/>
       <c r="S396" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="T396" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN</t>
-        </is>
-      </c>
-      <c r="U396" t="inlineStr"/>
-      <c r="V396" t="inlineStr"/>
+          <t>GOIAS SILAGEM</t>
+        </is>
+      </c>
+      <c r="U396" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V396" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 20/07/2026 15:31</t>
+        </is>
+      </c>
       <c r="W396" t="inlineStr"/>
       <c r="X396" t="inlineStr"/>
       <c r="Y396" t="inlineStr"/>
@@ -43313,22 +43312,22 @@
       <c r="AE396" t="inlineStr"/>
       <c r="AF396" t="inlineStr">
         <is>
-          <t>Imposto</t>
+          <t>Obrigação Acessória</t>
         </is>
       </c>
       <c r="AG396" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Erika Santana</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="n">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
@@ -43343,7 +43342,7 @@
       </c>
       <c r="E397" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
@@ -43373,7 +43372,7 @@
       </c>
       <c r="M397" t="inlineStr">
         <is>
-          <t>23/07/2026</t>
+          <t>24/07/2026</t>
         </is>
       </c>
       <c r="N397" t="inlineStr">
@@ -43382,11 +43381,11 @@
         </is>
       </c>
       <c r="O397" t="n">
-        <v>17968051</v>
+        <v>17042660</v>
       </c>
       <c r="P397" t="inlineStr">
         <is>
-          <t>Thais Souza</t>
+          <t>Nathalia Lourenco</t>
         </is>
       </c>
       <c r="Q397" t="inlineStr">
@@ -43400,7 +43399,7 @@
       </c>
       <c r="T397" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U397" t="inlineStr">
@@ -43410,7 +43409,7 @@
       </c>
       <c r="V397" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 20/07/2026 15:31</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 24/07/2026 - Data Comentário: 20/07/2026 15:12</t>
         </is>
       </c>
       <c r="W397" t="inlineStr"/>
@@ -43431,17 +43430,17 @@
       </c>
       <c r="AG397" t="inlineStr">
         <is>
-          <t>Erika Santana</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="n">
-        <v>6627</v>
+        <v>6962</v>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
@@ -43456,12 +43455,12 @@
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G398" t="n">
@@ -43486,7 +43485,7 @@
       </c>
       <c r="M398" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>29/07/2026</t>
         </is>
       </c>
       <c r="N398" t="inlineStr">
@@ -43495,11 +43494,11 @@
         </is>
       </c>
       <c r="O398" t="n">
-        <v>17042660</v>
+        <v>18187983</v>
       </c>
       <c r="P398" t="inlineStr">
         <is>
-          <t>Nathalia Lourenco</t>
+          <t>Mirian Lima</t>
         </is>
       </c>
       <c r="Q398" t="inlineStr">
@@ -43513,17 +43512,14 @@
       </c>
       <c r="T398" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
-        </is>
-      </c>
-      <c r="U398" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+          <t>PROMOTORAS GYN</t>
+        </is>
+      </c>
+      <c r="U398" t="inlineStr"/>
       <c r="V398" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 24/07/2026 - Data Comentário: 20/07/2026 15:12</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
+Aguardando apuração do PIS/COFINS/IRPJ e CSLL - Data Comentário: 20/07/2026 16:15</t>
         </is>
       </c>
       <c r="W398" t="inlineStr"/>
@@ -43550,11 +43546,11 @@
     </row>
     <row r="399">
       <c r="A399" t="n">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
+          <t>PROMOTORAS GYN LTDA</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
@@ -43608,7 +43604,7 @@
         </is>
       </c>
       <c r="O399" t="n">
-        <v>18187983</v>
+        <v>18187921</v>
       </c>
       <c r="P399" t="inlineStr">
         <is>
@@ -43660,11 +43656,11 @@
     </row>
     <row r="400">
       <c r="A400" t="n">
-        <v>6963</v>
+        <v>6627</v>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -43679,16 +43675,16 @@
       </c>
       <c r="E400" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G400" t="n">
-        <v>11516</v>
+        <v>7875</v>
       </c>
       <c r="H400" t="n">
         <v>0</v>
@@ -43700,29 +43696,25 @@
       </c>
       <c r="J400" t="inlineStr">
         <is>
-          <t>Módulo de Inclusão Tributária (MIT)</t>
+          <t>Movimento - Analise de Balanço Lucro Real</t>
         </is>
       </c>
       <c r="K400" t="inlineStr"/>
       <c r="L400" s="1" t="n">
-        <v>46233</v>
-      </c>
-      <c r="M400" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
+        <v>46230</v>
+      </c>
+      <c r="M400" t="inlineStr"/>
       <c r="N400" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O400" t="n">
-        <v>18187921</v>
+        <v>18096485</v>
       </c>
       <c r="P400" t="inlineStr">
         <is>
-          <t>Mirian Lima</t>
+          <t>Nathalia Lourenco</t>
         </is>
       </c>
       <c r="Q400" t="inlineStr">
@@ -43732,20 +43724,19 @@
       </c>
       <c r="R400" t="inlineStr"/>
       <c r="S400" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="T400" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN</t>
-        </is>
-      </c>
-      <c r="U400" t="inlineStr"/>
-      <c r="V400" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
-Aguardando apuração do PIS/COFINS/IRPJ e CSLL - Data Comentário: 20/07/2026 16:15</t>
-        </is>
-      </c>
+          <t xml:space="preserve">GTG </t>
+        </is>
+      </c>
+      <c r="U400" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V400" t="inlineStr"/>
       <c r="W400" t="inlineStr"/>
       <c r="X400" t="inlineStr"/>
       <c r="Y400" t="inlineStr"/>
@@ -43759,7 +43750,7 @@
       <c r="AE400" t="inlineStr"/>
       <c r="AF400" t="inlineStr">
         <is>
-          <t>Obrigação Acessória</t>
+          <t>Tarefa</t>
         </is>
       </c>
       <c r="AG400" t="inlineStr">
@@ -43770,11 +43761,11 @@
     </row>
     <row r="401">
       <c r="A401" t="n">
-        <v>6627</v>
+        <v>6962</v>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
@@ -43789,12 +43780,12 @@
       </c>
       <c r="E401" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G401" t="n">
@@ -43824,11 +43815,11 @@
         </is>
       </c>
       <c r="O401" t="n">
-        <v>18096485</v>
+        <v>18200035</v>
       </c>
       <c r="P401" t="inlineStr">
         <is>
-          <t>Nathalia Lourenco</t>
+          <t>Mirian Lima</t>
         </is>
       </c>
       <c r="Q401" t="inlineStr">
@@ -43842,14 +43833,10 @@
       </c>
       <c r="T401" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
-        </is>
-      </c>
-      <c r="U401" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+          <t>PROMOTORAS GYN</t>
+        </is>
+      </c>
+      <c r="U401" t="inlineStr"/>
       <c r="V401" t="inlineStr"/>
       <c r="W401" t="inlineStr"/>
       <c r="X401" t="inlineStr"/>
@@ -43875,11 +43862,11 @@
     </row>
     <row r="402">
       <c r="A402" t="n">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
+          <t>PROMOTORAS GYN LTDA</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
@@ -43929,7 +43916,7 @@
         </is>
       </c>
       <c r="O402" t="n">
-        <v>18200035</v>
+        <v>18200054</v>
       </c>
       <c r="P402" t="inlineStr">
         <is>
@@ -43976,11 +43963,11 @@
     </row>
     <row r="403">
       <c r="A403" t="n">
-        <v>6963</v>
+        <v>6628</v>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN LTDA</t>
+          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
@@ -43990,21 +43977,21 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G403" t="n">
-        <v>7875</v>
+        <v>9764</v>
       </c>
       <c r="H403" t="n">
         <v>0</v>
@@ -44016,7 +44003,7 @@
       </c>
       <c r="J403" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Lucro Real</t>
+          <t>Movimento - Analise de Balanço Simples Nacional</t>
         </is>
       </c>
       <c r="K403" t="inlineStr"/>
@@ -44030,11 +44017,11 @@
         </is>
       </c>
       <c r="O403" t="n">
-        <v>18200054</v>
+        <v>18096420</v>
       </c>
       <c r="P403" t="inlineStr">
         <is>
-          <t>Mirian Lima</t>
+          <t>Nathalia Lourenco</t>
         </is>
       </c>
       <c r="Q403" t="inlineStr">
@@ -44048,10 +44035,14 @@
       </c>
       <c r="T403" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN</t>
-        </is>
-      </c>
-      <c r="U403" t="inlineStr"/>
+          <t xml:space="preserve">GTG </t>
+        </is>
+      </c>
+      <c r="U403" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="V403" t="inlineStr"/>
       <c r="W403" t="inlineStr"/>
       <c r="X403" t="inlineStr"/>
@@ -44077,11 +44068,11 @@
     </row>
     <row r="404">
       <c r="A404" t="n">
-        <v>6628</v>
+        <v>6945</v>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
+          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -44124,18 +44115,22 @@
       <c r="L404" s="1" t="n">
         <v>46230</v>
       </c>
-      <c r="M404" t="inlineStr"/>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
       <c r="N404" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O404" t="n">
-        <v>18096420</v>
+        <v>18200043</v>
       </c>
       <c r="P404" t="inlineStr">
         <is>
-          <t>Nathalia Lourenco</t>
+          <t>Laisa Rocha</t>
         </is>
       </c>
       <c r="Q404" t="inlineStr">
@@ -44149,15 +44144,15 @@
       </c>
       <c r="T404" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
-        </is>
-      </c>
-      <c r="U404" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="V404" t="inlineStr"/>
+          <t>BRASIL DISTRIBUIDORA</t>
+        </is>
+      </c>
+      <c r="U404" t="inlineStr"/>
+      <c r="V404" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 20/07/2026 15:54</t>
+        </is>
+      </c>
       <c r="W404" t="inlineStr"/>
       <c r="X404" t="inlineStr"/>
       <c r="Y404" t="inlineStr"/>
@@ -44182,11 +44177,11 @@
     </row>
     <row r="405">
       <c r="A405" t="n">
-        <v>6945</v>
+        <v>5417</v>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
@@ -44196,55 +44191,51 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E405" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G405" t="n">
-        <v>9764</v>
+        <v>6890</v>
       </c>
       <c r="H405" t="n">
         <v>0</v>
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J405" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Simples Nacional</t>
+          <t>Fed - DCTFWEB</t>
         </is>
       </c>
       <c r="K405" t="inlineStr"/>
       <c r="L405" s="1" t="n">
-        <v>46230</v>
-      </c>
-      <c r="M405" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
+        <v>46233</v>
+      </c>
+      <c r="M405" t="inlineStr"/>
       <c r="N405" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O405" t="n">
-        <v>18200043</v>
+        <v>17399258</v>
       </c>
       <c r="P405" t="inlineStr">
         <is>
-          <t>Laisa Rocha</t>
+          <t>Eveny Silva</t>
         </is>
       </c>
       <c r="Q405" t="inlineStr">
@@ -44254,17 +44245,21 @@
       </c>
       <c r="R405" t="inlineStr"/>
       <c r="S405" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="T405" t="inlineStr">
         <is>
-          <t>BRASIL DISTRIBUIDORA</t>
-        </is>
-      </c>
-      <c r="U405" t="inlineStr"/>
+          <t>NOSSO NOVO SUPERMERCADO</t>
+        </is>
+      </c>
+      <c r="U405" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="V405" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 20/07/2026 15:54</t>
+          <t>Aguardando a Liberação da Gerência de Contas - Data Comentário: 20/07/2026 14:21</t>
         </is>
       </c>
       <c r="W405" t="inlineStr"/>
@@ -44280,22 +44275,22 @@
       <c r="AE405" t="inlineStr"/>
       <c r="AF405" t="inlineStr">
         <is>
-          <t>Tarefa</t>
+          <t>Obrigação Acessória</t>
         </is>
       </c>
       <c r="AG405" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="n">
-        <v>5417</v>
+        <v>5617</v>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -44315,7 +44310,7 @@
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G406" t="n">
@@ -44338,18 +44333,22 @@
       <c r="L406" s="1" t="n">
         <v>46233</v>
       </c>
-      <c r="M406" t="inlineStr"/>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
       <c r="N406" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O406" t="n">
-        <v>17399258</v>
+        <v>17407809</v>
       </c>
       <c r="P406" t="inlineStr">
         <is>
-          <t>Eveny Silva</t>
+          <t>Jackson Silva</t>
         </is>
       </c>
       <c r="Q406" t="inlineStr">
@@ -44363,7 +44362,7 @@
       </c>
       <c r="T406" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U406" t="inlineStr">
@@ -44373,7 +44372,7 @@
       </c>
       <c r="V406" t="inlineStr">
         <is>
-          <t>Aguardando a Liberação da Gerência de Contas - Data Comentário: 20/07/2026 14:21</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 22/07/2026 15:47</t>
         </is>
       </c>
       <c r="W406" t="inlineStr"/>
@@ -44394,17 +44393,17 @@
       </c>
       <c r="AG406" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Edileide Dias</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="n">
-        <v>5617</v>
+        <v>6224</v>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -44424,7 +44423,7 @@
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G407" t="n">
@@ -44458,7 +44457,7 @@
         </is>
       </c>
       <c r="O407" t="n">
-        <v>17407809</v>
+        <v>17688937</v>
       </c>
       <c r="P407" t="inlineStr">
         <is>
@@ -44513,11 +44512,11 @@
     </row>
     <row r="408">
       <c r="A408" t="n">
-        <v>6224</v>
+        <v>6278</v>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -44527,7 +44526,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Real - Anual</t>
         </is>
       </c>
       <c r="E408" t="inlineStr">
@@ -44537,7 +44536,7 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G408" t="n">
@@ -44560,22 +44559,18 @@
       <c r="L408" s="1" t="n">
         <v>46233</v>
       </c>
-      <c r="M408" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
+      <c r="M408" t="inlineStr"/>
       <c r="N408" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O408" t="n">
-        <v>17688937</v>
+        <v>17539766</v>
       </c>
       <c r="P408" t="inlineStr">
         <is>
-          <t>Jackson Silva</t>
+          <t>Isabela Lemos</t>
         </is>
       </c>
       <c r="Q408" t="inlineStr">
@@ -44589,7 +44584,7 @@
       </c>
       <c r="T408" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U408" t="inlineStr">
@@ -44597,11 +44592,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V408" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 22/07/2026 15:47</t>
-        </is>
-      </c>
+      <c r="V408" t="inlineStr"/>
       <c r="W408" t="inlineStr"/>
       <c r="X408" t="inlineStr"/>
       <c r="Y408" t="inlineStr"/>
@@ -44620,17 +44611,17 @@
       </c>
       <c r="AG408" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="n">
-        <v>6278</v>
+        <v>6279</v>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>DIENNYFER DA S PEREIRA</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -44640,7 +44631,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>Federal - Lucro Real - Anual</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E409" t="inlineStr">
@@ -44650,7 +44641,7 @@
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G409" t="n">
@@ -44680,7 +44671,7 @@
         </is>
       </c>
       <c r="O409" t="n">
-        <v>17539766</v>
+        <v>17646082</v>
       </c>
       <c r="P409" t="inlineStr">
         <is>
@@ -44731,11 +44722,11 @@
     </row>
     <row r="410">
       <c r="A410" t="n">
-        <v>6279</v>
+        <v>6404</v>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>DIENNYFER DA S PEREIRA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -44755,7 +44746,7 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G410" t="n">
@@ -44785,7 +44776,7 @@
         </is>
       </c>
       <c r="O410" t="n">
-        <v>17646082</v>
+        <v>16962326</v>
       </c>
       <c r="P410" t="inlineStr">
         <is>
@@ -44803,7 +44794,7 @@
       </c>
       <c r="T410" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>SOLAR INVESTIMENTOS</t>
         </is>
       </c>
       <c r="U410" t="inlineStr">
@@ -44836,11 +44827,11 @@
     </row>
     <row r="411">
       <c r="A411" t="n">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
@@ -44850,7 +44841,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E411" t="inlineStr">
@@ -44890,11 +44881,11 @@
         </is>
       </c>
       <c r="O411" t="n">
-        <v>16962326</v>
+        <v>18152536</v>
       </c>
       <c r="P411" t="inlineStr">
         <is>
-          <t>Isabela Lemos</t>
+          <t>Nathany Barreto</t>
         </is>
       </c>
       <c r="Q411" t="inlineStr">
@@ -44908,7 +44899,7 @@
       </c>
       <c r="T411" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U411" t="inlineStr">
@@ -44916,7 +44907,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V411" t="inlineStr"/>
+      <c r="V411" t="inlineStr">
+        <is>
+          <t>Aguardando a Liberação da Gerência de Contas - Data Comentário: 20/07/2026 17:55</t>
+        </is>
+      </c>
       <c r="W411" t="inlineStr"/>
       <c r="X411" t="inlineStr"/>
       <c r="Y411" t="inlineStr"/>
@@ -44935,17 +44930,17 @@
       </c>
       <c r="AG411" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="n">
-        <v>6486</v>
+        <v>6703</v>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>PC GAMER GOIANIA LTDA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -44955,7 +44950,7 @@
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E412" t="inlineStr">
@@ -44995,7 +44990,7 @@
         </is>
       </c>
       <c r="O412" t="n">
-        <v>18152536</v>
+        <v>17955184</v>
       </c>
       <c r="P412" t="inlineStr">
         <is>
@@ -45013,7 +45008,7 @@
       </c>
       <c r="T412" t="inlineStr">
         <is>
-          <t>PC GAMER</t>
+          <t>LIMA MOTA</t>
         </is>
       </c>
       <c r="U412" t="inlineStr">
@@ -45050,11 +45045,11 @@
     </row>
     <row r="413">
       <c r="A413" t="n">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -45064,7 +45059,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E413" t="inlineStr">
@@ -45097,18 +45092,22 @@
       <c r="L413" s="1" t="n">
         <v>46233</v>
       </c>
-      <c r="M413" t="inlineStr"/>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
       <c r="N413" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O413" t="n">
-        <v>17955184</v>
+        <v>17955397</v>
       </c>
       <c r="P413" t="inlineStr">
         <is>
-          <t>Nathany Barreto</t>
+          <t>Paulo Silva</t>
         </is>
       </c>
       <c r="Q413" t="inlineStr">
@@ -45122,7 +45121,7 @@
       </c>
       <c r="T413" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U413" t="inlineStr">
@@ -45132,7 +45131,7 @@
       </c>
       <c r="V413" t="inlineStr">
         <is>
-          <t>Aguardando a Liberação da Gerência de Contas - Data Comentário: 20/07/2026 17:55</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 22/07/2026 13:13</t>
         </is>
       </c>
       <c r="W413" t="inlineStr"/>
@@ -45153,17 +45152,17 @@
       </c>
       <c r="AG413" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="n">
-        <v>6704</v>
+        <v>6885</v>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -45173,7 +45172,7 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E414" t="inlineStr">
@@ -45217,11 +45216,11 @@
         </is>
       </c>
       <c r="O414" t="n">
-        <v>17955397</v>
+        <v>18128808</v>
       </c>
       <c r="P414" t="inlineStr">
         <is>
-          <t>Paulo Silva</t>
+          <t>Isabela Lemos</t>
         </is>
       </c>
       <c r="Q414" t="inlineStr">
@@ -45235,17 +45234,13 @@
       </c>
       <c r="T414" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
-        </is>
-      </c>
-      <c r="U414" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+          <t>EMPORIO DOS FRIOS</t>
+        </is>
+      </c>
+      <c r="U414" t="inlineStr"/>
       <c r="V414" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 22/07/2026 13:13</t>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 23/07/2026 - Data Comentário: 22/07/2026 19:56</t>
         </is>
       </c>
       <c r="W414" t="inlineStr"/>
@@ -45272,11 +45267,11 @@
     </row>
     <row r="415">
       <c r="A415" t="n">
-        <v>6885</v>
+        <v>5417</v>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
@@ -45286,7 +45281,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E415" t="inlineStr">
@@ -45296,11 +45291,11 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G415" t="n">
-        <v>6890</v>
+        <v>1582</v>
       </c>
       <c r="H415" t="n">
         <v>0</v>
@@ -45312,29 +45307,25 @@
       </c>
       <c r="J415" t="inlineStr">
         <is>
-          <t>Fed - DCTFWEB</t>
+          <t>Fed - IRPJ/CSLL</t>
         </is>
       </c>
       <c r="K415" t="inlineStr"/>
       <c r="L415" s="1" t="n">
-        <v>46233</v>
-      </c>
-      <c r="M415" t="inlineStr">
-        <is>
-          <t>23/07/2026</t>
-        </is>
-      </c>
+        <v>46232</v>
+      </c>
+      <c r="M415" t="inlineStr"/>
       <c r="N415" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O415" t="n">
-        <v>18128808</v>
+        <v>17398913</v>
       </c>
       <c r="P415" t="inlineStr">
         <is>
-          <t>Isabela Lemos</t>
+          <t>Eveny Silva</t>
         </is>
       </c>
       <c r="Q415" t="inlineStr">
@@ -45344,17 +45335,22 @@
       </c>
       <c r="R415" t="inlineStr"/>
       <c r="S415" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T415" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
-        </is>
-      </c>
-      <c r="U415" t="inlineStr"/>
+          <t>NOSSO NOVO SUPERMERCADO</t>
+        </is>
+      </c>
+      <c r="U415" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="V415" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 23/07/2026 - Data Comentário: 22/07/2026 19:56</t>
+          <t>Aguardando a Liberação da Gerência de Contas  
+Aguardando liberação da Lucratividade - Data Comentário: 21/07/2026 11:31</t>
         </is>
       </c>
       <c r="W415" t="inlineStr"/>
@@ -45370,22 +45366,22 @@
       <c r="AE415" t="inlineStr"/>
       <c r="AF415" t="inlineStr">
         <is>
-          <t>Obrigação Acessória</t>
+          <t>Imposto</t>
         </is>
       </c>
       <c r="AG415" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="n">
-        <v>5417</v>
+        <v>5617</v>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
@@ -45405,7 +45401,7 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G416" t="n">
@@ -45435,11 +45431,11 @@
         </is>
       </c>
       <c r="O416" t="n">
-        <v>17398913</v>
+        <v>17407549</v>
       </c>
       <c r="P416" t="inlineStr">
         <is>
-          <t>Eveny Silva</t>
+          <t>Jackson Silva</t>
         </is>
       </c>
       <c r="Q416" t="inlineStr">
@@ -45453,7 +45449,7 @@
       </c>
       <c r="T416" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U416" t="inlineStr">
@@ -45461,12 +45457,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V416" t="inlineStr">
-        <is>
-          <t>Aguardando a Liberação da Gerência de Contas  
-Aguardando liberação da Lucratividade - Data Comentário: 21/07/2026 11:31</t>
-        </is>
-      </c>
+      <c r="V416" t="inlineStr"/>
       <c r="W416" t="inlineStr"/>
       <c r="X416" t="inlineStr"/>
       <c r="Y416" t="inlineStr"/>
@@ -45485,17 +45476,17 @@
       </c>
       <c r="AG416" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Edileide Dias</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="n">
-        <v>5617</v>
+        <v>6224</v>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -45515,7 +45506,7 @@
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G417" t="n">
@@ -45545,7 +45536,7 @@
         </is>
       </c>
       <c r="O417" t="n">
-        <v>17407549</v>
+        <v>17688641</v>
       </c>
       <c r="P417" t="inlineStr">
         <is>
@@ -45596,11 +45587,11 @@
     </row>
     <row r="418">
       <c r="A418" t="n">
-        <v>6224</v>
+        <v>6278</v>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -45610,7 +45601,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Real - Anual</t>
         </is>
       </c>
       <c r="E418" t="inlineStr">
@@ -45620,7 +45611,7 @@
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G418" t="n">
@@ -45650,11 +45641,11 @@
         </is>
       </c>
       <c r="O418" t="n">
-        <v>17688641</v>
+        <v>18166309</v>
       </c>
       <c r="P418" t="inlineStr">
         <is>
-          <t>Jackson Silva</t>
+          <t>Isabela Lemos</t>
         </is>
       </c>
       <c r="Q418" t="inlineStr">
@@ -45668,7 +45659,7 @@
       </c>
       <c r="T418" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U418" t="inlineStr">
@@ -45676,7 +45667,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V418" t="inlineStr"/>
+      <c r="V418" t="inlineStr">
+        <is>
+          <t>Aguardando a Liberação da Gerência de Contas - Data Comentário: 22/07/2026 19:09</t>
+        </is>
+      </c>
       <c r="W418" t="inlineStr"/>
       <c r="X418" t="inlineStr"/>
       <c r="Y418" t="inlineStr"/>
@@ -45695,17 +45690,17 @@
       </c>
       <c r="AG418" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="n">
-        <v>6278</v>
+        <v>6486</v>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -45715,7 +45710,7 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>Federal - Lucro Real - Anual</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E419" t="inlineStr">
@@ -45755,11 +45750,11 @@
         </is>
       </c>
       <c r="O419" t="n">
-        <v>18166309</v>
+        <v>18114205</v>
       </c>
       <c r="P419" t="inlineStr">
         <is>
-          <t>Isabela Lemos</t>
+          <t>Nathany Barreto</t>
         </is>
       </c>
       <c r="Q419" t="inlineStr">
@@ -45773,7 +45768,7 @@
       </c>
       <c r="T419" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U419" t="inlineStr">
@@ -45783,7 +45778,8 @@
       </c>
       <c r="V419" t="inlineStr">
         <is>
-          <t>Aguardando a Liberação da Gerência de Contas - Data Comentário: 22/07/2026 19:09</t>
+          <t>Aguardando a Liberação da Gerência de Contas  
+Aguardando liberação da Lucratividade - Data Comentário: 21/07/2026 11:31</t>
         </is>
       </c>
       <c r="W419" t="inlineStr"/>
@@ -45804,17 +45800,17 @@
       </c>
       <c r="AG419" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="n">
-        <v>6486</v>
+        <v>6704</v>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>PC GAMER GOIANIA LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -45864,11 +45860,11 @@
         </is>
       </c>
       <c r="O420" t="n">
-        <v>18114205</v>
+        <v>17955369</v>
       </c>
       <c r="P420" t="inlineStr">
         <is>
-          <t>Nathany Barreto</t>
+          <t>Paulo Silva</t>
         </is>
       </c>
       <c r="Q420" t="inlineStr">
@@ -45882,7 +45878,7 @@
       </c>
       <c r="T420" t="inlineStr">
         <is>
-          <t>PC GAMER</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U420" t="inlineStr">
@@ -45893,7 +45889,7 @@
       <c r="V420" t="inlineStr">
         <is>
           <t>Aguardando a Liberação da Gerência de Contas  
-Aguardando liberação da Lucratividade - Data Comentário: 21/07/2026 11:31</t>
+Precisão conclusão 30/07/2026 - Data Comentário: 22/07/2026 13:15</t>
         </is>
       </c>
       <c r="W420" t="inlineStr"/>
@@ -45914,17 +45910,17 @@
       </c>
       <c r="AG420" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="n">
-        <v>6704</v>
+        <v>5417</v>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -45944,11 +45940,11 @@
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G421" t="n">
-        <v>1582</v>
+        <v>11514</v>
       </c>
       <c r="H421" t="n">
         <v>0</v>
@@ -45960,25 +45956,29 @@
       </c>
       <c r="J421" t="inlineStr">
         <is>
-          <t>Fed - IRPJ/CSLL</t>
+          <t>Módulo de Inclusão Tributária (MIT)</t>
         </is>
       </c>
       <c r="K421" t="inlineStr"/>
       <c r="L421" s="1" t="n">
-        <v>46232</v>
-      </c>
-      <c r="M421" t="inlineStr"/>
+        <v>46233</v>
+      </c>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
       <c r="N421" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O421" t="n">
-        <v>17955369</v>
+        <v>17399463</v>
       </c>
       <c r="P421" t="inlineStr">
         <is>
-          <t>Paulo Silva</t>
+          <t>Eveny Silva</t>
         </is>
       </c>
       <c r="Q421" t="inlineStr">
@@ -45988,11 +45988,11 @@
       </c>
       <c r="R421" t="inlineStr"/>
       <c r="S421" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="T421" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U421" t="inlineStr">
@@ -46002,8 +46002,8 @@
       </c>
       <c r="V421" t="inlineStr">
         <is>
-          <t>Aguardando a Liberação da Gerência de Contas  
-Precisão conclusão 30/07/2026 - Data Comentário: 22/07/2026 13:15</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
+Aguardando liberação do PIS/COFINS/IRPJ E CSLL - Data Comentário: 21/07/2026 11:36</t>
         </is>
       </c>
       <c r="W421" t="inlineStr"/>
@@ -46019,22 +46019,22 @@
       <c r="AE421" t="inlineStr"/>
       <c r="AF421" t="inlineStr">
         <is>
-          <t>Imposto</t>
+          <t>Obrigação Acessória</t>
         </is>
       </c>
       <c r="AG421" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="n">
-        <v>5417</v>
+        <v>5617</v>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -46054,7 +46054,7 @@
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G422" t="n">
@@ -46088,11 +46088,11 @@
         </is>
       </c>
       <c r="O422" t="n">
-        <v>17399463</v>
+        <v>17407974</v>
       </c>
       <c r="P422" t="inlineStr">
         <is>
-          <t>Eveny Silva</t>
+          <t>Jackson Silva</t>
         </is>
       </c>
       <c r="Q422" t="inlineStr">
@@ -46106,7 +46106,7 @@
       </c>
       <c r="T422" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U422" t="inlineStr">
@@ -46116,8 +46116,7 @@
       </c>
       <c r="V422" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
-Aguardando liberação do PIS/COFINS/IRPJ E CSLL - Data Comentário: 21/07/2026 11:36</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 22/07/2026 15:47</t>
         </is>
       </c>
       <c r="W422" t="inlineStr"/>
@@ -46138,17 +46137,17 @@
       </c>
       <c r="AG422" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Edileide Dias</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="n">
-        <v>5617</v>
+        <v>6224</v>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -46168,7 +46167,7 @@
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G423" t="n">
@@ -46202,7 +46201,7 @@
         </is>
       </c>
       <c r="O423" t="n">
-        <v>17407974</v>
+        <v>17689071</v>
       </c>
       <c r="P423" t="inlineStr">
         <is>
@@ -46257,11 +46256,11 @@
     </row>
     <row r="424">
       <c r="A424" t="n">
-        <v>6224</v>
+        <v>6278</v>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -46271,7 +46270,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Real - Anual</t>
         </is>
       </c>
       <c r="E424" t="inlineStr">
@@ -46281,7 +46280,7 @@
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G424" t="n">
@@ -46306,7 +46305,7 @@
       </c>
       <c r="M424" t="inlineStr">
         <is>
-          <t>29/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="N424" t="inlineStr">
@@ -46315,11 +46314,11 @@
         </is>
       </c>
       <c r="O424" t="n">
-        <v>17689071</v>
+        <v>17539898</v>
       </c>
       <c r="P424" t="inlineStr">
         <is>
-          <t>Jackson Silva</t>
+          <t>Isabela Lemos</t>
         </is>
       </c>
       <c r="Q424" t="inlineStr">
@@ -46333,7 +46332,7 @@
       </c>
       <c r="T424" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U424" t="inlineStr">
@@ -46343,7 +46342,7 @@
       </c>
       <c r="V424" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 22/07/2026 15:47</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 - Data Comentário: 22/07/2026 20:00</t>
         </is>
       </c>
       <c r="W424" t="inlineStr"/>
@@ -46364,17 +46363,17 @@
       </c>
       <c r="AG424" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="n">
-        <v>6278</v>
+        <v>6279</v>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>DIENNYFER DA S PEREIRA</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -46384,7 +46383,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>Federal - Lucro Real - Anual</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E425" t="inlineStr">
@@ -46394,7 +46393,7 @@
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G425" t="n">
@@ -46428,7 +46427,7 @@
         </is>
       </c>
       <c r="O425" t="n">
-        <v>17539898</v>
+        <v>18056291</v>
       </c>
       <c r="P425" t="inlineStr">
         <is>
@@ -46483,11 +46482,11 @@
     </row>
     <row r="426">
       <c r="A426" t="n">
-        <v>6279</v>
+        <v>6404</v>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>DIENNYFER DA S PEREIRA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -46507,7 +46506,7 @@
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G426" t="n">
@@ -46541,7 +46540,7 @@
         </is>
       </c>
       <c r="O426" t="n">
-        <v>18056291</v>
+        <v>16962472</v>
       </c>
       <c r="P426" t="inlineStr">
         <is>
@@ -46559,7 +46558,7 @@
       </c>
       <c r="T426" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>SOLAR INVESTIMENTOS</t>
         </is>
       </c>
       <c r="U426" t="inlineStr">
@@ -46596,11 +46595,11 @@
     </row>
     <row r="427">
       <c r="A427" t="n">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
@@ -46610,7 +46609,7 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E427" t="inlineStr">
@@ -46645,7 +46644,7 @@
       </c>
       <c r="M427" t="inlineStr">
         <is>
-          <t>30/07/2026</t>
+          <t>29/07/2026</t>
         </is>
       </c>
       <c r="N427" t="inlineStr">
@@ -46654,11 +46653,11 @@
         </is>
       </c>
       <c r="O427" t="n">
-        <v>16962472</v>
+        <v>18114225</v>
       </c>
       <c r="P427" t="inlineStr">
         <is>
-          <t>Isabela Lemos</t>
+          <t>Nathany Barreto</t>
         </is>
       </c>
       <c r="Q427" t="inlineStr">
@@ -46672,7 +46671,7 @@
       </c>
       <c r="T427" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U427" t="inlineStr">
@@ -46682,7 +46681,8 @@
       </c>
       <c r="V427" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 - Data Comentário: 22/07/2026 20:00</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
+Aguardando liberação do PIS/COFINS/IRPJ E CSLL - Data Comentário: 21/07/2026 11:36</t>
         </is>
       </c>
       <c r="W427" t="inlineStr"/>
@@ -46703,17 +46703,17 @@
       </c>
       <c r="AG427" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="n">
-        <v>6486</v>
+        <v>6703</v>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>PC GAMER GOIANIA LTDA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
@@ -46723,7 +46723,7 @@
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E428" t="inlineStr">
@@ -46767,7 +46767,7 @@
         </is>
       </c>
       <c r="O428" t="n">
-        <v>18114225</v>
+        <v>17955210</v>
       </c>
       <c r="P428" t="inlineStr">
         <is>
@@ -46785,7 +46785,7 @@
       </c>
       <c r="T428" t="inlineStr">
         <is>
-          <t>PC GAMER</t>
+          <t>LIMA MOTA</t>
         </is>
       </c>
       <c r="U428" t="inlineStr">
@@ -46823,11 +46823,11 @@
     </row>
     <row r="429">
       <c r="A429" t="n">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -46837,7 +46837,7 @@
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E429" t="inlineStr">
@@ -46872,7 +46872,7 @@
       </c>
       <c r="M429" t="inlineStr">
         <is>
-          <t>29/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="N429" t="inlineStr">
@@ -46881,11 +46881,11 @@
         </is>
       </c>
       <c r="O429" t="n">
-        <v>17955210</v>
+        <v>17955443</v>
       </c>
       <c r="P429" t="inlineStr">
         <is>
-          <t>Nathany Barreto</t>
+          <t>Paulo Silva</t>
         </is>
       </c>
       <c r="Q429" t="inlineStr">
@@ -46899,7 +46899,7 @@
       </c>
       <c r="T429" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U429" t="inlineStr">
@@ -46909,8 +46909,7 @@
       </c>
       <c r="V429" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
-Aguardando liberação do PIS/COFINS/IRPJ E CSLL - Data Comentário: 21/07/2026 11:36</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 - Data Comentário: 22/07/2026 13:16</t>
         </is>
       </c>
       <c r="W429" t="inlineStr"/>
@@ -46931,17 +46930,17 @@
       </c>
       <c r="AG429" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="n">
-        <v>6704</v>
+        <v>6279</v>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>DIENNYFER DA S PEREIRA</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
@@ -46951,7 +46950,7 @@
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E430" t="inlineStr">
@@ -46961,11 +46960,11 @@
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G430" t="n">
-        <v>11514</v>
+        <v>10988</v>
       </c>
       <c r="H430" t="n">
         <v>0</v>
@@ -46977,16 +46976,16 @@
       </c>
       <c r="J430" t="inlineStr">
         <is>
-          <t>Módulo de Inclusão Tributária (MIT)</t>
+          <t>Movimento - Analise de Balanço Lucro Presumido</t>
         </is>
       </c>
       <c r="K430" t="inlineStr"/>
       <c r="L430" s="1" t="n">
-        <v>46233</v>
+        <v>46230</v>
       </c>
       <c r="M430" t="inlineStr">
         <is>
-          <t>30/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="N430" t="inlineStr">
@@ -46995,11 +46994,11 @@
         </is>
       </c>
       <c r="O430" t="n">
-        <v>17955443</v>
+        <v>18097173</v>
       </c>
       <c r="P430" t="inlineStr">
         <is>
-          <t>Paulo Silva</t>
+          <t>Isabela Lemos</t>
         </is>
       </c>
       <c r="Q430" t="inlineStr">
@@ -47009,11 +47008,11 @@
       </c>
       <c r="R430" t="inlineStr"/>
       <c r="S430" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="T430" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U430" t="inlineStr">
@@ -47023,7 +47022,7 @@
       </c>
       <c r="V430" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 - Data Comentário: 22/07/2026 13:16</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 - Data Comentário: 22/07/2026 19:16</t>
         </is>
       </c>
       <c r="W430" t="inlineStr"/>
@@ -47039,7 +47038,7 @@
       <c r="AE430" t="inlineStr"/>
       <c r="AF430" t="inlineStr">
         <is>
-          <t>Obrigação Acessória</t>
+          <t>Tarefa</t>
         </is>
       </c>
       <c r="AG430" t="inlineStr">
@@ -47050,11 +47049,11 @@
     </row>
     <row r="431">
       <c r="A431" t="n">
-        <v>6279</v>
+        <v>6703</v>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>DIENNYFER DA S PEREIRA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
@@ -47074,7 +47073,7 @@
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G431" t="n">
@@ -47097,22 +47096,18 @@
       <c r="L431" s="1" t="n">
         <v>46230</v>
       </c>
-      <c r="M431" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
+      <c r="M431" t="inlineStr"/>
       <c r="N431" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O431" t="n">
-        <v>18097173</v>
+        <v>18112916</v>
       </c>
       <c r="P431" t="inlineStr">
         <is>
-          <t>Isabela Lemos</t>
+          <t>Nathany Barreto</t>
         </is>
       </c>
       <c r="Q431" t="inlineStr">
@@ -47126,7 +47121,7 @@
       </c>
       <c r="T431" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>LIMA MOTA</t>
         </is>
       </c>
       <c r="U431" t="inlineStr">
@@ -47134,11 +47129,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V431" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 - Data Comentário: 22/07/2026 19:16</t>
-        </is>
-      </c>
+      <c r="V431" t="inlineStr"/>
       <c r="W431" t="inlineStr"/>
       <c r="X431" t="inlineStr"/>
       <c r="Y431" t="inlineStr"/>
@@ -47157,17 +47148,17 @@
       </c>
       <c r="AG431" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="n">
-        <v>6703</v>
+        <v>5417</v>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
@@ -47177,7 +47168,7 @@
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E432" t="inlineStr">
@@ -47187,11 +47178,11 @@
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G432" t="n">
-        <v>10988</v>
+        <v>7874</v>
       </c>
       <c r="H432" t="n">
         <v>0</v>
@@ -47203,7 +47194,7 @@
       </c>
       <c r="J432" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Lucro Presumido</t>
+          <t>Movimento - Analise de Balanço Lucro Real</t>
         </is>
       </c>
       <c r="K432" t="inlineStr"/>
@@ -47217,11 +47208,11 @@
         </is>
       </c>
       <c r="O432" t="n">
-        <v>18112916</v>
+        <v>17399318</v>
       </c>
       <c r="P432" t="inlineStr">
         <is>
-          <t>Nathany Barreto</t>
+          <t>Eveny Silva</t>
         </is>
       </c>
       <c r="Q432" t="inlineStr">
@@ -47235,7 +47226,7 @@
       </c>
       <c r="T432" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U432" t="inlineStr">
@@ -47268,11 +47259,11 @@
     </row>
     <row r="433">
       <c r="A433" t="n">
-        <v>5417</v>
+        <v>5617</v>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
@@ -47292,7 +47283,7 @@
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G433" t="n">
@@ -47315,18 +47306,22 @@
       <c r="L433" s="1" t="n">
         <v>46230</v>
       </c>
-      <c r="M433" t="inlineStr"/>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
       <c r="N433" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O433" t="n">
-        <v>17399318</v>
+        <v>17407859</v>
       </c>
       <c r="P433" t="inlineStr">
         <is>
-          <t>Eveny Silva</t>
+          <t>Jackson Silva</t>
         </is>
       </c>
       <c r="Q433" t="inlineStr">
@@ -47340,7 +47335,7 @@
       </c>
       <c r="T433" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U433" t="inlineStr">
@@ -47348,7 +47343,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V433" t="inlineStr"/>
+      <c r="V433" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 22/07/2026 16:28</t>
+        </is>
+      </c>
       <c r="W433" t="inlineStr"/>
       <c r="X433" t="inlineStr"/>
       <c r="Y433" t="inlineStr"/>
@@ -47367,17 +47366,17 @@
       </c>
       <c r="AG433" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Edileide Dias</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="n">
-        <v>5617</v>
+        <v>6224</v>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
@@ -47397,7 +47396,7 @@
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G434" t="n">
@@ -47431,7 +47430,7 @@
         </is>
       </c>
       <c r="O434" t="n">
-        <v>17407859</v>
+        <v>17206042</v>
       </c>
       <c r="P434" t="inlineStr">
         <is>
@@ -47486,11 +47485,11 @@
     </row>
     <row r="435">
       <c r="A435" t="n">
-        <v>6224</v>
+        <v>6278</v>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
@@ -47500,7 +47499,7 @@
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Real - Anual</t>
         </is>
       </c>
       <c r="E435" t="inlineStr">
@@ -47510,7 +47509,7 @@
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G435" t="n">
@@ -47535,7 +47534,7 @@
       </c>
       <c r="M435" t="inlineStr">
         <is>
-          <t>29/07/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="N435" t="inlineStr">
@@ -47544,11 +47543,11 @@
         </is>
       </c>
       <c r="O435" t="n">
-        <v>17206042</v>
+        <v>17539826</v>
       </c>
       <c r="P435" t="inlineStr">
         <is>
-          <t>Jackson Silva</t>
+          <t>Isabela Lemos</t>
         </is>
       </c>
       <c r="Q435" t="inlineStr">
@@ -47562,7 +47561,7 @@
       </c>
       <c r="T435" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U435" t="inlineStr">
@@ -47572,7 +47571,7 @@
       </c>
       <c r="V435" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 22/07/2026 16:28</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 - Data Comentário: 22/07/2026 19:16</t>
         </is>
       </c>
       <c r="W435" t="inlineStr"/>
@@ -47593,17 +47592,17 @@
       </c>
       <c r="AG435" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="n">
-        <v>6278</v>
+        <v>6486</v>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
@@ -47613,7 +47612,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>Federal - Lucro Real - Anual</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E436" t="inlineStr">
@@ -47646,22 +47645,18 @@
       <c r="L436" s="1" t="n">
         <v>46230</v>
       </c>
-      <c r="M436" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
+      <c r="M436" t="inlineStr"/>
       <c r="N436" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O436" t="n">
-        <v>17539826</v>
+        <v>18130461</v>
       </c>
       <c r="P436" t="inlineStr">
         <is>
-          <t>Isabela Lemos</t>
+          <t>Nathany Barreto</t>
         </is>
       </c>
       <c r="Q436" t="inlineStr">
@@ -47675,7 +47670,7 @@
       </c>
       <c r="T436" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U436" t="inlineStr">
@@ -47683,11 +47678,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V436" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 - Data Comentário: 22/07/2026 19:16</t>
-        </is>
-      </c>
+      <c r="V436" t="inlineStr"/>
       <c r="W436" t="inlineStr"/>
       <c r="X436" t="inlineStr"/>
       <c r="Y436" t="inlineStr"/>
@@ -47706,7 +47697,7 @@
       </c>
       <c r="AG436" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
@@ -47740,37 +47731,41 @@
         </is>
       </c>
       <c r="G437" t="n">
-        <v>7874</v>
+        <v>5800</v>
       </c>
       <c r="H437" t="n">
-        <v>0</v>
+        <v>5776</v>
       </c>
       <c r="I437" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J437" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Lucro Real</t>
+          <t>CCT Lançamento Sd.663</t>
         </is>
       </c>
       <c r="K437" t="inlineStr"/>
       <c r="L437" s="1" t="n">
-        <v>46230</v>
-      </c>
-      <c r="M437" t="inlineStr"/>
+        <v>46233</v>
+      </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
       <c r="N437" t="inlineStr">
         <is>
-          <t>06/2026</t>
+          <t>00/2026</t>
         </is>
       </c>
       <c r="O437" t="n">
-        <v>18130461</v>
+        <v>17901201</v>
       </c>
       <c r="P437" t="inlineStr">
         <is>
-          <t>Nathany Barreto</t>
+          <t>Jakeline Silva</t>
         </is>
       </c>
       <c r="Q437" t="inlineStr">
@@ -47780,7 +47775,7 @@
       </c>
       <c r="R437" t="inlineStr"/>
       <c r="S437" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="T437" t="inlineStr">
         <is>
@@ -47792,7 +47787,12 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V437" t="inlineStr"/>
+      <c r="V437" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 30/07/2026 
+O retorno do cliente foi recebido. Estamos realizando os trâmites para a aplicação do reajuste. - Data Comentário: 27/07/2026 09:51</t>
+        </is>
+      </c>
       <c r="W437" t="inlineStr"/>
       <c r="X437" t="inlineStr"/>
       <c r="Y437" t="inlineStr"/>
@@ -47811,7 +47811,7 @@
       </c>
       <c r="AG437" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>David Bragança</t>
         </is>
       </c>
     </row>
@@ -83793,12 +83793,12 @@
       <c r="AC766" t="inlineStr"/>
       <c r="AD766" t="inlineStr">
         <is>
-          <t>Atraso do cliente, o atraso do cliente já é recorrente e de ciência do Master e do Gerente de Contas. - Data Comentário: 20/07/2026 08:57</t>
+          <t>Atraso do cliente, o atraso do cliente já é recorrente e de ciência do Master e do Gerente de Contas. - Data Comentário: 27/07/2026 12:36</t>
         </is>
       </c>
       <c r="AE766" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="AF766" t="inlineStr">
@@ -83908,12 +83908,12 @@
       <c r="AC767" t="inlineStr"/>
       <c r="AD767" t="inlineStr">
         <is>
-          <t>Atraso do cliente, o atraso do cliente já é recorrente e de ciência do Master e do Gerente de Contas. - Data Comentário: 23/07/2026 09:19</t>
+          <t>Atraso do cliente, o atraso do cliente já é recorrente e de ciência do Master e do Gerente de Contas. - Data Comentário: 27/07/2026 12:36</t>
         </is>
       </c>
       <c r="AE767" t="inlineStr">
         <is>
-          <t>23/07/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="AF767" t="inlineStr">
@@ -84024,12 +84024,12 @@
       <c r="AC768" t="inlineStr"/>
       <c r="AD768" t="inlineStr">
         <is>
-          <t>Aguardando o agendamento da implantação. - Data Comentário: 20/07/2026 08:57</t>
+          <t>Aguardando o agendamento da implantação. - Data Comentário: 27/07/2026 12:36</t>
         </is>
       </c>
       <c r="AE768" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>27/07/2026</t>
         </is>
       </c>
       <c r="AF768" t="inlineStr">
@@ -84136,12 +84136,12 @@
       <c r="AC769" t="inlineStr"/>
       <c r="AD769" t="inlineStr">
         <is>
-          <t>Aguardando o agendamento da implantação. - Data Comentário: 20/07/2026 08:57</t>
+          <t>Aguardando o agendamento da implantação. - Data Comentário: 27/07/2026 12:36</t>
         </is>
       </c>
       <c r="AE769" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>27/07/2026</t>
         </is>
       </c>
       <c r="AF769" t="inlineStr">
@@ -84248,12 +84248,12 @@
       <c r="AC770" t="inlineStr"/>
       <c r="AD770" t="inlineStr">
         <is>
-          <t>Aguardando o agendamento da implantação. - Data Comentário: 20/07/2026 08:57</t>
+          <t>Aguardando o agendamento da implantação. - Data Comentário: 27/07/2026 12:36</t>
         </is>
       </c>
       <c r="AE770" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>27/07/2026</t>
         </is>
       </c>
       <c r="AF770" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-27 15:45
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -47096,7 +47096,11 @@
       <c r="L431" s="1" t="n">
         <v>46230</v>
       </c>
-      <c r="M431" t="inlineStr"/>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
       <c r="N431" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -47129,7 +47133,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V431" t="inlineStr"/>
+      <c r="V431" t="inlineStr">
+        <is>
+          <t>Atraso da Operação, processo em elaboração conforme data prevista  Previsão para conclusão dia 29/07/2026 - Data Comentário: 27/07/2026 14:01</t>
+        </is>
+      </c>
       <c r="W431" t="inlineStr"/>
       <c r="X431" t="inlineStr"/>
       <c r="Y431" t="inlineStr"/>
@@ -47761,7 +47769,7 @@
       </c>
       <c r="M437" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="N437" t="inlineStr">
@@ -47798,8 +47806,8 @@
       </c>
       <c r="V437" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 
-Previsão para concluir em 28/07/2026 - Data Comentário: 27/07/2026 09:15</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 
+Data provisionada. - Data Comentário: 27/07/2026 15:32</t>
         </is>
       </c>
       <c r="W437" t="inlineStr"/>
@@ -48088,7 +48096,11 @@
       <c r="L440" s="1" t="n">
         <v>46234</v>
       </c>
-      <c r="M440" t="inlineStr"/>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
       <c r="N440" t="inlineStr">
         <is>
           <t>08/2026</t>
@@ -48117,7 +48129,12 @@
         </is>
       </c>
       <c r="U440" t="inlineStr"/>
-      <c r="V440" t="inlineStr"/>
+      <c r="V440" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
+Previsão de conclusão: 29/07/2026 - Data Comentário: 27/07/2026 14:34</t>
+        </is>
+      </c>
       <c r="W440" t="inlineStr"/>
       <c r="X440" t="inlineStr"/>
       <c r="Y440" t="inlineStr"/>
@@ -48735,7 +48752,11 @@
       <c r="L446" s="1" t="n">
         <v>46234</v>
       </c>
-      <c r="M446" t="inlineStr"/>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
       <c r="N446" t="inlineStr">
         <is>
           <t>08/2026</t>
@@ -48764,7 +48785,12 @@
         </is>
       </c>
       <c r="U446" t="inlineStr"/>
-      <c r="V446" t="inlineStr"/>
+      <c r="V446" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
+Previsão de conclusão: 29/07/2026 - Data Comentário: 27/07/2026 14:34</t>
+        </is>
+      </c>
       <c r="W446" t="inlineStr"/>
       <c r="X446" t="inlineStr"/>
       <c r="Y446" t="inlineStr"/>
@@ -83666,7 +83692,11 @@
           <t>HELBRAZ</t>
         </is>
       </c>
-      <c r="U765" t="inlineStr"/>
+      <c r="U765" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V765" t="inlineStr">
         <is>
           <t>Sem informações para a realização da tarefa  
@@ -83774,7 +83804,11 @@
           <t>HELBRAZ</t>
         </is>
       </c>
-      <c r="U766" t="inlineStr"/>
+      <c r="U766" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V766" t="inlineStr">
         <is>
           <t>Sem informações para a realização da tarefa  
@@ -84236,7 +84270,11 @@
           <t>HELBRAZ</t>
         </is>
       </c>
-      <c r="U770" t="inlineStr"/>
+      <c r="U770" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V770" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 17/07/2026 
@@ -84348,7 +84386,11 @@
           <t>HELBRAZ</t>
         </is>
       </c>
-      <c r="U771" t="inlineStr"/>
+      <c r="U771" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V771" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 17/07/2026 
@@ -84572,7 +84614,11 @@
           <t>HELBRAZ</t>
         </is>
       </c>
-      <c r="U773" t="inlineStr"/>
+      <c r="U773" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V773" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 27/07/2026 
@@ -84688,7 +84734,11 @@
           <t>HELBRAZ</t>
         </is>
       </c>
-      <c r="U774" t="inlineStr"/>
+      <c r="U774" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V774" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 27/07/2026 

</xml_diff>

<commit_message>
Atualização automática: 2026-07-27 16:47
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -884,7 +884,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 26/06/2026 
@@ -988,7 +992,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6962; Tarefa Incluida: 11615; Vencimento: 17/06/2026 00:00:00; UsuarioResponsavel: erikas - Data Comentário: 17/06/2026 11:09</t>
@@ -1091,7 +1099,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V6" t="inlineStr">
         <is>
           <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6963; Tarefa Incluida: 11615; Vencimento: 17/06/2026 00:00:00; UsuarioResponsavel: erikas - Data Comentário: 17/06/2026 11:09</t>
@@ -1531,7 +1543,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
@@ -1638,7 +1654,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
@@ -1745,7 +1765,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
@@ -2494,7 +2518,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr"/>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
@@ -2803,7 +2831,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V22" t="inlineStr">
         <is>
           <t>Sem informações para a realização da tarefa  
@@ -2907,7 +2939,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V23" t="inlineStr">
         <is>
           <t>Sem informações para a realização da tarefa  
@@ -3217,7 +3253,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr"/>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V26" t="inlineStr">
         <is>
           <t>Férias de 02/07/2026 a 10/07/2026. - Data Comentário: 01/07/2026 11:26</t>
@@ -3649,7 +3689,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr"/>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V30" t="inlineStr"/>
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr"/>
@@ -3855,7 +3899,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr"/>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V32" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 07/07/2026 
@@ -4300,7 +4348,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr"/>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V36" t="inlineStr"/>
       <c r="W36" t="inlineStr"/>
       <c r="X36" t="inlineStr"/>
@@ -4407,7 +4459,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr"/>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V37" t="inlineStr"/>
       <c r="W37" t="inlineStr"/>
       <c r="X37" t="inlineStr"/>
@@ -4514,7 +4570,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr"/>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V38" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 20/07/2026 
@@ -5675,7 +5735,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr"/>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V48" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 10/07/2026 
@@ -5899,7 +5963,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr"/>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V50" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 13/07/2026 
@@ -6932,7 +7000,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr"/>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V59" t="inlineStr">
         <is>
           <t>2. Folha Processada aguardando OK do cliente para finalização   Previsão para conclusão dia 06/07/2026 - Data Comentário: 03/07/2026 14:18</t>
@@ -7154,7 +7226,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr"/>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V61" t="inlineStr">
         <is>
           <t>2. Folha Processada aguardando OK do cliente para finalização   Previsão para conclusão dia 03/07/2026 - Data Comentário: 03/07/2026 16:19</t>
@@ -8034,7 +8110,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U69" t="inlineStr"/>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V69" t="inlineStr">
         <is>
           <t>2. Folha Processada aguardando OK do cliente para finalização   Previsão para conclusão dia 06/07/2026 - Data Comentário: 03/07/2026 14:17</t>
@@ -8244,7 +8324,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr"/>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V71" t="inlineStr"/>
       <c r="W71" t="inlineStr"/>
       <c r="X71" t="inlineStr"/>
@@ -9378,7 +9462,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U81" t="inlineStr"/>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V81" t="inlineStr">
         <is>
           <t>Imposto enviado via SCI Report - Data Comentário: 14/07/2026 17:57</t>
@@ -9592,7 +9680,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U83" t="inlineStr"/>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V83" t="inlineStr">
         <is>
           <t>Imposto enviado via SCI Report - Data Comentário: 13/07/2026 17:54</t>
@@ -10036,7 +10128,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U87" t="inlineStr"/>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V87" t="inlineStr"/>
       <c r="W87" t="inlineStr"/>
       <c r="X87" t="inlineStr"/>
@@ -10143,7 +10239,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U88" t="inlineStr"/>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V88" t="inlineStr"/>
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr"/>
@@ -10246,7 +10346,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U89" t="inlineStr"/>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V89" t="inlineStr">
         <is>
           <t>Atestado de dois dias em 26/06/2026. - Data Comentário: 01/07/2026 11:15</t>
@@ -11213,7 +11317,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U98" t="inlineStr"/>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V98" t="inlineStr"/>
       <c r="W98" t="inlineStr"/>
       <c r="X98" t="inlineStr"/>
@@ -11419,7 +11527,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U100" t="inlineStr"/>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V100" t="inlineStr"/>
       <c r="W100" t="inlineStr"/>
       <c r="X100" t="inlineStr"/>
@@ -12997,7 +13109,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U114" t="inlineStr"/>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V114" t="inlineStr">
         <is>
           <t>2. Folha Processada aguardando OK do cliente para finalização   Previsão para conclusão dia 06/07/2026 - Data Comentário: 03/07/2026 14:18</t>
@@ -13207,7 +13323,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U116" t="inlineStr"/>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V116" t="inlineStr"/>
       <c r="W116" t="inlineStr"/>
       <c r="X116" t="inlineStr"/>
@@ -14202,7 +14322,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U125" t="inlineStr"/>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V125" t="inlineStr">
         <is>
           <t>2. Folha Processada aguardando OK do cliente para finalização   Previsão para conclusão dia 06/07/2026 - Data Comentário: 03/07/2026 14:18</t>
@@ -14412,7 +14536,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U127" t="inlineStr"/>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V127" t="inlineStr"/>
       <c r="W127" t="inlineStr"/>
       <c r="X127" t="inlineStr"/>
@@ -14738,7 +14866,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U130" t="inlineStr"/>
+      <c r="U130" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V130" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 08/07/2026 
@@ -14842,7 +14974,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U131" t="inlineStr"/>
+      <c r="U131" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V131" t="inlineStr">
         <is>
           <t>Pedido de demissão - Desconto de Aviso em 07/07/2026 - Pgto 17/07/2026 - Data Comentário: 08/07/2026 11:16</t>
@@ -15163,7 +15299,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U134" t="inlineStr"/>
+      <c r="U134" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V134" t="inlineStr"/>
       <c r="W134" t="inlineStr"/>
       <c r="X134" t="inlineStr"/>
@@ -15262,7 +15402,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U135" t="inlineStr"/>
+      <c r="U135" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V135" t="inlineStr"/>
       <c r="W135" t="inlineStr"/>
       <c r="X135" t="inlineStr"/>
@@ -15583,7 +15727,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U138" t="inlineStr"/>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V138" t="inlineStr"/>
       <c r="W138" t="inlineStr"/>
       <c r="X138" t="inlineStr"/>
@@ -15682,7 +15830,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U139" t="inlineStr"/>
+      <c r="U139" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V139" t="inlineStr"/>
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr"/>
@@ -16003,7 +16155,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U142" t="inlineStr"/>
+      <c r="U142" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V142" t="inlineStr"/>
       <c r="W142" t="inlineStr"/>
       <c r="X142" t="inlineStr"/>
@@ -16102,7 +16258,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U143" t="inlineStr"/>
+      <c r="U143" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V143" t="inlineStr"/>
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr"/>
@@ -16316,7 +16476,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U145" t="inlineStr"/>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V145" t="inlineStr"/>
       <c r="W145" t="inlineStr"/>
       <c r="X145" t="inlineStr"/>
@@ -16423,7 +16587,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U146" t="inlineStr"/>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V146" t="inlineStr"/>
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr"/>
@@ -16526,7 +16694,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U147" t="inlineStr"/>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V147" t="inlineStr"/>
       <c r="W147" t="inlineStr"/>
       <c r="X147" t="inlineStr"/>
@@ -16625,7 +16797,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U148" t="inlineStr"/>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V148" t="inlineStr"/>
       <c r="W148" t="inlineStr"/>
       <c r="X148" t="inlineStr"/>
@@ -16946,7 +17122,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U151" t="inlineStr"/>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V151" t="inlineStr"/>
       <c r="W151" t="inlineStr"/>
       <c r="X151" t="inlineStr"/>
@@ -17045,7 +17225,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U152" t="inlineStr"/>
+      <c r="U152" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V152" t="inlineStr"/>
       <c r="W152" t="inlineStr"/>
       <c r="X152" t="inlineStr"/>
@@ -17144,7 +17328,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U153" t="inlineStr"/>
+      <c r="U153" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V153" t="inlineStr"/>
       <c r="W153" t="inlineStr"/>
       <c r="X153" t="inlineStr"/>
@@ -17243,7 +17431,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U154" t="inlineStr"/>
+      <c r="U154" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V154" t="inlineStr"/>
       <c r="W154" t="inlineStr"/>
       <c r="X154" t="inlineStr"/>
@@ -17342,7 +17534,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U155" t="inlineStr"/>
+      <c r="U155" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V155" t="inlineStr"/>
       <c r="W155" t="inlineStr"/>
       <c r="X155" t="inlineStr"/>
@@ -17441,7 +17637,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U156" t="inlineStr"/>
+      <c r="U156" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V156" t="inlineStr"/>
       <c r="W156" t="inlineStr"/>
       <c r="X156" t="inlineStr"/>
@@ -17540,7 +17740,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U157" t="inlineStr"/>
+      <c r="U157" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V157" t="inlineStr"/>
       <c r="W157" t="inlineStr"/>
       <c r="X157" t="inlineStr"/>
@@ -17639,7 +17843,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U158" t="inlineStr"/>
+      <c r="U158" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V158" t="inlineStr"/>
       <c r="W158" t="inlineStr"/>
       <c r="X158" t="inlineStr"/>
@@ -17960,7 +18168,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U161" t="inlineStr"/>
+      <c r="U161" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V161" t="inlineStr"/>
       <c r="W161" t="inlineStr"/>
       <c r="X161" t="inlineStr"/>
@@ -18059,7 +18271,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U162" t="inlineStr"/>
+      <c r="U162" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V162" t="inlineStr"/>
       <c r="W162" t="inlineStr"/>
       <c r="X162" t="inlineStr"/>
@@ -18380,7 +18596,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U165" t="inlineStr"/>
+      <c r="U165" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V165" t="inlineStr"/>
       <c r="W165" t="inlineStr"/>
       <c r="X165" t="inlineStr"/>
@@ -18479,7 +18699,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U166" t="inlineStr"/>
+      <c r="U166" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V166" t="inlineStr"/>
       <c r="W166" t="inlineStr"/>
       <c r="X166" t="inlineStr"/>
@@ -19065,7 +19289,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U171" t="inlineStr"/>
+      <c r="U171" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V171" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 
@@ -19181,7 +19409,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U172" t="inlineStr"/>
+      <c r="U172" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V172" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 
@@ -19416,7 +19648,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U174" t="inlineStr"/>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V174" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 06/07/2026 - Data Comentário: 06/07/2026 10:20</t>
@@ -19531,7 +19767,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U175" t="inlineStr"/>
+      <c r="U175" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V175" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 06/07/2026 - Data Comentário: 06/07/2026 10:20</t>
@@ -19885,7 +20125,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U178" t="inlineStr"/>
+      <c r="U178" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V178" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 07/07/2026 - Data Comentário: 06/07/2026 10:20</t>
@@ -20000,7 +20244,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U179" t="inlineStr"/>
+      <c r="U179" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V179" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 07/07/2026 - Data Comentário: 06/07/2026 10:20</t>
@@ -20107,7 +20355,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U180" t="inlineStr"/>
+      <c r="U180" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V180" t="inlineStr"/>
       <c r="W180" t="inlineStr"/>
       <c r="X180" t="inlineStr"/>
@@ -20206,7 +20458,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U181" t="inlineStr"/>
+      <c r="U181" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V181" t="inlineStr"/>
       <c r="W181" t="inlineStr"/>
       <c r="X181" t="inlineStr"/>
@@ -20433,7 +20689,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U183" t="inlineStr"/>
+      <c r="U183" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V183" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 17/07/2026 - Data Comentário: 14/07/2026 09:50</t>
@@ -20544,7 +20804,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U184" t="inlineStr"/>
+      <c r="U184" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V184" t="inlineStr">
         <is>
           <t>Atraso de envio do cliente, consultar pendências no check list - Data Comentário: 14/07/2026 09:51</t>
@@ -23667,7 +23931,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U213" t="inlineStr"/>
+      <c r="U213" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V213" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 17:18</t>
@@ -26447,7 +26715,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U238" t="inlineStr"/>
+      <c r="U238" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V238" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 13/07/2026 - Data Comentário: 13/07/2026 12:04</t>
@@ -28366,7 +28638,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U255" t="inlineStr"/>
+      <c r="U255" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V255" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 08/07/2026 - Data Comentário: 06/07/2026 15:51</t>
@@ -30419,7 +30695,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U274" t="inlineStr"/>
+      <c r="U274" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V274" t="inlineStr">
         <is>
           <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1866] sendo a ultima baixa feita [1866]-08/07/2026 18:25:05.. - Data Comentário: 08/07/2026 18:24</t>
@@ -30522,7 +30802,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U275" t="inlineStr"/>
+      <c r="U275" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V275" t="inlineStr">
         <is>
           <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1866] sendo a ultima baixa feita [1866]-08/07/2026 18:24:46.. - Data Comentário: 08/07/2026 18:24</t>
@@ -31172,7 +31456,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U281" t="inlineStr"/>
+      <c r="U281" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V281" t="inlineStr">
         <is>
           <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1793] sendo a ultima baixa feita [1793]-10/07/2026 09:57:11.. - Data Comentário: 10/07/2026 09:56</t>
@@ -31382,7 +31670,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U283" t="inlineStr"/>
+      <c r="U283" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V283" t="inlineStr"/>
       <c r="W283" t="inlineStr"/>
       <c r="X283" t="inlineStr"/>
@@ -31481,7 +31773,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U284" t="inlineStr"/>
+      <c r="U284" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V284" t="inlineStr">
         <is>
           <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-08/07/2026 18:24:14.. - Data Comentário: 08/07/2026 18:23</t>
@@ -31584,7 +31880,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U285" t="inlineStr"/>
+      <c r="U285" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V285" t="inlineStr">
         <is>
           <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1867] sendo a ultima baixa feita [1867]-08/07/2026 18:24:49.. - Data Comentário: 08/07/2026 18:24</t>
@@ -33066,7 +33366,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U299" t="inlineStr"/>
+      <c r="U299" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V299" t="inlineStr"/>
       <c r="W299" t="inlineStr"/>
       <c r="X299" t="inlineStr"/>
@@ -33268,7 +33572,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U301" t="inlineStr"/>
+      <c r="U301" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V301" t="inlineStr"/>
       <c r="W301" t="inlineStr"/>
       <c r="X301" t="inlineStr"/>
@@ -33371,7 +33679,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U302" t="inlineStr"/>
+      <c r="U302" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V302" t="inlineStr"/>
       <c r="W302" t="inlineStr"/>
       <c r="X302" t="inlineStr"/>
@@ -33474,7 +33786,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U303" t="inlineStr"/>
+      <c r="U303" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V303" t="inlineStr"/>
       <c r="W303" t="inlineStr"/>
       <c r="X303" t="inlineStr"/>
@@ -33577,7 +33893,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U304" t="inlineStr"/>
+      <c r="U304" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V304" t="inlineStr"/>
       <c r="W304" t="inlineStr"/>
       <c r="X304" t="inlineStr"/>
@@ -34849,7 +35169,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U316" t="inlineStr"/>
+      <c r="U316" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V316" t="inlineStr"/>
       <c r="W316" t="inlineStr"/>
       <c r="X316" t="inlineStr"/>
@@ -35051,7 +35375,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U318" t="inlineStr"/>
+      <c r="U318" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V318" t="inlineStr"/>
       <c r="W318" t="inlineStr"/>
       <c r="X318" t="inlineStr"/>
@@ -35154,7 +35482,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U319" t="inlineStr"/>
+      <c r="U319" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V319" t="inlineStr"/>
       <c r="W319" t="inlineStr"/>
       <c r="X319" t="inlineStr"/>
@@ -35257,7 +35589,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U320" t="inlineStr"/>
+      <c r="U320" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V320" t="inlineStr"/>
       <c r="W320" t="inlineStr"/>
       <c r="X320" t="inlineStr"/>
@@ -35360,7 +35696,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U321" t="inlineStr"/>
+      <c r="U321" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V321" t="inlineStr"/>
       <c r="W321" t="inlineStr"/>
       <c r="X321" t="inlineStr"/>
@@ -36616,7 +36956,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U333" t="inlineStr"/>
+      <c r="U333" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V333" t="inlineStr"/>
       <c r="W333" t="inlineStr"/>
       <c r="X333" t="inlineStr"/>
@@ -38094,7 +38438,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U347" t="inlineStr"/>
+      <c r="U347" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V347" t="inlineStr"/>
       <c r="W347" t="inlineStr"/>
       <c r="X347" t="inlineStr"/>
@@ -38296,7 +38644,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U349" t="inlineStr"/>
+      <c r="U349" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V349" t="inlineStr"/>
       <c r="W349" t="inlineStr"/>
       <c r="X349" t="inlineStr"/>
@@ -38399,7 +38751,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U350" t="inlineStr"/>
+      <c r="U350" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V350" t="inlineStr"/>
       <c r="W350" t="inlineStr"/>
       <c r="X350" t="inlineStr"/>
@@ -38502,7 +38858,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U351" t="inlineStr"/>
+      <c r="U351" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V351" t="inlineStr"/>
       <c r="W351" t="inlineStr"/>
       <c r="X351" t="inlineStr"/>
@@ -38605,7 +38965,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U352" t="inlineStr"/>
+      <c r="U352" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V352" t="inlineStr"/>
       <c r="W352" t="inlineStr"/>
       <c r="X352" t="inlineStr"/>
@@ -39877,7 +40241,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U364" t="inlineStr"/>
+      <c r="U364" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V364" t="inlineStr"/>
       <c r="W364" t="inlineStr"/>
       <c r="X364" t="inlineStr"/>
@@ -40079,7 +40447,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U366" t="inlineStr"/>
+      <c r="U366" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V366" t="inlineStr"/>
       <c r="W366" t="inlineStr"/>
       <c r="X366" t="inlineStr"/>
@@ -40182,7 +40554,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U367" t="inlineStr"/>
+      <c r="U367" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V367" t="inlineStr"/>
       <c r="W367" t="inlineStr"/>
       <c r="X367" t="inlineStr"/>
@@ -40285,7 +40661,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U368" t="inlineStr"/>
+      <c r="U368" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V368" t="inlineStr"/>
       <c r="W368" t="inlineStr"/>
       <c r="X368" t="inlineStr"/>
@@ -40388,7 +40768,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U369" t="inlineStr"/>
+      <c r="U369" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V369" t="inlineStr"/>
       <c r="W369" t="inlineStr"/>
       <c r="X369" t="inlineStr"/>
@@ -42657,7 +43041,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U390" t="inlineStr"/>
+      <c r="U390" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V390" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 
@@ -42767,7 +43155,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U391" t="inlineStr"/>
+      <c r="U391" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V391" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 
@@ -43083,7 +43475,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U394" t="inlineStr"/>
+      <c r="U394" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V394" t="inlineStr"/>
       <c r="W394" t="inlineStr"/>
       <c r="X394" t="inlineStr"/>
@@ -43184,7 +43580,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U395" t="inlineStr"/>
+      <c r="U395" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V395" t="inlineStr"/>
       <c r="W395" t="inlineStr"/>
       <c r="X395" t="inlineStr"/>
@@ -43515,7 +43915,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U398" t="inlineStr"/>
+      <c r="U398" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V398" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
@@ -43625,7 +44029,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U399" t="inlineStr"/>
+      <c r="U399" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V399" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
@@ -43836,7 +44244,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U401" t="inlineStr"/>
+      <c r="U401" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V401" t="inlineStr"/>
       <c r="W401" t="inlineStr"/>
       <c r="X401" t="inlineStr"/>
@@ -43937,7 +44349,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U402" t="inlineStr"/>
+      <c r="U402" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V402" t="inlineStr"/>
       <c r="W402" t="inlineStr"/>
       <c r="X402" t="inlineStr"/>
@@ -44042,7 +44458,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U403" t="inlineStr"/>
+      <c r="U403" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V403" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 20/07/2026 15:54</t>
@@ -46991,7 +47411,11 @@
       <c r="L430" s="1" t="n">
         <v>46230</v>
       </c>
-      <c r="M430" t="inlineStr"/>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
       <c r="N430" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -47024,7 +47448,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V430" t="inlineStr"/>
+      <c r="V430" t="inlineStr">
+        <is>
+          <t>Atraso da Operação, processo em elaboração conforme data prevista  Previsão para conclusão dia 29/07/2026 - Data Comentário: 27/07/2026 16:33</t>
+        </is>
+      </c>
       <c r="W430" t="inlineStr"/>
       <c r="X430" t="inlineStr"/>
       <c r="Y430" t="inlineStr"/>
@@ -47548,7 +47976,11 @@
       <c r="L435" s="1" t="n">
         <v>46230</v>
       </c>
-      <c r="M435" t="inlineStr"/>
+      <c r="M435" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
       <c r="N435" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -47581,7 +48013,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V435" t="inlineStr"/>
+      <c r="V435" t="inlineStr">
+        <is>
+          <t>Atraso da Operação, processo em elaboração conforme data prevista   Previsão para conclusão dia 30/07/2026 - Data Comentário: 27/07/2026 16:34</t>
+        </is>
+      </c>
       <c r="W435" t="inlineStr"/>
       <c r="X435" t="inlineStr"/>
       <c r="Y435" t="inlineStr"/>
@@ -48023,7 +48459,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U439" t="inlineStr"/>
+      <c r="U439" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V439" t="inlineStr"/>
       <c r="W439" t="inlineStr"/>
       <c r="X439" t="inlineStr"/>
@@ -48128,7 +48568,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U440" t="inlineStr"/>
+      <c r="U440" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V440" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
@@ -48679,7 +49123,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U445" t="inlineStr"/>
+      <c r="U445" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V445" t="inlineStr"/>
       <c r="W445" t="inlineStr"/>
       <c r="X445" t="inlineStr"/>
@@ -48784,7 +49232,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U446" t="inlineStr"/>
+      <c r="U446" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V446" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
@@ -48991,7 +49443,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U448" t="inlineStr"/>
+      <c r="U448" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V448" t="inlineStr"/>
       <c r="W448" t="inlineStr"/>
       <c r="X448" t="inlineStr"/>
@@ -49752,7 +50208,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U455" t="inlineStr"/>
+      <c r="U455" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V455" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
@@ -49862,7 +50322,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U456" t="inlineStr"/>
+      <c r="U456" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V456" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
@@ -49972,7 +50436,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U457" t="inlineStr"/>
+      <c r="U457" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V457" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
@@ -51158,7 +51626,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U468" t="inlineStr"/>
+      <c r="U468" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V468" t="inlineStr">
         <is>
           <t>Imposto enviado via SCI Report - Data Comentário: 17/07/2026 08:27</t>
@@ -51269,7 +51741,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U469" t="inlineStr"/>
+      <c r="U469" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V469" t="inlineStr">
         <is>
           <t>Aguardando Liberação do Fiscal  
@@ -51381,7 +51857,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U470" t="inlineStr"/>
+      <c r="U470" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V470" t="inlineStr">
         <is>
           <t>Aguardando Liberação do Fiscal  
@@ -51826,7 +52306,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U474" t="inlineStr"/>
+      <c r="U474" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V474" t="inlineStr"/>
       <c r="W474" t="inlineStr"/>
       <c r="X474" t="inlineStr"/>
@@ -51937,7 +52421,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U475" t="inlineStr"/>
+      <c r="U475" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V475" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 27/07/2026 - Data Comentário: 20/07/2026 15:48</t>
@@ -52500,7 +52988,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U480" t="inlineStr"/>
+      <c r="U480" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V480" t="inlineStr"/>
       <c r="W480" t="inlineStr"/>
       <c r="X480" t="inlineStr"/>
@@ -52607,7 +53099,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U481" t="inlineStr"/>
+      <c r="U481" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V481" t="inlineStr"/>
       <c r="W481" t="inlineStr"/>
       <c r="X481" t="inlineStr"/>
@@ -53842,7 +54338,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U492" t="inlineStr"/>
+      <c r="U492" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V492" t="inlineStr">
         <is>
           <t>Imposto enviado via SCI Report - Data Comentário: 15/07/2026 18:26</t>
@@ -54837,7 +55337,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U501" t="inlineStr"/>
+      <c r="U501" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V501" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 22/07/2026 13:13</t>
@@ -56062,7 +56566,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U512" t="inlineStr"/>
+      <c r="U512" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V512" t="inlineStr">
         <is>
           <t>Baixado via API integração MGC x Analise Balanço em 20/07/2026 18:22:04. - Data Comentário: 20/07/2026 18:17</t>
@@ -57148,7 +57656,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U522" t="inlineStr"/>
+      <c r="U522" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V522" t="inlineStr"/>
       <c r="W522" t="inlineStr"/>
       <c r="X522" t="inlineStr"/>
@@ -58138,7 +58650,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U531" t="inlineStr"/>
+      <c r="U531" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V531" t="inlineStr"/>
       <c r="W531" t="inlineStr"/>
       <c r="X531" t="inlineStr"/>
@@ -58703,7 +59219,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U536" t="inlineStr"/>
+      <c r="U536" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V536" t="inlineStr"/>
       <c r="W536" t="inlineStr"/>
       <c r="X536" t="inlineStr"/>
@@ -59490,7 +60010,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U543" t="inlineStr"/>
+      <c r="U543" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V543" t="inlineStr"/>
       <c r="W543" t="inlineStr"/>
       <c r="X543" t="inlineStr"/>
@@ -59597,7 +60121,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U544" t="inlineStr"/>
+      <c r="U544" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V544" t="inlineStr"/>
       <c r="W544" t="inlineStr"/>
       <c r="X544" t="inlineStr"/>
@@ -59708,7 +60236,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U545" t="inlineStr"/>
+      <c r="U545" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V545" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 20/07/2026 
@@ -60500,7 +61032,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U552" t="inlineStr"/>
+      <c r="U552" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V552" t="inlineStr"/>
       <c r="W552" t="inlineStr"/>
       <c r="X552" t="inlineStr"/>
@@ -60607,7 +61143,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U553" t="inlineStr"/>
+      <c r="U553" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V553" t="inlineStr"/>
       <c r="W553" t="inlineStr"/>
       <c r="X553" t="inlineStr"/>
@@ -60718,7 +61258,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U554" t="inlineStr"/>
+      <c r="U554" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V554" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 20/07/2026 
@@ -60946,7 +61490,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U556" t="inlineStr"/>
+      <c r="U556" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V556" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 03/08/2026 
@@ -61054,7 +61602,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U557" t="inlineStr"/>
+      <c r="U557" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V557" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 03/08/2026 
@@ -61842,7 +62394,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U564" t="inlineStr"/>
+      <c r="U564" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V564" t="inlineStr"/>
       <c r="W564" t="inlineStr"/>
       <c r="X564" t="inlineStr"/>
@@ -61949,7 +62505,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U565" t="inlineStr"/>
+      <c r="U565" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V565" t="inlineStr"/>
       <c r="W565" t="inlineStr"/>
       <c r="X565" t="inlineStr"/>
@@ -62060,7 +62620,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U566" t="inlineStr"/>
+      <c r="U566" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V566" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 21/07/2026 
@@ -62628,7 +63192,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U571" t="inlineStr"/>
+      <c r="U571" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V571" t="inlineStr"/>
       <c r="W571" t="inlineStr"/>
       <c r="X571" t="inlineStr"/>
@@ -63073,7 +63641,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U575" t="inlineStr"/>
+      <c r="U575" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V575" t="inlineStr">
         <is>
           <t>63 - Isaak Pinheiro Dias, Pedido de demissão - Aviso Trabalhado - pagamento em 22/07/2026. - Data Comentário: 16/06/2026 13:28</t>
@@ -63180,7 +63752,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U576" t="inlineStr"/>
+      <c r="U576" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V576" t="inlineStr">
         <is>
           <t>Pedido de demissão - Desconto de Aviso em 10/07/2026 - Pgto 20/07/2026 - Data Comentário: 13/07/2026 17:57</t>
@@ -63283,7 +63859,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U577" t="inlineStr"/>
+      <c r="U577" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V577" t="inlineStr">
         <is>
           <t>Demissão Por Justa Causa em 16/07/2026 - Pgto 24/07/2026 - Data Comentário: 17/07/2026 09:53</t>
@@ -63838,7 +64418,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U582" t="inlineStr"/>
+      <c r="U582" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V582" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 21/07/2026 
@@ -63954,7 +64538,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U583" t="inlineStr"/>
+      <c r="U583" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V583" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 20/07/2026 
@@ -64757,7 +65345,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U590" t="inlineStr"/>
+      <c r="U590" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V590" t="inlineStr">
         <is>
           <t>Imposto enviado via SCI Report - Data Comentário: 23/07/2026 17:14</t>
@@ -64868,7 +65460,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U591" t="inlineStr"/>
+      <c r="U591" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V591" t="inlineStr">
         <is>
           <t>Imposto enviado via SCI Report - Data Comentário: 23/07/2026 17:32</t>
@@ -65435,7 +66031,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U596" t="inlineStr"/>
+      <c r="U596" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V596" t="inlineStr"/>
       <c r="W596" t="inlineStr"/>
       <c r="X596" t="inlineStr"/>
@@ -65542,7 +66142,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U597" t="inlineStr"/>
+      <c r="U597" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V597" t="inlineStr"/>
       <c r="W597" t="inlineStr"/>
       <c r="X597" t="inlineStr"/>
@@ -68424,7 +69028,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U623" t="inlineStr"/>
+      <c r="U623" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V623" t="inlineStr">
         <is>
           <t>Imposto enviado via SCI Report - Data Comentário: 14/07/2026 09:03</t>
@@ -70658,7 +71266,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U643" t="inlineStr"/>
+      <c r="U643" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V643" t="inlineStr">
         <is>
           <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1805] sendo a ultima baixa feita [1805]-14/07/2026 10:55:52.. - Data Comentário: 14/07/2026 10:54</t>
@@ -70868,7 +71480,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U645" t="inlineStr"/>
+      <c r="U645" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V645" t="inlineStr"/>
       <c r="W645" t="inlineStr"/>
       <c r="X645" t="inlineStr"/>
@@ -71724,7 +72340,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U653" t="inlineStr"/>
+      <c r="U653" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V653" t="inlineStr"/>
       <c r="W653" t="inlineStr"/>
       <c r="X653" t="inlineStr"/>
@@ -73250,7 +73870,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U667" t="inlineStr"/>
+      <c r="U667" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V667" t="inlineStr">
         <is>
           <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1882] sendo a ultima baixa feita [1882]-23/07/2026 17:22:20.. - Data Comentário: 23/07/2026 17:21</t>
@@ -73357,7 +73981,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U668" t="inlineStr"/>
+      <c r="U668" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V668" t="inlineStr">
         <is>
           <t>Reaberto via Rotina Configuração Após Baixa de tarefa [1882] sendo a ultima baixa feita [1882]-23/07/2026 17:54:50.. - Data Comentário: 23/07/2026 17:54</t>
@@ -74011,7 +74639,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U674" t="inlineStr"/>
+      <c r="U674" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V674" t="inlineStr">
         <is>
           <t>Reaberto via Rotina Configuração Após Baixa de tarefa [7237] sendo a ultima baixa feita [7237]-17/07/2026 10:28:51.. - Data Comentário: 17/07/2026 10:28</t>
@@ -74114,7 +74746,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U675" t="inlineStr"/>
+      <c r="U675" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V675" t="inlineStr">
         <is>
           <t>Reaberto via Rotina Configuração Após Baixa de tarefa [7237] sendo a ultima baixa feita [7237]-17/07/2026 13:59:31.. - Data Comentário: 17/07/2026 13:58</t>
@@ -74217,7 +74853,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U676" t="inlineStr"/>
+      <c r="U676" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V676" t="inlineStr">
         <is>
           <t>Reaberto via Rotina Configuração Após Baixa de tarefa [7237] sendo a ultima baixa feita [7237]-17/07/2026 13:59:31.. - Data Comentário: 17/07/2026 13:58</t>
@@ -75287,7 +75927,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U686" t="inlineStr"/>
+      <c r="U686" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V686" t="inlineStr"/>
       <c r="W686" t="inlineStr"/>
       <c r="X686" t="inlineStr"/>
@@ -75390,7 +76034,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U687" t="inlineStr"/>
+      <c r="U687" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V687" t="inlineStr"/>
       <c r="W687" t="inlineStr"/>
       <c r="X687" t="inlineStr"/>
@@ -75493,7 +76141,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U688" t="inlineStr"/>
+      <c r="U688" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V688" t="inlineStr"/>
       <c r="W688" t="inlineStr"/>
       <c r="X688" t="inlineStr"/>
@@ -75596,7 +76248,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U689" t="inlineStr"/>
+      <c r="U689" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V689" t="inlineStr"/>
       <c r="W689" t="inlineStr"/>
       <c r="X689" t="inlineStr"/>
@@ -75699,7 +76355,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U690" t="inlineStr"/>
+      <c r="U690" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V690" t="inlineStr"/>
       <c r="W690" t="inlineStr"/>
       <c r="X690" t="inlineStr"/>
@@ -76971,7 +77631,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U702" t="inlineStr"/>
+      <c r="U702" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V702" t="inlineStr"/>
       <c r="W702" t="inlineStr"/>
       <c r="X702" t="inlineStr"/>
@@ -77173,7 +77837,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U704" t="inlineStr"/>
+      <c r="U704" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V704" t="inlineStr"/>
       <c r="W704" t="inlineStr"/>
       <c r="X704" t="inlineStr"/>
@@ -77276,7 +77944,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U705" t="inlineStr"/>
+      <c r="U705" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V705" t="inlineStr"/>
       <c r="W705" t="inlineStr"/>
       <c r="X705" t="inlineStr"/>
@@ -77379,7 +78051,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U706" t="inlineStr"/>
+      <c r="U706" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V706" t="inlineStr"/>
       <c r="W706" t="inlineStr"/>
       <c r="X706" t="inlineStr"/>
@@ -77482,7 +78158,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U707" t="inlineStr"/>
+      <c r="U707" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V707" t="inlineStr"/>
       <c r="W707" t="inlineStr"/>
       <c r="X707" t="inlineStr"/>
@@ -78631,7 +79311,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U718" t="inlineStr"/>
+      <c r="U718" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V718" t="inlineStr"/>
       <c r="W718" t="inlineStr"/>
       <c r="X718" t="inlineStr"/>
@@ -78734,7 +79418,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U719" t="inlineStr"/>
+      <c r="U719" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V719" t="inlineStr"/>
       <c r="W719" t="inlineStr"/>
       <c r="X719" t="inlineStr"/>
@@ -79867,7 +80555,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U729" t="inlineStr"/>
+      <c r="U729" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V729" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 20/07/2026 
@@ -79975,7 +80667,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U730" t="inlineStr"/>
+      <c r="U730" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V730" t="inlineStr"/>
       <c r="W730" t="inlineStr"/>
       <c r="X730" t="inlineStr"/>
@@ -80082,7 +80778,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U731" t="inlineStr"/>
+      <c r="U731" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V731" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 20/07/2026 
@@ -80190,7 +80890,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U732" t="inlineStr"/>
+      <c r="U732" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V732" t="inlineStr"/>
       <c r="W732" t="inlineStr"/>
       <c r="X732" t="inlineStr"/>
@@ -80293,7 +80997,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U733" t="inlineStr"/>
+      <c r="U733" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V733" t="inlineStr"/>
       <c r="W733" t="inlineStr"/>
       <c r="X733" t="inlineStr"/>
@@ -81565,7 +82273,11 @@
           <t>TECNO COM</t>
         </is>
       </c>
-      <c r="U745" t="inlineStr"/>
+      <c r="U745" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V745" t="inlineStr"/>
       <c r="W745" t="inlineStr"/>
       <c r="X745" t="inlineStr"/>
@@ -81767,7 +82479,11 @@
           <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
-      <c r="U747" t="inlineStr"/>
+      <c r="U747" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V747" t="inlineStr"/>
       <c r="W747" t="inlineStr"/>
       <c r="X747" t="inlineStr"/>
@@ -81870,7 +82586,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U748" t="inlineStr"/>
+      <c r="U748" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V748" t="inlineStr"/>
       <c r="W748" t="inlineStr"/>
       <c r="X748" t="inlineStr"/>
@@ -81973,7 +82693,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U749" t="inlineStr"/>
+      <c r="U749" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V749" t="inlineStr"/>
       <c r="W749" t="inlineStr"/>
       <c r="X749" t="inlineStr"/>
@@ -82076,7 +82800,11 @@
           <t>PROMOTORAS GYN</t>
         </is>
       </c>
-      <c r="U750" t="inlineStr"/>
+      <c r="U750" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V750" t="inlineStr"/>
       <c r="W750" t="inlineStr"/>
       <c r="X750" t="inlineStr"/>
@@ -83586,7 +84314,11 @@
           <t>TEC GRUA</t>
         </is>
       </c>
-      <c r="U764" t="inlineStr"/>
+      <c r="U764" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
       <c r="V764" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 22/07/2026 
@@ -83712,12 +84444,12 @@
       <c r="AC765" t="inlineStr"/>
       <c r="AD765" t="inlineStr">
         <is>
-          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09. - Data Comentário: 20/07/2026 08:57</t>
+          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09. - Data Comentário: 27/07/2026 16:25</t>
         </is>
       </c>
       <c r="AE765" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="AF765" t="inlineStr">
@@ -83824,12 +84556,12 @@
       <c r="AC766" t="inlineStr"/>
       <c r="AD766" t="inlineStr">
         <is>
-          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09. - Data Comentário: 20/07/2026 08:57</t>
+          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09. - Data Comentário: 27/07/2026 16:25</t>
         </is>
       </c>
       <c r="AE766" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="AF766" t="inlineStr">
@@ -83940,12 +84672,12 @@
       <c r="AC767" t="inlineStr"/>
       <c r="AD767" t="inlineStr">
         <is>
-          <t>A gerente Priscila Volpe, a GC Beatriz e o Afonso estão trabalhando em maneiras para ajustar os valores de saldo credor de meses anteriores, por conta de conflito no sys analise. - Data Comentário: 20/07/2026 08:57</t>
+          <t>A gerente Priscila Volpe, a GC Beatriz e o Afonso estão trabalhando em maneiras para ajustar os valores de saldo credor de meses anteriores, por conta de conflito no sys analise. - Data Comentário: 27/07/2026 16:25</t>
         </is>
       </c>
       <c r="AE767" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>27/07/2026</t>
         </is>
       </c>
       <c r="AF767" t="inlineStr">
@@ -84240,7 +84972,7 @@
       </c>
       <c r="M770" t="inlineStr">
         <is>
-          <t>17/07/2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
       <c r="N770" t="inlineStr">
@@ -84277,8 +85009,8 @@
       </c>
       <c r="V770" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 17/07/2026 
-implantação não foi marcada ainda. - Data Comentário: 10/07/2026 17:02</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 07/08/2026 
+As reuniões de implantação estão agendadas para agosto - Data Comentário: 27/07/2026 16:43</t>
         </is>
       </c>
       <c r="W770" t="inlineStr"/>
@@ -84356,7 +85088,7 @@
       </c>
       <c r="M771" t="inlineStr">
         <is>
-          <t>17/07/2026</t>
+          <t>07/08/2026</t>
         </is>
       </c>
       <c r="N771" t="inlineStr">
@@ -84393,8 +85125,8 @@
       </c>
       <c r="V771" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 17/07/2026 
-implantação não foi marcada ainda. - Data Comentário: 10/07/2026 17:02</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 07/08/2026 
+As reuniões de implantação estão agendadas para agosto - Data Comentário: 27/07/2026 16:43</t>
         </is>
       </c>
       <c r="W771" t="inlineStr"/>
@@ -84634,12 +85366,12 @@
       <c r="AC773" t="inlineStr"/>
       <c r="AD773" t="inlineStr">
         <is>
-          <t>Aguardando agendamento da implantação   - Data Comentário: 20/07/2026 08:58</t>
+          <t>Aguardando agendamento da implantação do cliente. - Data Comentário: 27/07/2026 16:26</t>
         </is>
       </c>
       <c r="AE773" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>27/07/2026</t>
         </is>
       </c>
       <c r="AF773" t="inlineStr">
@@ -84754,12 +85486,12 @@
       <c r="AC774" t="inlineStr"/>
       <c r="AD774" t="inlineStr">
         <is>
-          <t>Aguardando agendamento da implantação   - Data Comentário: 20/07/2026 08:58</t>
+          <t>Aguardando agendamento da implantação do cliente. - Data Comentário: 27/07/2026 16:26</t>
         </is>
       </c>
       <c r="AE774" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>27/07/2026</t>
         </is>
       </c>
       <c r="AF774" t="inlineStr">
@@ -84869,12 +85601,12 @@
       <c r="AC775" t="inlineStr"/>
       <c r="AD775" t="inlineStr">
         <is>
-          <t>Aguardando agendamento da implantação   - Data Comentário: 20/07/2026 08:58</t>
+          <t>Aguardando agendamento da implantação do cliente. - Data Comentário: 27/07/2026 16:26</t>
         </is>
       </c>
       <c r="AE775" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>27/07/2026</t>
         </is>
       </c>
       <c r="AF775" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-28 09:51
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -44423,11 +44423,11 @@
     </row>
     <row r="403">
       <c r="A403" t="n">
-        <v>6628</v>
+        <v>6962</v>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
+          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
@@ -44437,17 +44437,17 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G403" t="n">
@@ -44472,7 +44472,7 @@
       </c>
       <c r="M403" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="N403" t="inlineStr">
@@ -44481,11 +44481,11 @@
         </is>
       </c>
       <c r="O403" t="n">
-        <v>16960022</v>
+        <v>18187953</v>
       </c>
       <c r="P403" t="inlineStr">
         <is>
-          <t>Nathalia Lourenco</t>
+          <t>Mirian Lima</t>
         </is>
       </c>
       <c r="Q403" t="inlineStr">
@@ -44499,17 +44499,18 @@
       </c>
       <c r="T403" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>PROMOTORAS GYN</t>
         </is>
       </c>
       <c r="U403" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="V403" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 - Data Comentário: 28/07/2026 07:36</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 
+Aguardando apurações PIS/COFINS/IRPJ/CSLL - Data Comentário: 21/07/2026 10:05</t>
         </is>
       </c>
       <c r="W403" t="inlineStr"/>
@@ -44536,11 +44537,11 @@
     </row>
     <row r="404">
       <c r="A404" t="n">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
+          <t>PROMOTORAS GYN LTDA</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -44594,7 +44595,7 @@
         </is>
       </c>
       <c r="O404" t="n">
-        <v>18187953</v>
+        <v>18187891</v>
       </c>
       <c r="P404" t="inlineStr">
         <is>
@@ -44650,11 +44651,11 @@
     </row>
     <row r="405">
       <c r="A405" t="n">
-        <v>6963</v>
+        <v>6548</v>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN LTDA</t>
+          <t>GOIAS SILAGEM LTDA</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
@@ -44674,11 +44675,11 @@
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G405" t="n">
-        <v>6892</v>
+        <v>1651</v>
       </c>
       <c r="H405" t="n">
         <v>0</v>
@@ -44690,29 +44691,25 @@
       </c>
       <c r="J405" t="inlineStr">
         <is>
-          <t>Fed - DCTFWEB</t>
+          <t>Fed - IRPJ/CSLL</t>
         </is>
       </c>
       <c r="K405" t="inlineStr"/>
       <c r="L405" s="1" t="n">
-        <v>46233</v>
-      </c>
-      <c r="M405" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
+        <v>46232</v>
+      </c>
+      <c r="M405" t="inlineStr"/>
       <c r="N405" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O405" t="n">
-        <v>18187891</v>
+        <v>17967985</v>
       </c>
       <c r="P405" t="inlineStr">
         <is>
-          <t>Mirian Lima</t>
+          <t>Thais Souza</t>
         </is>
       </c>
       <c r="Q405" t="inlineStr">
@@ -44722,24 +44719,19 @@
       </c>
       <c r="R405" t="inlineStr"/>
       <c r="S405" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="T405" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN</t>
+          <t>GOIAS SILAGEM</t>
         </is>
       </c>
       <c r="U405" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="V405" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 
-Aguardando apurações PIS/COFINS/IRPJ/CSLL - Data Comentário: 21/07/2026 10:05</t>
-        </is>
-      </c>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V405" t="inlineStr"/>
       <c r="W405" t="inlineStr"/>
       <c r="X405" t="inlineStr"/>
       <c r="Y405" t="inlineStr"/>
@@ -44753,22 +44745,22 @@
       <c r="AE405" t="inlineStr"/>
       <c r="AF405" t="inlineStr">
         <is>
-          <t>Obrigação Acessória</t>
+          <t>Imposto</t>
         </is>
       </c>
       <c r="AG405" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Erika Santana</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="n">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -44783,7 +44775,7 @@
       </c>
       <c r="E406" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
@@ -44818,11 +44810,11 @@
         </is>
       </c>
       <c r="O406" t="n">
-        <v>17967985</v>
+        <v>17042385</v>
       </c>
       <c r="P406" t="inlineStr">
         <is>
-          <t>Thais Souza</t>
+          <t>Nathalia Lourenco</t>
         </is>
       </c>
       <c r="Q406" t="inlineStr">
@@ -44836,7 +44828,7 @@
       </c>
       <c r="T406" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U406" t="inlineStr">
@@ -44863,17 +44855,17 @@
       </c>
       <c r="AG406" t="inlineStr">
         <is>
-          <t>Erika Santana</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="n">
-        <v>6627</v>
+        <v>6962</v>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -44888,12 +44880,12 @@
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G407" t="n">
@@ -44923,11 +44915,11 @@
         </is>
       </c>
       <c r="O407" t="n">
-        <v>17042385</v>
+        <v>18187935</v>
       </c>
       <c r="P407" t="inlineStr">
         <is>
-          <t>Nathalia Lourenco</t>
+          <t>Mirian Lima</t>
         </is>
       </c>
       <c r="Q407" t="inlineStr">
@@ -44941,12 +44933,12 @@
       </c>
       <c r="T407" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>PROMOTORAS GYN</t>
         </is>
       </c>
       <c r="U407" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="V407" t="inlineStr"/>
@@ -44974,11 +44966,11 @@
     </row>
     <row r="408">
       <c r="A408" t="n">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
+          <t>PROMOTORAS GYN LTDA</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -45028,7 +45020,7 @@
         </is>
       </c>
       <c r="O408" t="n">
-        <v>18187935</v>
+        <v>18187873</v>
       </c>
       <c r="P408" t="inlineStr">
         <is>
@@ -45079,11 +45071,11 @@
     </row>
     <row r="409">
       <c r="A409" t="n">
-        <v>6963</v>
+        <v>6548</v>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN LTDA</t>
+          <t>GOIAS SILAGEM LTDA</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -45103,11 +45095,11 @@
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G409" t="n">
-        <v>1651</v>
+        <v>11516</v>
       </c>
       <c r="H409" t="n">
         <v>0</v>
@@ -45119,25 +45111,29 @@
       </c>
       <c r="J409" t="inlineStr">
         <is>
-          <t>Fed - IRPJ/CSLL</t>
+          <t>Módulo de Inclusão Tributária (MIT)</t>
         </is>
       </c>
       <c r="K409" t="inlineStr"/>
       <c r="L409" s="1" t="n">
-        <v>46232</v>
-      </c>
-      <c r="M409" t="inlineStr"/>
+        <v>46233</v>
+      </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>23/07/2026</t>
+        </is>
+      </c>
       <c r="N409" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O409" t="n">
-        <v>18187873</v>
+        <v>17968051</v>
       </c>
       <c r="P409" t="inlineStr">
         <is>
-          <t>Mirian Lima</t>
+          <t>Thais Souza</t>
         </is>
       </c>
       <c r="Q409" t="inlineStr">
@@ -45147,19 +45143,23 @@
       </c>
       <c r="R409" t="inlineStr"/>
       <c r="S409" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="T409" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN</t>
+          <t>GOIAS SILAGEM</t>
         </is>
       </c>
       <c r="U409" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="V409" t="inlineStr"/>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V409" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 20/07/2026 15:31</t>
+        </is>
+      </c>
       <c r="W409" t="inlineStr"/>
       <c r="X409" t="inlineStr"/>
       <c r="Y409" t="inlineStr"/>
@@ -45173,22 +45173,22 @@
       <c r="AE409" t="inlineStr"/>
       <c r="AF409" t="inlineStr">
         <is>
-          <t>Imposto</t>
+          <t>Obrigação Acessória</t>
         </is>
       </c>
       <c r="AG409" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Erika Santana</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="n">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -45203,7 +45203,7 @@
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
@@ -45233,7 +45233,7 @@
       </c>
       <c r="M410" t="inlineStr">
         <is>
-          <t>23/07/2026</t>
+          <t>24/07/2026</t>
         </is>
       </c>
       <c r="N410" t="inlineStr">
@@ -45242,11 +45242,11 @@
         </is>
       </c>
       <c r="O410" t="n">
-        <v>17968051</v>
+        <v>17042660</v>
       </c>
       <c r="P410" t="inlineStr">
         <is>
-          <t>Thais Souza</t>
+          <t>Nathalia Lourenco</t>
         </is>
       </c>
       <c r="Q410" t="inlineStr">
@@ -45260,7 +45260,7 @@
       </c>
       <c r="T410" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U410" t="inlineStr">
@@ -45270,7 +45270,7 @@
       </c>
       <c r="V410" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 20/07/2026 15:31</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 24/07/2026 - Data Comentário: 20/07/2026 15:12</t>
         </is>
       </c>
       <c r="W410" t="inlineStr"/>
@@ -45291,17 +45291,17 @@
       </c>
       <c r="AG410" t="inlineStr">
         <is>
-          <t>Erika Santana</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="n">
-        <v>6627</v>
+        <v>6962</v>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
@@ -45316,12 +45316,12 @@
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G411" t="n">
@@ -45346,7 +45346,7 @@
       </c>
       <c r="M411" t="inlineStr">
         <is>
-          <t>24/07/2026</t>
+          <t>29/07/2026</t>
         </is>
       </c>
       <c r="N411" t="inlineStr">
@@ -45355,11 +45355,11 @@
         </is>
       </c>
       <c r="O411" t="n">
-        <v>17042660</v>
+        <v>18187983</v>
       </c>
       <c r="P411" t="inlineStr">
         <is>
-          <t>Nathalia Lourenco</t>
+          <t>Mirian Lima</t>
         </is>
       </c>
       <c r="Q411" t="inlineStr">
@@ -45373,17 +45373,18 @@
       </c>
       <c r="T411" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>PROMOTORAS GYN</t>
         </is>
       </c>
       <c r="U411" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="V411" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 24/07/2026 - Data Comentário: 20/07/2026 15:12</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
+Aguardando apuração do PIS/COFINS/IRPJ e CSLL - Data Comentário: 20/07/2026 16:15</t>
         </is>
       </c>
       <c r="W411" t="inlineStr"/>
@@ -45410,11 +45411,11 @@
     </row>
     <row r="412">
       <c r="A412" t="n">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
+          <t>PROMOTORAS GYN LTDA</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -45468,7 +45469,7 @@
         </is>
       </c>
       <c r="O412" t="n">
-        <v>18187983</v>
+        <v>18187921</v>
       </c>
       <c r="P412" t="inlineStr">
         <is>
@@ -45524,11 +45525,11 @@
     </row>
     <row r="413">
       <c r="A413" t="n">
-        <v>6963</v>
+        <v>5417</v>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -45548,45 +45549,41 @@
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G413" t="n">
-        <v>11516</v>
+        <v>6890</v>
       </c>
       <c r="H413" t="n">
         <v>0</v>
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J413" t="inlineStr">
         <is>
-          <t>Módulo de Inclusão Tributária (MIT)</t>
+          <t>Fed - DCTFWEB</t>
         </is>
       </c>
       <c r="K413" t="inlineStr"/>
       <c r="L413" s="1" t="n">
         <v>46233</v>
       </c>
-      <c r="M413" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
+      <c r="M413" t="inlineStr"/>
       <c r="N413" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O413" t="n">
-        <v>18187921</v>
+        <v>17399258</v>
       </c>
       <c r="P413" t="inlineStr">
         <is>
-          <t>Mirian Lima</t>
+          <t>Eveny Silva</t>
         </is>
       </c>
       <c r="Q413" t="inlineStr">
@@ -45600,18 +45597,17 @@
       </c>
       <c r="T413" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U413" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="V413" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
-Aguardando apuração do PIS/COFINS/IRPJ e CSLL - Data Comentário: 20/07/2026 16:15</t>
+          <t>Aguardando a Liberação da Gerência de Contas - Data Comentário: 20/07/2026 14:21</t>
         </is>
       </c>
       <c r="W413" t="inlineStr"/>
@@ -45632,17 +45628,17 @@
       </c>
       <c r="AG413" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="n">
-        <v>5417</v>
+        <v>5617</v>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -45662,7 +45658,7 @@
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G414" t="n">
@@ -45685,18 +45681,22 @@
       <c r="L414" s="1" t="n">
         <v>46233</v>
       </c>
-      <c r="M414" t="inlineStr"/>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
       <c r="N414" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O414" t="n">
-        <v>17399258</v>
+        <v>17407809</v>
       </c>
       <c r="P414" t="inlineStr">
         <is>
-          <t>Eveny Silva</t>
+          <t>Jackson Silva</t>
         </is>
       </c>
       <c r="Q414" t="inlineStr">
@@ -45710,7 +45710,7 @@
       </c>
       <c r="T414" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U414" t="inlineStr">
@@ -45720,7 +45720,7 @@
       </c>
       <c r="V414" t="inlineStr">
         <is>
-          <t>Aguardando a Liberação da Gerência de Contas - Data Comentário: 20/07/2026 14:21</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 22/07/2026 15:47</t>
         </is>
       </c>
       <c r="W414" t="inlineStr"/>
@@ -45741,17 +45741,17 @@
       </c>
       <c r="AG414" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Edileide Dias</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="n">
-        <v>5617</v>
+        <v>6224</v>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
@@ -45771,7 +45771,7 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G415" t="n">
@@ -45805,7 +45805,7 @@
         </is>
       </c>
       <c r="O415" t="n">
-        <v>17407809</v>
+        <v>17688937</v>
       </c>
       <c r="P415" t="inlineStr">
         <is>
@@ -45860,11 +45860,11 @@
     </row>
     <row r="416">
       <c r="A416" t="n">
-        <v>6224</v>
+        <v>6278</v>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
@@ -45874,7 +45874,7 @@
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Real - Anual</t>
         </is>
       </c>
       <c r="E416" t="inlineStr">
@@ -45884,7 +45884,7 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G416" t="n">
@@ -45907,22 +45907,18 @@
       <c r="L416" s="1" t="n">
         <v>46233</v>
       </c>
-      <c r="M416" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
+      <c r="M416" t="inlineStr"/>
       <c r="N416" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O416" t="n">
-        <v>17688937</v>
+        <v>17539766</v>
       </c>
       <c r="P416" t="inlineStr">
         <is>
-          <t>Jackson Silva</t>
+          <t>Isabela Lemos</t>
         </is>
       </c>
       <c r="Q416" t="inlineStr">
@@ -45936,7 +45932,7 @@
       </c>
       <c r="T416" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U416" t="inlineStr">
@@ -45944,11 +45940,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V416" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 22/07/2026 15:47</t>
-        </is>
-      </c>
+      <c r="V416" t="inlineStr"/>
       <c r="W416" t="inlineStr"/>
       <c r="X416" t="inlineStr"/>
       <c r="Y416" t="inlineStr"/>
@@ -45967,17 +45959,17 @@
       </c>
       <c r="AG416" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="n">
-        <v>6278</v>
+        <v>6279</v>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>DIENNYFER DA S PEREIRA</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -45987,7 +45979,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>Federal - Lucro Real - Anual</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E417" t="inlineStr">
@@ -45997,7 +45989,7 @@
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G417" t="n">
@@ -46027,7 +46019,7 @@
         </is>
       </c>
       <c r="O417" t="n">
-        <v>17539766</v>
+        <v>17646082</v>
       </c>
       <c r="P417" t="inlineStr">
         <is>
@@ -46078,11 +46070,11 @@
     </row>
     <row r="418">
       <c r="A418" t="n">
-        <v>6279</v>
+        <v>6404</v>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>DIENNYFER DA S PEREIRA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -46102,7 +46094,7 @@
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G418" t="n">
@@ -46125,14 +46117,18 @@
       <c r="L418" s="1" t="n">
         <v>46233</v>
       </c>
-      <c r="M418" t="inlineStr"/>
+      <c r="M418" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
       <c r="N418" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O418" t="n">
-        <v>17646082</v>
+        <v>16962326</v>
       </c>
       <c r="P418" t="inlineStr">
         <is>
@@ -46150,7 +46146,7 @@
       </c>
       <c r="T418" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>SOLAR INVESTIMENTOS</t>
         </is>
       </c>
       <c r="U418" t="inlineStr">
@@ -46158,7 +46154,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V418" t="inlineStr"/>
+      <c r="V418" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 - Data Comentário: 27/07/2026 16:50</t>
+        </is>
+      </c>
       <c r="W418" t="inlineStr"/>
       <c r="X418" t="inlineStr"/>
       <c r="Y418" t="inlineStr"/>
@@ -46183,11 +46183,11 @@
     </row>
     <row r="419">
       <c r="A419" t="n">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -46197,7 +46197,7 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E419" t="inlineStr">
@@ -46230,22 +46230,18 @@
       <c r="L419" s="1" t="n">
         <v>46233</v>
       </c>
-      <c r="M419" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
+      <c r="M419" t="inlineStr"/>
       <c r="N419" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O419" t="n">
-        <v>16962326</v>
+        <v>18152536</v>
       </c>
       <c r="P419" t="inlineStr">
         <is>
-          <t>Isabela Lemos</t>
+          <t>Nathany Barreto</t>
         </is>
       </c>
       <c r="Q419" t="inlineStr">
@@ -46259,7 +46255,7 @@
       </c>
       <c r="T419" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U419" t="inlineStr">
@@ -46269,7 +46265,7 @@
       </c>
       <c r="V419" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 - Data Comentário: 27/07/2026 16:50</t>
+          <t>Aguardando a Liberação da Gerência de Contas - Data Comentário: 20/07/2026 17:55</t>
         </is>
       </c>
       <c r="W419" t="inlineStr"/>
@@ -46290,17 +46286,17 @@
       </c>
       <c r="AG419" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="n">
-        <v>6486</v>
+        <v>6703</v>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>PC GAMER GOIANIA LTDA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -46310,7 +46306,7 @@
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E420" t="inlineStr">
@@ -46350,7 +46346,7 @@
         </is>
       </c>
       <c r="O420" t="n">
-        <v>18152536</v>
+        <v>17955184</v>
       </c>
       <c r="P420" t="inlineStr">
         <is>
@@ -46368,7 +46364,7 @@
       </c>
       <c r="T420" t="inlineStr">
         <is>
-          <t>PC GAMER</t>
+          <t>LIMA MOTA</t>
         </is>
       </c>
       <c r="U420" t="inlineStr">
@@ -46405,11 +46401,11 @@
     </row>
     <row r="421">
       <c r="A421" t="n">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -46419,7 +46415,7 @@
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E421" t="inlineStr">
@@ -46452,18 +46448,22 @@
       <c r="L421" s="1" t="n">
         <v>46233</v>
       </c>
-      <c r="M421" t="inlineStr"/>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
       <c r="N421" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O421" t="n">
-        <v>17955184</v>
+        <v>17955397</v>
       </c>
       <c r="P421" t="inlineStr">
         <is>
-          <t>Nathany Barreto</t>
+          <t>Paulo Silva</t>
         </is>
       </c>
       <c r="Q421" t="inlineStr">
@@ -46477,7 +46477,7 @@
       </c>
       <c r="T421" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U421" t="inlineStr">
@@ -46487,7 +46487,7 @@
       </c>
       <c r="V421" t="inlineStr">
         <is>
-          <t>Aguardando a Liberação da Gerência de Contas - Data Comentário: 20/07/2026 17:55</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 - Data Comentário: 28/07/2026 08:27</t>
         </is>
       </c>
       <c r="W421" t="inlineStr"/>
@@ -46508,17 +46508,17 @@
       </c>
       <c r="AG421" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="n">
-        <v>6704</v>
+        <v>6885</v>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -46528,7 +46528,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E422" t="inlineStr">
@@ -46563,7 +46563,7 @@
       </c>
       <c r="M422" t="inlineStr">
         <is>
-          <t>30/07/2026</t>
+          <t>23/07/2026</t>
         </is>
       </c>
       <c r="N422" t="inlineStr">
@@ -46572,11 +46572,11 @@
         </is>
       </c>
       <c r="O422" t="n">
-        <v>17955397</v>
+        <v>18128808</v>
       </c>
       <c r="P422" t="inlineStr">
         <is>
-          <t>Paulo Silva</t>
+          <t>Isabela Lemos</t>
         </is>
       </c>
       <c r="Q422" t="inlineStr">
@@ -46590,17 +46590,13 @@
       </c>
       <c r="T422" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
-        </is>
-      </c>
-      <c r="U422" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+          <t>EMPORIO DOS FRIOS</t>
+        </is>
+      </c>
+      <c r="U422" t="inlineStr"/>
       <c r="V422" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 - Data Comentário: 28/07/2026 08:27</t>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 23/07/2026 - Data Comentário: 22/07/2026 19:56</t>
         </is>
       </c>
       <c r="W422" t="inlineStr"/>
@@ -46627,11 +46623,11 @@
     </row>
     <row r="423">
       <c r="A423" t="n">
-        <v>6885</v>
+        <v>5417</v>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t xml:space="preserve">EMPORIO MENDANHA LTDA </t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -46641,7 +46637,7 @@
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E423" t="inlineStr">
@@ -46651,11 +46647,11 @@
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G423" t="n">
-        <v>6890</v>
+        <v>1582</v>
       </c>
       <c r="H423" t="n">
         <v>0</v>
@@ -46667,16 +46663,16 @@
       </c>
       <c r="J423" t="inlineStr">
         <is>
-          <t>Fed - DCTFWEB</t>
+          <t>Fed - IRPJ/CSLL</t>
         </is>
       </c>
       <c r="K423" t="inlineStr"/>
       <c r="L423" s="1" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="M423" t="inlineStr">
         <is>
-          <t>23/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="N423" t="inlineStr">
@@ -46685,11 +46681,11 @@
         </is>
       </c>
       <c r="O423" t="n">
-        <v>18128808</v>
+        <v>17398913</v>
       </c>
       <c r="P423" t="inlineStr">
         <is>
-          <t>Isabela Lemos</t>
+          <t>Eveny Silva</t>
         </is>
       </c>
       <c r="Q423" t="inlineStr">
@@ -46699,17 +46695,22 @@
       </c>
       <c r="R423" t="inlineStr"/>
       <c r="S423" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="T423" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
-        </is>
-      </c>
-      <c r="U423" t="inlineStr"/>
+          <t>NOSSO NOVO SUPERMERCADO</t>
+        </is>
+      </c>
+      <c r="U423" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="V423" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 23/07/2026 - Data Comentário: 22/07/2026 19:56</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 
+aguardando liberação - Data Comentário: 28/07/2026 09:32</t>
         </is>
       </c>
       <c r="W423" t="inlineStr"/>
@@ -46725,22 +46726,22 @@
       <c r="AE423" t="inlineStr"/>
       <c r="AF423" t="inlineStr">
         <is>
-          <t>Obrigação Acessória</t>
+          <t>Imposto</t>
         </is>
       </c>
       <c r="AG423" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="n">
-        <v>5417</v>
+        <v>5617</v>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -46760,7 +46761,7 @@
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G424" t="n">
@@ -46783,18 +46784,22 @@
       <c r="L424" s="1" t="n">
         <v>46232</v>
       </c>
-      <c r="M424" t="inlineStr"/>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
       <c r="N424" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O424" t="n">
-        <v>17398913</v>
+        <v>17407549</v>
       </c>
       <c r="P424" t="inlineStr">
         <is>
-          <t>Eveny Silva</t>
+          <t>Jackson Silva</t>
         </is>
       </c>
       <c r="Q424" t="inlineStr">
@@ -46808,7 +46813,7 @@
       </c>
       <c r="T424" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U424" t="inlineStr">
@@ -46818,8 +46823,8 @@
       </c>
       <c r="V424" t="inlineStr">
         <is>
-          <t>Aguardando a Liberação da Gerência de Contas  
-Aguardando liberação da Lucratividade - Data Comentário: 21/07/2026 11:31</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 
+aguardando liberação - Data Comentário: 28/07/2026 09:32</t>
         </is>
       </c>
       <c r="W424" t="inlineStr"/>
@@ -46840,17 +46845,17 @@
       </c>
       <c r="AG424" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Edileide Dias</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="n">
-        <v>5617</v>
+        <v>6224</v>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -46870,7 +46875,7 @@
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G425" t="n">
@@ -46893,14 +46898,18 @@
       <c r="L425" s="1" t="n">
         <v>46232</v>
       </c>
-      <c r="M425" t="inlineStr"/>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
       <c r="N425" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O425" t="n">
-        <v>17407549</v>
+        <v>17688641</v>
       </c>
       <c r="P425" t="inlineStr">
         <is>
@@ -46926,7 +46935,12 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V425" t="inlineStr"/>
+      <c r="V425" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 
+aguardando liberação - Data Comentário: 28/07/2026 09:32</t>
+        </is>
+      </c>
       <c r="W425" t="inlineStr"/>
       <c r="X425" t="inlineStr"/>
       <c r="Y425" t="inlineStr"/>
@@ -46951,11 +46965,11 @@
     </row>
     <row r="426">
       <c r="A426" t="n">
-        <v>6224</v>
+        <v>6278</v>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -46965,7 +46979,7 @@
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Real - Anual</t>
         </is>
       </c>
       <c r="E426" t="inlineStr">
@@ -46975,7 +46989,7 @@
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G426" t="n">
@@ -46998,18 +47012,22 @@
       <c r="L426" s="1" t="n">
         <v>46232</v>
       </c>
-      <c r="M426" t="inlineStr"/>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
       <c r="N426" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O426" t="n">
-        <v>17688641</v>
+        <v>18166309</v>
       </c>
       <c r="P426" t="inlineStr">
         <is>
-          <t>Jackson Silva</t>
+          <t>Isabela Lemos</t>
         </is>
       </c>
       <c r="Q426" t="inlineStr">
@@ -47023,7 +47041,7 @@
       </c>
       <c r="T426" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U426" t="inlineStr">
@@ -47031,7 +47049,12 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V426" t="inlineStr"/>
+      <c r="V426" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 
+aguardando liberação - Data Comentário: 28/07/2026 09:32</t>
+        </is>
+      </c>
       <c r="W426" t="inlineStr"/>
       <c r="X426" t="inlineStr"/>
       <c r="Y426" t="inlineStr"/>
@@ -47050,17 +47073,17 @@
       </c>
       <c r="AG426" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="n">
-        <v>6278</v>
+        <v>6486</v>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
@@ -47070,7 +47093,7 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Federal - Lucro Real - Anual</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E427" t="inlineStr">
@@ -47103,18 +47126,22 @@
       <c r="L427" s="1" t="n">
         <v>46232</v>
       </c>
-      <c r="M427" t="inlineStr"/>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
       <c r="N427" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O427" t="n">
-        <v>18166309</v>
+        <v>18114205</v>
       </c>
       <c r="P427" t="inlineStr">
         <is>
-          <t>Isabela Lemos</t>
+          <t>Nathany Barreto</t>
         </is>
       </c>
       <c r="Q427" t="inlineStr">
@@ -47128,7 +47155,7 @@
       </c>
       <c r="T427" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U427" t="inlineStr">
@@ -47138,7 +47165,8 @@
       </c>
       <c r="V427" t="inlineStr">
         <is>
-          <t>Aguardando a Liberação da Gerência de Contas - Data Comentário: 22/07/2026 19:09</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 
+aguardando liberação - Data Comentário: 28/07/2026 09:32</t>
         </is>
       </c>
       <c r="W427" t="inlineStr"/>
@@ -47159,17 +47187,17 @@
       </c>
       <c r="AG427" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="n">
-        <v>6486</v>
+        <v>6704</v>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>PC GAMER GOIANIA LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
@@ -47212,18 +47240,22 @@
       <c r="L428" s="1" t="n">
         <v>46232</v>
       </c>
-      <c r="M428" t="inlineStr"/>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
       <c r="N428" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O428" t="n">
-        <v>18114205</v>
+        <v>17955369</v>
       </c>
       <c r="P428" t="inlineStr">
         <is>
-          <t>Nathany Barreto</t>
+          <t>Paulo Silva</t>
         </is>
       </c>
       <c r="Q428" t="inlineStr">
@@ -47237,7 +47269,7 @@
       </c>
       <c r="T428" t="inlineStr">
         <is>
-          <t>PC GAMER</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U428" t="inlineStr">
@@ -47247,8 +47279,8 @@
       </c>
       <c r="V428" t="inlineStr">
         <is>
-          <t>Aguardando a Liberação da Gerência de Contas  
-Aguardando liberação da Lucratividade - Data Comentário: 21/07/2026 11:31</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 
+aguardando liberação - Data Comentário: 28/07/2026 09:32</t>
         </is>
       </c>
       <c r="W428" t="inlineStr"/>
@@ -47269,17 +47301,17 @@
       </c>
       <c r="AG428" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="n">
-        <v>6704</v>
+        <v>5417</v>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -47299,11 +47331,11 @@
       </c>
       <c r="F429" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G429" t="n">
-        <v>1582</v>
+        <v>11514</v>
       </c>
       <c r="H429" t="n">
         <v>0</v>
@@ -47315,25 +47347,29 @@
       </c>
       <c r="J429" t="inlineStr">
         <is>
-          <t>Fed - IRPJ/CSLL</t>
+          <t>Módulo de Inclusão Tributária (MIT)</t>
         </is>
       </c>
       <c r="K429" t="inlineStr"/>
       <c r="L429" s="1" t="n">
-        <v>46232</v>
-      </c>
-      <c r="M429" t="inlineStr"/>
+        <v>46233</v>
+      </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t>29/07/2026</t>
+        </is>
+      </c>
       <c r="N429" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O429" t="n">
-        <v>17955369</v>
+        <v>17399463</v>
       </c>
       <c r="P429" t="inlineStr">
         <is>
-          <t>Paulo Silva</t>
+          <t>Eveny Silva</t>
         </is>
       </c>
       <c r="Q429" t="inlineStr">
@@ -47343,11 +47379,11 @@
       </c>
       <c r="R429" t="inlineStr"/>
       <c r="S429" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="T429" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U429" t="inlineStr">
@@ -47357,8 +47393,8 @@
       </c>
       <c r="V429" t="inlineStr">
         <is>
-          <t>Aguardando a Liberação da Gerência de Contas  
-Precisão conclusão 30/07/2026 - Data Comentário: 22/07/2026 13:15</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
+Aguardando liberação do PIS/COFINS/IRPJ E CSLL - Data Comentário: 21/07/2026 11:36</t>
         </is>
       </c>
       <c r="W429" t="inlineStr"/>
@@ -47374,22 +47410,22 @@
       <c r="AE429" t="inlineStr"/>
       <c r="AF429" t="inlineStr">
         <is>
-          <t>Imposto</t>
+          <t>Obrigação Acessória</t>
         </is>
       </c>
       <c r="AG429" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="n">
-        <v>5417</v>
+        <v>5617</v>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
@@ -47409,7 +47445,7 @@
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G430" t="n">
@@ -47443,11 +47479,11 @@
         </is>
       </c>
       <c r="O430" t="n">
-        <v>17399463</v>
+        <v>17407974</v>
       </c>
       <c r="P430" t="inlineStr">
         <is>
-          <t>Eveny Silva</t>
+          <t>Jackson Silva</t>
         </is>
       </c>
       <c r="Q430" t="inlineStr">
@@ -47461,7 +47497,7 @@
       </c>
       <c r="T430" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U430" t="inlineStr">
@@ -47471,8 +47507,7 @@
       </c>
       <c r="V430" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
-Aguardando liberação do PIS/COFINS/IRPJ E CSLL - Data Comentário: 21/07/2026 11:36</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 22/07/2026 15:47</t>
         </is>
       </c>
       <c r="W430" t="inlineStr"/>
@@ -47493,17 +47528,17 @@
       </c>
       <c r="AG430" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Edileide Dias</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="n">
-        <v>5617</v>
+        <v>6224</v>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
@@ -47523,7 +47558,7 @@
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G431" t="n">
@@ -47557,7 +47592,7 @@
         </is>
       </c>
       <c r="O431" t="n">
-        <v>17407974</v>
+        <v>17689071</v>
       </c>
       <c r="P431" t="inlineStr">
         <is>
@@ -47612,11 +47647,11 @@
     </row>
     <row r="432">
       <c r="A432" t="n">
-        <v>6224</v>
+        <v>6278</v>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>EMPORIO DOS FRIOS LTDA</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
@@ -47626,7 +47661,7 @@
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Real - Anual</t>
         </is>
       </c>
       <c r="E432" t="inlineStr">
@@ -47636,7 +47671,7 @@
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G432" t="n">
@@ -47661,7 +47696,7 @@
       </c>
       <c r="M432" t="inlineStr">
         <is>
-          <t>29/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="N432" t="inlineStr">
@@ -47670,11 +47705,11 @@
         </is>
       </c>
       <c r="O432" t="n">
-        <v>17689071</v>
+        <v>17539898</v>
       </c>
       <c r="P432" t="inlineStr">
         <is>
-          <t>Jackson Silva</t>
+          <t>Isabela Lemos</t>
         </is>
       </c>
       <c r="Q432" t="inlineStr">
@@ -47688,7 +47723,7 @@
       </c>
       <c r="T432" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U432" t="inlineStr">
@@ -47698,7 +47733,7 @@
       </c>
       <c r="V432" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 22/07/2026 15:47</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 - Data Comentário: 22/07/2026 20:00</t>
         </is>
       </c>
       <c r="W432" t="inlineStr"/>
@@ -47719,17 +47754,17 @@
       </c>
       <c r="AG432" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="n">
-        <v>6278</v>
+        <v>6279</v>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS LTDA</t>
+          <t>DIENNYFER DA S PEREIRA</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
@@ -47739,7 +47774,7 @@
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>Federal - Lucro Real - Anual</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E433" t="inlineStr">
@@ -47749,7 +47784,7 @@
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G433" t="n">
@@ -47783,7 +47818,7 @@
         </is>
       </c>
       <c r="O433" t="n">
-        <v>17539898</v>
+        <v>18056291</v>
       </c>
       <c r="P433" t="inlineStr">
         <is>
@@ -47838,11 +47873,11 @@
     </row>
     <row r="434">
       <c r="A434" t="n">
-        <v>6279</v>
+        <v>6404</v>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>DIENNYFER DA S PEREIRA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
@@ -47862,7 +47897,7 @@
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G434" t="n">
@@ -47896,7 +47931,7 @@
         </is>
       </c>
       <c r="O434" t="n">
-        <v>18056291</v>
+        <v>16962472</v>
       </c>
       <c r="P434" t="inlineStr">
         <is>
@@ -47914,7 +47949,7 @@
       </c>
       <c r="T434" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>SOLAR INVESTIMENTOS</t>
         </is>
       </c>
       <c r="U434" t="inlineStr">
@@ -47951,11 +47986,11 @@
     </row>
     <row r="435">
       <c r="A435" t="n">
-        <v>6404</v>
+        <v>6486</v>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
@@ -47965,7 +48000,7 @@
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E435" t="inlineStr">
@@ -48000,7 +48035,7 @@
       </c>
       <c r="M435" t="inlineStr">
         <is>
-          <t>30/07/2026</t>
+          <t>29/07/2026</t>
         </is>
       </c>
       <c r="N435" t="inlineStr">
@@ -48009,11 +48044,11 @@
         </is>
       </c>
       <c r="O435" t="n">
-        <v>16962472</v>
+        <v>18114225</v>
       </c>
       <c r="P435" t="inlineStr">
         <is>
-          <t>Isabela Lemos</t>
+          <t>Nathany Barreto</t>
         </is>
       </c>
       <c r="Q435" t="inlineStr">
@@ -48027,7 +48062,7 @@
       </c>
       <c r="T435" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U435" t="inlineStr">
@@ -48037,7 +48072,8 @@
       </c>
       <c r="V435" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 - Data Comentário: 22/07/2026 20:00</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
+Aguardando liberação do PIS/COFINS/IRPJ E CSLL - Data Comentário: 21/07/2026 11:36</t>
         </is>
       </c>
       <c r="W435" t="inlineStr"/>
@@ -48058,17 +48094,17 @@
       </c>
       <c r="AG435" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>Karina Santos</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="n">
-        <v>6486</v>
+        <v>6703</v>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>PC GAMER GOIANIA LTDA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
@@ -48078,7 +48114,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E436" t="inlineStr">
@@ -48122,7 +48158,7 @@
         </is>
       </c>
       <c r="O436" t="n">
-        <v>18114225</v>
+        <v>17955210</v>
       </c>
       <c r="P436" t="inlineStr">
         <is>
@@ -48140,7 +48176,7 @@
       </c>
       <c r="T436" t="inlineStr">
         <is>
-          <t>PC GAMER</t>
+          <t>LIMA MOTA</t>
         </is>
       </c>
       <c r="U436" t="inlineStr">
@@ -48178,11 +48214,11 @@
     </row>
     <row r="437">
       <c r="A437" t="n">
-        <v>6703</v>
+        <v>6704</v>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
@@ -48192,7 +48228,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
@@ -48227,7 +48263,7 @@
       </c>
       <c r="M437" t="inlineStr">
         <is>
-          <t>29/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="N437" t="inlineStr">
@@ -48236,11 +48272,11 @@
         </is>
       </c>
       <c r="O437" t="n">
-        <v>17955210</v>
+        <v>17955443</v>
       </c>
       <c r="P437" t="inlineStr">
         <is>
-          <t>Nathany Barreto</t>
+          <t>Paulo Silva</t>
         </is>
       </c>
       <c r="Q437" t="inlineStr">
@@ -48254,7 +48290,7 @@
       </c>
       <c r="T437" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U437" t="inlineStr">
@@ -48264,8 +48300,7 @@
       </c>
       <c r="V437" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 
-Aguardando liberação do PIS/COFINS/IRPJ E CSLL - Data Comentário: 21/07/2026 11:36</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 - Data Comentário: 22/07/2026 13:16</t>
         </is>
       </c>
       <c r="W437" t="inlineStr"/>
@@ -48286,17 +48321,17 @@
       </c>
       <c r="AG437" t="inlineStr">
         <is>
-          <t>Karina Santos</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="n">
-        <v>6704</v>
+        <v>6486</v>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>PC GAMER GOIANIA LTDA</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
@@ -48320,19 +48355,19 @@
         </is>
       </c>
       <c r="G438" t="n">
-        <v>11514</v>
+        <v>5800</v>
       </c>
       <c r="H438" t="n">
-        <v>0</v>
+        <v>5776</v>
       </c>
       <c r="I438" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J438" t="inlineStr">
         <is>
-          <t>Módulo de Inclusão Tributária (MIT)</t>
+          <t>CCT Lançamento Sd.663</t>
         </is>
       </c>
       <c r="K438" t="inlineStr"/>
@@ -48346,15 +48381,15 @@
       </c>
       <c r="N438" t="inlineStr">
         <is>
-          <t>06/2026</t>
+          <t>00/2026</t>
         </is>
       </c>
       <c r="O438" t="n">
-        <v>17955443</v>
+        <v>17901201</v>
       </c>
       <c r="P438" t="inlineStr">
         <is>
-          <t>Paulo Silva</t>
+          <t>Jakeline Silva</t>
         </is>
       </c>
       <c r="Q438" t="inlineStr">
@@ -48368,7 +48403,7 @@
       </c>
       <c r="T438" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>PC GAMER</t>
         </is>
       </c>
       <c r="U438" t="inlineStr">
@@ -48378,7 +48413,8 @@
       </c>
       <c r="V438" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 - Data Comentário: 22/07/2026 13:16</t>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 30/07/2026 
+O retorno do cliente foi recebido. Estamos realizando os trâmites para a aplicação do reajuste. - Data Comentário: 27/07/2026 09:51</t>
         </is>
       </c>
       <c r="W438" t="inlineStr"/>
@@ -48394,22 +48430,22 @@
       <c r="AE438" t="inlineStr"/>
       <c r="AF438" t="inlineStr">
         <is>
-          <t>Obrigação Acessória</t>
+          <t>Tarefa</t>
         </is>
       </c>
       <c r="AG438" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>David Bragança</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="n">
-        <v>6486</v>
+        <v>6548</v>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>PC GAMER GOIANIA LTDA</t>
+          <t>GOIAS SILAGEM LTDA</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
@@ -48433,10 +48469,10 @@
         </is>
       </c>
       <c r="G439" t="n">
-        <v>5800</v>
+        <v>11542</v>
       </c>
       <c r="H439" t="n">
-        <v>5776</v>
+        <v>0</v>
       </c>
       <c r="I439" t="inlineStr">
         <is>
@@ -48445,12 +48481,12 @@
       </c>
       <c r="J439" t="inlineStr">
         <is>
-          <t>CCT Lançamento Sd.663</t>
+          <t>Envio Arq. eConsignado Cliente</t>
         </is>
       </c>
       <c r="K439" t="inlineStr"/>
       <c r="L439" s="1" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="M439" t="inlineStr">
         <is>
@@ -48459,15 +48495,15 @@
       </c>
       <c r="N439" t="inlineStr">
         <is>
-          <t>00/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="O439" t="n">
-        <v>17901201</v>
+        <v>17222967</v>
       </c>
       <c r="P439" t="inlineStr">
         <is>
-          <t>Jakeline Silva</t>
+          <t>Evellin Bispo</t>
         </is>
       </c>
       <c r="Q439" t="inlineStr">
@@ -48477,11 +48513,11 @@
       </c>
       <c r="R439" t="inlineStr"/>
       <c r="S439" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="T439" t="inlineStr">
         <is>
-          <t>PC GAMER</t>
+          <t>GOIAS SILAGEM</t>
         </is>
       </c>
       <c r="U439" t="inlineStr">
@@ -48491,8 +48527,8 @@
       </c>
       <c r="V439" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 30/07/2026 
-O retorno do cliente foi recebido. Estamos realizando os trâmites para a aplicação do reajuste. - Data Comentário: 27/07/2026 09:51</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 
+Data provisionada. - Data Comentário: 27/07/2026 15:32</t>
         </is>
       </c>
       <c r="W439" t="inlineStr"/>
@@ -48508,7 +48544,7 @@
       <c r="AE439" t="inlineStr"/>
       <c r="AF439" t="inlineStr">
         <is>
-          <t>Tarefa</t>
+          <t>Obrigação Acessória</t>
         </is>
       </c>
       <c r="AG439" t="inlineStr">
@@ -48519,11 +48555,11 @@
     </row>
     <row r="440">
       <c r="A440" t="n">
-        <v>6548</v>
+        <v>6703</v>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM LTDA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
@@ -48533,7 +48569,7 @@
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E440" t="inlineStr">
@@ -48568,7 +48604,7 @@
       </c>
       <c r="M440" t="inlineStr">
         <is>
-          <t>30/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="N440" t="inlineStr">
@@ -48577,11 +48613,11 @@
         </is>
       </c>
       <c r="O440" t="n">
-        <v>17222967</v>
+        <v>18077184</v>
       </c>
       <c r="P440" t="inlineStr">
         <is>
-          <t>Evellin Bispo</t>
+          <t>Ana Marcelino</t>
         </is>
       </c>
       <c r="Q440" t="inlineStr">
@@ -48595,7 +48631,7 @@
       </c>
       <c r="T440" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM</t>
+          <t>LIMA MOTA</t>
         </is>
       </c>
       <c r="U440" t="inlineStr">
@@ -48605,8 +48641,8 @@
       </c>
       <c r="V440" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 
-Data provisionada. - Data Comentário: 27/07/2026 15:32</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 
+previsão - Data Comentário: 27/07/2026 09:33</t>
         </is>
       </c>
       <c r="W440" t="inlineStr"/>
@@ -48627,17 +48663,17 @@
       </c>
       <c r="AG440" t="inlineStr">
         <is>
-          <t>David Bragança</t>
+          <t>Sara Cavalheiro</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="n">
-        <v>6703</v>
+        <v>6779</v>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>CORDEIRO E CIA LTDA</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
@@ -48647,7 +48683,7 @@
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E441" t="inlineStr">
@@ -48691,11 +48727,11 @@
         </is>
       </c>
       <c r="O441" t="n">
-        <v>18077184</v>
+        <v>18090271</v>
       </c>
       <c r="P441" t="inlineStr">
         <is>
-          <t>Ana Marcelino</t>
+          <t>Kaique Souza</t>
         </is>
       </c>
       <c r="Q441" t="inlineStr">
@@ -48709,18 +48745,18 @@
       </c>
       <c r="T441" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U441" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="V441" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 
-previsão - Data Comentário: 27/07/2026 09:33</t>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 28/07/2026 
+Será enviado ao cliente em 28/07/2026. - Data Comentário: 27/07/2026 18:16</t>
         </is>
       </c>
       <c r="W441" t="inlineStr"/>
@@ -48747,11 +48783,11 @@
     </row>
     <row r="442">
       <c r="A442" t="n">
-        <v>6779</v>
+        <v>6949</v>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>CORDEIRO E CIA LTDA</t>
+          <t>TEC GRUA LOCAÇÃO E COMERCIO DE EQUIPAMENTOS PARA CONSTRUÇÃO LTDA</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
@@ -48761,7 +48797,7 @@
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E442" t="inlineStr">
@@ -48771,7 +48807,7 @@
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G442" t="n">
@@ -48796,7 +48832,7 @@
       </c>
       <c r="M442" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="N442" t="inlineStr">
@@ -48805,11 +48841,11 @@
         </is>
       </c>
       <c r="O442" t="n">
-        <v>18090271</v>
+        <v>18190470</v>
       </c>
       <c r="P442" t="inlineStr">
         <is>
-          <t>Kaique Souza</t>
+          <t>Gabriela Peres</t>
         </is>
       </c>
       <c r="Q442" t="inlineStr">
@@ -48823,7 +48859,7 @@
       </c>
       <c r="T442" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>TEC GRUA</t>
         </is>
       </c>
       <c r="U442" t="inlineStr">
@@ -48833,8 +48869,8 @@
       </c>
       <c r="V442" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 28/07/2026 
-Será enviado ao cliente em 28/07/2026. - Data Comentário: 27/07/2026 18:16</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
+Previsão de conclusão: 29/07/2026 - Data Comentário: 27/07/2026 14:34</t>
         </is>
       </c>
       <c r="W442" t="inlineStr"/>
@@ -48855,17 +48891,17 @@
       </c>
       <c r="AG442" t="inlineStr">
         <is>
-          <t>Sara Cavalheiro</t>
+          <t>Leandro Matos</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="n">
-        <v>6949</v>
+        <v>6548</v>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>TEC GRUA LOCAÇÃO E COMERCIO DE EQUIPAMENTOS PARA CONSTRUÇÃO LTDA</t>
+          <t>GOIAS SILAGEM LTDA</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
@@ -48885,14 +48921,14 @@
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G443" t="n">
-        <v>11542</v>
+        <v>5905</v>
       </c>
       <c r="H443" t="n">
-        <v>0</v>
+        <v>5784</v>
       </c>
       <c r="I443" t="inlineStr">
         <is>
@@ -48901,29 +48937,29 @@
       </c>
       <c r="J443" t="inlineStr">
         <is>
-          <t>Envio Arq. eConsignado Cliente</t>
+          <t>Folha Mensal/Pró-Labore</t>
         </is>
       </c>
       <c r="K443" t="inlineStr"/>
       <c r="L443" s="1" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="M443" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="N443" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="O443" t="n">
-        <v>18190470</v>
+        <v>17222668</v>
       </c>
       <c r="P443" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Evellin Bispo</t>
         </is>
       </c>
       <c r="Q443" t="inlineStr">
@@ -48933,22 +48969,21 @@
       </c>
       <c r="R443" t="inlineStr"/>
       <c r="S443" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T443" t="inlineStr">
         <is>
-          <t>TEC GRUA</t>
+          <t>GOIAS SILAGEM</t>
         </is>
       </c>
       <c r="U443" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="V443" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
-Previsão de conclusão: 29/07/2026 - Data Comentário: 27/07/2026 14:34</t>
+          <t>2. Folha Processada aguardando OK do cliente para finalização   Previsão para conclusão dia 30/07/2026 - Data Comentário: 27/07/2026 17:24</t>
         </is>
       </c>
       <c r="W443" t="inlineStr"/>
@@ -48969,7 +49004,7 @@
       </c>
       <c r="AG443" t="inlineStr">
         <is>
-          <t>Leandro Matos</t>
+          <t>David Bragança</t>
         </is>
       </c>
     </row>
@@ -49003,7 +49038,7 @@
         </is>
       </c>
       <c r="G444" t="n">
-        <v>5905</v>
+        <v>5853</v>
       </c>
       <c r="H444" t="n">
         <v>5784</v>
@@ -49015,7 +49050,7 @@
       </c>
       <c r="J444" t="inlineStr">
         <is>
-          <t>Folha Mensal/Pró-Labore</t>
+          <t>FOPAG Impressão PDF</t>
         </is>
       </c>
       <c r="K444" t="inlineStr"/>
@@ -49033,7 +49068,7 @@
         </is>
       </c>
       <c r="O444" t="n">
-        <v>17222668</v>
+        <v>17222587</v>
       </c>
       <c r="P444" t="inlineStr">
         <is>
@@ -49061,7 +49096,7 @@
       </c>
       <c r="V444" t="inlineStr">
         <is>
-          <t>2. Folha Processada aguardando OK do cliente para finalização   Previsão para conclusão dia 30/07/2026 - Data Comentário: 27/07/2026 17:24</t>
+          <t>3. Folha, Aguardando Resumo p/ Processamento   Previsão para conclusão dia 30/07/2026 - Data Comentário: 27/07/2026 09:32</t>
         </is>
       </c>
       <c r="W444" t="inlineStr"/>
@@ -49077,7 +49112,7 @@
       <c r="AE444" t="inlineStr"/>
       <c r="AF444" t="inlineStr">
         <is>
-          <t>Obrigação Acessória</t>
+          <t>Tarefa</t>
         </is>
       </c>
       <c r="AG444" t="inlineStr">
@@ -49116,10 +49151,10 @@
         </is>
       </c>
       <c r="G445" t="n">
-        <v>5853</v>
+        <v>11541</v>
       </c>
       <c r="H445" t="n">
-        <v>5784</v>
+        <v>0</v>
       </c>
       <c r="I445" t="inlineStr">
         <is>
@@ -49128,25 +49163,25 @@
       </c>
       <c r="J445" t="inlineStr">
         <is>
-          <t>FOPAG Impressão PDF</t>
+          <t>Importação Arq. eConsignado Único</t>
         </is>
       </c>
       <c r="K445" t="inlineStr"/>
       <c r="L445" s="1" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="M445" t="inlineStr">
         <is>
-          <t>30/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="N445" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="O445" t="n">
-        <v>17222587</v>
+        <v>17222947</v>
       </c>
       <c r="P445" t="inlineStr">
         <is>
@@ -49160,7 +49195,7 @@
       </c>
       <c r="R445" t="inlineStr"/>
       <c r="S445" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="T445" t="inlineStr">
         <is>
@@ -49174,7 +49209,8 @@
       </c>
       <c r="V445" t="inlineStr">
         <is>
-          <t>3. Folha, Aguardando Resumo p/ Processamento   Previsão para conclusão dia 30/07/2026 - Data Comentário: 27/07/2026 09:32</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 
+Previsão para concluir em 28/07/2026 - Data Comentário: 27/07/2026 09:17</t>
         </is>
       </c>
       <c r="W445" t="inlineStr"/>
@@ -49190,7 +49226,7 @@
       <c r="AE445" t="inlineStr"/>
       <c r="AF445" t="inlineStr">
         <is>
-          <t>Tarefa</t>
+          <t>Obrigação Acessória</t>
         </is>
       </c>
       <c r="AG445" t="inlineStr">
@@ -49201,11 +49237,11 @@
     </row>
     <row r="446">
       <c r="A446" t="n">
-        <v>6548</v>
+        <v>6703</v>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM LTDA</t>
+          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -49215,7 +49251,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E446" t="inlineStr">
@@ -49248,22 +49284,18 @@
       <c r="L446" s="1" t="n">
         <v>46234</v>
       </c>
-      <c r="M446" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
+      <c r="M446" t="inlineStr"/>
       <c r="N446" t="inlineStr">
         <is>
           <t>08/2026</t>
         </is>
       </c>
       <c r="O446" t="n">
-        <v>17222947</v>
+        <v>18077174</v>
       </c>
       <c r="P446" t="inlineStr">
         <is>
-          <t>Evellin Bispo</t>
+          <t>Ana Marcelino</t>
         </is>
       </c>
       <c r="Q446" t="inlineStr">
@@ -49277,7 +49309,7 @@
       </c>
       <c r="T446" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM</t>
+          <t>LIMA MOTA</t>
         </is>
       </c>
       <c r="U446" t="inlineStr">
@@ -49285,12 +49317,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V446" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 28/07/2026 
-Previsão para concluir em 28/07/2026 - Data Comentário: 27/07/2026 09:17</t>
-        </is>
-      </c>
+      <c r="V446" t="inlineStr"/>
       <c r="W446" t="inlineStr"/>
       <c r="X446" t="inlineStr"/>
       <c r="Y446" t="inlineStr"/>
@@ -49309,17 +49336,17 @@
       </c>
       <c r="AG446" t="inlineStr">
         <is>
-          <t>David Bragança</t>
+          <t>Sara Cavalheiro</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="n">
-        <v>6703</v>
+        <v>6779</v>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>LIMA MOTA LOCAÇÕES, SERVIÇOS E COMERCIO LTDA</t>
+          <t>CORDEIRO E CIA LTDA</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
@@ -49329,7 +49356,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
@@ -49362,18 +49389,22 @@
       <c r="L447" s="1" t="n">
         <v>46234</v>
       </c>
-      <c r="M447" t="inlineStr"/>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
       <c r="N447" t="inlineStr">
         <is>
           <t>08/2026</t>
         </is>
       </c>
       <c r="O447" t="n">
-        <v>18077174</v>
+        <v>18090261</v>
       </c>
       <c r="P447" t="inlineStr">
         <is>
-          <t>Ana Marcelino</t>
+          <t>Kaique Souza</t>
         </is>
       </c>
       <c r="Q447" t="inlineStr">
@@ -49387,15 +49418,20 @@
       </c>
       <c r="T447" t="inlineStr">
         <is>
-          <t>LIMA MOTA</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U447" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="V447" t="inlineStr"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="V447" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 28/07/2026 
+Será enviado ao cliente em 28/07/2026. - Data Comentário: 27/07/2026 18:16</t>
+        </is>
+      </c>
       <c r="W447" t="inlineStr"/>
       <c r="X447" t="inlineStr"/>
       <c r="Y447" t="inlineStr"/>
@@ -49420,11 +49456,11 @@
     </row>
     <row r="448">
       <c r="A448" t="n">
-        <v>6779</v>
+        <v>6949</v>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>CORDEIRO E CIA LTDA</t>
+          <t>TEC GRUA LOCAÇÃO E COMERCIO DE EQUIPAMENTOS PARA CONSTRUÇÃO LTDA</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
@@ -49434,7 +49470,7 @@
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E448" t="inlineStr">
@@ -49444,7 +49480,7 @@
       </c>
       <c r="F448" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G448" t="n">
@@ -49469,7 +49505,7 @@
       </c>
       <c r="M448" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="N448" t="inlineStr">
@@ -49478,11 +49514,11 @@
         </is>
       </c>
       <c r="O448" t="n">
-        <v>18090261</v>
+        <v>18190464</v>
       </c>
       <c r="P448" t="inlineStr">
         <is>
-          <t>Kaique Souza</t>
+          <t>Gabriela Peres</t>
         </is>
       </c>
       <c r="Q448" t="inlineStr">
@@ -49496,7 +49532,7 @@
       </c>
       <c r="T448" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>TEC GRUA</t>
         </is>
       </c>
       <c r="U448" t="inlineStr">
@@ -49506,8 +49542,8 @@
       </c>
       <c r="V448" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 28/07/2026 
-Será enviado ao cliente em 28/07/2026. - Data Comentário: 27/07/2026 18:16</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
+Previsão de conclusão: 29/07/2026 - Data Comentário: 27/07/2026 14:34</t>
         </is>
       </c>
       <c r="W448" t="inlineStr"/>
@@ -49528,17 +49564,17 @@
       </c>
       <c r="AG448" t="inlineStr">
         <is>
-          <t>Sara Cavalheiro</t>
+          <t>Leandro Matos</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="n">
-        <v>6949</v>
+        <v>5417</v>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>TEC GRUA LOCAÇÃO E COMERCIO DE EQUIPAMENTOS PARA CONSTRUÇÃO LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
@@ -49558,14 +49594,14 @@
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G449" t="n">
-        <v>11541</v>
+        <v>5847</v>
       </c>
       <c r="H449" t="n">
-        <v>0</v>
+        <v>5784</v>
       </c>
       <c r="I449" t="inlineStr">
         <is>
@@ -49574,29 +49610,29 @@
       </c>
       <c r="J449" t="inlineStr">
         <is>
-          <t>Importação Arq. eConsignado Único</t>
+          <t>Rebto planilha/Resumo de Folha (28)</t>
         </is>
       </c>
       <c r="K449" t="inlineStr"/>
       <c r="L449" s="1" t="n">
-        <v>46234</v>
+        <v>46231</v>
       </c>
       <c r="M449" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="N449" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="O449" t="n">
-        <v>18190464</v>
+        <v>18158415</v>
       </c>
       <c r="P449" t="inlineStr">
         <is>
-          <t>Gabriela Peres</t>
+          <t>Mikael Teixeira</t>
         </is>
       </c>
       <c r="Q449" t="inlineStr">
@@ -49606,22 +49642,21 @@
       </c>
       <c r="R449" t="inlineStr"/>
       <c r="S449" t="n">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="T449" t="inlineStr">
         <is>
-          <t>TEC GRUA</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U449" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="V449" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
-Previsão de conclusão: 29/07/2026 - Data Comentário: 27/07/2026 14:34</t>
+          <t>3. Folha, Aguardando Resumo p/ Processamento   Previsão para conclusão dia 28/07/2026 - Data Comentário: 27/07/2026 17:53</t>
         </is>
       </c>
       <c r="W449" t="inlineStr"/>
@@ -49637,22 +49672,18 @@
       <c r="AE449" t="inlineStr"/>
       <c r="AF449" t="inlineStr">
         <is>
-          <t>Obrigação Acessória</t>
-        </is>
-      </c>
-      <c r="AG449" t="inlineStr">
-        <is>
-          <t>Leandro Matos</t>
-        </is>
-      </c>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AG449" t="inlineStr"/>
     </row>
     <row r="450">
       <c r="A450" t="n">
-        <v>5417</v>
+        <v>6779</v>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>CORDEIRO E CIA LTDA</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
@@ -49662,7 +49693,7 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E450" t="inlineStr">
@@ -49672,7 +49703,7 @@
       </c>
       <c r="F450" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G450" t="n">
@@ -49706,11 +49737,11 @@
         </is>
       </c>
       <c r="O450" t="n">
-        <v>18158415</v>
+        <v>18158762</v>
       </c>
       <c r="P450" t="inlineStr">
         <is>
-          <t>Mikael Teixeira</t>
+          <t>Kaique Souza</t>
         </is>
       </c>
       <c r="Q450" t="inlineStr">
@@ -49724,17 +49755,18 @@
       </c>
       <c r="T450" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U450" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="V450" t="inlineStr">
         <is>
-          <t>3. Folha, Aguardando Resumo p/ Processamento   Previsão para conclusão dia 28/07/2026 - Data Comentário: 27/07/2026 17:53</t>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 28/07/2026 
+Aguardando envio do cliente. - Data Comentário: 27/07/2026 17:59</t>
         </is>
       </c>
       <c r="W450" t="inlineStr"/>
@@ -49753,15 +49785,19 @@
           <t>Tarefa</t>
         </is>
       </c>
-      <c r="AG450" t="inlineStr"/>
+      <c r="AG450" t="inlineStr">
+        <is>
+          <t>Sara Cavalheiro</t>
+        </is>
+      </c>
     </row>
     <row r="451">
       <c r="A451" t="n">
-        <v>6779</v>
+        <v>6548</v>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>CORDEIRO E CIA LTDA</t>
+          <t>GOIAS SILAGEM LTDA</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
@@ -49771,7 +49807,7 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E451" t="inlineStr">
@@ -49785,7 +49821,7 @@
         </is>
       </c>
       <c r="G451" t="n">
-        <v>5847</v>
+        <v>5906</v>
       </c>
       <c r="H451" t="n">
         <v>5784</v>
@@ -49797,16 +49833,16 @@
       </c>
       <c r="J451" t="inlineStr">
         <is>
-          <t>Rebto planilha/Resumo de Folha (28)</t>
+          <t>Recibo de Pagamento</t>
         </is>
       </c>
       <c r="K451" t="inlineStr"/>
       <c r="L451" s="1" t="n">
-        <v>46231</v>
+        <v>46233</v>
       </c>
       <c r="M451" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="N451" t="inlineStr">
@@ -49815,11 +49851,11 @@
         </is>
       </c>
       <c r="O451" t="n">
-        <v>18158762</v>
+        <v>17222684</v>
       </c>
       <c r="P451" t="inlineStr">
         <is>
-          <t>Kaique Souza</t>
+          <t>Evellin Bispo</t>
         </is>
       </c>
       <c r="Q451" t="inlineStr">
@@ -49829,22 +49865,22 @@
       </c>
       <c r="R451" t="inlineStr"/>
       <c r="S451" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="T451" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>GOIAS SILAGEM</t>
         </is>
       </c>
       <c r="U451" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="V451" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 28/07/2026 
-Aguardando envio do cliente. - Data Comentário: 27/07/2026 17:59</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 
+Previsão para concluir em 30/07/2026 - Data Comentário: 27/07/2026 09:24</t>
         </is>
       </c>
       <c r="W451" t="inlineStr"/>
@@ -49865,7 +49901,7 @@
       </c>
       <c r="AG451" t="inlineStr">
         <is>
-          <t>Sara Cavalheiro</t>
+          <t>David Bragança</t>
         </is>
       </c>
     </row>
@@ -49899,7 +49935,7 @@
         </is>
       </c>
       <c r="G452" t="n">
-        <v>5906</v>
+        <v>5907</v>
       </c>
       <c r="H452" t="n">
         <v>5784</v>
@@ -49911,7 +49947,7 @@
       </c>
       <c r="J452" t="inlineStr">
         <is>
-          <t>Recibo de Pagamento</t>
+          <t>Relação Bancária - Salário</t>
         </is>
       </c>
       <c r="K452" t="inlineStr"/>
@@ -49929,7 +49965,7 @@
         </is>
       </c>
       <c r="O452" t="n">
-        <v>17222684</v>
+        <v>17222697</v>
       </c>
       <c r="P452" t="inlineStr">
         <is>
@@ -49958,7 +49994,7 @@
       <c r="V452" t="inlineStr">
         <is>
           <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 
-Previsão para concluir em 30/07/2026 - Data Comentário: 27/07/2026 09:24</t>
+Previsão para concluir em 30/07/2026 - Data Comentário: 27/07/2026 09:25</t>
         </is>
       </c>
       <c r="W452" t="inlineStr"/>
@@ -49985,11 +50021,11 @@
     </row>
     <row r="453">
       <c r="A453" t="n">
-        <v>6548</v>
+        <v>5417</v>
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
@@ -50009,14 +50045,14 @@
       </c>
       <c r="F453" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G453" t="n">
-        <v>5907</v>
+        <v>6348</v>
       </c>
       <c r="H453" t="n">
-        <v>5784</v>
+        <v>0</v>
       </c>
       <c r="I453" t="inlineStr">
         <is>
@@ -50025,7 +50061,7 @@
       </c>
       <c r="J453" t="inlineStr">
         <is>
-          <t>Relação Bancária - Salário</t>
+          <t>RESCISÃO - RESCISÃO</t>
         </is>
       </c>
       <c r="K453" t="inlineStr"/>
@@ -50034,7 +50070,7 @@
       </c>
       <c r="M453" t="inlineStr">
         <is>
-          <t>30/07/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="N453" t="inlineStr">
@@ -50043,11 +50079,11 @@
         </is>
       </c>
       <c r="O453" t="n">
-        <v>17222697</v>
+        <v>18202319</v>
       </c>
       <c r="P453" t="inlineStr">
         <is>
-          <t>Evellin Bispo</t>
+          <t>Mikael Teixeira</t>
         </is>
       </c>
       <c r="Q453" t="inlineStr">
@@ -50061,7 +50097,7 @@
       </c>
       <c r="T453" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U453" t="inlineStr">
@@ -50071,8 +50107,8 @@
       </c>
       <c r="V453" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 
-Previsão para concluir em 30/07/2026 - Data Comentário: 27/07/2026 09:25</t>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 28/07/2026 
+aguardando cliente enviar informações - Data Comentário: 27/07/2026 18:00</t>
         </is>
       </c>
       <c r="W453" t="inlineStr"/>
@@ -50088,22 +50124,18 @@
       <c r="AE453" t="inlineStr"/>
       <c r="AF453" t="inlineStr">
         <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AG453" t="inlineStr">
-        <is>
-          <t>David Bragança</t>
-        </is>
-      </c>
+          <t>Imposto</t>
+        </is>
+      </c>
+      <c r="AG453" t="inlineStr"/>
     </row>
     <row r="454">
       <c r="A454" t="n">
-        <v>5417</v>
+        <v>6949</v>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>TEC GRUA LOCAÇÃO E COMERCIO DE EQUIPAMENTOS PARA CONSTRUÇÃO LTDA</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
@@ -50123,45 +50155,45 @@
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G454" t="n">
-        <v>6348</v>
+        <v>11617</v>
       </c>
       <c r="H454" t="n">
         <v>0</v>
       </c>
       <c r="I454" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J454" t="inlineStr">
         <is>
-          <t>RESCISÃO - RESCISÃO</t>
+          <t>Envio de ATA de Implantação - EF I</t>
         </is>
       </c>
       <c r="K454" t="inlineStr"/>
       <c r="L454" s="1" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="M454" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="N454" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>06/2026</t>
         </is>
       </c>
       <c r="O454" t="n">
-        <v>18202319</v>
+        <v>18166588</v>
       </c>
       <c r="P454" t="inlineStr">
         <is>
-          <t>Mikael Teixeira</t>
+          <t>Priscila Volpe</t>
         </is>
       </c>
       <c r="Q454" t="inlineStr">
@@ -50171,22 +50203,22 @@
       </c>
       <c r="R454" t="inlineStr"/>
       <c r="S454" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="T454" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>TEC GRUA</t>
         </is>
       </c>
       <c r="U454" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="V454" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 28/07/2026 
-aguardando cliente enviar informações - Data Comentário: 27/07/2026 18:00</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
+ainda não foi realizado as implantações - Data Comentário: 01/07/2026 13:38</t>
         </is>
       </c>
       <c r="W454" t="inlineStr"/>
@@ -50202,18 +50234,22 @@
       <c r="AE454" t="inlineStr"/>
       <c r="AF454" t="inlineStr">
         <is>
-          <t>Imposto</t>
-        </is>
-      </c>
-      <c r="AG454" t="inlineStr"/>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AG454" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" t="n">
-        <v>6949</v>
+        <v>6962</v>
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>TEC GRUA LOCAÇÃO E COMERCIO DE EQUIPAMENTOS PARA CONSTRUÇÃO LTDA</t>
+          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
@@ -50267,7 +50303,7 @@
         </is>
       </c>
       <c r="O455" t="n">
-        <v>18166588</v>
+        <v>18186565</v>
       </c>
       <c r="P455" t="inlineStr">
         <is>
@@ -50285,7 +50321,7 @@
       </c>
       <c r="T455" t="inlineStr">
         <is>
-          <t>TEC GRUA</t>
+          <t>PROMOTORAS GYN</t>
         </is>
       </c>
       <c r="U455" t="inlineStr">
@@ -50323,11 +50359,11 @@
     </row>
     <row r="456">
       <c r="A456" t="n">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
+          <t>PROMOTORAS GYN LTDA</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
@@ -50381,7 +50417,7 @@
         </is>
       </c>
       <c r="O456" t="n">
-        <v>18186565</v>
+        <v>18186566</v>
       </c>
       <c r="P456" t="inlineStr">
         <is>
@@ -50437,11 +50473,11 @@
     </row>
     <row r="457">
       <c r="A457" t="n">
-        <v>6963</v>
+        <v>5417</v>
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
@@ -50461,45 +50497,41 @@
       </c>
       <c r="F457" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G457" t="n">
-        <v>11617</v>
+        <v>957</v>
       </c>
       <c r="H457" t="n">
         <v>0</v>
       </c>
       <c r="I457" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J457" t="inlineStr">
         <is>
-          <t>Envio de ATA de Implantação - EF I</t>
+          <t>Definição do Lucro Trimestral</t>
         </is>
       </c>
       <c r="K457" t="inlineStr"/>
       <c r="L457" s="1" t="n">
-        <v>46234</v>
-      </c>
-      <c r="M457" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
+        <v>46233</v>
+      </c>
+      <c r="M457" t="inlineStr"/>
       <c r="N457" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O457" t="n">
-        <v>18186566</v>
+        <v>17398899</v>
       </c>
       <c r="P457" t="inlineStr">
         <is>
-          <t>Priscila Volpe</t>
+          <t>Sergio Fernandes</t>
         </is>
       </c>
       <c r="Q457" t="inlineStr">
@@ -50509,24 +50541,19 @@
       </c>
       <c r="R457" t="inlineStr"/>
       <c r="S457" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="T457" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U457" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="V457" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
-ainda não foi realizado as implantações - Data Comentário: 01/07/2026 13:38</t>
-        </is>
-      </c>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V457" t="inlineStr"/>
       <c r="W457" t="inlineStr"/>
       <c r="X457" t="inlineStr"/>
       <c r="Y457" t="inlineStr"/>
@@ -50543,19 +50570,15 @@
           <t>Tarefa</t>
         </is>
       </c>
-      <c r="AG457" t="inlineStr">
-        <is>
-          <t>Nayara Oliveira</t>
-        </is>
-      </c>
+      <c r="AG457" t="inlineStr"/>
     </row>
     <row r="458">
       <c r="A458" t="n">
-        <v>5417</v>
+        <v>5617</v>
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
@@ -50575,7 +50598,7 @@
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G458" t="n">
@@ -50605,7 +50628,7 @@
         </is>
       </c>
       <c r="O458" t="n">
-        <v>17398899</v>
+        <v>17407535</v>
       </c>
       <c r="P458" t="inlineStr">
         <is>
@@ -50623,7 +50646,7 @@
       </c>
       <c r="T458" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U458" t="inlineStr">
@@ -50652,11 +50675,11 @@
     </row>
     <row r="459">
       <c r="A459" t="n">
-        <v>5617</v>
+        <v>6627</v>
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
@@ -50671,7 +50694,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F459" t="inlineStr">
@@ -50706,7 +50729,7 @@
         </is>
       </c>
       <c r="O459" t="n">
-        <v>17407535</v>
+        <v>17042325</v>
       </c>
       <c r="P459" t="inlineStr">
         <is>
@@ -50724,7 +50747,7 @@
       </c>
       <c r="T459" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U459" t="inlineStr">
@@ -50753,11 +50776,11 @@
     </row>
     <row r="460">
       <c r="A460" t="n">
-        <v>6627</v>
+        <v>6359</v>
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>MACHADO PRESTACAO DE SERVICOS LTDA</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
@@ -50767,12 +50790,12 @@
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F460" t="inlineStr">
@@ -50781,19 +50804,19 @@
         </is>
       </c>
       <c r="G460" t="n">
-        <v>957</v>
+        <v>1662</v>
       </c>
       <c r="H460" t="n">
         <v>0</v>
       </c>
       <c r="I460" t="inlineStr">
         <is>
-          <t>GERENCIA DE CONTAS</t>
+          <t>CTB - CONTÁBIL INDUSTRIA</t>
         </is>
       </c>
       <c r="J460" t="inlineStr">
         <is>
-          <t>Definição do Lucro Trimestral</t>
+          <t>Devolução de Documentos</t>
         </is>
       </c>
       <c r="K460" t="inlineStr"/>
@@ -50807,32 +50830,26 @@
         </is>
       </c>
       <c r="O460" t="n">
-        <v>17042325</v>
-      </c>
-      <c r="P460" t="inlineStr">
-        <is>
-          <t>Sergio Fernandes</t>
-        </is>
-      </c>
+        <v>17108122</v>
+      </c>
+      <c r="P460" t="inlineStr"/>
       <c r="Q460" t="inlineStr">
         <is>
-          <t>Em Aberto</t>
-        </is>
-      </c>
-      <c r="R460" t="inlineStr"/>
+          <t>Baixado</t>
+        </is>
+      </c>
+      <c r="R460" s="1" t="n">
+        <v>46209.66158305555</v>
+      </c>
       <c r="S460" t="n">
         <v>-2</v>
       </c>
       <c r="T460" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
-        </is>
-      </c>
-      <c r="U460" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
+          <t>MACHADO</t>
+        </is>
+      </c>
+      <c r="U460" t="inlineStr"/>
       <c r="V460" t="inlineStr"/>
       <c r="W460" t="inlineStr"/>
       <c r="X460" t="inlineStr"/>
@@ -50840,7 +50857,11 @@
       <c r="Z460" t="n">
         <v>0</v>
       </c>
-      <c r="AA460" t="inlineStr"/>
+      <c r="AA460" t="inlineStr">
+        <is>
+          <t>Isabella Nascimento</t>
+        </is>
+      </c>
       <c r="AB460" t="inlineStr"/>
       <c r="AC460" t="inlineStr"/>
       <c r="AD460" t="inlineStr"/>
@@ -50854,11 +50875,11 @@
     </row>
     <row r="461">
       <c r="A461" t="n">
-        <v>6359</v>
+        <v>6548</v>
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>MACHADO PRESTACAO DE SERVICOS LTDA</t>
+          <t>GOIAS SILAGEM LTDA</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
@@ -50868,7 +50889,7 @@
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E461" t="inlineStr">
@@ -50882,7 +50903,7 @@
         </is>
       </c>
       <c r="G461" t="n">
-        <v>1662</v>
+        <v>7237</v>
       </c>
       <c r="H461" t="n">
         <v>0</v>
@@ -50894,12 +50915,12 @@
       </c>
       <c r="J461" t="inlineStr">
         <is>
-          <t>Devolução de Documentos</t>
+          <t>Envio de Impostos - DCTF Web</t>
         </is>
       </c>
       <c r="K461" t="inlineStr"/>
       <c r="L461" s="1" t="n">
-        <v>46233</v>
+        <v>46223</v>
       </c>
       <c r="M461" t="inlineStr"/>
       <c r="N461" t="inlineStr">
@@ -50908,27 +50929,39 @@
         </is>
       </c>
       <c r="O461" t="n">
-        <v>17108122</v>
-      </c>
-      <c r="P461" t="inlineStr"/>
+        <v>17968026</v>
+      </c>
+      <c r="P461" t="inlineStr">
+        <is>
+          <t>Thais Souza</t>
+        </is>
+      </c>
       <c r="Q461" t="inlineStr">
         <is>
           <t>Baixado</t>
         </is>
       </c>
       <c r="R461" s="1" t="n">
-        <v>46209.66158305555</v>
+        <v>46219.68663078704</v>
       </c>
       <c r="S461" t="n">
-        <v>-2</v>
+        <v>8</v>
       </c>
       <c r="T461" t="inlineStr">
         <is>
-          <t>MACHADO</t>
-        </is>
-      </c>
-      <c r="U461" t="inlineStr"/>
-      <c r="V461" t="inlineStr"/>
+          <t>GOIAS SILAGEM</t>
+        </is>
+      </c>
+      <c r="U461" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V461" t="inlineStr">
+        <is>
+          <t>Imposto enviado via SCI Report - Data Comentário: 16/07/2026 11:35</t>
+        </is>
+      </c>
       <c r="W461" t="inlineStr"/>
       <c r="X461" t="inlineStr"/>
       <c r="Y461" t="inlineStr"/>
@@ -50937,7 +50970,7 @@
       </c>
       <c r="AA461" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Juan Rodrigues</t>
         </is>
       </c>
       <c r="AB461" t="inlineStr"/>
@@ -50946,18 +50979,22 @@
       <c r="AE461" t="inlineStr"/>
       <c r="AF461" t="inlineStr">
         <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AG461" t="inlineStr"/>
+          <t>Imposto</t>
+        </is>
+      </c>
+      <c r="AG461" t="inlineStr">
+        <is>
+          <t>Erika Santana</t>
+        </is>
+      </c>
     </row>
     <row r="462">
       <c r="A462" t="n">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
@@ -50972,7 +51009,7 @@
       </c>
       <c r="E462" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F462" t="inlineStr">
@@ -50998,7 +51035,7 @@
       </c>
       <c r="K462" t="inlineStr"/>
       <c r="L462" s="1" t="n">
-        <v>46223</v>
+        <v>46219</v>
       </c>
       <c r="M462" t="inlineStr"/>
       <c r="N462" t="inlineStr">
@@ -51007,11 +51044,11 @@
         </is>
       </c>
       <c r="O462" t="n">
-        <v>17968026</v>
+        <v>17042520</v>
       </c>
       <c r="P462" t="inlineStr">
         <is>
-          <t>Thais Souza</t>
+          <t>Nathalia Lourenco</t>
         </is>
       </c>
       <c r="Q462" t="inlineStr">
@@ -51020,14 +51057,14 @@
         </is>
       </c>
       <c r="R462" s="1" t="n">
-        <v>46219.68663078704</v>
+        <v>46218.73863668981</v>
       </c>
       <c r="S462" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="T462" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U462" t="inlineStr">
@@ -51037,7 +51074,7 @@
       </c>
       <c r="V462" t="inlineStr">
         <is>
-          <t>Imposto enviado via SCI Report - Data Comentário: 16/07/2026 11:35</t>
+          <t>Imposto enviado via SCI Report - Data Comentário: 15/07/2026 16:01</t>
         </is>
       </c>
       <c r="W462" t="inlineStr"/>
@@ -51062,17 +51099,17 @@
       </c>
       <c r="AG462" t="inlineStr">
         <is>
-          <t>Erika Santana</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="n">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
@@ -51082,7 +51119,7 @@
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E463" t="inlineStr">
@@ -51122,7 +51159,7 @@
         </is>
       </c>
       <c r="O463" t="n">
-        <v>17042520</v>
+        <v>16960034</v>
       </c>
       <c r="P463" t="inlineStr">
         <is>
@@ -51135,7 +51172,7 @@
         </is>
       </c>
       <c r="R463" s="1" t="n">
-        <v>46218.73863668981</v>
+        <v>46218.73864609954</v>
       </c>
       <c r="S463" t="n">
         <v>12</v>
@@ -51183,11 +51220,11 @@
     </row>
     <row r="464">
       <c r="A464" t="n">
-        <v>6628</v>
+        <v>6945</v>
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
+          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
@@ -51228,7 +51265,7 @@
       </c>
       <c r="K464" t="inlineStr"/>
       <c r="L464" s="1" t="n">
-        <v>46219</v>
+        <v>46223</v>
       </c>
       <c r="M464" t="inlineStr"/>
       <c r="N464" t="inlineStr">
@@ -51237,11 +51274,11 @@
         </is>
       </c>
       <c r="O464" t="n">
-        <v>16960034</v>
+        <v>18163681</v>
       </c>
       <c r="P464" t="inlineStr">
         <is>
-          <t>Nathalia Lourenco</t>
+          <t>Laisa Rocha</t>
         </is>
       </c>
       <c r="Q464" t="inlineStr">
@@ -51250,24 +51287,24 @@
         </is>
       </c>
       <c r="R464" s="1" t="n">
-        <v>46218.73864609954</v>
+        <v>46220.43670297453</v>
       </c>
       <c r="S464" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="T464" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
       <c r="U464" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="V464" t="inlineStr">
         <is>
-          <t>Imposto enviado via SCI Report - Data Comentário: 15/07/2026 16:01</t>
+          <t>Imposto enviado via SCI Report - Data Comentário: 17/07/2026 08:27</t>
         </is>
       </c>
       <c r="W464" t="inlineStr"/>
@@ -51298,11 +51335,11 @@
     </row>
     <row r="465">
       <c r="A465" t="n">
-        <v>6945</v>
+        <v>6962</v>
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
+          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
@@ -51312,17 +51349,17 @@
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F465" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Reynaldo Santos</t>
         </is>
       </c>
       <c r="G465" t="n">
@@ -51352,11 +51389,11 @@
         </is>
       </c>
       <c r="O465" t="n">
-        <v>18163681</v>
+        <v>18187960</v>
       </c>
       <c r="P465" t="inlineStr">
         <is>
-          <t>Laisa Rocha</t>
+          <t>Mirian Lima</t>
         </is>
       </c>
       <c r="Q465" t="inlineStr">
@@ -51365,14 +51402,14 @@
         </is>
       </c>
       <c r="R465" s="1" t="n">
-        <v>46220.43670297453</v>
+        <v>46220.58299991898</v>
       </c>
       <c r="S465" t="n">
         <v>8</v>
       </c>
       <c r="T465" t="inlineStr">
         <is>
-          <t>BRASIL DISTRIBUIDORA</t>
+          <t>PROMOTORAS GYN</t>
         </is>
       </c>
       <c r="U465" t="inlineStr">
@@ -51382,7 +51419,8 @@
       </c>
       <c r="V465" t="inlineStr">
         <is>
-          <t>Imposto enviado via SCI Report - Data Comentário: 17/07/2026 08:27</t>
+          <t>Aguardando Liberação do Fiscal  
+RETIFICAÇÃO REINF- AGUARDANDO OK - Data Comentário: 17/07/2026 10:39</t>
         </is>
       </c>
       <c r="W465" t="inlineStr"/>
@@ -51393,7 +51431,7 @@
       </c>
       <c r="AA465" t="inlineStr">
         <is>
-          <t>Juan Rodrigues</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
       <c r="AB465" t="inlineStr"/>
@@ -51413,11 +51451,11 @@
     </row>
     <row r="466">
       <c r="A466" t="n">
-        <v>6962</v>
+        <v>6963</v>
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>INOVAR CONSULTORIA EM VAREJO LTDA</t>
+          <t>PROMOTORAS GYN LTDA</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
@@ -51467,7 +51505,7 @@
         </is>
       </c>
       <c r="O466" t="n">
-        <v>18187960</v>
+        <v>18187898</v>
       </c>
       <c r="P466" t="inlineStr">
         <is>
@@ -51480,7 +51518,7 @@
         </is>
       </c>
       <c r="R466" s="1" t="n">
-        <v>46220.58299991898</v>
+        <v>46220.58300498842</v>
       </c>
       <c r="S466" t="n">
         <v>8</v>
@@ -51529,11 +51567,11 @@
     </row>
     <row r="467">
       <c r="A467" t="n">
-        <v>6963</v>
+        <v>6627</v>
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
@@ -51548,16 +51586,16 @@
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F467" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G467" t="n">
-        <v>7237</v>
+        <v>7869</v>
       </c>
       <c r="H467" t="n">
         <v>0</v>
@@ -51569,12 +51607,12 @@
       </c>
       <c r="J467" t="inlineStr">
         <is>
-          <t>Envio de Impostos - DCTF Web</t>
+          <t xml:space="preserve">Envio do Razão Conta - Valores à Classificar </t>
         </is>
       </c>
       <c r="K467" t="inlineStr"/>
       <c r="L467" s="1" t="n">
-        <v>46223</v>
+        <v>46230</v>
       </c>
       <c r="M467" t="inlineStr"/>
       <c r="N467" t="inlineStr">
@@ -51583,11 +51621,11 @@
         </is>
       </c>
       <c r="O467" t="n">
-        <v>18187898</v>
+        <v>17042540</v>
       </c>
       <c r="P467" t="inlineStr">
         <is>
-          <t>Mirian Lima</t>
+          <t>Nathalia Lourenco</t>
         </is>
       </c>
       <c r="Q467" t="inlineStr">
@@ -51596,27 +51634,22 @@
         </is>
       </c>
       <c r="R467" s="1" t="n">
-        <v>46220.58300498842</v>
+        <v>46223.56737932871</v>
       </c>
       <c r="S467" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="T467" t="inlineStr">
         <is>
-          <t>PROMOTORAS GYN</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U467" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="V467" t="inlineStr">
-        <is>
-          <t>Aguardando Liberação do Fiscal  
-RETIFICAÇÃO REINF- AGUARDANDO OK - Data Comentário: 17/07/2026 10:39</t>
-        </is>
-      </c>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V467" t="inlineStr"/>
       <c r="W467" t="inlineStr"/>
       <c r="X467" t="inlineStr"/>
       <c r="Y467" t="inlineStr"/>
@@ -51634,7 +51667,7 @@
       <c r="AE467" t="inlineStr"/>
       <c r="AF467" t="inlineStr">
         <is>
-          <t>Imposto</t>
+          <t>Tarefa</t>
         </is>
       </c>
       <c r="AG467" t="inlineStr">
@@ -51645,11 +51678,11 @@
     </row>
     <row r="468">
       <c r="A468" t="n">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
@@ -51659,7 +51692,7 @@
       </c>
       <c r="D468" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E468" t="inlineStr">
@@ -51699,7 +51732,7 @@
         </is>
       </c>
       <c r="O468" t="n">
-        <v>17042540</v>
+        <v>16960046</v>
       </c>
       <c r="P468" t="inlineStr">
         <is>
@@ -51712,7 +51745,7 @@
         </is>
       </c>
       <c r="R468" s="1" t="n">
-        <v>46223.56737932871</v>
+        <v>46223.56864207176</v>
       </c>
       <c r="S468" t="n">
         <v>1</v>
@@ -51784,7 +51817,7 @@
         </is>
       </c>
       <c r="G469" t="n">
-        <v>7869</v>
+        <v>1650</v>
       </c>
       <c r="H469" t="n">
         <v>0</v>
@@ -51796,12 +51829,12 @@
       </c>
       <c r="J469" t="inlineStr">
         <is>
-          <t xml:space="preserve">Envio do Razão Conta - Valores à Classificar </t>
+          <t>Fechamento Mensal</t>
         </is>
       </c>
       <c r="K469" t="inlineStr"/>
       <c r="L469" s="1" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="M469" t="inlineStr"/>
       <c r="N469" t="inlineStr">
@@ -51810,7 +51843,7 @@
         </is>
       </c>
       <c r="O469" t="n">
-        <v>16960046</v>
+        <v>16959972</v>
       </c>
       <c r="P469" t="inlineStr">
         <is>
@@ -51823,10 +51856,10 @@
         </is>
       </c>
       <c r="R469" s="1" t="n">
-        <v>46223.56864207176</v>
+        <v>46203.00285659722</v>
       </c>
       <c r="S469" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T469" t="inlineStr">
         <is>
@@ -51847,7 +51880,7 @@
       </c>
       <c r="AA469" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>ex-funcionario</t>
         </is>
       </c>
       <c r="AB469" t="inlineStr"/>
@@ -51867,11 +51900,11 @@
     </row>
     <row r="470">
       <c r="A470" t="n">
-        <v>6628</v>
+        <v>6945</v>
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
+          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
@@ -51921,11 +51954,11 @@
         </is>
       </c>
       <c r="O470" t="n">
-        <v>16959972</v>
+        <v>18163665</v>
       </c>
       <c r="P470" t="inlineStr">
         <is>
-          <t>Nathalia Lourenco</t>
+          <t>Laisa Rocha</t>
         </is>
       </c>
       <c r="Q470" t="inlineStr">
@@ -51934,19 +51967,19 @@
         </is>
       </c>
       <c r="R470" s="1" t="n">
-        <v>46203.00285659722</v>
+        <v>46203.00296711805</v>
       </c>
       <c r="S470" t="n">
         <v>0</v>
       </c>
       <c r="T470" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>BRASIL DISTRIBUIDORA</t>
         </is>
       </c>
       <c r="U470" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="V470" t="inlineStr"/>
@@ -51978,11 +52011,11 @@
     </row>
     <row r="471">
       <c r="A471" t="n">
-        <v>6945</v>
+        <v>6628</v>
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>BRASIL DISTRIBUIDORA DE PEÇAS LTDA</t>
+          <t>TSN TECHNICAL SERVICE NETWORK LTDA</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
@@ -52006,7 +52039,7 @@
         </is>
       </c>
       <c r="G471" t="n">
-        <v>1650</v>
+        <v>6892</v>
       </c>
       <c r="H471" t="n">
         <v>0</v>
@@ -52018,25 +52051,29 @@
       </c>
       <c r="J471" t="inlineStr">
         <is>
-          <t>Fechamento Mensal</t>
+          <t>Fed - DCTFWEB</t>
         </is>
       </c>
       <c r="K471" t="inlineStr"/>
       <c r="L471" s="1" t="n">
-        <v>46231</v>
-      </c>
-      <c r="M471" t="inlineStr"/>
+        <v>46233</v>
+      </c>
+      <c r="M471" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
       <c r="N471" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O471" t="n">
-        <v>18163665</v>
+        <v>16960022</v>
       </c>
       <c r="P471" t="inlineStr">
         <is>
-          <t>Laisa Rocha</t>
+          <t>Nathalia Lourenco</t>
         </is>
       </c>
       <c r="Q471" t="inlineStr">
@@ -52045,22 +52082,26 @@
         </is>
       </c>
       <c r="R471" s="1" t="n">
-        <v>46203.00296711805</v>
+        <v>46231.37417729167</v>
       </c>
       <c r="S471" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="T471" t="inlineStr">
         <is>
-          <t>BRASIL DISTRIBUIDORA</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U471" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="V471" t="inlineStr"/>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="V471" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 - Data Comentário: 28/07/2026 07:36</t>
+        </is>
+      </c>
       <c r="W471" t="inlineStr"/>
       <c r="X471" t="inlineStr"/>
       <c r="Y471" t="inlineStr"/>
@@ -52069,7 +52110,7 @@
       </c>
       <c r="AA471" t="inlineStr">
         <is>
-          <t>ex-funcionario</t>
+          <t>Nathalia Lourenco</t>
         </is>
       </c>
       <c r="AB471" t="inlineStr"/>
@@ -52078,7 +52119,7 @@
       <c r="AE471" t="inlineStr"/>
       <c r="AF471" t="inlineStr">
         <is>
-          <t>Tarefa</t>
+          <t>Obrigação Acessória</t>
         </is>
       </c>
       <c r="AG471" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-28 11:49
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG775"/>
+  <dimension ref="A1:AG769"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42787,11 +42787,7 @@
       <c r="L388" s="1" t="n">
         <v>46230</v>
       </c>
-      <c r="M388" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
+      <c r="M388" t="inlineStr"/>
       <c r="N388" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -42826,7 +42822,7 @@
       </c>
       <c r="V388" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 29/07/2026 - Data Comentário: 20/07/2026 15:54</t>
+          <t>Aguardando Liberação do Fiscal - Data Comentário: 28/07/2026 11:36</t>
         </is>
       </c>
       <c r="W388" t="inlineStr"/>
@@ -44133,7 +44129,7 @@
       </c>
       <c r="M400" t="inlineStr">
         <is>
-          <t>23/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="N400" t="inlineStr">
@@ -44170,7 +44166,7 @@
       </c>
       <c r="V400" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 20/07/2026 15:29</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 - Data Comentário: 28/07/2026 11:32</t>
         </is>
       </c>
       <c r="W400" t="inlineStr"/>
@@ -44618,7 +44614,11 @@
           <t>B</t>
         </is>
       </c>
-      <c r="V404" t="inlineStr"/>
+      <c r="V404" t="inlineStr">
+        <is>
+          <t>Fechamento Contábil já liberado - Aguardando liberação da gerência de contas - Data Comentário: 28/07/2026 11:36</t>
+        </is>
+      </c>
       <c r="W404" t="inlineStr"/>
       <c r="X404" t="inlineStr"/>
       <c r="Y404" t="inlineStr"/>
@@ -45007,7 +45007,7 @@
       </c>
       <c r="M408" t="inlineStr">
         <is>
-          <t>23/07/2026</t>
+          <t>30/07/2026</t>
         </is>
       </c>
       <c r="N408" t="inlineStr">
@@ -45044,7 +45044,7 @@
       </c>
       <c r="V408" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 23/07/2026 - Data Comentário: 20/07/2026 15:31</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/07/2026 - Data Comentário: 28/07/2026 11:36</t>
         </is>
       </c>
       <c r="W408" t="inlineStr"/>
@@ -84498,41 +84498,37 @@
         </is>
       </c>
       <c r="G765" t="n">
-        <v>11613</v>
+        <v>9791</v>
       </c>
       <c r="H765" t="n">
         <v>0</v>
       </c>
       <c r="I765" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J765" t="inlineStr">
         <is>
-          <t>Envio de ATA de Implantação - CTB V - GOIAS</t>
+          <t>Aplicação de Modelo - Pendente - GOIAS</t>
         </is>
       </c>
       <c r="K765" t="inlineStr"/>
       <c r="L765" s="1" t="n">
-        <v>46230</v>
-      </c>
-      <c r="M765" t="inlineStr">
-        <is>
-          <t>07/08/2026</t>
-        </is>
-      </c>
+        <v>46206</v>
+      </c>
+      <c r="M765" t="inlineStr"/>
       <c r="N765" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O765" t="n">
-        <v>18189089</v>
+        <v>18189077</v>
       </c>
       <c r="P765" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Mauricio Lermen</t>
         </is>
       </c>
       <c r="Q765" t="inlineStr">
@@ -84542,7 +84538,7 @@
       </c>
       <c r="R765" t="inlineStr"/>
       <c r="S765" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="T765" t="inlineStr">
         <is>
@@ -84556,8 +84552,8 @@
       </c>
       <c r="V765" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 07/08/2026 
-As reuniões de implantação estão agendadas para agosto - Data Comentário: 27/07/2026 16:43</t>
+          <t>Sem informações para a realização da tarefa  
+Não recebemos as informações e documentos do cliente. Conforme consulta hoje, não temos sequer a procuração até o momento. Previsão de conclusão, 02 dias úteis após recebimento. - Data Comentário: 27/07/2026 18:16</t>
         </is>
       </c>
       <c r="W765" t="inlineStr"/>
@@ -84569,12 +84565,12 @@
       <c r="AC765" t="inlineStr"/>
       <c r="AD765" t="inlineStr">
         <is>
-          <t>Aguardando o agendamento da implantação. - Data Comentário: 27/07/2026 12:36</t>
+          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09. - Data Comentário: 27/07/2026 16:25</t>
         </is>
       </c>
       <c r="AE765" t="inlineStr">
         <is>
-          <t>27/07/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="AF765" t="inlineStr">
@@ -84614,41 +84610,37 @@
         </is>
       </c>
       <c r="G766" t="n">
-        <v>11613</v>
+        <v>9791</v>
       </c>
       <c r="H766" t="n">
         <v>0</v>
       </c>
       <c r="I766" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J766" t="inlineStr">
         <is>
-          <t>Envio de ATA de Implantação - CTB V - GOIAS</t>
+          <t>Aplicação de Modelo - Pendente - GOIAS</t>
         </is>
       </c>
       <c r="K766" t="inlineStr"/>
       <c r="L766" s="1" t="n">
-        <v>46230</v>
-      </c>
-      <c r="M766" t="inlineStr">
-        <is>
-          <t>07/08/2026</t>
-        </is>
-      </c>
+        <v>46206</v>
+      </c>
+      <c r="M766" t="inlineStr"/>
       <c r="N766" t="inlineStr">
         <is>
           <t>06/2026</t>
         </is>
       </c>
       <c r="O766" t="n">
-        <v>18189088</v>
+        <v>18189076</v>
       </c>
       <c r="P766" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Mauricio Lermen</t>
         </is>
       </c>
       <c r="Q766" t="inlineStr">
@@ -84658,7 +84650,7 @@
       </c>
       <c r="R766" t="inlineStr"/>
       <c r="S766" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="T766" t="inlineStr">
         <is>
@@ -84672,8 +84664,8 @@
       </c>
       <c r="V766" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 07/08/2026 
-As reuniões de implantação estão agendadas para agosto - Data Comentário: 27/07/2026 16:43</t>
+          <t>Sem informações para a realização da tarefa  
+Não recebemos as informações e documentos do cliente. Conforme consulta hoje, não temos sequer a procuração até o momento. Previsão de conclusão, 02 dias úteis após recebimento. - Data Comentário: 27/07/2026 18:16</t>
         </is>
       </c>
       <c r="W766" t="inlineStr"/>
@@ -84685,12 +84677,12 @@
       <c r="AC766" t="inlineStr"/>
       <c r="AD766" t="inlineStr">
         <is>
-          <t>Aguardando o agendamento da implantação. - Data Comentário: 27/07/2026 12:36</t>
+          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09. - Data Comentário: 27/07/2026 16:25</t>
         </is>
       </c>
       <c r="AE766" t="inlineStr">
         <is>
-          <t>27/07/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="AF766" t="inlineStr">
@@ -84702,11 +84694,11 @@
     </row>
     <row r="767">
       <c r="A767" t="n">
-        <v>6981</v>
+        <v>6627</v>
       </c>
       <c r="B767" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUIZ GOMES DA SILVA - O GOIANO </t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C767" t="inlineStr">
@@ -84721,50 +84713,50 @@
       </c>
       <c r="E767" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F767" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G767" t="n">
-        <v>11613</v>
+        <v>7026</v>
       </c>
       <c r="H767" t="n">
         <v>0</v>
       </c>
       <c r="I767" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J767" t="inlineStr">
         <is>
-          <t>Envio de ATA de Implantação - CTB V - SP</t>
+          <t>Movimento - Sistema de Análise</t>
         </is>
       </c>
       <c r="K767" t="inlineStr"/>
       <c r="L767" s="1" t="n">
-        <v>46230</v>
+        <v>46167</v>
       </c>
       <c r="M767" t="inlineStr">
         <is>
-          <t>17/07/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="N767" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="O767" t="n">
-        <v>18195072</v>
+        <v>18048469</v>
       </c>
       <c r="P767" t="inlineStr">
         <is>
-          <t>Tatiana Linardi</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="Q767" t="inlineStr">
@@ -84774,18 +84766,22 @@
       </c>
       <c r="R767" t="inlineStr"/>
       <c r="S767" t="n">
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="T767" t="inlineStr">
         <is>
-          <t>SUPERMERCADO AVENIDA</t>
-        </is>
-      </c>
-      <c r="U767" t="inlineStr"/>
+          <t xml:space="preserve">GTG </t>
+        </is>
+      </c>
+      <c r="U767" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
       <c r="V767" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 17/07/2026 
-implantação não foi marcada ainda. - Data Comentário: 10/07/2026 17:02</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
+validando com o GC - Data Comentário: 27/07/2026 18:38</t>
         </is>
       </c>
       <c r="W767" t="inlineStr"/>
@@ -84797,7 +84793,7 @@
       <c r="AC767" t="inlineStr"/>
       <c r="AD767" t="inlineStr">
         <is>
-          <t>Aguardando o agendamento da implantação. - Data Comentário: 27/07/2026 12:36</t>
+          <t>A gerente Priscila Volpe, a GC Beatriz e o Afonso estão trabalhando em maneiras para ajustar os valores de saldo credor de meses anteriores, por conta de conflito no sys analise. - Data Comentário: 27/07/2026 16:25</t>
         </is>
       </c>
       <c r="AE767" t="inlineStr">
@@ -84810,15 +84806,19 @@
           <t>Tarefa</t>
         </is>
       </c>
-      <c r="AG767" t="inlineStr"/>
+      <c r="AG767" t="inlineStr">
+        <is>
+          <t>Nayara Oliveira</t>
+        </is>
+      </c>
     </row>
     <row r="768">
       <c r="A768" t="n">
-        <v>6966</v>
+        <v>6224</v>
       </c>
       <c r="B768" t="inlineStr">
         <is>
-          <t>HELBRAZ COMERCIO DE PAPELARIA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C768" t="inlineStr">
@@ -84828,7 +84828,7 @@
       </c>
       <c r="D768" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E768" t="inlineStr">
@@ -84838,41 +84838,41 @@
       </c>
       <c r="F768" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G768" t="n">
-        <v>9791</v>
+        <v>1802</v>
       </c>
       <c r="H768" t="n">
         <v>0</v>
       </c>
       <c r="I768" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J768" t="inlineStr">
         <is>
-          <t>Aplicação de Modelo - Pendente - GOIAS</t>
+          <t>Est - ICMS RPA - CÓD. 046-2</t>
         </is>
       </c>
       <c r="K768" t="inlineStr"/>
       <c r="L768" s="1" t="n">
-        <v>46206</v>
+        <v>46182</v>
       </c>
       <c r="M768" t="inlineStr"/>
       <c r="N768" t="inlineStr">
         <is>
-          <t>06/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="O768" t="n">
-        <v>18189077</v>
+        <v>17688680</v>
       </c>
       <c r="P768" t="inlineStr">
         <is>
-          <t>Mauricio Lermen</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="Q768" t="inlineStr">
@@ -84882,22 +84882,21 @@
       </c>
       <c r="R768" t="inlineStr"/>
       <c r="S768" t="n">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="T768" t="inlineStr">
         <is>
-          <t>HELBRAZ</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U768" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="V768" t="inlineStr">
         <is>
-          <t>Sem informações para a realização da tarefa  
-Não recebemos as informações e documentos do cliente. Conforme consulta hoje, não temos sequer a procuração até o momento. Previsão de conclusão, 02 dias úteis após recebimento. - Data Comentário: 27/07/2026 18:16</t>
+          <t>Atraso do Cliente, cobrança ativa, GC e GM ciente do atraso - Data Comentário: 25/06/2026 16:00</t>
         </is>
       </c>
       <c r="W768" t="inlineStr"/>
@@ -84909,7 +84908,7 @@
       <c r="AC768" t="inlineStr"/>
       <c r="AD768" t="inlineStr">
         <is>
-          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09. - Data Comentário: 27/07/2026 16:25</t>
+          <t>Atraso do cliente, o atraso do cliente já é recorrente e de ciência do Master e do Gerente de Contas. - Data Comentário: 27/07/2026 12:36</t>
         </is>
       </c>
       <c r="AE768" t="inlineStr">
@@ -84919,18 +84918,22 @@
       </c>
       <c r="AF768" t="inlineStr">
         <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AG768" t="inlineStr"/>
+          <t>Imposto</t>
+        </is>
+      </c>
+      <c r="AG768" t="inlineStr">
+        <is>
+          <t>Ricardo Fischer</t>
+        </is>
+      </c>
     </row>
     <row r="769">
       <c r="A769" t="n">
-        <v>6967</v>
+        <v>6224</v>
       </c>
       <c r="B769" t="inlineStr">
         <is>
-          <t>JL DISTRIBUIDORA DE PAPELARIA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C769" t="inlineStr">
@@ -84940,7 +84943,7 @@
       </c>
       <c r="D769" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E769" t="inlineStr">
@@ -84950,41 +84953,41 @@
       </c>
       <c r="F769" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G769" t="n">
-        <v>9791</v>
+        <v>1808</v>
       </c>
       <c r="H769" t="n">
         <v>0</v>
       </c>
       <c r="I769" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J769" t="inlineStr">
         <is>
-          <t>Aplicação de Modelo - Pendente - GOIAS</t>
+          <t>Fed - PIS/COFINS Não Cumul/Mon - 5856</t>
         </is>
       </c>
       <c r="K769" t="inlineStr"/>
       <c r="L769" s="1" t="n">
-        <v>46206</v>
+        <v>46195</v>
       </c>
       <c r="M769" t="inlineStr"/>
       <c r="N769" t="inlineStr">
         <is>
-          <t>06/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="O769" t="n">
-        <v>18189076</v>
+        <v>17688690</v>
       </c>
       <c r="P769" t="inlineStr">
         <is>
-          <t>Mauricio Lermen</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="Q769" t="inlineStr">
@@ -84994,22 +84997,21 @@
       </c>
       <c r="R769" t="inlineStr"/>
       <c r="S769" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="T769" t="inlineStr">
         <is>
-          <t>HELBRAZ</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U769" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="V769" t="inlineStr">
         <is>
-          <t>Sem informações para a realização da tarefa  
-Não recebemos as informações e documentos do cliente. Conforme consulta hoje, não temos sequer a procuração até o momento. Previsão de conclusão, 02 dias úteis após recebimento. - Data Comentário: 27/07/2026 18:16</t>
+          <t>Atraso de envio do cliente, consultar pendências no check list - Data Comentário: 23/06/2026 15:41</t>
         </is>
       </c>
       <c r="W769" t="inlineStr"/>
@@ -85021,7 +85023,7 @@
       <c r="AC769" t="inlineStr"/>
       <c r="AD769" t="inlineStr">
         <is>
-          <t>Aguardando implantação do cliente para que seja possível a realização da tarefa - AI09. - Data Comentário: 27/07/2026 16:25</t>
+          <t>Atraso do cliente, o atraso do cliente já é recorrente e de ciência do Master e do Gerente de Contas. - Data Comentário: 27/07/2026 12:36</t>
         </is>
       </c>
       <c r="AE769" t="inlineStr">
@@ -85031,713 +85033,12 @@
       </c>
       <c r="AF769" t="inlineStr">
         <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AG769" t="inlineStr"/>
-    </row>
-    <row r="770">
-      <c r="A770" t="n">
-        <v>6627</v>
-      </c>
-      <c r="B770" t="inlineStr">
-        <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
-        </is>
-      </c>
-      <c r="C770" t="inlineStr">
-        <is>
-          <t>GOIAS</t>
-        </is>
-      </c>
-      <c r="D770" t="inlineStr">
-        <is>
-          <t>Federal - L Real -Trimestral</t>
-        </is>
-      </c>
-      <c r="E770" t="inlineStr">
-        <is>
-          <t>Vander Silva</t>
-        </is>
-      </c>
-      <c r="F770" t="inlineStr">
-        <is>
-          <t>Edimir Santos</t>
-        </is>
-      </c>
-      <c r="G770" t="n">
-        <v>7026</v>
-      </c>
-      <c r="H770" t="n">
-        <v>0</v>
-      </c>
-      <c r="I770" t="inlineStr">
-        <is>
-          <t>EF - INDUSTRIA</t>
-        </is>
-      </c>
-      <c r="J770" t="inlineStr">
-        <is>
-          <t>Movimento - Sistema de Análise</t>
-        </is>
-      </c>
-      <c r="K770" t="inlineStr"/>
-      <c r="L770" s="1" t="n">
-        <v>46167</v>
-      </c>
-      <c r="M770" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="N770" t="inlineStr">
-        <is>
-          <t>04/2026</t>
-        </is>
-      </c>
-      <c r="O770" t="n">
-        <v>18048469</v>
-      </c>
-      <c r="P770" t="inlineStr">
-        <is>
-          <t>Denis Reis</t>
-        </is>
-      </c>
-      <c r="Q770" t="inlineStr">
-        <is>
-          <t>Em Atraso</t>
-        </is>
-      </c>
-      <c r="R770" t="inlineStr"/>
-      <c r="S770" t="n">
-        <v>64</v>
-      </c>
-      <c r="T770" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GTG </t>
-        </is>
-      </c>
-      <c r="U770" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="V770" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
-validando com o GC - Data Comentário: 27/07/2026 18:38</t>
-        </is>
-      </c>
-      <c r="W770" t="inlineStr"/>
-      <c r="X770" t="inlineStr"/>
-      <c r="Y770" t="inlineStr"/>
-      <c r="Z770" t="inlineStr"/>
-      <c r="AA770" t="inlineStr"/>
-      <c r="AB770" t="inlineStr"/>
-      <c r="AC770" t="inlineStr"/>
-      <c r="AD770" t="inlineStr">
-        <is>
-          <t>A gerente Priscila Volpe, a GC Beatriz e o Afonso estão trabalhando em maneiras para ajustar os valores de saldo credor de meses anteriores, por conta de conflito no sys analise. - Data Comentário: 27/07/2026 16:25</t>
-        </is>
-      </c>
-      <c r="AE770" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="AF770" t="inlineStr">
-        <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AG770" t="inlineStr">
-        <is>
-          <t>Nayara Oliveira</t>
-        </is>
-      </c>
-    </row>
-    <row r="771">
-      <c r="A771" t="n">
-        <v>6224</v>
-      </c>
-      <c r="B771" t="inlineStr">
-        <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
-        </is>
-      </c>
-      <c r="C771" t="inlineStr">
-        <is>
-          <t>GOIAS</t>
-        </is>
-      </c>
-      <c r="D771" t="inlineStr">
-        <is>
-          <t>Federal - L Real -Trimestral</t>
-        </is>
-      </c>
-      <c r="E771" t="inlineStr">
-        <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="F771" t="inlineStr">
-        <is>
-          <t>Sem Master</t>
-        </is>
-      </c>
-      <c r="G771" t="n">
-        <v>1802</v>
-      </c>
-      <c r="H771" t="n">
-        <v>0</v>
-      </c>
-      <c r="I771" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="J771" t="inlineStr">
-        <is>
-          <t>Est - ICMS RPA - CÓD. 046-2</t>
-        </is>
-      </c>
-      <c r="K771" t="inlineStr"/>
-      <c r="L771" s="1" t="n">
-        <v>46182</v>
-      </c>
-      <c r="M771" t="inlineStr"/>
-      <c r="N771" t="inlineStr">
-        <is>
-          <t>05/2026</t>
-        </is>
-      </c>
-      <c r="O771" t="n">
-        <v>17688680</v>
-      </c>
-      <c r="P771" t="inlineStr">
-        <is>
-          <t>Cristina Leite</t>
-        </is>
-      </c>
-      <c r="Q771" t="inlineStr">
-        <is>
-          <t>Em Atraso</t>
-        </is>
-      </c>
-      <c r="R771" t="inlineStr"/>
-      <c r="S771" t="n">
-        <v>49</v>
-      </c>
-      <c r="T771" t="inlineStr">
-        <is>
-          <t>SUPER MAIS DO GOIÁS</t>
-        </is>
-      </c>
-      <c r="U771" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="V771" t="inlineStr">
-        <is>
-          <t>Atraso do Cliente, cobrança ativa, GC e GM ciente do atraso - Data Comentário: 25/06/2026 16:00</t>
-        </is>
-      </c>
-      <c r="W771" t="inlineStr"/>
-      <c r="X771" t="inlineStr"/>
-      <c r="Y771" t="inlineStr"/>
-      <c r="Z771" t="inlineStr"/>
-      <c r="AA771" t="inlineStr"/>
-      <c r="AB771" t="inlineStr"/>
-      <c r="AC771" t="inlineStr"/>
-      <c r="AD771" t="inlineStr">
-        <is>
-          <t>Atraso do cliente, o atraso do cliente já é recorrente e de ciência do Master e do Gerente de Contas. - Data Comentário: 27/07/2026 12:36</t>
-        </is>
-      </c>
-      <c r="AE771" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="AF771" t="inlineStr">
-        <is>
           <t>Imposto</t>
         </is>
       </c>
-      <c r="AG771" t="inlineStr">
+      <c r="AG769" t="inlineStr">
         <is>
           <t>Ricardo Fischer</t>
-        </is>
-      </c>
-    </row>
-    <row r="772">
-      <c r="A772" t="n">
-        <v>6224</v>
-      </c>
-      <c r="B772" t="inlineStr">
-        <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
-        </is>
-      </c>
-      <c r="C772" t="inlineStr">
-        <is>
-          <t>GOIAS</t>
-        </is>
-      </c>
-      <c r="D772" t="inlineStr">
-        <is>
-          <t>Federal - L Real -Trimestral</t>
-        </is>
-      </c>
-      <c r="E772" t="inlineStr">
-        <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="F772" t="inlineStr">
-        <is>
-          <t>Sem Master</t>
-        </is>
-      </c>
-      <c r="G772" t="n">
-        <v>1808</v>
-      </c>
-      <c r="H772" t="n">
-        <v>0</v>
-      </c>
-      <c r="I772" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="J772" t="inlineStr">
-        <is>
-          <t>Fed - PIS/COFINS Não Cumul/Mon - 5856</t>
-        </is>
-      </c>
-      <c r="K772" t="inlineStr"/>
-      <c r="L772" s="1" t="n">
-        <v>46195</v>
-      </c>
-      <c r="M772" t="inlineStr"/>
-      <c r="N772" t="inlineStr">
-        <is>
-          <t>05/2026</t>
-        </is>
-      </c>
-      <c r="O772" t="n">
-        <v>17688690</v>
-      </c>
-      <c r="P772" t="inlineStr">
-        <is>
-          <t>Cristina Leite</t>
-        </is>
-      </c>
-      <c r="Q772" t="inlineStr">
-        <is>
-          <t>Em Atraso</t>
-        </is>
-      </c>
-      <c r="R772" t="inlineStr"/>
-      <c r="S772" t="n">
-        <v>36</v>
-      </c>
-      <c r="T772" t="inlineStr">
-        <is>
-          <t>SUPER MAIS DO GOIÁS</t>
-        </is>
-      </c>
-      <c r="U772" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="V772" t="inlineStr">
-        <is>
-          <t>Atraso de envio do cliente, consultar pendências no check list - Data Comentário: 23/06/2026 15:41</t>
-        </is>
-      </c>
-      <c r="W772" t="inlineStr"/>
-      <c r="X772" t="inlineStr"/>
-      <c r="Y772" t="inlineStr"/>
-      <c r="Z772" t="inlineStr"/>
-      <c r="AA772" t="inlineStr"/>
-      <c r="AB772" t="inlineStr"/>
-      <c r="AC772" t="inlineStr"/>
-      <c r="AD772" t="inlineStr">
-        <is>
-          <t>Atraso do cliente, o atraso do cliente já é recorrente e de ciência do Master e do Gerente de Contas. - Data Comentário: 27/07/2026 12:36</t>
-        </is>
-      </c>
-      <c r="AE772" t="inlineStr">
-        <is>
-          <t>31/07/2026</t>
-        </is>
-      </c>
-      <c r="AF772" t="inlineStr">
-        <is>
-          <t>Imposto</t>
-        </is>
-      </c>
-      <c r="AG772" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
-    </row>
-    <row r="773">
-      <c r="A773" t="n">
-        <v>6966</v>
-      </c>
-      <c r="B773" t="inlineStr">
-        <is>
-          <t>HELBRAZ COMERCIO DE PAPELARIA LTDA</t>
-        </is>
-      </c>
-      <c r="C773" t="inlineStr">
-        <is>
-          <t>GOIAS</t>
-        </is>
-      </c>
-      <c r="D773" t="inlineStr">
-        <is>
-          <t>Federal - SN</t>
-        </is>
-      </c>
-      <c r="E773" t="inlineStr">
-        <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="F773" t="inlineStr">
-        <is>
-          <t>Reynaldo Santos</t>
-        </is>
-      </c>
-      <c r="G773" t="n">
-        <v>11618</v>
-      </c>
-      <c r="H773" t="n">
-        <v>0</v>
-      </c>
-      <c r="I773" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="J773" t="inlineStr">
-        <is>
-          <t>Envio de ATA de Implantação - EF V - GOIAS</t>
-        </is>
-      </c>
-      <c r="K773" t="inlineStr"/>
-      <c r="L773" s="1" t="n">
-        <v>46230</v>
-      </c>
-      <c r="M773" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="N773" t="inlineStr">
-        <is>
-          <t>06/2026</t>
-        </is>
-      </c>
-      <c r="O773" t="n">
-        <v>18189093</v>
-      </c>
-      <c r="P773" t="inlineStr">
-        <is>
-          <t>Claudineia Rodrigues</t>
-        </is>
-      </c>
-      <c r="Q773" t="inlineStr">
-        <is>
-          <t>Em Atraso</t>
-        </is>
-      </c>
-      <c r="R773" t="inlineStr"/>
-      <c r="S773" t="n">
-        <v>1</v>
-      </c>
-      <c r="T773" t="inlineStr">
-        <is>
-          <t>HELBRAZ</t>
-        </is>
-      </c>
-      <c r="U773" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="V773" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 27/07/2026 
-Reunião de implantação ainda não agendada. - Data Comentário: 23/07/2026 18:48</t>
-        </is>
-      </c>
-      <c r="W773" t="inlineStr"/>
-      <c r="X773" t="inlineStr"/>
-      <c r="Y773" t="inlineStr"/>
-      <c r="Z773" t="inlineStr"/>
-      <c r="AA773" t="inlineStr"/>
-      <c r="AB773" t="inlineStr"/>
-      <c r="AC773" t="inlineStr"/>
-      <c r="AD773" t="inlineStr">
-        <is>
-          <t>Aguardando agendamento da implantação do cliente. - Data Comentário: 27/07/2026 16:26</t>
-        </is>
-      </c>
-      <c r="AE773" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="AF773" t="inlineStr">
-        <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AG773" t="inlineStr">
-        <is>
-          <t>Claudineia Rodrigues</t>
-        </is>
-      </c>
-    </row>
-    <row r="774">
-      <c r="A774" t="n">
-        <v>6967</v>
-      </c>
-      <c r="B774" t="inlineStr">
-        <is>
-          <t>JL DISTRIBUIDORA DE PAPELARIA LTDA</t>
-        </is>
-      </c>
-      <c r="C774" t="inlineStr">
-        <is>
-          <t>GOIAS</t>
-        </is>
-      </c>
-      <c r="D774" t="inlineStr">
-        <is>
-          <t>Federal - SN</t>
-        </is>
-      </c>
-      <c r="E774" t="inlineStr">
-        <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="F774" t="inlineStr">
-        <is>
-          <t>Reynaldo Santos</t>
-        </is>
-      </c>
-      <c r="G774" t="n">
-        <v>11618</v>
-      </c>
-      <c r="H774" t="n">
-        <v>0</v>
-      </c>
-      <c r="I774" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="J774" t="inlineStr">
-        <is>
-          <t>Envio de ATA de Implantação - EF V - GOIAS</t>
-        </is>
-      </c>
-      <c r="K774" t="inlineStr"/>
-      <c r="L774" s="1" t="n">
-        <v>46230</v>
-      </c>
-      <c r="M774" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="N774" t="inlineStr">
-        <is>
-          <t>06/2026</t>
-        </is>
-      </c>
-      <c r="O774" t="n">
-        <v>18189092</v>
-      </c>
-      <c r="P774" t="inlineStr">
-        <is>
-          <t>Claudineia Rodrigues</t>
-        </is>
-      </c>
-      <c r="Q774" t="inlineStr">
-        <is>
-          <t>Em Atraso</t>
-        </is>
-      </c>
-      <c r="R774" t="inlineStr"/>
-      <c r="S774" t="n">
-        <v>1</v>
-      </c>
-      <c r="T774" t="inlineStr">
-        <is>
-          <t>HELBRAZ</t>
-        </is>
-      </c>
-      <c r="U774" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="V774" t="inlineStr">
-        <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 27/07/2026 
-Reunião de implantação ainda não agendada. - Data Comentário: 23/07/2026 18:48</t>
-        </is>
-      </c>
-      <c r="W774" t="inlineStr"/>
-      <c r="X774" t="inlineStr"/>
-      <c r="Y774" t="inlineStr"/>
-      <c r="Z774" t="inlineStr"/>
-      <c r="AA774" t="inlineStr"/>
-      <c r="AB774" t="inlineStr"/>
-      <c r="AC774" t="inlineStr"/>
-      <c r="AD774" t="inlineStr">
-        <is>
-          <t>Aguardando agendamento da implantação do cliente. - Data Comentário: 27/07/2026 16:26</t>
-        </is>
-      </c>
-      <c r="AE774" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="AF774" t="inlineStr">
-        <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AG774" t="inlineStr">
-        <is>
-          <t>Claudineia Rodrigues</t>
-        </is>
-      </c>
-    </row>
-    <row r="775">
-      <c r="A775" t="n">
-        <v>6981</v>
-      </c>
-      <c r="B775" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUIZ GOMES DA SILVA - O GOIANO </t>
-        </is>
-      </c>
-      <c r="C775" t="inlineStr">
-        <is>
-          <t>GOIAS</t>
-        </is>
-      </c>
-      <c r="D775" t="inlineStr">
-        <is>
-          <t>Federal - L Real -Trimestral</t>
-        </is>
-      </c>
-      <c r="E775" t="inlineStr">
-        <is>
-          <t>Ricardo Ferreira</t>
-        </is>
-      </c>
-      <c r="F775" t="inlineStr">
-        <is>
-          <t>Reynaldo Santos</t>
-        </is>
-      </c>
-      <c r="G775" t="n">
-        <v>11618</v>
-      </c>
-      <c r="H775" t="n">
-        <v>0</v>
-      </c>
-      <c r="I775" t="inlineStr">
-        <is>
-          <t>EF - VAREJO</t>
-        </is>
-      </c>
-      <c r="J775" t="inlineStr">
-        <is>
-          <t>Envio de ATA de Implantação - EF V - SP</t>
-        </is>
-      </c>
-      <c r="K775" t="inlineStr"/>
-      <c r="L775" s="1" t="n">
-        <v>46230</v>
-      </c>
-      <c r="M775" t="inlineStr">
-        <is>
-          <t>17/07/2026</t>
-        </is>
-      </c>
-      <c r="N775" t="inlineStr">
-        <is>
-          <t>07/2026</t>
-        </is>
-      </c>
-      <c r="O775" t="n">
-        <v>18195073</v>
-      </c>
-      <c r="P775" t="inlineStr">
-        <is>
-          <t>Claudineia Rodrigues</t>
-        </is>
-      </c>
-      <c r="Q775" t="inlineStr">
-        <is>
-          <t>Em Atraso</t>
-        </is>
-      </c>
-      <c r="R775" t="inlineStr"/>
-      <c r="S775" t="n">
-        <v>1</v>
-      </c>
-      <c r="T775" t="inlineStr">
-        <is>
-          <t>SUPERMERCADO AVENIDA</t>
-        </is>
-      </c>
-      <c r="U775" t="inlineStr"/>
-      <c r="V775" t="inlineStr">
-        <is>
-          <t>Reunião de implantação ainda não agendada. - Data Comentário: 13/07/2026 08:26</t>
-        </is>
-      </c>
-      <c r="W775" t="inlineStr"/>
-      <c r="X775" t="inlineStr"/>
-      <c r="Y775" t="inlineStr"/>
-      <c r="Z775" t="inlineStr"/>
-      <c r="AA775" t="inlineStr"/>
-      <c r="AB775" t="inlineStr"/>
-      <c r="AC775" t="inlineStr"/>
-      <c r="AD775" t="inlineStr">
-        <is>
-          <t>Aguardando agendamento da implantação do cliente. - Data Comentário: 27/07/2026 16:26</t>
-        </is>
-      </c>
-      <c r="AE775" t="inlineStr">
-        <is>
-          <t>27/07/2026</t>
-        </is>
-      </c>
-      <c r="AF775" t="inlineStr">
-        <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AG775" t="inlineStr">
-        <is>
-          <t>Claudineia Rodrigues</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-28 12:49
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG769"/>
+  <dimension ref="A1:AG775"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -85042,6 +85042,608 @@
         </is>
       </c>
     </row>
+    <row r="770">
+      <c r="A770" t="n">
+        <v>6992</v>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>ALDENIR VENANCIO DE OLIVEIRA LTDA</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>GOIAS</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>Federal - L Real -Trimestral</t>
+        </is>
+      </c>
+      <c r="E770" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="F770" t="inlineStr">
+        <is>
+          <t>Reynaldo Santos</t>
+        </is>
+      </c>
+      <c r="G770" t="n">
+        <v>11613</v>
+      </c>
+      <c r="H770" t="n">
+        <v>0</v>
+      </c>
+      <c r="I770" t="inlineStr">
+        <is>
+          <t>CTB - CONTÁBIL VAREJO</t>
+        </is>
+      </c>
+      <c r="J770" t="inlineStr">
+        <is>
+          <t>Envio de ATA de Implantação - CTB V - GOIAS</t>
+        </is>
+      </c>
+      <c r="K770" t="inlineStr"/>
+      <c r="L770" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="M770" t="inlineStr"/>
+      <c r="N770" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
+      <c r="O770" t="n">
+        <v>18210693</v>
+      </c>
+      <c r="P770" t="inlineStr">
+        <is>
+          <t>Tatiana Linardi</t>
+        </is>
+      </c>
+      <c r="Q770" t="inlineStr">
+        <is>
+          <t>Em Aberto</t>
+        </is>
+      </c>
+      <c r="R770" t="inlineStr"/>
+      <c r="S770" t="n">
+        <v>0</v>
+      </c>
+      <c r="T770" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO CRISTO REI</t>
+        </is>
+      </c>
+      <c r="U770" t="inlineStr"/>
+      <c r="V770" t="inlineStr">
+        <is>
+          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6992; Tarefa Incluida: 11613; Vencimento: 28/07/2026 00:00:00; UsuarioResponsavel: tatiana - Data Comentário: 28/07/2026 12:02</t>
+        </is>
+      </c>
+      <c r="W770" t="inlineStr"/>
+      <c r="X770" t="inlineStr"/>
+      <c r="Y770" t="inlineStr"/>
+      <c r="Z770" t="inlineStr"/>
+      <c r="AA770" t="inlineStr"/>
+      <c r="AB770" t="inlineStr"/>
+      <c r="AC770" t="inlineStr"/>
+      <c r="AD770" t="inlineStr"/>
+      <c r="AE770" t="inlineStr"/>
+      <c r="AF770" t="inlineStr">
+        <is>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AG770" t="inlineStr"/>
+    </row>
+    <row r="771">
+      <c r="A771" t="n">
+        <v>6993</v>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>GOMES SERVIÇOS - LTDA</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>GOIAS</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>Federal - SN</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="F771" t="inlineStr">
+        <is>
+          <t>Reynaldo Santos</t>
+        </is>
+      </c>
+      <c r="G771" t="n">
+        <v>11613</v>
+      </c>
+      <c r="H771" t="n">
+        <v>0</v>
+      </c>
+      <c r="I771" t="inlineStr">
+        <is>
+          <t>CTB - CONTÁBIL VAREJO</t>
+        </is>
+      </c>
+      <c r="J771" t="inlineStr">
+        <is>
+          <t>Envio de ATA de Implantação - CTB V - GOIAS</t>
+        </is>
+      </c>
+      <c r="K771" t="inlineStr"/>
+      <c r="L771" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="M771" t="inlineStr"/>
+      <c r="N771" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
+      <c r="O771" t="n">
+        <v>18210694</v>
+      </c>
+      <c r="P771" t="inlineStr">
+        <is>
+          <t>Tatiana Linardi</t>
+        </is>
+      </c>
+      <c r="Q771" t="inlineStr">
+        <is>
+          <t>Em Aberto</t>
+        </is>
+      </c>
+      <c r="R771" t="inlineStr"/>
+      <c r="S771" t="n">
+        <v>0</v>
+      </c>
+      <c r="T771" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO CRISTO REI</t>
+        </is>
+      </c>
+      <c r="U771" t="inlineStr"/>
+      <c r="V771" t="inlineStr">
+        <is>
+          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6993; Tarefa Incluida: 11613; Vencimento: 28/07/2026 00:00:00; UsuarioResponsavel: tatiana - Data Comentário: 28/07/2026 12:02</t>
+        </is>
+      </c>
+      <c r="W771" t="inlineStr"/>
+      <c r="X771" t="inlineStr"/>
+      <c r="Y771" t="inlineStr"/>
+      <c r="Z771" t="inlineStr"/>
+      <c r="AA771" t="inlineStr"/>
+      <c r="AB771" t="inlineStr"/>
+      <c r="AC771" t="inlineStr"/>
+      <c r="AD771" t="inlineStr"/>
+      <c r="AE771" t="inlineStr"/>
+      <c r="AF771" t="inlineStr">
+        <is>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AG771" t="inlineStr"/>
+    </row>
+    <row r="772">
+      <c r="A772" t="n">
+        <v>6992</v>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>ALDENIR VENANCIO DE OLIVEIRA LTDA</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>GOIAS</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>Federal - L Real -Trimestral</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="F772" t="inlineStr">
+        <is>
+          <t>Reynaldo Santos</t>
+        </is>
+      </c>
+      <c r="G772" t="n">
+        <v>11616</v>
+      </c>
+      <c r="H772" t="n">
+        <v>0</v>
+      </c>
+      <c r="I772" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="J772" t="inlineStr">
+        <is>
+          <t>Envio de ATA de Implantação - DP - GOIAS</t>
+        </is>
+      </c>
+      <c r="K772" t="inlineStr"/>
+      <c r="L772" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="M772" t="inlineStr"/>
+      <c r="N772" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
+      <c r="O772" t="n">
+        <v>18210691</v>
+      </c>
+      <c r="P772" t="inlineStr">
+        <is>
+          <t>Mauricio Lermen</t>
+        </is>
+      </c>
+      <c r="Q772" t="inlineStr">
+        <is>
+          <t>Em Aberto</t>
+        </is>
+      </c>
+      <c r="R772" t="inlineStr"/>
+      <c r="S772" t="n">
+        <v>0</v>
+      </c>
+      <c r="T772" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO CRISTO REI</t>
+        </is>
+      </c>
+      <c r="U772" t="inlineStr"/>
+      <c r="V772" t="inlineStr">
+        <is>
+          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6992; Tarefa Incluida: 11616; Vencimento: 28/07/2026 00:00:00; UsuarioResponsavel: mauricio - Data Comentário: 28/07/2026 12:02</t>
+        </is>
+      </c>
+      <c r="W772" t="inlineStr"/>
+      <c r="X772" t="inlineStr"/>
+      <c r="Y772" t="inlineStr"/>
+      <c r="Z772" t="inlineStr"/>
+      <c r="AA772" t="inlineStr"/>
+      <c r="AB772" t="inlineStr"/>
+      <c r="AC772" t="inlineStr"/>
+      <c r="AD772" t="inlineStr"/>
+      <c r="AE772" t="inlineStr"/>
+      <c r="AF772" t="inlineStr">
+        <is>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AG772" t="inlineStr"/>
+    </row>
+    <row r="773">
+      <c r="A773" t="n">
+        <v>6993</v>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>GOMES SERVIÇOS - LTDA</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>GOIAS</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>Federal - SN</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="F773" t="inlineStr">
+        <is>
+          <t>Reynaldo Santos</t>
+        </is>
+      </c>
+      <c r="G773" t="n">
+        <v>11616</v>
+      </c>
+      <c r="H773" t="n">
+        <v>0</v>
+      </c>
+      <c r="I773" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="J773" t="inlineStr">
+        <is>
+          <t>Envio de ATA de Implantação - DP - GOIAS</t>
+        </is>
+      </c>
+      <c r="K773" t="inlineStr"/>
+      <c r="L773" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="M773" t="inlineStr"/>
+      <c r="N773" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
+      <c r="O773" t="n">
+        <v>18210692</v>
+      </c>
+      <c r="P773" t="inlineStr">
+        <is>
+          <t>Mauricio Lermen</t>
+        </is>
+      </c>
+      <c r="Q773" t="inlineStr">
+        <is>
+          <t>Em Aberto</t>
+        </is>
+      </c>
+      <c r="R773" t="inlineStr"/>
+      <c r="S773" t="n">
+        <v>0</v>
+      </c>
+      <c r="T773" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO CRISTO REI</t>
+        </is>
+      </c>
+      <c r="U773" t="inlineStr"/>
+      <c r="V773" t="inlineStr">
+        <is>
+          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6993; Tarefa Incluida: 11616; Vencimento: 28/07/2026 00:00:00; UsuarioResponsavel: mauricio - Data Comentário: 28/07/2026 12:02</t>
+        </is>
+      </c>
+      <c r="W773" t="inlineStr"/>
+      <c r="X773" t="inlineStr"/>
+      <c r="Y773" t="inlineStr"/>
+      <c r="Z773" t="inlineStr"/>
+      <c r="AA773" t="inlineStr"/>
+      <c r="AB773" t="inlineStr"/>
+      <c r="AC773" t="inlineStr"/>
+      <c r="AD773" t="inlineStr"/>
+      <c r="AE773" t="inlineStr"/>
+      <c r="AF773" t="inlineStr">
+        <is>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AG773" t="inlineStr"/>
+    </row>
+    <row r="774">
+      <c r="A774" t="n">
+        <v>6992</v>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>ALDENIR VENANCIO DE OLIVEIRA LTDA</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>GOIAS</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>Federal - L Real -Trimestral</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="F774" t="inlineStr">
+        <is>
+          <t>Reynaldo Santos</t>
+        </is>
+      </c>
+      <c r="G774" t="n">
+        <v>11618</v>
+      </c>
+      <c r="H774" t="n">
+        <v>0</v>
+      </c>
+      <c r="I774" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="J774" t="inlineStr">
+        <is>
+          <t>Envio de ATA de Implantação - EF V - GOIAS</t>
+        </is>
+      </c>
+      <c r="K774" t="inlineStr"/>
+      <c r="L774" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="M774" t="inlineStr"/>
+      <c r="N774" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
+      <c r="O774" t="n">
+        <v>18210695</v>
+      </c>
+      <c r="P774" t="inlineStr">
+        <is>
+          <t>Claudineia Rodrigues</t>
+        </is>
+      </c>
+      <c r="Q774" t="inlineStr">
+        <is>
+          <t>Em Aberto</t>
+        </is>
+      </c>
+      <c r="R774" t="inlineStr"/>
+      <c r="S774" t="n">
+        <v>0</v>
+      </c>
+      <c r="T774" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO CRISTO REI</t>
+        </is>
+      </c>
+      <c r="U774" t="inlineStr"/>
+      <c r="V774" t="inlineStr">
+        <is>
+          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6992; Tarefa Incluida: 11618; Vencimento: 28/07/2026 00:00:00; UsuarioResponsavel: Claudineia - Data Comentário: 28/07/2026 12:02</t>
+        </is>
+      </c>
+      <c r="W774" t="inlineStr"/>
+      <c r="X774" t="inlineStr"/>
+      <c r="Y774" t="inlineStr"/>
+      <c r="Z774" t="inlineStr"/>
+      <c r="AA774" t="inlineStr"/>
+      <c r="AB774" t="inlineStr"/>
+      <c r="AC774" t="inlineStr"/>
+      <c r="AD774" t="inlineStr"/>
+      <c r="AE774" t="inlineStr"/>
+      <c r="AF774" t="inlineStr">
+        <is>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AG774" t="inlineStr">
+        <is>
+          <t>Claudineia Rodrigues</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="n">
+        <v>6993</v>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>GOMES SERVIÇOS - LTDA</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>GOIAS</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>Federal - SN</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="F775" t="inlineStr">
+        <is>
+          <t>Reynaldo Santos</t>
+        </is>
+      </c>
+      <c r="G775" t="n">
+        <v>11618</v>
+      </c>
+      <c r="H775" t="n">
+        <v>0</v>
+      </c>
+      <c r="I775" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="J775" t="inlineStr">
+        <is>
+          <t>Envio de ATA de Implantação - EF V - GOIAS</t>
+        </is>
+      </c>
+      <c r="K775" t="inlineStr"/>
+      <c r="L775" s="1" t="n">
+        <v>46231</v>
+      </c>
+      <c r="M775" t="inlineStr"/>
+      <c r="N775" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
+      <c r="O775" t="n">
+        <v>18210696</v>
+      </c>
+      <c r="P775" t="inlineStr">
+        <is>
+          <t>Claudineia Rodrigues</t>
+        </is>
+      </c>
+      <c r="Q775" t="inlineStr">
+        <is>
+          <t>Em Aberto</t>
+        </is>
+      </c>
+      <c r="R775" t="inlineStr"/>
+      <c r="S775" t="n">
+        <v>0</v>
+      </c>
+      <c r="T775" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO CRISTO REI</t>
+        </is>
+      </c>
+      <c r="U775" t="inlineStr"/>
+      <c r="V775" t="inlineStr">
+        <is>
+          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6993; Tarefa Incluida: 11618; Vencimento: 28/07/2026 00:00:00; UsuarioResponsavel: Claudineia - Data Comentário: 28/07/2026 12:02</t>
+        </is>
+      </c>
+      <c r="W775" t="inlineStr"/>
+      <c r="X775" t="inlineStr"/>
+      <c r="Y775" t="inlineStr"/>
+      <c r="Z775" t="inlineStr"/>
+      <c r="AA775" t="inlineStr"/>
+      <c r="AB775" t="inlineStr"/>
+      <c r="AC775" t="inlineStr"/>
+      <c r="AD775" t="inlineStr"/>
+      <c r="AE775" t="inlineStr"/>
+      <c r="AF775" t="inlineStr">
+        <is>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AG775" t="inlineStr">
+        <is>
+          <t>Claudineia Rodrigues</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização automática: 2026-07-28 17:54
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -85107,7 +85107,11 @@
       <c r="L770" s="1" t="n">
         <v>46231</v>
       </c>
-      <c r="M770" t="inlineStr"/>
+      <c r="M770" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
       <c r="N770" t="inlineStr">
         <is>
           <t>07/2026</t>
@@ -85138,7 +85142,8 @@
       <c r="U770" t="inlineStr"/>
       <c r="V770" t="inlineStr">
         <is>
-          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6992; Tarefa Incluida: 11613; Vencimento: 28/07/2026 00:00:00; UsuarioResponsavel: tatiana - Data Comentário: 28/07/2026 12:02</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 07/08/2026 
+vamos marcar a reunião de implantação em agosto - Data Comentário: 28/07/2026 17:29</t>
         </is>
       </c>
       <c r="W770" t="inlineStr"/>
@@ -85206,7 +85211,11 @@
       <c r="L771" s="1" t="n">
         <v>46231</v>
       </c>
-      <c r="M771" t="inlineStr"/>
+      <c r="M771" t="inlineStr">
+        <is>
+          <t>07/08/2026</t>
+        </is>
+      </c>
       <c r="N771" t="inlineStr">
         <is>
           <t>07/2026</t>
@@ -85237,7 +85246,8 @@
       <c r="U771" t="inlineStr"/>
       <c r="V771" t="inlineStr">
         <is>
-          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6993; Tarefa Incluida: 11613; Vencimento: 28/07/2026 00:00:00; UsuarioResponsavel: tatiana - Data Comentário: 28/07/2026 12:02</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 07/08/2026 
+vamos marcar a reunião de implantação em agosto - Data Comentário: 28/07/2026 17:29</t>
         </is>
       </c>
       <c r="W771" t="inlineStr"/>

</xml_diff>